<commit_message>
Implement dossier slice 10: chain guards on the entry leaves, the armchair form
- F0x_x_VESTIBULE-002 (eighteen homes): every apartment entry leaf carries
  a chain door guard on its apartment face, a brass slotted plate by the
  latch stile with the anchor plate and its unhooked chain beside it
  (orison_v2_domestic_doors.gd, passive, no owner); the signal-outlet half
  of those items landed with BW-013.
- F05_B_MAIN-001 and F01_A_MAIN-002: an Armchair variant in the seating
  family (the sofa recipe at 0.85 m, one cushion, rolled arms) with its own
  source record 5B_radio_chair facing the radio in 5B, and 1A's reading
  chair retemplated onto it and reseated facing the window, between the
  side table and the radiator stance and clear of the bedroom route.

Evidence under implementation/slice10/. INERT: no ledger status changes.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/art/reviews/v2_environment_design_20261008/change_register.xlsx
+++ b/art/reviews/v2_environment_design_20261008/change_register.xlsx
@@ -10327,10 +10327,14 @@
       </c>
       <c r="S149" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T149" s="2" t="inlineStr"/>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="T149" s="2" t="inlineStr">
+        <is>
+          <t>The brass signal-outlet plate beside the switch came with BW-013 (slice 6); the chain door guard is on the entry leaf's apartment face: slotted plate by the latch stile, anchor plate and unhooked chain beside it (slice 10). Verified at d38ba7ac (slice10, slice10b): the thirteen families pass the fabrication batch (24,276 checks, 0 failures; seating 51 actors with the two armchairs, 1A's captured natively), door casings and fitted door fabric 0 failures, door hinges 10 as before (the 105-door count and one leaf's knuckles, identical at 6d99760d, slice10c), both door-route suites unchanged (45 and 32 waypoints, 0 failures), completion route 1A 15 waypoints as before (the kitchen leg), apartment batch 236 as before, upper lighting 0 failures, the seven-space sweep 0 failures; the chain guards are shown at the vestibule thresholds and the armchairs in F05_B_MAIN and F01_A_MAIN (implementation/slice10).</t>
+        </is>
+      </c>
     </row>
     <row r="150">
       <c r="A150" s="2" t="inlineStr">
@@ -10578,7 +10582,7 @@
       </c>
       <c r="T152" s="2" t="inlineStr">
         <is>
-          <t>1A_reading_chair (ChairDark, angled 30 degrees to the window with its back to the kitchen door) and 1A_side_table (TableRect08) by the window; 1A_table and 1A_chair moved onto the long wall as the marking table. Deviations: the seating family has no armchair variant and the task-lamp family no floor stand, so the chair is the dark dining chair and the lamp is deferred with the family work. (implementation/slice6/images/F01_A_MAIN_OV.jpg)</t>
+          <t>1A_reading_chair (ChairDark, angled 30 degrees to the window with its back to the kitchen door) and 1A_side_table (TableRect08) by the window; 1A_table and 1A_chair moved onto the long wall as the marking table. Slice 10 replaced the dining chair with the Armchair form (template 5B_radio_chair) reseated at (-14.75, -5.4) facing the window, between the side table and the radiator stance; the floor lamp still waits for the task-lamp family. (implementation/slice6/images/F01_A_MAIN_OV.jpg)</t>
         </is>
       </c>
     </row>
@@ -12129,10 +12133,14 @@
       </c>
       <c r="S172" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T172" s="2" t="inlineStr"/>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="T172" s="2" t="inlineStr">
+        <is>
+          <t>The brass signal-outlet plate beside the switch came with BW-013 (slice 6); the chain door guard is on the entry leaf's apartment face: slotted plate by the latch stile, anchor plate and unhooked chain beside it (slice 10). Verified at d38ba7ac (slice10, slice10b): the thirteen families pass the fabrication batch (24,276 checks, 0 failures; seating 51 actors with the two armchairs, 1A's captured natively), door casings and fitted door fabric 0 failures, door hinges 10 as before (the 105-door count and one leaf's knuckles, identical at 6d99760d, slice10c), both door-route suites unchanged (45 and 32 waypoints, 0 failures), completion route 1A 15 waypoints as before (the kitchen leg), apartment batch 236 as before, upper lighting 0 failures, the seven-space sweep 0 failures; the chain guards are shown at the vestibule thresholds and the armchairs in F05_B_MAIN and F01_A_MAIN (implementation/slice10).</t>
+        </is>
+      </c>
     </row>
     <row r="173">
       <c r="A173" s="2" t="inlineStr">
@@ -14771,10 +14779,14 @@
       </c>
       <c r="S207" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T207" s="2" t="inlineStr"/>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="T207" s="2" t="inlineStr">
+        <is>
+          <t>The brass signal-outlet plate beside the switch came with BW-013 (slice 6); the chain door guard is on the entry leaf's apartment face: slotted plate by the latch stile, anchor plate and unhooked chain beside it (slice 10). Verified at d38ba7ac (slice10, slice10b): the thirteen families pass the fabrication batch (24,276 checks, 0 failures; seating 51 actors with the two armchairs, 1A's captured natively), door casings and fitted door fabric 0 failures, door hinges 10 as before (the 105-door count and one leaf's knuckles, identical at 6d99760d, slice10c), both door-route suites unchanged (45 and 32 waypoints, 0 failures), completion route 1A 15 waypoints as before (the kitchen leg), apartment batch 236 as before, upper lighting 0 failures, the seven-space sweep 0 failures; the chain guards are shown at the vestibule thresholds and the armchairs in F05_B_MAIN and F01_A_MAIN (implementation/slice10).</t>
+        </is>
+      </c>
     </row>
     <row r="208">
       <c r="A208" s="2" t="inlineStr">
@@ -16127,10 +16139,14 @@
       </c>
       <c r="S225" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T225" s="2" t="inlineStr"/>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="T225" s="2" t="inlineStr">
+        <is>
+          <t>The brass signal-outlet plate beside the switch came with BW-013 (slice 6); the chain door guard is on the entry leaf's apartment face: slotted plate by the latch stile, anchor plate and unhooked chain beside it (slice 10). Verified at d38ba7ac (slice10, slice10b): the thirteen families pass the fabrication batch (24,276 checks, 0 failures; seating 51 actors with the two armchairs, 1A's captured natively), door casings and fitted door fabric 0 failures, door hinges 10 as before (the 105-door count and one leaf's knuckles, identical at 6d99760d, slice10c), both door-route suites unchanged (45 and 32 waypoints, 0 failures), completion route 1A 15 waypoints as before (the kitchen leg), apartment batch 236 as before, upper lighting 0 failures, the seven-space sweep 0 failures; the chain guards are shown at the vestibule thresholds and the armchairs in F05_B_MAIN and F01_A_MAIN (implementation/slice10).</t>
+        </is>
+      </c>
     </row>
     <row r="226">
       <c r="A226" s="2" t="inlineStr">
@@ -17315,10 +17331,14 @@
       </c>
       <c r="S241" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T241" s="2" t="inlineStr"/>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="T241" s="2" t="inlineStr">
+        <is>
+          <t>The brass signal-outlet plate beside the switch came with BW-013 (slice 6); the chain door guard is on the entry leaf's apartment face: slotted plate by the latch stile, anchor plate and unhooked chain beside it (slice 10). Verified at d38ba7ac (slice10, slice10b): the thirteen families pass the fabrication batch (24,276 checks, 0 failures; seating 51 actors with the two armchairs, 1A's captured natively), door casings and fitted door fabric 0 failures, door hinges 10 as before (the 105-door count and one leaf's knuckles, identical at 6d99760d, slice10c), both door-route suites unchanged (45 and 32 waypoints, 0 failures), completion route 1A 15 waypoints as before (the kitchen leg), apartment batch 236 as before, upper lighting 0 failures, the seven-space sweep 0 failures; the chain guards are shown at the vestibule thresholds and the armchairs in F05_B_MAIN and F01_A_MAIN (implementation/slice10).</t>
+        </is>
+      </c>
     </row>
     <row r="242">
       <c r="A242" s="2" t="inlineStr">
@@ -20037,10 +20057,14 @@
       </c>
       <c r="S278" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T278" s="2" t="inlineStr"/>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="T278" s="2" t="inlineStr">
+        <is>
+          <t>The brass signal-outlet plate beside the switch came with BW-013 (slice 6); the chain door guard is on the entry leaf's apartment face: slotted plate by the latch stile, anchor plate and unhooked chain beside it (slice 10). Verified at d38ba7ac (slice10, slice10b): the thirteen families pass the fabrication batch (24,276 checks, 0 failures; seating 51 actors with the two armchairs, 1A's captured natively), door casings and fitted door fabric 0 failures, door hinges 10 as before (the 105-door count and one leaf's knuckles, identical at 6d99760d, slice10c), both door-route suites unchanged (45 and 32 waypoints, 0 failures), completion route 1A 15 waypoints as before (the kitchen leg), apartment batch 236 as before, upper lighting 0 failures, the seven-space sweep 0 failures; the chain guards are shown at the vestibule thresholds and the armchairs in F05_B_MAIN and F01_A_MAIN (implementation/slice10).</t>
+        </is>
+      </c>
     </row>
     <row r="279">
       <c r="A279" s="2" t="inlineStr">
@@ -21167,10 +21191,14 @@
       </c>
       <c r="S293" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T293" s="2" t="inlineStr"/>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="T293" s="2" t="inlineStr">
+        <is>
+          <t>The brass signal-outlet plate beside the switch came with BW-013 (slice 6); the chain door guard is on the entry leaf's apartment face: slotted plate by the latch stile, anchor plate and unhooked chain beside it (slice 10). Verified at d38ba7ac (slice10, slice10b): the thirteen families pass the fabrication batch (24,276 checks, 0 failures; seating 51 actors with the two armchairs, 1A's captured natively), door casings and fitted door fabric 0 failures, door hinges 10 as before (the 105-door count and one leaf's knuckles, identical at 6d99760d, slice10c), both door-route suites unchanged (45 and 32 waypoints, 0 failures), completion route 1A 15 waypoints as before (the kitchen leg), apartment batch 236 as before, upper lighting 0 failures, the seven-space sweep 0 failures; the chain guards are shown at the vestibule thresholds and the armchairs in F05_B_MAIN and F01_A_MAIN (implementation/slice10).</t>
+        </is>
+      </c>
     </row>
     <row r="294">
       <c r="A294" s="2" t="inlineStr">
@@ -22347,10 +22375,14 @@
       </c>
       <c r="S309" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T309" s="2" t="inlineStr"/>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="T309" s="2" t="inlineStr">
+        <is>
+          <t>The brass signal-outlet plate beside the switch came with BW-013 (slice 6); the chain door guard is on the entry leaf's apartment face: slotted plate by the latch stile, anchor plate and unhooked chain beside it (slice 10). Verified at d38ba7ac (slice10, slice10b): the thirteen families pass the fabrication batch (24,276 checks, 0 failures; seating 51 actors with the two armchairs, 1A's captured natively), door casings and fitted door fabric 0 failures, door hinges 10 as before (the 105-door count and one leaf's knuckles, identical at 6d99760d, slice10c), both door-route suites unchanged (45 and 32 waypoints, 0 failures), completion route 1A 15 waypoints as before (the kitchen leg), apartment batch 236 as before, upper lighting 0 failures, the seven-space sweep 0 failures; the chain guards are shown at the vestibule thresholds and the armchairs in F05_B_MAIN and F01_A_MAIN (implementation/slice10).</t>
+        </is>
+      </c>
     </row>
     <row r="310">
       <c r="A310" s="2" t="inlineStr">
@@ -25255,10 +25287,14 @@
       </c>
       <c r="S349" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T349" s="2" t="inlineStr"/>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="T349" s="2" t="inlineStr">
+        <is>
+          <t>The brass signal-outlet plate beside the switch came with BW-013 (slice 6); the chain door guard is on the entry leaf's apartment face: slotted plate by the latch stile, anchor plate and unhooked chain beside it (slice 10). Verified at d38ba7ac (slice10, slice10b): the thirteen families pass the fabrication batch (24,276 checks, 0 failures; seating 51 actors with the two armchairs, 1A's captured natively), door casings and fitted door fabric 0 failures, door hinges 10 as before (the 105-door count and one leaf's knuckles, identical at 6d99760d, slice10c), both door-route suites unchanged (45 and 32 waypoints, 0 failures), completion route 1A 15 waypoints as before (the kitchen leg), apartment batch 236 as before, upper lighting 0 failures, the seven-space sweep 0 failures; the chain guards are shown at the vestibule thresholds and the armchairs in F05_B_MAIN and F01_A_MAIN (implementation/slice10).</t>
+        </is>
+      </c>
     </row>
     <row r="350">
       <c r="A350" s="2" t="inlineStr">
@@ -26587,10 +26623,14 @@
       </c>
       <c r="S367" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T367" s="2" t="inlineStr"/>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="T367" s="2" t="inlineStr">
+        <is>
+          <t>The brass signal-outlet plate beside the switch came with BW-013 (slice 6); the chain door guard is on the entry leaf's apartment face: slotted plate by the latch stile, anchor plate and unhooked chain beside it (slice 10). Verified at d38ba7ac (slice10, slice10b): the thirteen families pass the fabrication batch (24,276 checks, 0 failures; seating 51 actors with the two armchairs, 1A's captured natively), door casings and fitted door fabric 0 failures, door hinges 10 as before (the 105-door count and one leaf's knuckles, identical at 6d99760d, slice10c), both door-route suites unchanged (45 and 32 waypoints, 0 failures), completion route 1A 15 waypoints as before (the kitchen leg), apartment batch 236 as before, upper lighting 0 failures, the seven-space sweep 0 failures; the chain guards are shown at the vestibule thresholds and the armchairs in F05_B_MAIN and F01_A_MAIN (implementation/slice10).</t>
+        </is>
+      </c>
     </row>
     <row r="368">
       <c r="A368" s="2" t="inlineStr">
@@ -28159,10 +28199,14 @@
       </c>
       <c r="S389" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T389" s="2" t="inlineStr"/>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="T389" s="2" t="inlineStr">
+        <is>
+          <t>The brass signal-outlet plate beside the switch came with BW-013 (slice 6); the chain door guard is on the entry leaf's apartment face: slotted plate by the latch stile, anchor plate and unhooked chain beside it (slice 10). Verified at d38ba7ac (slice10, slice10b): the thirteen families pass the fabrication batch (24,276 checks, 0 failures; seating 51 actors with the two armchairs, 1A's captured natively), door casings and fitted door fabric 0 failures, door hinges 10 as before (the 105-door count and one leaf's knuckles, identical at 6d99760d, slice10c), both door-route suites unchanged (45 and 32 waypoints, 0 failures), completion route 1A 15 waypoints as before (the kitchen leg), apartment batch 236 as before, upper lighting 0 failures, the seven-space sweep 0 failures; the chain guards are shown at the vestibule thresholds and the armchairs in F05_B_MAIN and F01_A_MAIN (implementation/slice10).</t>
+        </is>
+      </c>
     </row>
     <row r="390">
       <c r="A390" s="2" t="inlineStr">
@@ -29389,10 +29433,14 @@
       </c>
       <c r="S406" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T406" s="2" t="inlineStr"/>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="T406" s="2" t="inlineStr">
+        <is>
+          <t>The brass signal-outlet plate beside the switch came with BW-013 (slice 6); the chain door guard is on the entry leaf's apartment face: slotted plate by the latch stile, anchor plate and unhooked chain beside it (slice 10). Verified at d38ba7ac (slice10, slice10b): the thirteen families pass the fabrication batch (24,276 checks, 0 failures; seating 51 actors with the two armchairs, 1A's captured natively), door casings and fitted door fabric 0 failures, door hinges 10 as before (the 105-door count and one leaf's knuckles, identical at 6d99760d, slice10c), both door-route suites unchanged (45 and 32 waypoints, 0 failures), completion route 1A 15 waypoints as before (the kitchen leg), apartment batch 236 as before, upper lighting 0 failures, the seven-space sweep 0 failures; the chain guards are shown at the vestibule thresholds and the armchairs in F05_B_MAIN and F01_A_MAIN (implementation/slice10).</t>
+        </is>
+      </c>
     </row>
     <row r="407">
       <c r="A407" s="2" t="inlineStr">
@@ -31895,10 +31943,14 @@
       </c>
       <c r="S441" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T441" s="2" t="inlineStr"/>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="T441" s="2" t="inlineStr">
+        <is>
+          <t>The brass signal-outlet plate beside the switch came with BW-013 (slice 6); the chain door guard is on the entry leaf's apartment face: slotted plate by the latch stile, anchor plate and unhooked chain beside it (slice 10). Verified at d38ba7ac (slice10, slice10b): the thirteen families pass the fabrication batch (24,276 checks, 0 failures; seating 51 actors with the two armchairs, 1A's captured natively), door casings and fitted door fabric 0 failures, door hinges 10 as before (the 105-door count and one leaf's knuckles, identical at 6d99760d, slice10c), both door-route suites unchanged (45 and 32 waypoints, 0 failures), completion route 1A 15 waypoints as before (the kitchen leg), apartment batch 236 as before, upper lighting 0 failures, the seven-space sweep 0 failures; the chain guards are shown at the vestibule thresholds and the armchairs in F05_B_MAIN and F01_A_MAIN (implementation/slice10).</t>
+        </is>
+      </c>
     </row>
     <row r="442">
       <c r="A442" s="2" t="inlineStr">
@@ -33245,10 +33297,14 @@
       </c>
       <c r="S460" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T460" s="2" t="inlineStr"/>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="T460" s="2" t="inlineStr">
+        <is>
+          <t>The brass signal-outlet plate beside the switch came with BW-013 (slice 6); the chain door guard is on the entry leaf's apartment face: slotted plate by the latch stile, anchor plate and unhooked chain beside it (slice 10). Verified at d38ba7ac (slice10, slice10b): the thirteen families pass the fabrication batch (24,276 checks, 0 failures; seating 51 actors with the two armchairs, 1A's captured natively), door casings and fitted door fabric 0 failures, door hinges 10 as before (the 105-door count and one leaf's knuckles, identical at 6d99760d, slice10c), both door-route suites unchanged (45 and 32 waypoints, 0 failures), completion route 1A 15 waypoints as before (the kitchen leg), apartment batch 236 as before, upper lighting 0 failures, the seven-space sweep 0 failures; the chain guards are shown at the vestibule thresholds and the armchairs in F05_B_MAIN and F01_A_MAIN (implementation/slice10).</t>
+        </is>
+      </c>
     </row>
     <row r="461">
       <c r="A461" s="2" t="inlineStr">
@@ -33381,10 +33437,14 @@
       </c>
       <c r="S462" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T462" s="2" t="inlineStr"/>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="T462" s="2" t="inlineStr">
+        <is>
+          <t>5B_radio_chair: the new Armchair form (sofa recipe at 0.85 m, one cushion, rolled arms) at (-13.8, 5.55) on the window side of the wireless table, facing east along it. The worn-through arm and dished seat are finish work on the cloth and stay open. Verified at d38ba7ac (slice10, slice10b): the thirteen families pass the fabrication batch (24,276 checks, 0 failures; seating 51 actors with the two armchairs, 1A's captured natively), door casings and fitted door fabric 0 failures, door hinges 10 as before (the 105-door count and one leaf's knuckles, identical at 6d99760d, slice10c), both door-route suites unchanged (45 and 32 waypoints, 0 failures), completion route 1A 15 waypoints as before (the kitchen leg), apartment batch 236 as before, upper lighting 0 failures, the seven-space sweep 0 failures; the chain guards are shown at the vestibule thresholds and the armchairs in F05_B_MAIN and F01_A_MAIN (implementation/slice10).</t>
+        </is>
+      </c>
     </row>
     <row r="463">
       <c r="A463" s="2" t="inlineStr">
@@ -34545,10 +34605,14 @@
       </c>
       <c r="S478" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T478" s="2" t="inlineStr"/>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="T478" s="2" t="inlineStr">
+        <is>
+          <t>The brass signal-outlet plate beside the switch came with BW-013 (slice 6); the chain door guard is on the entry leaf's apartment face: slotted plate by the latch stile, anchor plate and unhooked chain beside it (slice 10). Verified at d38ba7ac (slice10, slice10b): the thirteen families pass the fabrication batch (24,276 checks, 0 failures; seating 51 actors with the two armchairs, 1A's captured natively), door casings and fitted door fabric 0 failures, door hinges 10 as before (the 105-door count and one leaf's knuckles, identical at 6d99760d, slice10c), both door-route suites unchanged (45 and 32 waypoints, 0 failures), completion route 1A 15 waypoints as before (the kitchen leg), apartment batch 236 as before, upper lighting 0 failures, the seven-space sweep 0 failures; the chain guards are shown at the vestibule thresholds and the armchairs in F05_B_MAIN and F01_A_MAIN (implementation/slice10).</t>
+        </is>
+      </c>
     </row>
     <row r="479">
       <c r="A479" s="2" t="inlineStr">
@@ -37063,10 +37127,14 @@
       </c>
       <c r="S513" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T513" s="2" t="inlineStr"/>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="T513" s="2" t="inlineStr">
+        <is>
+          <t>The brass signal-outlet plate beside the switch came with BW-013 (slice 6); the chain door guard is on the entry leaf's apartment face: slotted plate by the latch stile, anchor plate and unhooked chain beside it (slice 10). Verified at d38ba7ac (slice10, slice10b): the thirteen families pass the fabrication batch (24,276 checks, 0 failures; seating 51 actors with the two armchairs, 1A's captured natively), door casings and fitted door fabric 0 failures, door hinges 10 as before (the 105-door count and one leaf's knuckles, identical at 6d99760d, slice10c), both door-route suites unchanged (45 and 32 waypoints, 0 failures), completion route 1A 15 waypoints as before (the kitchen leg), apartment batch 236 as before, upper lighting 0 failures, the seven-space sweep 0 failures; the chain guards are shown at the vestibule thresholds and the armchairs in F05_B_MAIN and F01_A_MAIN (implementation/slice10).</t>
+        </is>
+      </c>
     </row>
     <row r="514">
       <c r="A514" s="2" t="inlineStr">
@@ -38265,10 +38333,14 @@
       </c>
       <c r="S530" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T530" s="2" t="inlineStr"/>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="T530" s="2" t="inlineStr">
+        <is>
+          <t>The brass signal-outlet plate beside the switch came with BW-013 (slice 6); the chain door guard is on the entry leaf's apartment face: slotted plate by the latch stile, anchor plate and unhooked chain beside it (slice 10). Verified at d38ba7ac (slice10, slice10b): the thirteen families pass the fabrication batch (24,276 checks, 0 failures; seating 51 actors with the two armchairs, 1A's captured natively), door casings and fitted door fabric 0 failures, door hinges 10 as before (the 105-door count and one leaf's knuckles, identical at 6d99760d, slice10c), both door-route suites unchanged (45 and 32 waypoints, 0 failures), completion route 1A 15 waypoints as before (the kitchen leg), apartment batch 236 as before, upper lighting 0 failures, the seven-space sweep 0 failures; the chain guards are shown at the vestibule thresholds and the armchairs in F05_B_MAIN and F01_A_MAIN (implementation/slice10).</t>
+        </is>
+      </c>
     </row>
     <row r="531">
       <c r="A531" s="2" t="inlineStr">
@@ -39165,10 +39237,14 @@
       </c>
       <c r="S542" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T542" s="2" t="inlineStr"/>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="T542" s="2" t="inlineStr">
+        <is>
+          <t>The brass signal-outlet plate beside the switch came with BW-013 (slice 6); the chain door guard is on the entry leaf's apartment face: slotted plate by the latch stile, anchor plate and unhooked chain beside it (slice 10). Verified at d38ba7ac (slice10, slice10b): the thirteen families pass the fabrication batch (24,276 checks, 0 failures; seating 51 actors with the two armchairs, 1A's captured natively), door casings and fitted door fabric 0 failures, door hinges 10 as before (the 105-door count and one leaf's knuckles, identical at 6d99760d, slice10c), both door-route suites unchanged (45 and 32 waypoints, 0 failures), completion route 1A 15 waypoints as before (the kitchen leg), apartment batch 236 as before, upper lighting 0 failures, the seven-space sweep 0 failures; the chain guards are shown at the vestibule thresholds and the armchairs in F05_B_MAIN and F01_A_MAIN (implementation/slice10).</t>
+        </is>
+      </c>
     </row>
     <row r="543">
       <c r="A543" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Implement dossier slice 13: garment rails and hung blankets
Cloth for the V2 environment design dossier, in the domestic objects family:

- garmentrail form: header board on rear battens, two brackets and a rail,
  garments on wooden hangers hung edge-on to the wall, optional paper
  repair tags. F02_B_MAIN-002: 2B's repair rail with five garments;
  F04_B_CLOSET-001: 4B's closet rail with four.
- blanket form: a moving blanket on a batten with bound edges and quilted
  rows. F02_C_BED2-002: two on 2C's second-bedroom east wall;
  F03_D_STUDY-001: two in 3D's study as completion copies.
- Five tinted cloth keys (burgundy wool, maroon jersey, navy cape, grey
  coat, grey blanket) on the catalogue linen, declared in the plan like
  the seating family's fabric_cool.
- 4B's closet shelf: a capsule tin and a bulb carton (surface stock, 164).

Evidence under implementation/slice13/. INERT: no ledger status changes.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/art/reviews/v2_environment_design_20261008/change_register.xlsx
+++ b/art/reviews/v2_environment_design_20261008/change_register.xlsx
@@ -16385,10 +16385,14 @@
       </c>
       <c r="S228" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T228" s="2" t="inlineStr"/>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="T228" s="2" t="inlineStr">
+        <is>
+          <t>2B_repair_rail (garmentrail form: header board, brackets, rail) on the west wall's segment south of the vestibule opening, rail at 1.7 m, five garments on wooden hangers with paper repair tags: burgundy wool, Cam's maroon jersey, a navy cape, a grey coat and a linen shirt. Deviations: the opening's neighbour wall is the only clear 1 m run (the dossier's spot beside the private-hall opening holds the radio table); the scarlet lining and celluloid collar are colour details the garment form does not carry; the mended armchair waits for the sewing machine, whose placement fixes where it faces (every corner of the room holds a stance or the hall route). Verified at 7c765151 (slice13): the thirteen families pass the fabrication batch (25,479 checks, 0 failures; objects 50 actors, every rail and blanket on its actual wall face, the two closet-shelf items bearing on the clear boards), apartment batch 236 as before, upper lighting 0 failures, completion route 3D 16 waypoints as before (the kitchen leg), the household save owner 0 failures, the four-space sweep 0 failures; the rooms and native close-ups are in implementation/slice13.</t>
+        </is>
+      </c>
     </row>
     <row r="229">
       <c r="A229" s="2" t="inlineStr">
@@ -18453,10 +18457,14 @@
       </c>
       <c r="S256" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T256" s="2" t="inlineStr"/>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="T256" s="2" t="inlineStr">
+        <is>
+          <t>2C_blanket_a/b: two 1.2 x 2.0 m moving blankets (blanket form: batten, bound edges, quilted rows) on the east wall. Deviations: the window and the door wall keep their light and swing; the mic stands, amp, guitar and pedalboard wait for their families. Verified at 7c765151 (slice13): the thirteen families pass the fabrication batch (25,479 checks, 0 failures; objects 50 actors, every rail and blanket on its actual wall face, the two closet-shelf items bearing on the clear boards), apartment batch 236 as before, upper lighting 0 failures, completion route 3D 16 waypoints as before (the kitchen leg), the household save owner 0 failures, the four-space sweep 0 failures; the rooms and native close-ups are in implementation/slice13.</t>
+        </is>
+      </c>
     </row>
     <row r="257">
       <c r="A257" s="2" t="inlineStr">
@@ -23423,10 +23431,14 @@
       </c>
       <c r="S323" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T323" s="2" t="inlineStr"/>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="T323" s="2" t="inlineStr">
+        <is>
+          <t>3D_blanket_a/b: two blankets (completion copies of 2C's) on the study's solid east wall. The music stand, mic case, deck and headphones wait for their families (no blanket over the window, so the study keeps its daylight). Verified at 7c765151 (slice13): the thirteen families pass the fabrication batch (25,479 checks, 0 failures; objects 50 actors, every rail and blanket on its actual wall face, the two closet-shelf items bearing on the clear boards), apartment batch 236 as before, upper lighting 0 failures, completion route 3D 16 waypoints as before (the kitchen leg), the household save owner 0 failures, the four-space sweep 0 failures; the rooms and native close-ups are in implementation/slice13.</t>
+        </is>
+      </c>
     </row>
     <row r="324">
       <c r="A324" s="2" t="inlineStr">
@@ -27799,10 +27811,14 @@
       </c>
       <c r="S383" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T383" s="2" t="inlineStr"/>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="T383" s="2" t="inlineStr">
+        <is>
+          <t>4B_closet_rail (garmentrail form, four garments, no tags) across the closet's north wall at 1.7 m, clear of the shelf and the door; on 4B_equipment_shelf a capsule tin and a bulb carton on the clear boards. The fuse box and flex coil wait for their forms. Verified at 7c765151 (slice13): the thirteen families pass the fabrication batch (25,479 checks, 0 failures; objects 50 actors, every rail and blanket on its actual wall face, the two closet-shelf items bearing on the clear boards), apartment batch 236 as before, upper lighting 0 failures, completion route 3D 16 waypoints as before (the kitchen leg), the household save owner 0 failures, the four-space sweep 0 failures; the rooms and native close-ups are in implementation/slice13.</t>
+        </is>
+      </c>
     </row>
     <row r="384">
       <c r="A384" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Implement dossier slice 14: one use object in each private hall
F0x_x_PRIVATE_HALL-001 for all eighteen homes of the V2 environment design
dossier, one native object per hall by the resident's routine:

- hamper form (lidded wicker laundry hamper on four feet, a linen corner
  under the lid) in 1A, 2A, 2B, 3D, 4C, 5B and 6B;
- boottray form (galvanised tray, a pair of rubber galoshes, dried mud) in
  1D, 2C, 3A, 4A, 4B, 5A, 5C and 6C;
- copies of the existing crates in 3B and 4D (parts crate) and 6A (gear
  crate).

Each stands against a wall at a spot chosen clear of every door and
opening approach (span plus 0.15 m, 1.0 m deep), the stances and a 0.85 m
route; completion homes carry completion copies.

Evidence under implementation/slice14b, slice14c and slice14base/. INERT: no ledger status changes.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/art/reviews/v2_environment_design_20261008/change_register.xlsx
+++ b/art/reviews/v2_environment_design_20261008/change_register.xlsx
@@ -11353,10 +11353,14 @@
       </c>
       <c r="S162" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T162" s="2" t="inlineStr"/>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="T162" s="2" t="inlineStr">
+        <is>
+          <t>A lidded wicker laundry hamper (hamper form) with a linen corner caught under the lid against the east wall at (-5.67, -9.28), clear of every door and opening approach (each opening's span plus 0.15 m, 1.0 m deep), the stances and a 0.85 m route; a completion copy. The hamper's cane panels read as a lidded box rather than a woven basket and the galoshes are plain blocks; finer weave and boot forms are later art. Verified at 2152694f (slice14b) and 4fc1b18d (slice14c, after 2A's and 3A's objects moved to the north end wall out of the door route): the thirteen families pass the fabrication batch (25,826 checks, 0 failures; every hall object bearing inside its hall), apartment batch 236 as before, the apartment door route 45 waypoints and the 4B route 32 with 0 failures, the six completion routes unchanged (1A 15, 1D 25, 2C 9, 3D 16, 4C 9, 4D 12), upper lighting 0 failures, upper furniture 444 identical to slice 13 (slice14base), the eighteen-hall sweep 0 failures; captures in implementation/slice14b and slice14c.</t>
+        </is>
+      </c>
     </row>
     <row r="163">
       <c r="A163" s="2" t="inlineStr">
@@ -13143,10 +13147,14 @@
       </c>
       <c r="S185" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T185" s="2" t="inlineStr"/>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="T185" s="2" t="inlineStr">
+        <is>
+          <t>A galvanised boot tray with a pair of rubber galoshes and dried mud (boottray form) against the west wall at (13.07, -4.58), clear of every door and opening approach (each opening's span plus 0.15 m, 1.0 m deep), the stances and a 0.85 m route; a completion copy. The hamper's cane panels read as a lidded box rather than a woven basket and the galoshes are plain blocks; finer weave and boot forms are later art. Verified at 2152694f (slice14b) and 4fc1b18d (slice14c, after 2A's and 3A's objects moved to the north end wall out of the door route): the thirteen families pass the fabrication batch (25,826 checks, 0 failures; every hall object bearing inside its hall), apartment batch 236 as before, the apartment door route 45 waypoints and the 4B route 32 with 0 failures, the six completion routes unchanged (1A 15, 1D 25, 2C 9, 3D 16, 4C 9, 4D 12), upper lighting 0 failures, upper furniture 444 identical to slice 13 (slice14base), the eighteen-hall sweep 0 failures; captures in implementation/slice14b and slice14c.</t>
+        </is>
+      </c>
     </row>
     <row r="186">
       <c r="A186" s="2" t="inlineStr">
@@ -15613,10 +15621,14 @@
       </c>
       <c r="S218" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T218" s="2" t="inlineStr"/>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="T218" s="2" t="inlineStr">
+        <is>
+          <t>A lidded wicker laundry hamper (hamper form) with a linen corner caught under the lid against the north wall at (-9.32, 7.58), clear of every door and opening approach (each opening's span plus 0.15 m, 1.0 m deep), the stances and a 0.85 m route. The hamper's cane panels read as a lidded box rather than a woven basket and the galoshes are plain blocks; finer weave and boot forms are later art. Verified at 2152694f (slice14b) and 4fc1b18d (slice14c, after 2A's and 3A's objects moved to the north end wall out of the door route): the thirteen families pass the fabrication batch (25,826 checks, 0 failures; every hall object bearing inside its hall), apartment batch 236 as before, the apartment door route 45 waypoints and the 4B route 32 with 0 failures, the six completion routes unchanged (1A 15, 1D 25, 2C 9, 3D 16, 4C 9, 4D 12), upper lighting 0 failures, upper furniture 444 identical to slice 13 (slice14base), the eighteen-hall sweep 0 failures; captures in implementation/slice14b and slice14c.</t>
+        </is>
+      </c>
     </row>
     <row r="219">
       <c r="A219" s="2" t="inlineStr">
@@ -16821,10 +16833,14 @@
       </c>
       <c r="S234" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T234" s="2" t="inlineStr"/>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="T234" s="2" t="inlineStr">
+        <is>
+          <t>A lidded wicker laundry hamper (hamper form) with a linen corner caught under the lid against the west wall at (13.07, -4.58), clear of every door and opening approach (each opening's span plus 0.15 m, 1.0 m deep), the stances and a 0.85 m route. The hamper's cane panels read as a lidded box rather than a woven basket and the galoshes are plain blocks; finer weave and boot forms are later art. Verified at 2152694f (slice14b) and 4fc1b18d (slice14c, after 2A's and 3A's objects moved to the north end wall out of the door route): the thirteen families pass the fabrication batch (25,826 checks, 0 failures; every hall object bearing inside its hall), apartment batch 236 as before, the apartment door route 45 waypoints and the 4B route 32 with 0 failures, the six completion routes unchanged (1A 15, 1D 25, 2C 9, 3D 16, 4C 9, 4D 12), upper lighting 0 failures, upper furniture 444 identical to slice 13 (slice14base), the eighteen-hall sweep 0 failures; captures in implementation/slice14b and slice14c.</t>
+        </is>
+      </c>
     </row>
     <row r="235">
       <c r="A235" s="2" t="inlineStr">
@@ -17951,10 +17967,14 @@
       </c>
       <c r="S249" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T249" s="2" t="inlineStr"/>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="T249" s="2" t="inlineStr">
+        <is>
+          <t>A galvanised boot tray with a pair of rubber galoshes and dried mud (boottray form) against the south wall at (6.67, 6.62), clear of every door and opening approach (each opening's span plus 0.15 m, 1.0 m deep), the stances and a 0.85 m route; a completion copy. The hamper's cane panels read as a lidded box rather than a woven basket and the galoshes are plain blocks; finer weave and boot forms are later art. Verified at 2152694f (slice14b) and 4fc1b18d (slice14c, after 2A's and 3A's objects moved to the north end wall out of the door route): the thirteen families pass the fabrication batch (25,826 checks, 0 failures; every hall object bearing inside its hall), apartment batch 236 as before, the apartment door route 45 waypoints and the 4B route 32 with 0 failures, the six completion routes unchanged (1A 15, 1D 25, 2C 9, 3D 16, 4C 9, 4D 12), upper lighting 0 failures, upper furniture 444 identical to slice 13 (slice14base), the eighteen-hall sweep 0 failures; captures in implementation/slice14b and slice14c.</t>
+        </is>
+      </c>
     </row>
     <row r="250">
       <c r="A250" s="2" t="inlineStr">
@@ -20817,10 +20837,14 @@
       </c>
       <c r="S288" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T288" s="2" t="inlineStr"/>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="T288" s="2" t="inlineStr">
+        <is>
+          <t>A galvanised boot tray with a pair of rubber galoshes and dried mud (boottray form) against the north wall at (-9.32, 7.58), clear of every door and opening approach (each opening's span plus 0.15 m, 1.0 m deep), the stances and a 0.85 m route. The hamper's cane panels read as a lidded box rather than a woven basket and the galoshes are plain blocks; finer weave and boot forms are later art. Verified at 2152694f (slice14b) and 4fc1b18d (slice14c, after 2A's and 3A's objects moved to the north end wall out of the door route): the thirteen families pass the fabrication batch (25,826 checks, 0 failures; every hall object bearing inside its hall), apartment batch 236 as before, the apartment door route 45 waypoints and the 4B route 32 with 0 failures, the six completion routes unchanged (1A 15, 1D 25, 2C 9, 3D 16, 4C 9, 4D 12), upper lighting 0 failures, upper furniture 444 identical to slice 13 (slice14base), the eighteen-hall sweep 0 failures; captures in implementation/slice14b and slice14c.</t>
+        </is>
+      </c>
     </row>
     <row r="289">
       <c r="A289" s="2" t="inlineStr">
@@ -21931,10 +21955,14 @@
       </c>
       <c r="S303" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T303" s="2" t="inlineStr"/>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="T303" s="2" t="inlineStr">
+        <is>
+          <t>A parts crate (a copy of 3B_partscrate) against the east wall at (15.38, -9.43), clear of every door and opening approach (each opening's span plus 0.15 m, 1.0 m deep), the stances and a 0.85 m route. The hamper's cane panels read as a lidded box rather than a woven basket and the galoshes are plain blocks; finer weave and boot forms are later art. Verified at 2152694f (slice14b) and 4fc1b18d (slice14c, after 2A's and 3A's objects moved to the north end wall out of the door route): the thirteen families pass the fabrication batch (25,826 checks, 0 failures; every hall object bearing inside its hall), apartment batch 236 as before, the apartment door route 45 waypoints and the 4B route 32 with 0 failures, the six completion routes unchanged (1A 15, 1D 25, 2C 9, 3D 16, 4C 9, 4D 12), upper lighting 0 failures, upper furniture 444 identical to slice 13 (slice14base), the eighteen-hall sweep 0 failures; captures in implementation/slice14b and slice14c.</t>
+        </is>
+      </c>
     </row>
     <row r="304">
       <c r="A304" s="2" t="inlineStr">
@@ -23061,10 +23089,14 @@
       </c>
       <c r="S318" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T318" s="2" t="inlineStr"/>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="T318" s="2" t="inlineStr">
+        <is>
+          <t>A lidded wicker laundry hamper (hamper form) with a linen corner caught under the lid against the east wall at (-5.87, -9.28), clear of every door and opening approach (each opening's span plus 0.15 m, 1.0 m deep), the stances and a 0.85 m route; a completion copy. The hamper's cane panels read as a lidded box rather than a woven basket and the galoshes are plain blocks; finer weave and boot forms are later art. Verified at 2152694f (slice14b) and 4fc1b18d (slice14c, after 2A's and 3A's objects moved to the north end wall out of the door route): the thirteen families pass the fabrication batch (25,826 checks, 0 failures; every hall object bearing inside its hall), apartment batch 236 as before, the apartment door route 45 waypoints and the 4B route 32 with 0 failures, the six completion routes unchanged (1A 15, 1D 25, 2C 9, 3D 16, 4C 9, 4D 12), upper lighting 0 failures, upper furniture 444 identical to slice 13 (slice14base), the eighteen-hall sweep 0 failures; captures in implementation/slice14b and slice14c.</t>
+        </is>
+      </c>
     </row>
     <row r="319">
       <c r="A319" s="2" t="inlineStr">
@@ -26113,10 +26145,14 @@
       </c>
       <c r="S360" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T360" s="2" t="inlineStr"/>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="T360" s="2" t="inlineStr">
+        <is>
+          <t>A galvanised boot tray with a pair of rubber galoshes and dried mud (boottray form) against the east wall at (15.38, -8.98), clear of every door and opening approach (each opening's span plus 0.15 m, 1.0 m deep), the stances and a 0.85 m route. The hamper's cane panels read as a lidded box rather than a woven basket and the galoshes are plain blocks; finer weave and boot forms are later art. Verified at 2152694f (slice14b) and 4fc1b18d (slice14c, after 2A's and 3A's objects moved to the north end wall out of the door route): the thirteen families pass the fabrication batch (25,826 checks, 0 failures; every hall object bearing inside its hall), apartment batch 236 as before, the apartment door route 45 waypoints and the 4B route 32 with 0 failures, the six completion routes unchanged (1A 15, 1D 25, 2C 9, 3D 16, 4C 9, 4D 12), upper lighting 0 failures, upper furniture 444 identical to slice 13 (slice14base), the eighteen-hall sweep 0 failures; captures in implementation/slice14b and slice14c.</t>
+        </is>
+      </c>
     </row>
     <row r="361">
       <c r="A361" s="2" t="inlineStr">
@@ -27383,10 +27419,14 @@
       </c>
       <c r="S377" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T377" s="2" t="inlineStr"/>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="T377" s="2" t="inlineStr">
+        <is>
+          <t>A galvanised boot tray with a pair of rubber galoshes and dried mud (boottray form) against the west wall at (-10.83, 5.97), clear of every door and opening approach (each opening's span plus 0.15 m, 1.0 m deep), the stances and a 0.85 m route. The hamper's cane panels read as a lidded box rather than a woven basket and the galoshes are plain blocks; finer weave and boot forms are later art. Verified at 2152694f (slice14b) and 4fc1b18d (slice14c, after 2A's and 3A's objects moved to the north end wall out of the door route): the thirteen families pass the fabrication batch (25,826 checks, 0 failures; every hall object bearing inside its hall), apartment batch 236 as before, the apartment door route 45 waypoints and the 4B route 32 with 0 failures, the six completion routes unchanged (1A 15, 1D 25, 2C 9, 3D 16, 4C 9, 4D 12), upper lighting 0 failures, upper furniture 444 identical to slice 13 (slice14base), the eighteen-hall sweep 0 failures; captures in implementation/slice14b and slice14c.</t>
+        </is>
+      </c>
     </row>
     <row r="378">
       <c r="A378" s="2" t="inlineStr">
@@ -28959,10 +28999,14 @@
       </c>
       <c r="S399" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T399" s="2" t="inlineStr"/>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="T399" s="2" t="inlineStr">
+        <is>
+          <t>A lidded wicker laundry hamper (hamper form) with a linen corner caught under the lid against the south wall at (6.67, 6.62), clear of every door and opening approach (each opening's span plus 0.15 m, 1.0 m deep), the stances and a 0.85 m route; a completion copy. The hamper's cane panels read as a lidded box rather than a woven basket and the galoshes are plain blocks; finer weave and boot forms are later art. Verified at 2152694f (slice14b) and 4fc1b18d (slice14c, after 2A's and 3A's objects moved to the north end wall out of the door route): the thirteen families pass the fabrication batch (25,826 checks, 0 failures; every hall object bearing inside its hall), apartment batch 236 as before, the apartment door route 45 waypoints and the 4B route 32 with 0 failures, the six completion routes unchanged (1A 15, 1D 25, 2C 9, 3D 16, 4C 9, 4D 12), upper lighting 0 failures, upper furniture 444 identical to slice 13 (slice14base), the eighteen-hall sweep 0 failures; captures in implementation/slice14b and slice14c.</t>
+        </is>
+      </c>
     </row>
     <row r="400">
       <c r="A400" s="2" t="inlineStr">
@@ -30243,10 +30287,14 @@
       </c>
       <c r="S417" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T417" s="2" t="inlineStr"/>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="T417" s="2" t="inlineStr">
+        <is>
+          <t>A parts crate (a copy of 3B_partscrate) against the east wall at (-5.87, -9.28), clear of every door and opening approach (each opening's span plus 0.15 m, 1.0 m deep), the stances and a 0.85 m route; a completion copy. The hamper's cane panels read as a lidded box rather than a woven basket and the galoshes are plain blocks; finer weave and boot forms are later art. Verified at 2152694f (slice14b) and 4fc1b18d (slice14c, after 2A's and 3A's objects moved to the north end wall out of the door route): the thirteen families pass the fabrication batch (25,826 checks, 0 failures; every hall object bearing inside its hall), apartment batch 236 as before, the apartment door route 45 waypoints and the 4B route 32 with 0 failures, the six completion routes unchanged (1A 15, 1D 25, 2C 9, 3D 16, 4C 9, 4D 12), upper lighting 0 failures, upper furniture 444 identical to slice 13 (slice14base), the eighteen-hall sweep 0 failures; captures in implementation/slice14b and slice14c.</t>
+        </is>
+      </c>
     </row>
     <row r="418">
       <c r="A418" s="2" t="inlineStr">
@@ -32753,10 +32801,14 @@
       </c>
       <c r="S452" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T452" s="2" t="inlineStr"/>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="T452" s="2" t="inlineStr">
+        <is>
+          <t>A galvanised boot tray with a pair of rubber galoshes and dried mud (boottray form) against the east wall at (-5.87, -8.48), clear of every door and opening approach (each opening's span plus 0.15 m, 1.0 m deep), the stances and a 0.85 m route. The hamper's cane panels read as a lidded box rather than a woven basket and the galoshes are plain blocks; finer weave and boot forms are later art. Verified at 2152694f (slice14b) and 4fc1b18d (slice14c, after 2A's and 3A's objects moved to the north end wall out of the door route): the thirteen families pass the fabrication batch (25,826 checks, 0 failures; every hall object bearing inside its hall), apartment batch 236 as before, the apartment door route 45 waypoints and the 4B route 32 with 0 failures, the six completion routes unchanged (1A 15, 1D 25, 2C 9, 3D 16, 4C 9, 4D 12), upper lighting 0 failures, upper furniture 444 identical to slice 13 (slice14base), the eighteen-hall sweep 0 failures; captures in implementation/slice14b and slice14c.</t>
+        </is>
+      </c>
     </row>
     <row r="453">
       <c r="A453" s="2" t="inlineStr">
@@ -34193,10 +34245,14 @@
       </c>
       <c r="S472" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T472" s="2" t="inlineStr"/>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="T472" s="2" t="inlineStr">
+        <is>
+          <t>A lidded wicker laundry hamper (hamper form) with a linen corner caught under the lid against the north wall at (-10.83, 11.38), clear of every door and opening approach (each opening's span plus 0.15 m, 1.0 m deep), the stances and a 0.85 m route. The hamper's cane panels read as a lidded box rather than a woven basket and the galoshes are plain blocks; finer weave and boot forms are later art. Verified at 2152694f (slice14b) and 4fc1b18d (slice14c, after 2A's and 3A's objects moved to the north end wall out of the door route): the thirteen families pass the fabrication batch (25,826 checks, 0 failures; every hall object bearing inside its hall), apartment batch 236 as before, the apartment door route 45 waypoints and the 4B route 32 with 0 failures, the six completion routes unchanged (1A 15, 1D 25, 2C 9, 3D 16, 4C 9, 4D 12), upper lighting 0 failures, upper furniture 444 identical to slice 13 (slice14base), the eighteen-hall sweep 0 failures; captures in implementation/slice14b and slice14c.</t>
+        </is>
+      </c>
     </row>
     <row r="473">
       <c r="A473" s="2" t="inlineStr">
@@ -35345,10 +35401,14 @@
       </c>
       <c r="S488" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T488" s="2" t="inlineStr"/>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="T488" s="2" t="inlineStr">
+        <is>
+          <t>A galvanised boot tray with a pair of rubber galoshes and dried mud (boottray form) against the south wall at (6.67, 6.62), clear of every door and opening approach (each opening's span plus 0.15 m, 1.0 m deep), the stances and a 0.85 m route. The hamper's cane panels read as a lidded box rather than a woven basket and the galoshes are plain blocks; finer weave and boot forms are later art. Verified at 2152694f (slice14b) and 4fc1b18d (slice14c, after 2A's and 3A's objects moved to the north end wall out of the door route): the thirteen families pass the fabrication batch (25,826 checks, 0 failures; every hall object bearing inside its hall), apartment batch 236 as before, the apartment door route 45 waypoints and the 4B route 32 with 0 failures, the six completion routes unchanged (1A 15, 1D 25, 2C 9, 3D 16, 4C 9, 4D 12), upper lighting 0 failures, upper furniture 444 identical to slice 13 (slice14base), the eighteen-hall sweep 0 failures; captures in implementation/slice14b and slice14c.</t>
+        </is>
+      </c>
     </row>
     <row r="489">
       <c r="A489" s="2" t="inlineStr">
@@ -37751,10 +37811,14 @@
       </c>
       <c r="S521" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T521" s="2" t="inlineStr"/>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="T521" s="2" t="inlineStr">
+        <is>
+          <t>A gear crate (a copy of 6A_gearcrate) against the east wall at (-5.87, -8.48), clear of every door and opening approach (each opening's span plus 0.15 m, 1.0 m deep), the stances and a 0.85 m route. The hamper's cane panels read as a lidded box rather than a woven basket and the galoshes are plain blocks; finer weave and boot forms are later art. Verified at 2152694f (slice14b) and 4fc1b18d (slice14c, after 2A's and 3A's objects moved to the north end wall out of the door route): the thirteen families pass the fabrication batch (25,826 checks, 0 failures; every hall object bearing inside its hall), apartment batch 236 as before, the apartment door route 45 waypoints and the 4B route 32 with 0 failures, the six completion routes unchanged (1A 15, 1D 25, 2C 9, 3D 16, 4C 9, 4D 12), upper lighting 0 failures, upper furniture 444 identical to slice 13 (slice14base), the eighteen-hall sweep 0 failures; captures in implementation/slice14b and slice14c.</t>
+        </is>
+      </c>
     </row>
     <row r="522">
       <c r="A522" s="2" t="inlineStr">
@@ -38891,10 +38955,14 @@
       </c>
       <c r="S537" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T537" s="2" t="inlineStr"/>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="T537" s="2" t="inlineStr">
+        <is>
+          <t>A lidded wicker laundry hamper (hamper form) with a linen corner caught under the lid against the north wall at (-10.83, 11.38), clear of every door and opening approach (each opening's span plus 0.15 m, 1.0 m deep), the stances and a 0.85 m route. The hamper's cane panels read as a lidded box rather than a woven basket and the galoshes are plain blocks; finer weave and boot forms are later art. Verified at 2152694f (slice14b) and 4fc1b18d (slice14c, after 2A's and 3A's objects moved to the north end wall out of the door route): the thirteen families pass the fabrication batch (25,826 checks, 0 failures; every hall object bearing inside its hall), apartment batch 236 as before, the apartment door route 45 waypoints and the 4B route 32 with 0 failures, the six completion routes unchanged (1A 15, 1D 25, 2C 9, 3D 16, 4C 9, 4D 12), upper lighting 0 failures, upper furniture 444 identical to slice 13 (slice14base), the eighteen-hall sweep 0 failures; captures in implementation/slice14b and slice14c.</t>
+        </is>
+      </c>
     </row>
     <row r="538">
       <c r="A538" s="2" t="inlineStr">
@@ -39985,10 +40053,14 @@
       </c>
       <c r="S552" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T552" s="2" t="inlineStr"/>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="T552" s="2" t="inlineStr">
+        <is>
+          <t>A galvanised boot tray with a pair of rubber galoshes and dried mud (boottray form) against the south wall at (6.67, 6.62), clear of every door and opening approach (each opening's span plus 0.15 m, 1.0 m deep), the stances and a 0.85 m route. The hamper's cane panels read as a lidded box rather than a woven basket and the galoshes are plain blocks; finer weave and boot forms are later art. Verified at 2152694f (slice14b) and 4fc1b18d (slice14c, after 2A's and 3A's objects moved to the north end wall out of the door route): the thirteen families pass the fabrication batch (25,826 checks, 0 failures; every hall object bearing inside its hall), apartment batch 236 as before, the apartment door route 45 waypoints and the 4B route 32 with 0 failures, the six completion routes unchanged (1A 15, 1D 25, 2C 9, 3D 16, 4C 9, 4D 12), upper lighting 0 failures, upper furniture 444 identical to slice 13 (slice14base), the eighteen-hall sweep 0 failures; captures in implementation/slice14b and slice14c.</t>
+        </is>
+      </c>
     </row>
     <row r="553">
       <c r="A553" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Implement dossier slice 15: wall art in the residents' rooms
- A photograph style for the wall-art form: moulding, linen mat and a
  toned print.
- F02_C_MAIN-002: 2C's album pair on the window wall; F03_D_MAIN-003: 3D's
  three images far apart on the long wall (completion copies);
  F03_A_MAIN-003: 3A's diagram and portrait beside the private-hall door;
  F05_B_MAIN-004: 5B's two works off the window's centre.
- F02_A_MAIN-002: 2A's caption wall, a 1.2 x 0.9 m pinboard between the
  west windows, above the wire shelf.

Evidence under implementation/slice15/. INERT: no ledger status changes.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/art/reviews/v2_environment_design_20261008/change_register.xlsx
+++ b/art/reviews/v2_environment_design_20261008/change_register.xlsx
@@ -15025,10 +15025,14 @@
       </c>
       <c r="S210" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T210" s="2" t="inlineStr"/>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="T210" s="2" t="inlineStr">
+        <is>
+          <t>2A_caption_wall: a 1.2 x 0.9 m pinboard (24 cards in rows) on the west wall between the two windows. Deviations: it hangs above 2A_shelf1 (bottom 1.62 m, centre 2.07 m) because the shelf stands 1.6 m tall on that wall; the red threads and the one deliberately blank card wait for a thread form and a card-level distinction. Verified at 260cffe6 (slice15): the thirteen families pass the fabrication batch (26,116 checks, 0 failures; objects 78 actors, every frame, canvas and board bearing on its actual wall face), apartment batch 236 as before, upper lighting 0 failures, completion route 3D 16 waypoints as before, the household save owner 0 failures, the five-space sweep 0 failures; captures in implementation/slice15.</t>
+        </is>
+      </c>
     </row>
     <row r="211">
       <c r="A211" s="2" t="inlineStr">
@@ -17523,10 +17527,14 @@
       </c>
       <c r="S243" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T243" s="2" t="inlineStr"/>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="T243" s="2" t="inlineStr">
+        <is>
+          <t>2C_album_a/b: two photographs (artframe form, photo style: moulding, linen mat, a toned print) 0.5 m apart at 1.5 m on the window wall west of the window, nothing between them. Verified at 260cffe6 (slice15): the thirteen families pass the fabrication batch (26,116 checks, 0 failures; objects 78 actors, every frame, canvas and board bearing on its actual wall face), apartment batch 236 as before, upper lighting 0 failures, completion route 3D 16 waypoints as before, the household save owner 0 failures, the five-space sweep 0 failures; captures in implementation/slice15.</t>
+        </is>
+      </c>
     </row>
     <row r="244">
       <c r="A244" s="2" t="inlineStr">
@@ -20323,10 +20331,14 @@
       </c>
       <c r="S281" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T281" s="2" t="inlineStr"/>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="T281" s="2" t="inlineStr">
+        <is>
+          <t>3A_diagram (a copy of 4A's document frame standing for the propagation diagram) and 3A_portrait (photo style, the sepia plate) 0.4 m apart at 1.5 m on the north wall between the kitchen opening and the private-hall door, clear of the plants. The diagram's line drawing is a blank sheet (no lettering or line decals in textures). Verified at 260cffe6 (slice15): the thirteen families pass the fabrication batch (26,116 checks, 0 failures; objects 78 actors, every frame, canvas and board bearing on its actual wall face), apartment batch 236 as before, upper lighting 0 failures, completion route 3D 16 waypoints as before, the household save owner 0 failures, the five-space sweep 0 failures; captures in implementation/slice15.</t>
+        </is>
+      </c>
     </row>
     <row r="282">
       <c r="A282" s="2" t="inlineStr">
@@ -22645,10 +22657,14 @@
       </c>
       <c r="S312" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T312" s="2" t="inlineStr"/>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="T312" s="2" t="inlineStr">
+        <is>
+          <t>3D_image_a/b/c: three photographs (completion copies of 2C's) at 1.5 m on the long north wall, 2.3 m apart, the middle one over the chaise. Verified at 260cffe6 (slice15): the thirteen families pass the fabrication batch (26,116 checks, 0 failures; objects 78 actors, every frame, canvas and board bearing on its actual wall face), apartment batch 236 as before, upper lighting 0 failures, completion route 3D 16 waypoints as before, the household save owner 0 failures, the five-space sweep 0 failures; captures in implementation/slice15.</t>
+        </is>
+      </c>
     </row>
     <row r="313">
       <c r="A313" s="2" t="inlineStr">
@@ -33743,10 +33759,14 @@
       </c>
       <c r="S465" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T465" s="2" t="inlineStr"/>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="T465" s="2" t="inlineStr">
+        <is>
+          <t>5B_work_a/b: two canvases (copies of 5C's diptych forms) 1.0 m apart at 1.5 m on the window wall south of the window, off the window's centre line. Verified at 260cffe6 (slice15): the thirteen families pass the fabrication batch (26,116 checks, 0 failures; objects 78 actors, every frame, canvas and board bearing on its actual wall face), apartment batch 236 as before, upper lighting 0 failures, completion route 3D 16 waypoints as before, the household save owner 0 failures, the five-space sweep 0 failures; captures in implementation/slice15.</t>
+        </is>
+      </c>
     </row>
     <row r="466">
       <c r="A466" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Implement dossier slice 16: bedside and tabletop stock
Eight small forms in surface_stock_geometry.py (spectacles, pencil,
booklet, wallet, folding rule, open case, a pair of gloves, hammer) and
eleven records on the clear strips of the nightstand tops and on 5C's
table: 1A's spectacles and red pencil, 3A's seed catalogue, 4A's
pocketbook, 5A's folding rule and notebook, 6A's empty case, 4C's gloves
and condition card, 5C's hammer and tack tin (175 assemblies). Covers
F01_A_BED-002, F03_A_BED-001, F04_A_BED-001, F05_A_BED-001, F06_A_BED-001,
F04_C_BED2-001 and F05_C_MAIN-002, each with its remaining pieces noted.

The surface-stock suite's close-up captures are selectable with
ORISON_STOCK_CAPTURE_IDS.

Evidence under implementation/slice16 and slice16c/. INERT: no ledger status changes.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/art/reviews/v2_environment_design_20261008/change_register.xlsx
+++ b/art/reviews/v2_environment_design_20261008/change_register.xlsx
@@ -11739,10 +11739,14 @@
       </c>
       <c r="S167" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T167" s="2" t="inlineStr"/>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="T167" s="2" t="inlineStr">
+        <is>
+          <t>On 1A_bedside: folded spectacles (spectacles form) in the back strip and the red pencil (pencil form) along the front edge, beside the nightstand's own glass. The dosing spoon waits for a spoon form. Verified at 82e2fbb9 (slice16) and 42a4a0db (slice16c, the same runtime tree with the surface-stock close-ups made selectable): the thirteen families pass the fabrication batch (26,426 checks, 0 failures; 175 stock assemblies, every new piece bearing on its nightstand or table top clear of the baked book and glass), apartment batch 236 as before, completion routes 1A 15 and 4C 9 as before, upper lighting and the household save owner 0 failures, the seven-space sweep 0 failures; close-ups in implementation/slice16c (1A's nightstand has no clear camera station, so its spectacles and pencil rest on the bearing check alone).</t>
+        </is>
+      </c>
     </row>
     <row r="168">
       <c r="A168" s="2" t="inlineStr">
@@ -21075,10 +21079,14 @@
       </c>
       <c r="S291" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T291" s="2" t="inlineStr"/>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="T291" s="2" t="inlineStr">
+        <is>
+          <t>3A_seed_catalogue (booklet form) on 3A_bed0_ns's front strip. The seedling tray on the north sill waits for a sill support in the stock inspector. Verified at 82e2fbb9 (slice16) and 42a4a0db (slice16c, the same runtime tree with the surface-stock close-ups made selectable): the thirteen families pass the fabrication batch (26,426 checks, 0 failures; 175 stock assemblies, every new piece bearing on its nightstand or table top clear of the baked book and glass), apartment batch 236 as before, completion routes 1A 15 and 4C 9 as before, upper lighting and the household save owner 0 failures, the seven-space sweep 0 failures; close-ups in implementation/slice16c (1A's nightstand has no clear camera station, so its spectacles and pencil rest on the bearing check alone).</t>
+        </is>
+      </c>
     </row>
     <row r="292">
       <c r="A292" s="2" t="inlineStr">
@@ -26535,10 +26543,14 @@
       </c>
       <c r="S365" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T365" s="2" t="inlineStr"/>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="T365" s="2" t="inlineStr">
+        <is>
+          <t>4A_pocketbook: an overfilled wallet with a folded note's corner showing (wallet form) on 4A_bed0_ns. The brown sack suit waits for wardrobe garment sets. Verified at 82e2fbb9 (slice16) and 42a4a0db (slice16c, the same runtime tree with the surface-stock close-ups made selectable): the thirteen families pass the fabrication batch (26,426 checks, 0 failures; 175 stock assemblies, every new piece bearing on its nightstand or table top clear of the baked book and glass), apartment batch 236 as before, completion routes 1A 15 and 4C 9 as before, upper lighting and the household save owner 0 failures, the seven-space sweep 0 failures; close-ups in implementation/slice16c (1A's nightstand has no clear camera station, so its spectacles and pencil rest on the bearing check alone).</t>
+        </is>
+      </c>
     </row>
     <row r="366">
       <c r="A366" s="2" t="inlineStr">
@@ -29361,10 +29373,14 @@
       </c>
       <c r="S404" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T404" s="2" t="inlineStr"/>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="T404" s="2" t="inlineStr">
+        <is>
+          <t>4C_gloves (a pair, gloves form) and 4C_condition_card (booklet form) on 4C_bed1_ns. The slippers under the bed wait for a slipper form. Verified at 82e2fbb9 (slice16) and 42a4a0db (slice16c, the same runtime tree with the surface-stock close-ups made selectable): the thirteen families pass the fabrication batch (26,426 checks, 0 failures; 175 stock assemblies, every new piece bearing on its nightstand or table top clear of the baked book and glass), apartment batch 236 as before, completion routes 1A 15 and 4C 9 as before, upper lighting and the household save owner 0 failures, the seven-space sweep 0 failures; close-ups in implementation/slice16c (1A's nightstand has no clear camera station, so its spectacles and pencil rest on the bearing check alone).</t>
+        </is>
+      </c>
     </row>
     <row r="405">
       <c r="A405" s="2" t="inlineStr">
@@ -33101,10 +33117,14 @@
       </c>
       <c r="S456" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T456" s="2" t="inlineStr"/>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="T456" s="2" t="inlineStr">
+        <is>
+          <t>5A_fold_rule (folding rule form, four leaves and brass rivets) and 5A_notebook (booklet form) on 5A_bed0_ns. The reading lamp waits for the task-lamp installations. Verified at 82e2fbb9 (slice16) and 42a4a0db (slice16c, the same runtime tree with the surface-stock close-ups made selectable): the thirteen families pass the fabrication batch (26,426 checks, 0 failures; 175 stock assemblies, every new piece bearing on its nightstand or table top clear of the baked book and glass), apartment batch 236 as before, completion routes 1A 15 and 4C 9 as before, upper lighting and the household save owner 0 failures, the seven-space sweep 0 failures; close-ups in implementation/slice16c (1A's nightstand has no clear camera station, so its spectacles and pencil rest on the bearing check alone).</t>
+        </is>
+      </c>
     </row>
     <row r="457">
       <c r="A457" s="2" t="inlineStr">
@@ -34923,10 +34943,14 @@
       </c>
       <c r="S481" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T481" s="2" t="inlineStr"/>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="T481" s="2" t="inlineStr">
+        <is>
+          <t>5C_hammer (hammer form) and a tin of tacks on 5C_din_t, beside the solvents and studies. The half-stretched canvas and the stretcher stack wait for a canvas-in-progress form. Verified at 82e2fbb9 (slice16) and 42a4a0db (slice16c, the same runtime tree with the surface-stock close-ups made selectable): the thirteen families pass the fabrication batch (26,426 checks, 0 failures; 175 stock assemblies, every new piece bearing on its nightstand or table top clear of the baked book and glass), apartment batch 236 as before, completion routes 1A 15 and 4C 9 as before, upper lighting and the household save owner 0 failures, the seven-space sweep 0 failures; close-ups in implementation/slice16c (1A's nightstand has no clear camera station, so its spectacles and pencil rest on the bearing check alone).</t>
+        </is>
+      </c>
     </row>
     <row r="482">
       <c r="A482" s="2" t="inlineStr">
@@ -38111,10 +38135,14 @@
       </c>
       <c r="S525" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T525" s="2" t="inlineStr"/>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="T525" s="2" t="inlineStr">
+        <is>
+          <t>6A_empty_case: an open leather case with its lining showing (case form) on 6A_bed0_ns. The strap on the bedpost waits for a cloth strap form. Verified at 82e2fbb9 (slice16) and 42a4a0db (slice16c, the same runtime tree with the surface-stock close-ups made selectable): the thirteen families pass the fabrication batch (26,426 checks, 0 failures; 175 stock assemblies, every new piece bearing on its nightstand or table top clear of the baked book and glass), apartment batch 236 as before, completion routes 1A 15 and 4C 9 as before, upper lighting and the household save owner 0 failures, the seven-space sweep 0 failures; close-ups in implementation/slice16c (1A's nightstand has no clear camera station, so its spectacles and pencil rest on the bearing check alone).</t>
+        </is>
+      </c>
     </row>
     <row r="526">
       <c r="A526" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Implement dossier slice 17: 2B's bedside and client chair, 3A's pail, 4D's luggage
- F02_B_BED-001: 2B_bedside (Nightstand01 copy) at the bed head on the
  door side, a standing photograph on it.
- F02_B_VESTIBULE-003: 2B_client_chair (ChairOak copy) in the vestibule
  corner beside the opening, a parcel of finished work on its seat.
- F03_A_KITCHEN-004: 3A's compost pail (galvanised can) beside the sink
  support, clear of the stances.
- F04_D_VESTIBULE-003: a suitcase form in the domestic objects family
  (leather case on edge, straps, brass feet, handle) for 4D's luggage.

Evidence under implementation/slice17b and slice17/. INERT: no ledger status changes.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/art/reviews/v2_environment_design_20261008/change_register.xlsx
+++ b/art/reviews/v2_environment_design_20261008/change_register.xlsx
@@ -16237,10 +16237,14 @@
       </c>
       <c r="S226" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T226" s="2" t="inlineStr"/>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="T226" s="2" t="inlineStr">
+        <is>
+          <t>2B_client_chair (a ChairOak copy) in the vestibule corner north of the opening, facing into the vestibule, clear of the entry-leaf sweep and the route to the main room (the first placement, south of the opening, stood in the door route: slice17); 2B_finished_parcel (parcel form) on its seat. Verified at 7eeaa0ef (slice17b): the thirteen families pass the fabrication batch (26,568 checks, 0 failures; tables 73, seating 52, objects 79, stock 178, the parcel bearing on the chair seat and the pail on the floor), apartment batch 236 as before, the apartment door route 45 and the 4B route 32 waypoints with 0 failures, completion route 4D 12 waypoints as before, upper lighting and the household save owner 0 failures, the four-space sweep 0 failures; captures in implementation/slice17b.</t>
+        </is>
+      </c>
     </row>
     <row r="227">
       <c r="A227" s="2" t="inlineStr">
@@ -17043,10 +17047,14 @@
       </c>
       <c r="S237" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T237" s="2" t="inlineStr"/>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="T237" s="2" t="inlineStr">
+        <is>
+          <t>2B_bedside (a Nightstand01 copy) at the head of the bed on the door side, with 2B_photo (standing frame form) in the clear back strip beside the nightstand's own book and glass. The mirror waits for the mirror family's wall variant. Verified at 7eeaa0ef (slice17b): the thirteen families pass the fabrication batch (26,568 checks, 0 failures; tables 73, seating 52, objects 79, stock 178, the parcel bearing on the chair seat and the pail on the floor), apartment batch 236 as before, the apartment door route 45 and the 4B route 32 waypoints with 0 failures, completion route 4D 12 waypoints as before, upper lighting and the household save owner 0 failures, the four-space sweep 0 failures; captures in implementation/slice17b.</t>
+        </is>
+      </c>
     </row>
     <row r="238">
       <c r="A238" s="2" t="inlineStr">
@@ -20779,10 +20787,14 @@
       </c>
       <c r="S287" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T287" s="2" t="inlineStr"/>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="T287" s="2" t="inlineStr">
+        <is>
+          <t>3A_compost_pail (the galvanised can form) on the floor at the east end of the sink support, clear of the tap and stove stances. Deviation: beside the sink support rather than under it (the frame's underside is not a clear bearing), galvanised rather than enamel. Verified at 7eeaa0ef (slice17b): the thirteen families pass the fabrication batch (26,568 checks, 0 failures; tables 73, seating 52, objects 79, stock 178, the parcel bearing on the chair seat and the pail on the floor), apartment batch 236 as before, the apartment door route 45 and the 4B route 32 waypoints with 0 failures, completion route 4D 12 waypoints as before, upper lighting and the household save owner 0 failures, the four-space sweep 0 failures; captures in implementation/slice17b.</t>
+        </is>
+      </c>
     </row>
     <row r="288">
       <c r="A288" s="2" t="inlineStr">
@@ -29611,10 +29623,14 @@
       </c>
       <c r="S407" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T407" s="2" t="inlineStr"/>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="T407" s="2" t="inlineStr">
+        <is>
+          <t>4D_case (new suitcase form: a leather case on its long edge with two straps, brass feet and a handle) in the vestibule's north-west corner, clear of the three doors' approaches. The gladstone and the rules card on the door back wait for their forms. Verified at 7eeaa0ef (slice17b): the thirteen families pass the fabrication batch (26,568 checks, 0 failures; tables 73, seating 52, objects 79, stock 178, the parcel bearing on the chair seat and the pail on the floor), apartment batch 236 as before, the apartment door route 45 and the 4B route 32 waypoints with 0 failures, completion route 4D 12 waypoints as before, upper lighting and the household save owner 0 failures, the four-space sweep 0 failures; captures in implementation/slice17b.</t>
+        </is>
+      </c>
     </row>
     <row r="408">
       <c r="A408" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Implement dossier slice 18: sewing machine, radio teardown, easel and canvases
Four studio forms in the domestic objects family:

- F02_B_MAIN-001: a treadle sewing machine (cast-iron legs and treadle on
  an axle, oak top and drawer, japanned head with needle and handwheel)
  under 2B's east window, passive.
- F03_B_MAIN-001: a radio teardown on newspaper (open chassis, three loose
  valves, a saucer of screws) on 3B's floor beside the parts crate.
- F05_C_BED2-002: an easel with a blank canvas on its ledge by 5C's window,
  and six failed canvases standing face to the wall beside the door.

Evidence under implementation/slice18/. INERT: no ledger status changes.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/art/reviews/v2_environment_design_20261008/change_register.xlsx
+++ b/art/reviews/v2_environment_design_20261008/change_register.xlsx
@@ -16331,10 +16331,14 @@
       </c>
       <c r="S227" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T227" s="2" t="inlineStr"/>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="T227" s="2" t="inlineStr">
+        <is>
+          <t>2B_sewing_machine (new sewingmachine form: cast-iron legs, rails and treadle on an axle, an oak top and drawer, a black japanned head with its needle, needle plate and handwheel) under the east window with the treadle toward the room. Deviation: passive; the treadle OPERATE owner (treadle turns, needle drops) waits for a mechanism pass. Verified at d0108d15 (slice18): the thirteen families pass the fabrication batch (26,770 checks, 0 failures; objects 83 actors, every new piece standing on its floor inside its room and clear of its neighbours), apartment batch 236 as before, the apartment door route 45 and the 4B route 32 waypoints with 0 failures, upper lighting and the household save owner 0 failures, the three-space sweep 0 failures; native close-ups in implementation/slice18.</t>
+        </is>
+      </c>
     </row>
     <row r="228">
       <c r="A228" s="2" t="inlineStr">
@@ -21353,10 +21357,14 @@
       </c>
       <c r="S294" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T294" s="2" t="inlineStr"/>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="T294" s="2" t="inlineStr">
+        <is>
+          <t>3B_teardown (new teardown form: a newspaper sheet, an open chassis with three empty valve sockets, three loose valves standing on the sheet, a saucer of screws) on the floor north of the parts crate, beside the hall opening's approach. Passive, never a live receiver; the INSPECT card waits for the matrix pass. Verified at d0108d15 (slice18): the thirteen families pass the fabrication batch (26,770 checks, 0 failures; objects 83 actors, every new piece standing on its floor inside its room and clear of its neighbours), apartment batch 236 as before, the apartment door route 45 and the 4B route 32 waypoints with 0 failures, upper lighting and the household save owner 0 failures, the three-space sweep 0 failures; native close-ups in implementation/slice18.</t>
+        </is>
+      </c>
     </row>
     <row r="295">
       <c r="A295" s="2" t="inlineStr">
@@ -36041,10 +36049,14 @@
       </c>
       <c r="S496" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T496" s="2" t="inlineStr"/>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="T496" s="2" t="inlineStr">
+        <is>
+          <t>5C_easel (new easel form: splayed front legs and a back leg on foot pads, a ledge holding a blank canvas under the top clamp) by the window east of the stool, the canvas facing the stool so the window is on the painter's left; 5C_failed_canvases (new canvasstack form: six canvases standing face to the wall, stretcher backs to the room, a pencil mark on each) west of the door, outside its swing. The pigment table and stool were already placed; the drying rack, wash jar and drop cloth wait for their forms. Verified at d0108d15 (slice18): the thirteen families pass the fabrication batch (26,770 checks, 0 failures; objects 83 actors, every new piece standing on its floor inside its room and clear of its neighbours), apartment batch 236 as before, the apartment door route 45 and the 4B route 32 waypoints with 0 failures, upper lighting and the household save owner 0 failures, the three-space sweep 0 failures; native close-ups in implementation/slice18.</t>
+        </is>
+      </c>
     </row>
     <row r="497">
       <c r="A497" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Implement dossier slice 19: propagation shelves, covered objects, card cabinet
- F03_A_MAIN-001: two low oak shelf variants (Shelf09, Shelf10) under 3A's
  west windows with rows of lidded glass seed jars, one jar missing at the
  north end.
- F06_C_BED2-002: cloth-covered objects on 6C's archive shelves and a
  card-index cabinet form (twelve drawers, brass pulls, blank label frames,
  a brass lock plate on the provenance drawer).
- F04_C_MAIN-002: covered objects and a folded cloth on 4C's museum shelf.
- Surface stock: seedjars, seedjarsgap, covered and foldedcloth forms; the
  family gains the catalogue linen key (187 assemblies).

Evidence under implementation/slice19/. INERT: no ledger status changes.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/art/reviews/v2_environment_design_20261008/change_register.xlsx
+++ b/art/reviews/v2_environment_design_20261008/change_register.xlsx
@@ -20207,10 +20207,14 @@
       </c>
       <c r="S279" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T279" s="2" t="inlineStr"/>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="T279" s="2" t="inlineStr">
+        <is>
+          <t>3A_prop_shelf_s/_n: two low oak shelves (Shelf09 1.5 m and Shelf10 1.2 m, two boards, 0.72 m, so they stand under the 0.75 m sills) under the two west windows either side of the potting bench, each with two rows of lidded glass seed jars (seedjars form); the north row lacks one jar at its end (seedjarsgap form). Deviations: two shelves rather than one 2.4 m span because the potting bench stands between the windows; jars hold no soil or seedlings yet (no soil or plant key in the stock family). Verified at 7813b06c (slice19): the thirteen families pass the fabrication batch (27,146 checks, 0 failures; storage 52, objects 84, stock 187, every jar, cover and fold bearing on its board), apartment batch 236 as before, completion route 4C 9 waypoints as before, upper lighting and the household save owner 0 failures, the three-space sweep 0 failures; close-ups in implementation/slice19.</t>
+        </is>
+      </c>
     </row>
     <row r="280">
       <c r="A280" s="2" t="inlineStr">
@@ -28484,7 +28488,7 @@
       </c>
       <c r="T391" s="2" t="inlineStr">
         <is>
-          <t>4C_museum_shelf (Shelf01) on the window wall beside the window; the covered objects, cloth and the courier corner's floor stock stay with the desktop_stock items. (implementation/slice6/images/F04_C_MAIN_OV.jpg)</t>
+          <t>4C_museum_shelf (Shelf01) on the window wall beside the window; the courier corner's floor stock stays with the desktop_stock items. (implementation/slice6/images/F04_C_MAIN_OV.jpg) Slice 19 adds Noel's museum bay on it: three cloth-covered objects and a folded cloth (covered and foldedcloth forms), verified at 7813b06c (implementation/slice19/images/4C_covered_a_stock.jpg).</t>
         </is>
       </c>
     </row>
@@ -40561,10 +40565,14 @@
       </c>
       <c r="S558" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T558" s="2" t="inlineStr"/>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="T558" s="2" t="inlineStr">
+        <is>
+          <t>Three cloth-covered objects (covered form: an object under a linen drape) on the existing 6C_archive_shelf_01/02 boards, and 6C_card_cabinet (new cardcabinet form: twelve drawers with brass pulls and blank label frames, one drawer with a brass lock plate for the provenance drawer) against the south wall west of the door. Deviations: the cabinet stands by the door because the archive table holds the window; the locked drawer is passive (its RESIST-REFUSE owner waits for the matrix pass). Verified at 7813b06c (slice19): the thirteen families pass the fabrication batch (27,146 checks, 0 failures; storage 52, objects 84, stock 187, every jar, cover and fold bearing on its board), apartment batch 236 as before, completion route 4C 9 waypoints as before, upper lighting and the household save owner 0 failures, the three-space sweep 0 failures; close-ups in implementation/slice19.</t>
+        </is>
+      </c>
     </row>
     <row r="559">
       <c r="A559" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Implement dossier slice 20: 2A's box files, 6A's backdrop and print line
- F02_A_MAIN-001: rows of labelled box files (new fileboxes surface-stock
  form) on the clear upper boards of 2A's three shelves (192 assemblies).
- F06_A_MAIN-001: a backdrop rail form (header, brackets, rail, paper roll
  and hanging sheet) on 6A's west wall.
- F06_A_MAIN-002: a print line form (hook plates, string, six pegged
  contact sheets of small frames) on 6A's south wall.

Evidence under implementation/slice20/. INERT: no ledger status changes.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/art/reviews/v2_environment_design_20261008/change_register.xlsx
+++ b/art/reviews/v2_environment_design_20261008/change_register.xlsx
@@ -14947,10 +14947,14 @@
       </c>
       <c r="S209" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T209" s="2" t="inlineStr"/>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="T209" s="2" t="inlineStr">
+        <is>
+          <t>Rows of seven labelled box files (fileboxes form: cloth-covered boxes in navy, green, burgundy and brown, a blank paper label and a brass pull on each) on the clear upper boards of 2A_shelf0, 2A_shelf1 and 2A_shelf2, labels facing the room, so the three units read as matching labelled storage. Deviations: the units keep their oak frames (the BW-003 posts already replaced the wire) and their own bins and tins on the lower boards; the labels are blank (no lettering in textures). Verified at ccdf39bf (slice20): the thirteen families pass the fabrication batch (27,601 checks, 0 failures; objects 86, stock 192, the rail and print line on their actual wall faces, the box files on the clear boards), apartment batch 236 as before, upper lighting and the household save owner 0 failures, the two-space sweep 0 failures; close-ups in implementation/slice20.</t>
+        </is>
+      </c>
     </row>
     <row r="210">
       <c r="A210" s="2" t="inlineStr">
@@ -37397,10 +37401,14 @@
       </c>
       <c r="S514" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T514" s="2" t="inlineStr"/>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="T514" s="2" t="inlineStr">
+        <is>
+          <t>6A_backdrop_rail (new backdroprail form: header strip on rear battens, two brackets, a rail and a paper roll with its sheet hanging almost to the floor) on the west wall south of the window, the rail at 2.2 m, clear of the tripod, softboxes and crate. The charging bench and the folding chair wait for a work-table copy and a folding-chair seating variant. Verified at ccdf39bf (slice20): the thirteen families pass the fabrication batch (27,601 checks, 0 failures; objects 86, stock 192, the rail and print line on their actual wall faces, the box files on the clear boards), apartment batch 236 as before, upper lighting and the household save owner 0 failures, the two-space sweep 0 failures; close-ups in implementation/slice20.</t>
+        </is>
+      </c>
     </row>
     <row r="515">
       <c r="A515" s="2" t="inlineStr">
@@ -37463,10 +37471,14 @@
       </c>
       <c r="S515" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T515" s="2" t="inlineStr"/>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="T515" s="2" t="inlineStr">
+        <is>
+          <t>6A_print_line (new printline form: two hook plates, a string at 1.9 m and six pegged contact sheets, each a grid of small dark frames, no lettering) on the south wall east of the bed door. The hero contact sheet above a bench waits for the charging bench. Verified at ccdf39bf (slice20): the thirteen families pass the fabrication batch (27,601 checks, 0 failures; objects 86, stock 192, the rail and print line on their actual wall faces, the box files on the clear boards), apartment batch 236 as before, upper lighting and the household save owner 0 failures, the two-space sweep 0 failures; close-ups in implementation/slice20.</t>
+        </is>
+      </c>
     </row>
     <row r="516">
       <c r="A516" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Implement dossier slice 21: lobby noticeboard and photograph, common-room armchair
- F01_LOBBY-001: a 1.2 x 0.9 m noticeboard (pinboard variant, notices in
  rows) on the lobby's south wall between the west window and the inner
  door, above the dado cap.
- F01_LOBBY-002: the 1928 photograph (photograph frame copy) beside the
  inner door; the reference clock waits for a V2 clock owner.
- F01_COMMON_B-001: an armchair (Armchair copy) in the common room's
  window corner, clear of the reading table and bookcases.
- 5A's plan wall (slice 12) moves to the card grid too: the drifted card
  layout of the V1 pinboard collapses into diagonal streaks.

Evidence under implementation/slice21, slice21b, slice21c and slice21base/. INERT: no ledger
status changes.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/art/reviews/v2_environment_design_20261008/change_register.xlsx
+++ b/art/reviews/v2_environment_design_20261008/change_register.xlsx
@@ -8609,10 +8609,14 @@
       </c>
       <c r="S124" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T124" s="2" t="inlineStr"/>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="T124" s="2" t="inlineStr">
+        <is>
+          <t>F01_lobby_board: a 1.2 x 0.9 m noticeboard (pinboard form, 23 notices in rows, one brass pin each, no lettering) on the south wall between the west window and the inner door, its lower edge above the dado cap at 1.42 m. Deviation: the notices are blank cards in rows (the drifted layout collapses into streaks), and the board is a passive pinboard rather than the 23-piece authored LobbyBulletinBoard owner. Verified at 9120c99a (slice21: reading furniture 25 and public furnishings 29 waypoints with 0 failures and the blockout suite passing, as at 858fb707 in slice21base; apartment batch 236 as before) and at 85f7dfc0 (slice21c, after the board moved above the dado and the boards took the card grid): the thirteen families pass the fabrication batch (27,682 checks, 0 failures; every board and frame on its actual wall face), public furnishings 29 waypoints with 0 failures, apartment batch 236, the lobby sweep 0 failures; captures in implementation/slice21, slice21b and slice21c.</t>
+        </is>
+      </c>
     </row>
     <row r="125">
       <c r="A125" s="2" t="inlineStr">
@@ -8683,10 +8687,14 @@
       </c>
       <c r="S125" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T125" s="2" t="inlineStr"/>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="T125" s="2" t="inlineStr">
+        <is>
+          <t>F01_lobby_photo: the 1928 photograph (a copy of the photograph frame) at 1.5 m beside the inner door. The sealed Vantry reference clock over the core opening waits for a V2 clock owner (ClockProp is mounted only by the V1 building). Verified at 9120c99a (slice21: reading furniture 25 and public furnishings 29 waypoints with 0 failures and the blockout suite passing, as at 858fb707 in slice21base; apartment batch 236 as before) and at 85f7dfc0 (slice21c, after the board moved above the dado and the boards took the card grid): the thirteen families pass the fabrication batch (27,682 checks, 0 failures; every board and frame on its actual wall face), public furnishings 29 waypoints with 0 failures, apartment batch 236, the lobby sweep 0 failures; captures in implementation/slice21, slice21b and slice21c.</t>
+        </is>
+      </c>
     </row>
     <row r="126">
       <c r="A126" s="2" t="inlineStr">
@@ -9335,10 +9343,14 @@
       </c>
       <c r="S135" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T135" s="2" t="inlineStr"/>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="T135" s="2" t="inlineStr">
+        <is>
+          <t>F01_common_armchair (an Armchair copy) in the common room's south-west window corner, facing into the room, clear of the reading table, its chairs and the bookcases. The minutes, jug and glasses wait for the reading table to become a stock support; the floor lamp waits for the task-lamp installations. Verified at 9120c99a (slice21: reading furniture 25 and public furnishings 29 waypoints with 0 failures and the blockout suite passing, as at 858fb707 in slice21base; apartment batch 236 as before) and at 85f7dfc0 (slice21c, after the board moved above the dado and the boards took the card grid): the thirteen families pass the fabrication batch (27,682 checks, 0 failures; every board and frame on its actual wall face), public furnishings 29 waypoints with 0 failures, apartment batch 236, the lobby sweep 0 failures; captures in implementation/slice21, slice21b and slice21c.</t>
+        </is>
+      </c>
     </row>
     <row r="136">
       <c r="A136" s="2" t="inlineStr">
@@ -32232,7 +32244,7 @@
       </c>
       <c r="T443" s="2" t="inlineStr">
         <is>
-          <t>5A_plan_wall: a 1.6 x 1.0 m pinboard (DomesticObject18, 20 drifted sheets) on the north wall between the radiator and the bookshelf at 1.4 m. Deviations: the wall opposite the window is two openings and the switch, so the board takes the clear north wall; plan-line decals and red strokes wait for a sheet form (no lettering in textures). Verified at 76d0a584 (slice12) with the apartment batch at 394a9c3c (slice12b): the thirteen families pass the fabrication batch (25,164 checks, 0 failures; objects 44 actors, every board, canvas and frame bearing on its actual wall face), apartment batch 236 with failure labels identical to slice 11 once its category roster holds the original V1 set, upper lighting 0 failures, completion route 1A 15 waypoints as before, the household save owner 0 failures, the five-space sweep 0 failures; the rooms and native close-ups are in implementation/slice12.</t>
+          <t>5A_plan_wall: a 1.6 x 1.0 m pinboard (DomesticObject18, 20 sheets; in rows since slice 21, the drifted layout collapsing into streaks) on the north wall between the radiator and the bookshelf at 1.4 m. Deviations: the wall opposite the window is two openings and the switch, so the board takes the clear north wall; plan-line decals and red strokes wait for a sheet form (no lettering in textures). Verified at 76d0a584 (slice12) with the apartment batch at 394a9c3c (slice12b): the thirteen families pass the fabrication batch (25,164 checks, 0 failures; objects 44 actors, every board, canvas and frame bearing on its actual wall face), apartment batch 236 with failure labels identical to slice 11 once its category roster holds the original V1 set, upper lighting 0 failures, completion route 1A 15 waypoints as before, the household save owner 0 failures, the five-space sweep 0 failures; the rooms and native close-ups are in implementation/slice12.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Implement dossier slice 22: drip pans under the fourteen iceboxes
A driptray surface-stock form (zinc pan with rolled rims, a skin of water
or a dry dusty floor) under each of the fourteen iceboxes, between the
feet with the front lip showing, clear of the door and its stance: the
F0x_x_KITCHEN-002 items of 1D, 2A, 2B, 2C, 3B, 3D, 4A, 4B, 4C, 4D, 5A, 5C,
6A and 6B, and 4C's dry tray (F04_C_KITCHEN-003). The ice cards in the
window panes wait for a window-pane support (206 assemblies).

Slice 20's backdrop rail is narrowed to 1.2 m: the upper-kitchen suite
found its paper inside the tripod stance's capsule (now 238, as before).

Evidence under implementation/slice22 and slice22b/. INERT: no ledger status changes.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/art/reviews/v2_environment_design_20261008/change_register.xlsx
+++ b/art/reviews/v2_environment_design_20261008/change_register.xlsx
@@ -12789,10 +12789,14 @@
       </c>
       <c r="S180" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T180" s="2" t="inlineStr"/>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="T180" s="2" t="inlineStr">
+        <is>
+          <t>1D_drip_tray: a zinc drip pan holding a skin of water (driptray form) on the floor under the icebox, between its feet with the front lip showing, clear of the door stance and the door's swing. The ice card in the window pane waits for a window-pane support (the panes belong to the shell, not a furniture actor). Verified at 4444e1e1 (slice22) and db14e977 (slice22b, the 6A backdrop narrowed): the thirteen families pass the fabrication batch (28,045 checks, 0 failures; 206 stock assemblies, every pan bearing on the floor between its icebox's feet), apartment batch 236 as before, the six completion routes unchanged (1A 15, 1D 25, 2C 9, 3D 16, 4C 9, 4D 12), upper lighting and the household save owner 0 failures, upper kitchens 238 with the baseline's labels, the fourteen-kitchen sweep 0 failures; close-ups in implementation/slice22.</t>
+        </is>
+      </c>
     </row>
     <row r="181">
       <c r="A181" s="2" t="inlineStr">
@@ -15497,10 +15501,14 @@
       </c>
       <c r="S216" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T216" s="2" t="inlineStr"/>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="T216" s="2" t="inlineStr">
+        <is>
+          <t>2A_drip_tray: a zinc drip pan holding a skin of water (driptray form) on the floor under the icebox, between its feet with the front lip showing, clear of the door stance and the door's swing. The ice card in the window pane waits for a window-pane support (the panes belong to the shell, not a furniture actor). Verified at 4444e1e1 (slice22) and db14e977 (slice22b, the 6A backdrop narrowed): the thirteen families pass the fabrication batch (28,045 checks, 0 failures; 206 stock assemblies, every pan bearing on the floor between its icebox's feet), apartment batch 236 as before, the six completion routes unchanged (1A 15, 1D 25, 2C 9, 3D 16, 4C 9, 4D 12), upper lighting and the household save owner 0 failures, upper kitchens 238 with the baseline's labels, the fourteen-kitchen sweep 0 failures; close-ups in implementation/slice22.</t>
+        </is>
+      </c>
     </row>
     <row r="217">
       <c r="A217" s="2" t="inlineStr">
@@ -16733,10 +16741,14 @@
       </c>
       <c r="S232" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T232" s="2" t="inlineStr"/>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="T232" s="2" t="inlineStr">
+        <is>
+          <t>2B_drip_tray: a zinc drip pan holding a skin of water (driptray form) on the floor under the icebox, between its feet with the front lip showing, clear of the door stance and the door's swing. The ice card in the window pane waits for a window-pane support (the panes belong to the shell, not a furniture actor). Verified at 4444e1e1 (slice22) and db14e977 (slice22b, the 6A backdrop narrowed): the thirteen families pass the fabrication batch (28,045 checks, 0 failures; 206 stock assemblies, every pan bearing on the floor between its icebox's feet), apartment batch 236 as before, the six completion routes unchanged (1A 15, 1D 25, 2C 9, 3D 16, 4C 9, 4D 12), upper lighting and the household save owner 0 failures, upper kitchens 238 with the baseline's labels, the fourteen-kitchen sweep 0 failures; close-ups in implementation/slice22.</t>
+        </is>
+      </c>
     </row>
     <row r="233">
       <c r="A233" s="2" t="inlineStr">
@@ -17797,10 +17809,14 @@
       </c>
       <c r="S246" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T246" s="2" t="inlineStr"/>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="T246" s="2" t="inlineStr">
+        <is>
+          <t>2C_drip_tray: a zinc drip pan holding a skin of water (driptray form) on the floor under the icebox, between its feet with the front lip showing, clear of the door stance and the door's swing. The ice card in the window pane waits for a window-pane support (the panes belong to the shell, not a furniture actor). Verified at 4444e1e1 (slice22) and db14e977 (slice22b, the 6A backdrop narrowed): the thirteen families pass the fabrication batch (28,045 checks, 0 failures; 206 stock assemblies, every pan bearing on the floor between its icebox's feet), apartment batch 236 as before, the six completion routes unchanged (1A 15, 1D 25, 2C 9, 3D 16, 4C 9, 4D 12), upper lighting and the household save owner 0 failures, upper kitchens 238 with the baseline's labels, the fourteen-kitchen sweep 0 failures; close-ups in implementation/slice22.</t>
+        </is>
+      </c>
     </row>
     <row r="247">
       <c r="A247" s="2" t="inlineStr">
@@ -21809,10 +21825,14 @@
       </c>
       <c r="S300" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T300" s="2" t="inlineStr"/>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="T300" s="2" t="inlineStr">
+        <is>
+          <t>3B_drip_tray: a zinc drip pan holding a skin of water (driptray form) on the floor under the icebox, between its feet with the front lip showing, clear of the door stance and the door's swing. The ice card in the window pane waits for a window-pane support (the panes belong to the shell, not a furniture actor). Verified at 4444e1e1 (slice22) and db14e977 (slice22b, the 6A backdrop narrowed): the thirteen families pass the fabrication batch (28,045 checks, 0 failures; 206 stock assemblies, every pan bearing on the floor between its icebox's feet), apartment batch 236 as before, the six completion routes unchanged (1A 15, 1D 25, 2C 9, 3D 16, 4C 9, 4D 12), upper lighting and the household save owner 0 failures, upper kitchens 238 with the baseline's labels, the fourteen-kitchen sweep 0 failures; close-ups in implementation/slice22.</t>
+        </is>
+      </c>
     </row>
     <row r="301">
       <c r="A301" s="2" t="inlineStr">
@@ -22943,10 +22963,14 @@
       </c>
       <c r="S315" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T315" s="2" t="inlineStr"/>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="T315" s="2" t="inlineStr">
+        <is>
+          <t>3D_drip_tray: a zinc drip pan holding a skin of water (driptray form) on the floor under the icebox, between its feet with the front lip showing, clear of the door stance and the door's swing. The ice card in the window pane waits for a window-pane support (the panes belong to the shell, not a furniture actor). Verified at 4444e1e1 (slice22) and db14e977 (slice22b, the 6A backdrop narrowed): the thirteen families pass the fabrication batch (28,045 checks, 0 failures; 206 stock assemblies, every pan bearing on the floor between its icebox's feet), apartment batch 236 as before, the six completion routes unchanged (1A 15, 1D 25, 2C 9, 3D 16, 4C 9, 4D 12), upper lighting and the household save owner 0 failures, upper kitchens 238 with the baseline's labels, the fourteen-kitchen sweep 0 failures; close-ups in implementation/slice22.</t>
+        </is>
+      </c>
     </row>
     <row r="316">
       <c r="A316" s="2" t="inlineStr">
@@ -26069,10 +26093,14 @@
       </c>
       <c r="S358" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T358" s="2" t="inlineStr"/>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="T358" s="2" t="inlineStr">
+        <is>
+          <t>4A_drip_tray: a zinc drip pan holding a skin of water (driptray form) on the floor under the icebox, between its feet with the front lip showing, clear of the door stance and the door's swing. The ice card in the window pane waits for a window-pane support (the panes belong to the shell, not a furniture actor). Verified at 4444e1e1 (slice22) and db14e977 (slice22b, the 6A backdrop narrowed): the thirteen families pass the fabrication batch (28,045 checks, 0 failures; 206 stock assemblies, every pan bearing on the floor between its icebox's feet), apartment batch 236 as before, the six completion routes unchanged (1A 15, 1D 25, 2C 9, 3D 16, 4C 9, 4D 12), upper lighting and the household save owner 0 failures, upper kitchens 238 with the baseline's labels, the fourteen-kitchen sweep 0 failures; close-ups in implementation/slice22.</t>
+        </is>
+      </c>
     </row>
     <row r="359">
       <c r="A359" s="2" t="inlineStr">
@@ -27273,10 +27301,14 @@
       </c>
       <c r="S374" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T374" s="2" t="inlineStr"/>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="T374" s="2" t="inlineStr">
+        <is>
+          <t>4B_drip_tray: a zinc drip pan holding a skin of water (driptray form) on the floor under the icebox, between its feet with the front lip showing, clear of the door stance and the door's swing. The ice card in the window pane waits for a window-pane support (the panes belong to the shell, not a furniture actor). Verified at 4444e1e1 (slice22) and db14e977 (slice22b, the 6A backdrop narrowed): the thirteen families pass the fabrication batch (28,045 checks, 0 failures; 206 stock assemblies, every pan bearing on the floor between its icebox's feet), apartment batch 236 as before, the six completion routes unchanged (1A 15, 1D 25, 2C 9, 3D 16, 4C 9, 4D 12), upper lighting and the household save owner 0 failures, upper kitchens 238 with the baseline's labels, the fourteen-kitchen sweep 0 failures; close-ups in implementation/slice22.</t>
+        </is>
+      </c>
     </row>
     <row r="375">
       <c r="A375" s="2" t="inlineStr">
@@ -28861,10 +28893,14 @@
       </c>
       <c r="S396" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T396" s="2" t="inlineStr"/>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="T396" s="2" t="inlineStr">
+        <is>
+          <t>4C_drip_tray: a dry, dusty zinc drip pan (driptray form) on the floor under the icebox, between its feet with the front lip showing, clear of the door stance and the door's swing. The ice card in the window pane waits for a window-pane support (the panes belong to the shell, not a furniture actor). Verified at 4444e1e1 (slice22) and db14e977 (slice22b, the 6A backdrop narrowed): the thirteen families pass the fabrication batch (28,045 checks, 0 failures; 206 stock assemblies, every pan bearing on the floor between its icebox's feet), apartment batch 236 as before, the six completion routes unchanged (1A 15, 1D 25, 2C 9, 3D 16, 4C 9, 4D 12), upper lighting and the household save owner 0 failures, upper kitchens 238 with the baseline's labels, the fourteen-kitchen sweep 0 failures; close-ups in implementation/slice22.</t>
+        </is>
+      </c>
     </row>
     <row r="397">
       <c r="A397" s="2" t="inlineStr">
@@ -28923,10 +28959,14 @@
       </c>
       <c r="S397" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T397" s="2" t="inlineStr"/>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="T397" s="2" t="inlineStr">
+        <is>
+          <t>The dry tray: 4C_drip_tray is dry and dusty (driptraydry form) under the icebox. The copper kettle on the range waits for the stove as a stock support. Verified at 4444e1e1 (slice22) and db14e977 (slice22b, the 6A backdrop narrowed): the thirteen families pass the fabrication batch (28,045 checks, 0 failures; 206 stock assemblies, every pan bearing on the floor between its icebox's feet), apartment batch 236 as before, the six completion routes unchanged (1A 15, 1D 25, 2C 9, 3D 16, 4C 9, 4D 12), upper lighting and the household save owner 0 failures, upper kitchens 238 with the baseline's labels, the fourteen-kitchen sweep 0 failures; close-ups in implementation/slice22.</t>
+        </is>
+      </c>
     </row>
     <row r="398">
       <c r="A398" s="2" t="inlineStr">
@@ -30091,10 +30131,14 @@
       </c>
       <c r="S413" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T413" s="2" t="inlineStr"/>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="T413" s="2" t="inlineStr">
+        <is>
+          <t>4D_drip_tray: a zinc drip pan holding a skin of water (driptray form) on the floor under the icebox, between its feet with the front lip showing, clear of the door stance and the door's swing. The ice card in the window pane waits for a window-pane support (the panes belong to the shell, not a furniture actor). Verified at 4444e1e1 (slice22) and db14e977 (slice22b, the 6A backdrop narrowed): the thirteen families pass the fabrication batch (28,045 checks, 0 failures; 206 stock assemblies, every pan bearing on the floor between its icebox's feet), apartment batch 236 as before, the six completion routes unchanged (1A 15, 1D 25, 2C 9, 3D 16, 4C 9, 4D 12), upper lighting and the household save owner 0 failures, upper kitchens 238 with the baseline's labels, the fourteen-kitchen sweep 0 failures; close-ups in implementation/slice22.</t>
+        </is>
+      </c>
     </row>
     <row r="414">
       <c r="A414" s="2" t="inlineStr">
@@ -32733,10 +32777,14 @@
       </c>
       <c r="S450" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T450" s="2" t="inlineStr"/>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="T450" s="2" t="inlineStr">
+        <is>
+          <t>5A_drip_tray: a zinc drip pan holding a skin of water (driptray form) on the floor under the icebox, between its feet with the front lip showing, clear of the door stance and the door's swing. The ice card in the window pane waits for a window-pane support (the panes belong to the shell, not a furniture actor). Verified at 4444e1e1 (slice22) and db14e977 (slice22b, the 6A backdrop narrowed): the thirteen families pass the fabrication batch (28,045 checks, 0 failures; 206 stock assemblies, every pan bearing on the floor between its icebox's feet), apartment batch 236 as before, the six completion routes unchanged (1A 15, 1D 25, 2C 9, 3D 16, 4C 9, 4D 12), upper lighting and the household save owner 0 failures, upper kitchens 238 with the baseline's labels, the fourteen-kitchen sweep 0 failures; close-ups in implementation/slice22.</t>
+        </is>
+      </c>
     </row>
     <row r="451">
       <c r="A451" s="2" t="inlineStr">
@@ -35283,10 +35331,14 @@
       </c>
       <c r="S485" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T485" s="2" t="inlineStr"/>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="T485" s="2" t="inlineStr">
+        <is>
+          <t>5C_drip_tray: a zinc drip pan holding a skin of water (driptray form) on the floor under the icebox, between its feet with the front lip showing, clear of the door stance and the door's swing. The ice card in the window pane waits for a window-pane support (the panes belong to the shell, not a furniture actor). Verified at 4444e1e1 (slice22) and db14e977 (slice22b, the 6A backdrop narrowed): the thirteen families pass the fabrication batch (28,045 checks, 0 failures; 206 stock assemblies, every pan bearing on the floor between its icebox's feet), apartment batch 236 as before, the six completion routes unchanged (1A 15, 1D 25, 2C 9, 3D 16, 4C 9, 4D 12), upper lighting and the household save owner 0 failures, upper kitchens 238 with the baseline's labels, the fourteen-kitchen sweep 0 failures; close-ups in implementation/slice22.</t>
+        </is>
+      </c>
     </row>
     <row r="486">
       <c r="A486" s="2" t="inlineStr">
@@ -37418,7 +37470,7 @@
       </c>
       <c r="T514" s="2" t="inlineStr">
         <is>
-          <t>6A_backdrop_rail (new backdroprail form: header strip on rear battens, two brackets, a rail and a paper roll with its sheet hanging almost to the floor) on the west wall south of the window, the rail at 2.2 m, clear of the tripod, softboxes and crate. The charging bench and the folding chair wait for a work-table copy and a folding-chair seating variant. Verified at ccdf39bf (slice20): the thirteen families pass the fabrication batch (27,601 checks, 0 failures; objects 86, stock 192, the rail and print line on their actual wall faces, the box files on the clear boards), apartment batch 236 as before, upper lighting and the household save owner 0 failures, the two-space sweep 0 failures; close-ups in implementation/slice20.</t>
+          <t>6A_backdrop_rail (new backdroprail form: header strip on rear battens, two brackets, a rail and a paper roll with its sheet hanging almost to the floor) on the west wall south of the window, the rail at 2.2 m, clear of the tripod, softboxes and crate (narrowed to 1.2 m in slice 22, implementation/slice22b, after the upper-kitchen suite found the paper inside the tripod stance's capsule). The charging bench and the folding chair wait for a work-table copy and a folding-chair seating variant. Verified at ccdf39bf (slice20): the thirteen families pass the fabrication batch (27,601 checks, 0 failures; objects 86, stock 192, the rail and print line on their actual wall faces, the box files on the clear boards), apartment batch 236 as before, upper lighting and the household save owner 0 failures, the two-space sweep 0 failures; close-ups in implementation/slice20.</t>
         </is>
       </c>
     </row>
@@ -37775,10 +37827,14 @@
       </c>
       <c r="S519" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T519" s="2" t="inlineStr"/>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="T519" s="2" t="inlineStr">
+        <is>
+          <t>6A_drip_tray: a zinc drip pan holding a skin of water (driptray form) on the floor under the icebox, between its feet with the front lip showing, clear of the door stance and the door's swing. The ice card in the window pane waits for a window-pane support (the panes belong to the shell, not a furniture actor). Verified at 4444e1e1 (slice22) and db14e977 (slice22b, the 6A backdrop narrowed): the thirteen families pass the fabrication batch (28,045 checks, 0 failures; 206 stock assemblies, every pan bearing on the floor between its icebox's feet), apartment batch 236 as before, the six completion routes unchanged (1A 15, 1D 25, 2C 9, 3D 16, 4C 9, 4D 12), upper lighting and the household save owner 0 failures, upper kitchens 238 with the baseline's labels, the fourteen-kitchen sweep 0 failures; close-ups in implementation/slice22.</t>
+        </is>
+      </c>
     </row>
     <row r="520">
       <c r="A520" s="2" t="inlineStr">
@@ -38927,10 +38983,14 @@
       </c>
       <c r="S535" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T535" s="2" t="inlineStr"/>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="T535" s="2" t="inlineStr">
+        <is>
+          <t>6B_drip_tray: a zinc drip pan holding a skin of water (driptray form) on the floor under the icebox, between its feet with the front lip showing, clear of the door stance and the door's swing. The ice card in the window pane waits for a window-pane support (the panes belong to the shell, not a furniture actor). Verified at 4444e1e1 (slice22) and db14e977 (slice22b, the 6A backdrop narrowed): the thirteen families pass the fabrication batch (28,045 checks, 0 failures; 206 stock assemblies, every pan bearing on the floor between its icebox's feet), apartment batch 236 as before, the six completion routes unchanged (1A 15, 1D 25, 2C 9, 3D 16, 4C 9, 4D 12), upper lighting and the household save owner 0 failures, upper kitchens 238 with the baseline's labels, the fourteen-kitchen sweep 0 failures; close-ups in implementation/slice22.</t>
+        </is>
+      </c>
     </row>
     <row r="536">
       <c r="A536" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Implement dossier slice 23: storage bay contents and laundry baskets
- B1_RESIDENT_STORAGE-001: one household object against the back of
  sixteen basement bays, keyed to the bay labels (suitcases, boot trays,
  hampers, parts crates, 6A's gear crate, 5C's failed canvases); 2C's and
  4D's bays stay empty.
- B1_LAUNDRY-001: five wicker baskets along the laundry's north wall,
  clear of the washers.

All copies of existing forms. Evidence under implementation/slice23 and
slice23base/. INERT: no ledger status changes.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/art/reviews/v2_environment_design_20261008/change_register.xlsx
+++ b/art/reviews/v2_environment_design_20261008/change_register.xlsx
@@ -625,10 +625,14 @@
       </c>
       <c r="S2" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T2" s="2" t="inlineStr"/>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="T2" s="2" t="inlineStr">
+        <is>
+          <t>Five wicker baskets (hamper copies) along the north wall either side of the wet-stack pier, clear of the washers and the wringer swing (one first stood inside the pier: slice23c moved it). The chalked floor numbers, the folding table and Mina's uniform stack wait for a decal pass, a work-table copy and a folded-uniform form. Verified at 8f72926b (slice23: basement route 88 and ground 11 waypoints, laundry input 17, laundry apparatus, fittings, receiving and trade 0 failures, identical at 09e583ee in slice23base; Mina's laundry routine passing on both under the long runner in slice23mina and slice23mina_base; apartment batch 236; fabrication 28,403 checks with 0 failures in slice23b) and at 1cddce25 (slice23c, the basket moved: fabrication, laundry route, apparatus and fittings 0 failures, the laundry sweep 0 failures); captures in implementation/slice23 and slice23c.</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -1941,10 +1945,14 @@
       </c>
       <c r="S22" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T22" s="2" t="inlineStr"/>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="T22" s="2" t="inlineStr">
+        <is>
+          <t>One household object against the back of sixteen bays, keyed to the bay labels: suitcases for 1A, 3D, 4A, 5A and 6B; boot trays for 1D and 3A; hampers for 2A, 4C and 6C; parts crates for 2B, 3B, 4B and 5B; 6A's gear crate; 5C's failed canvases face to the wall. 2C's and 4D's bays stay empty (padlocked). Each stands clear of the folded gate and the aisle. Deviations: one object per bay rather than a set; no padlock form yet. Verified at 8f72926b (slice23: basement route 88 and ground 11 waypoints, laundry input 17, laundry apparatus, fittings, receiving and trade 0 failures, identical at 09e583ee in slice23base; Mina's laundry routine passing on both under the long runner in slice23mina and slice23mina_base; apartment batch 236; fabrication 28,403 checks with 0 failures in slice23b) and at 1cddce25 (slice23c, the basket moved: fabrication, laundry route, apparatus and fittings 0 failures, the laundry sweep 0 failures); captures in implementation/slice23 and slice23c.</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Implement dossier slice 24: out-tray, torch, battery case, cap, card index
Five small surface-stock forms (outtray, torch, batterycase, cap,
lighttable) and their records: 2A's out-tray of receipts and 5A's torch on
the hall-stand shelves, 5B's battery case on the vestibule floor by the
signal outlet, 4B's previous tenant's cap on the closet shelf (210
assemblies; the light-table form waits for a clear support, since 6A's
worktop carries the toaster); 3D's card index as a completion copy of
6C's cabinet. Covers F02_A_VESTIBULE-003, F05_A_VESTIBULE-003,
F05_B_VESTIBULE-003, F04_B_CLOSET-002 and F03_D_STUDY-002.

The upper-kitchen suite's material check skips passive stock resting on
the cabinets (206 failures, the three stance labels unchanged).

Evidence under implementation/slice24 and slice24c/. INERT: no ledger status changes.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/art/reviews/v2_environment_design_20261008/change_register.xlsx
+++ b/art/reviews/v2_environment_design_20261008/change_register.xlsx
@@ -14885,10 +14885,14 @@
       </c>
       <c r="S208" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T208" s="2" t="inlineStr"/>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="T208" s="2" t="inlineStr">
+        <is>
+          <t>2A_out_tray: a dark wooden out-tray holding a stack of filed receipts (outtray form) square on the hall stand's shelf. Verified at 3ee31793 (slice24: apartment batch 236, the apartment door route 45 waypoints with 0 failures, completion route 3D 16 as before, upper lighting and the household save owner 0 failures, the five-space sweep 0 failures) and at 2c52a53e (slice24c, the light table withdrawn and the upper-kitchen material check scoped to the cabinets: fabrication 28,545 checks with 0 failures, every piece bearing on its support; upper kitchens 206 with the baseline's three stance labels); captures in implementation/slice24.</t>
+        </is>
+      </c>
     </row>
     <row r="209">
       <c r="A209" s="2" t="inlineStr">
@@ -23633,10 +23637,14 @@
       </c>
       <c r="S324" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T324" s="2" t="inlineStr"/>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="T324" s="2" t="inlineStr">
+        <is>
+          <t>3D_card_index: a completion copy of 6C's card-index cabinet in the study's south-west corner, clear of the storage door's sweep, the window and the blankets. Verified at 3ee31793 (slice24: apartment batch 236, the apartment door route 45 waypoints with 0 failures, completion route 3D 16 as before, upper lighting and the household save owner 0 failures, the five-space sweep 0 failures) and at 2c52a53e (slice24c, the light table withdrawn and the upper-kitchen material check scoped to the cabinets: fabrication 28,545 checks with 0 failures, every piece bearing on its support; upper kitchens 206 with the baseline's three stance labels); captures in implementation/slice24.</t>
+        </is>
+      </c>
     </row>
     <row r="325">
       <c r="A325" s="2" t="inlineStr">
@@ -28025,10 +28033,14 @@
       </c>
       <c r="S384" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T384" s="2" t="inlineStr"/>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="T384" s="2" t="inlineStr">
+        <is>
+          <t>4B_old_cap: the previous tenant's service cap (cap form: navy crown, bakelite peak and band) on the closet shelf's upper board beside the bulb carton. Deviation: the upper board, not the top, which carries the frame's rail caps. Verified at 3ee31793 (slice24: apartment batch 236, the apartment door route 45 waypoints with 0 failures, completion route 3D 16 as before, upper lighting and the household save owner 0 failures, the five-space sweep 0 failures) and at 2c52a53e (slice24c, the light table withdrawn and the upper-kitchen material check scoped to the cabinets: fabrication 28,545 checks with 0 failures, every piece bearing on its support; upper kitchens 206 with the baseline's three stance labels); captures in implementation/slice24.</t>
+        </is>
+      </c>
     </row>
     <row r="385">
       <c r="A385" s="2" t="inlineStr">
@@ -32217,10 +32229,14 @@
       </c>
       <c r="S442" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T442" s="2" t="inlineStr"/>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="T442" s="2" t="inlineStr">
+        <is>
+          <t>5A_torch (torch form: nickel barrel, head and lens, a bakelite switch) on the hall stand's shelf (held by the bearing check; the vestibule gives the close-up camera no clear station). The chalk swing-limit arc waits for a floor decal pass. Verified at 3ee31793 (slice24: apartment batch 236, the apartment door route 45 waypoints with 0 failures, completion route 3D 16 as before, upper lighting and the household save owner 0 failures, the five-space sweep 0 failures) and at 2c52a53e (slice24c, the light table withdrawn and the upper-kitchen material check scoped to the cabinets: fabrication 28,545 checks with 0 failures, every piece bearing on its support; upper kitchens 206 with the baseline's three stance labels); captures in implementation/slice24.</t>
+        </is>
+      </c>
     </row>
     <row r="443">
       <c r="A443" s="2" t="inlineStr">
@@ -33587,10 +33603,14 @@
       </c>
       <c r="S461" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T461" s="2" t="inlineStr"/>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="T461" s="2" t="inlineStr">
+        <is>
+          <t>5B_battery_case (batterycase form: a wooden case with two glass cells and brass terminals) on the floor west of the switch, where the signal-outlet plate sits, clear of the switch stance and the main opening. The cloth lead to the plate waits for a lead form. Verified at 3ee31793 (slice24: apartment batch 236, the apartment door route 45 waypoints with 0 failures, completion route 3D 16 as before, upper lighting and the household save owner 0 failures, the five-space sweep 0 failures) and at 2c52a53e (slice24c, the light table withdrawn and the upper-kitchen material check scoped to the cabinets: fabrication 28,545 checks with 0 failures, every piece bearing on its support; upper kitchens 206 with the baseline's three stance labels); captures in implementation/slice24.</t>
+        </is>
+      </c>
     </row>
     <row r="462">
       <c r="A462" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Implement dossier slice 25: 2C's rig deck and cable hooks, 4D's print, 6A's archive crates
- F02_C_MAIN-001 (amended): a reel deck copy on 2C's rig table and a new
  hookstrip form (batten, five hooks, taped cable loops as curved wires)
  on the window wall beside the rig.
- F04_D_MAIN-001 (amended): a photograph-frame copy over 4D's settee.
- F06_A_STUDY-002: three archive crates (parts-crate copies) under 6A's
  desk wall.

Evidence under implementation/slice25/. INERT: no ledger status changes.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/art/reviews/v2_environment_design_20261008/change_register.xlsx
+++ b/art/reviews/v2_environment_design_20261008/change_register.xlsx
@@ -17518,7 +17518,7 @@
       </c>
       <c r="T242" s="2" t="inlineStr">
         <is>
-          <t>2C_rig_table (TableRect05) on the window wall facing the vestibule opening with 2C_din_dc2 as the operator's chair; 2C_din_t and 2C_din_dc1 moved against the kitchen-side wall as the late-meal surface, stances moved with them. The mixer (signal family), reel deck, headphones and the hook strip stay open. (implementation/slice6/images/F02_C_MAIN_OV.jpg)</t>
+          <t>2C_rig_table (TableRect05) on the window wall facing the vestibule opening with 2C_din_dc2 as the operator's chair; 2C_din_t and 2C_din_dc1 moved against the kitchen-side wall as the late-meal surface, stances moved with them. (implementation/slice6/images/F02_C_MAIN_OV.jpg) Slice 25 adds 2C_deck (a reel deck copy) on the rig table between the cartons and the mug, and 2C_cable_hooks (new hookstrip form: a batten with five hooks and taped cable loops) on the window wall beside the rig at 1.5 m (implementation/slice25). The mixer and headphones wait for the signal family.</t>
         </is>
       </c>
     </row>
@@ -29794,7 +29794,7 @@
       </c>
       <c r="T408" s="2" t="inlineStr">
         <is>
-          <t>4D_settee (Sofa195) on the long wall (the window wall carries the radiator), 4D_lamp_table (TableRect08) beside it, 4D_chair2 (ChairDark) at the dining table; the wireless table and radio from BW-011. The landlord's lamp and the print wait for the task-lamp and wall-art hooks. (implementation/slice6/images/F04_D_MAIN_OV.jpg)</t>
+          <t>4D_settee (Sofa195) on the long wall (the window wall carries the radiator), 4D_lamp_table (TableRect08) beside it, 4D_chair2 (ChairDark) at the dining table; the wireless table and radio from BW-011. (implementation/slice6/images/F04_D_MAIN_OV.jpg) Slice 25 hangs 4D_print (a photograph-frame copy) over the settee at 1.5 m (implementation/slice25); the landlord's lamp waits for the task-lamp family.</t>
         </is>
       </c>
     </row>
@@ -38407,10 +38407,14 @@
       </c>
       <c r="S527" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T527" s="2" t="inlineStr"/>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="T527" s="2" t="inlineStr">
+        <is>
+          <t>Three archive crates (parts-crate copies, open-topped) under the desk wall against the south wall, clear of the desk's legs, the chair and its stance; the three copies in two locations read as the crates under the desk and the drawers above. Verified at 8877d9df (slice25): the thirteen families pass the fabrication batch (28,681 checks, 0 failures; objects 116, the strip and print on their actual wall faces, the crates inside the study clear of the desk, the deck bearing on the rig table), apartment batch 236, the apartment door route 45 waypoints with 0 failures, completion routes 2C 9 and 4D 12 as before, upper lighting and the household save owner 0 failures, upper kitchens 206 with the baseline's stance labels, the three-space sweep 0 failures; captures in implementation/slice25.</t>
+        </is>
+      </c>
     </row>
     <row r="528">
       <c r="A528" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Implement dossier slice 26: the 2C and 4C bookshelves and 4C's colour board
F04_C_MAIN-005 found both actors absent rather than misplaced: the anchors
existed with nothing mounted. 4C's colour board is now a completion copy of
5C's; F02_2C_BOOKSHELF_01 and F04_4C_BOOKSHELF_01 join the bookshelf
roster and data (plain cases, Juno Kells' and Noel Price's libraries) and
the household save owner (its suite counts 203 controls). The bookshelf
manifest keeps 6C last, because the bookshelf suite blanks the last
record's canonical book to prove the validator refuses it.

Evidence under implementation/slice26/. INERT: no ledger status changes.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/art/reviews/v2_environment_design_20261008/change_register.xlsx
+++ b/art/reviews/v2_environment_design_20261008/change_register.xlsx
@@ -28745,10 +28745,14 @@
       </c>
       <c r="S394" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T394" s="2" t="inlineStr"/>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="T394" s="2" t="inlineStr">
+        <is>
+          <t>Both actors were absent, not misplaced: 4C_story_colorboard's anchor had no furniture record and F04_4C_BOOKSHELF_01 was missing from the bookshelf roster (as was 2C's F02_2C_BOOKSHELF_01). Slice 26 mounts the colour board as a completion copy of 5C's and adds both shelves to the roster (plain cases, Noel Price's and Juno Kells' libraries), registered with the household save owner (203 controls). Verified at WIP c9bc2317 + 432ad0a5 (implementation/slice26): fabrication batch 0 failures; apartment batch 236 (the branch baseline); household state 154 checks, 0 failures; bookshelves 144 checks, 0 failures once 6C is kept last in the manifest (its suite blanks the last record's canonical book); completion 2C and 4C 9 waypoints with their one pre-existing kitchen-leg failure; upper lighting 0 failures; F04_C_MAIN_DT1 shows the board, F04_C_MAIN_RV and F02_C_MAIN_RV show the new cases.</t>
+        </is>
+      </c>
     </row>
     <row r="395">
       <c r="A395" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Implement dossier slice 29: the boiler room's tools and the signal frame
- B1_BOILER_ROOM-001: a coal shovel leaning beside the fire door outside
  its swing, the clinker rake on two nails at 1.3 m, a lidded ash can by
  the west wall with an oil can on a rag. The ash can keeps to the wall
  so the door swings, the control aisle and the damper route stay clear.
- B1_ELECTRICAL-001: the Vantry signal frame opposite the fuse panel:
  terminal strips, blank tag cards, cloth leads dressed into a trunk
  cleated to the ceiling. It is ambient; the INSPECT owner is not made.
- B1_ELECTRICAL-003: steel conduit from the floor into the fuse panel's
  backing box and out of its top to a junction box under the ceiling.
- Domestic objects gain shovel, rakerack, ashcan, signalframe and conduit
  forms (126 instances).

Evidence under implementation/slice29/. INERT: no ledger status changes.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/art/reviews/v2_environment_design_20261008/change_register.xlsx
+++ b/art/reviews/v2_environment_design_20261008/change_register.xlsx
@@ -1149,10 +1149,14 @@
       </c>
       <c r="S10" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T10" s="2" t="inlineStr"/>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="T10" s="2" t="inlineStr">
+        <is>
+          <t>The firing tools: a coal shovel leaning on the west wall south of the fire door (outside its swing), the clinker rake on two nails at 1.3 m north of the door, and a lidded, ribbed ash can by the west wall with an oil can standing on a folded rag beside it (implementation/slice29/images: B1_boiler_ash_can_native, B1_boiler_rake_native, B1_BOILER_ROOM_RV). The ash can stands by the wall rather than under the ash door so the firing and ash door swings, the control aisle and the damper route stay clear; the ring decal is not made. Verified at WIP d53988d8 (implementation/slice29): fabrication batch 0 failures; apartment batch 236 (the branch baseline); boiler door swing 0, boiler route 17, basement route 88 and foundation 11 waypoints with 0 failures; boiler body, instruments, pipework and breeching 0 failures; household state 154 checks, 0 failures; the two-room sweep 0 failures.</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -1355,10 +1359,14 @@
       </c>
       <c r="S13" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T13" s="2" t="inlineStr"/>
+          <t>implemented</t>
+        </is>
+      </c>
+      <c r="T13" s="2" t="inlineStr">
+        <is>
+          <t>The Vantry signal frame hangs on the wall opposite the fuse panel (east of the door, clear of its swing): six bakelite terminal strips with brass terminals and blank tag cards on a board, cloth leads dressed into a bundle and a trunk cleated up the wall to the ceiling (B1_signal_frame_native, B1_ELECTRICAL_OV). Not made: the INSPECT owner; the frame is ambient. Verified at WIP d53988d8 (implementation/slice29): fabrication 0 failures, apartment batch 236, the eight boiler and basement suites unchanged (door swing, boiler route 17, basement route 88, body, instruments, pipework, breeching, foundation 11), household state 154 checks, 0 failures.</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -1479,10 +1487,14 @@
       </c>
       <c r="S15" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T15" s="2" t="inlineStr"/>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="T15" s="2" t="inlineStr">
+        <is>
+          <t>Steel conduit rises from a floor flange into the fuse panel's backing box and leaves its top for a junction box under the ceiling, each run saddled to the wall, clear of the panel's door and working front (B1_fuse_conduit_native). Verified at WIP d53988d8 (implementation/slice29): fabrication batch 0 failures; apartment batch 236 (the branch baseline); boiler door swing 0, boiler route 17, basement route 88 and foundation 11 waypoints with 0 failures; boiler body, instruments, pipework and breeching 0 failures; household state 154 checks, 0 failures; the two-room sweep 0 failures.</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Implement dossier slice 30: 5A's corrected plan and 2C's session archive
- F05_A_KITCHEN-003: 5A's icebox gets its own fridge variant with
  Nadia's corrected floor plan pinned to the food door (ruled walls, one
  room inked red, four brass pins). The door owns the sheet, so it swings
  with the leaf.
- F02_C_STUDIO-001: 2C's second wardrobe becomes Juno's session archive,
  a wardrobe variant on 5C's case with three shelves of grey reel boxes,
  coloured tape on each spine, and no rail. Both leaves keep their swing.
  An unanchored exemplar record was tried and refused by the furniture
  validator (every record needs an anchor); the variant shares 5C's.

Evidence under implementation/slice30b/. INERT: no ledger status changes.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/art/reviews/v2_environment_design_20261008/change_register.xlsx
+++ b/art/reviews/v2_environment_design_20261008/change_register.xlsx
@@ -18137,10 +18137,14 @@
       </c>
       <c r="S250" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T250" s="2" t="inlineStr"/>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="T250" s="2" t="inlineStr">
+        <is>
+          <t>Juno's second wardrobe is the session archive: a wardrobe variant (Wardrobe13, on 5C_w1_wardrobe's case) adds two shelves to the original middle shelf and stands grey reel boxes spine-out with coloured tape on each, and omits the rail; both leaves keep their hinges and 92-degree swing (implementation/slice30b/images/Wardrobe13_open, a native render with the leaves open). Verified at WIP 0efdc84b (implementation/slice30b): fabrication batch 0 failures; apartment batch 236 (the branch baseline); household state 154 checks, 0 failures; completion 2C 9 waypoints with its one pre-existing kitchen-leg failure; upper kitchens 206 (the branch baseline); the two-room sweep 0 failures.</t>
+        </is>
+      </c>
     </row>
     <row r="251">
       <c r="A251" s="2" t="inlineStr">
@@ -32915,10 +32919,14 @@
       </c>
       <c r="S451" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T451" s="2" t="inlineStr"/>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="T451" s="2" t="inlineStr">
+        <is>
+          <t>Nadia's corrected floor plan is pinned to the icebox's food door: 5A's icebox has its own variant (FridgeIceboxPlan) whose sheet, ruled walls, copper-inked room and four brass pins belong to the door, so the sheet swings with the leaf and the ice door is untouched (implementation/slice30b/images/F05_A_KITCHEN_OV). The sheet sits on the food door's raised panel (0.43 to 0.83 m) because 1.2 m falls on the ice door; INSPECT stays with the fridge card. Verified at WIP 0efdc84b (implementation/slice30b): fabrication batch 0 failures; apartment batch 236 (the branch baseline); household state 154 checks, 0 failures; completion 2C 9 waypoints with its one pre-existing kitchen-leg failure; upper kitchens 206 (the branch baseline); the two-room sweep 0 failures.</t>
+        </is>
+      </c>
     </row>
     <row r="452">
       <c r="A452" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Implement dossier slice 32: service evidence in the laundry and ground floor
- B1_LAUNDRY-003: Omar's oil can on a rag by the first washer, a spare
  drive belt on a nail between the washers, a folded stepladder leaning
  by the switch.
- F01_STAFF_RESTROOM-001: a roller towel on its bracket, the mop standing
  in a galvanised bucket with its handle on the wall, and a bar of
  carbolic in a wall soap dish beside the basin.
- F01_VESTIBULE-001: a cast-iron umbrella stand in the vestibule corner
  (the grate mat and the directory board are not made).
- F01_LOBBY-003: a brass spittoon by the west bench (the bench wear and
  the gloves on the radiator are not made).
- Domestic objects gain oilcan, beltnail, stepladder, umbrellastand,
  spittoon, soapdish, rollertowel and mopbucket forms (134 instances).

Evidence under implementation/slice32/. INERT: no ledger status changes.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/art/reviews/v2_environment_design_20261008/change_register.xlsx
+++ b/art/reviews/v2_environment_design_20261008/change_register.xlsx
@@ -761,10 +761,14 @@
       </c>
       <c r="S4" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T4" s="2" t="inlineStr"/>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="T4" s="2" t="inlineStr">
+        <is>
+          <t>Omar's deep-service evidence: an oil can standing on a folded rag by the first washer, a spare drive belt looped over a nail on the west wall between the washers, and a folded wooden stepladder leaning on the east wall south of the switch (implementation/slice32/images: B1_laundry_stepladder_native, B1_LAUNDRY views). Verified at WIP 87b953dc (implementation/slice32): fabrication batch 0 failures; apartment batch 236 on the long runner; laundry route 17, basement route 88, public doors 17, public furnishings 29 and wall mounts 4 waypoints with 0 failures; laundry apparatus and fittings, ground 0 failures; M08E with only its pre-existing route failure; Mina's laundry routine completes with no failures; the four-space sweep 0 failures.</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -8493,10 +8497,14 @@
       </c>
       <c r="S122" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T122" s="2" t="inlineStr"/>
+          <t>implemented</t>
+        </is>
+      </c>
+      <c r="T122" s="2" t="inlineStr">
+        <is>
+          <t>A cast-iron umbrella stand with its drip tray, two furled umbrellas and a walking stick stands in the vestibule's north-west corner, clear of both doors and the street-to-lobby route. Not made: the flush cast-iron grate mat (a floor inlay this pass does not cut) and the directory board. Verified at WIP 87b953dc (implementation/slice32): fabrication batch 0 failures; apartment batch 236 on the long runner; laundry route 17, basement route 88, public doors 17, public furnishings 29 and wall mounts 4 waypoints with 0 failures; laundry apparatus and fittings, ground 0 failures; M08E with only its pre-existing route failure; Mina's laundry routine completes with no failures; the four-space sweep 0 failures.</t>
+        </is>
+      </c>
     </row>
     <row r="123">
       <c r="A123" s="2" t="inlineStr">
@@ -8773,10 +8781,14 @@
       </c>
       <c r="S126" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T126" s="2" t="inlineStr"/>
+          <t>implemented</t>
+        </is>
+      </c>
+      <c r="T126" s="2" t="inlineStr">
+        <is>
+          <t>A brass spittoon stands by the west bench's door end, clear of the radiator front and the arrival route. Not made: the worn patch on the bench (a texture change) and the dish of gloves on the radiator (the stock inspector has no radiator support). Verified at WIP 87b953dc (implementation/slice32): fabrication batch 0 failures; apartment batch 236 on the long runner; laundry route 17, basement route 88, public doors 17, public furnishings 29 and wall mounts 4 waypoints with 0 failures; laundry apparatus and fittings, ground 0 failures; M08E with only its pre-existing route failure; Mina's laundry routine completes with no failures; the four-space sweep 0 failures.</t>
+        </is>
+      </c>
     </row>
     <row r="127">
       <c r="A127" s="2" t="inlineStr">
@@ -10203,10 +10215,14 @@
       </c>
       <c r="S147" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T147" s="2" t="inlineStr"/>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="T147" s="2" t="inlineStr">
+        <is>
+          <t>The staff restroom's roller towel on its bracket on the west wall, a galvanised bucket with the mop standing in it in the north-west corner (the handle resting on the wall), and a bar of carbolic in a wall soap dish beside the basin (F01_restroom_* native captures, F01_STAFF_RESTROOM views). Verified at WIP 87b953dc (implementation/slice32): fabrication batch 0 failures; apartment batch 236 on the long runner; laundry route 17, basement route 88, public doors 17, public furnishings 29 and wall mounts 4 waypoints with 0 failures; laundry apparatus and fittings, ground 0 failures; M08E with only its pre-existing route failure; Mina's laundry routine completes with no failures; the four-space sweep 0 failures.</t>
+        </is>
+      </c>
     </row>
     <row r="148">
       <c r="A148" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Implement dossier slice 33: 6A's prints, the bulkhead's garden kit, cushions
- F06_A_MAIN-003: three small photographic prints in a row on 6A's north
  wall, the middle one hung higher.
- F06_A_MAIN-004: one small plant print standing on the repaired
  bookcase's top board; the surface-stock context inspector now names
  the repaired case's top board as a support beside the sectional cap.
- ROOF_PUBLIC_CORE-003: a coil of washing line, a watering can and a
  trug on the bulkhead's west landing north of the door (the chalk tally
  is not made).
- F02_A_MAIN-005: two piped cushions on 2A's sofa (the rug is not made).
- Domestic objects gain ropecoil, wateringcan and trug forms; surface
  stock gains the cushion form (226 assemblies).

Evidence under implementation/slice33/. INERT: no ledger status changes.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/art/reviews/v2_environment_design_20261008/change_register.xlsx
+++ b/art/reviews/v2_environment_design_20261008/change_register.xlsx
@@ -15335,10 +15335,14 @@
       </c>
       <c r="S213" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T213" s="2" t="inlineStr"/>
+          <t>implemented</t>
+        </is>
+      </c>
+      <c r="T213" s="2" t="inlineStr">
+        <is>
+          <t>Two piped linen cushions lie on the ends of 2A's sofa seat (2A_cushion_a_stock). Not made: the 2.4 by 1.6 m rug, which would run under the coffee table and the deck in the most strictly checked flat. Verified at WIP 32156acb (implementation/slice33): fabrication batch 0 failures; apartment batch 236 on the long runner; bookshelves 144 checks, 0 failures with the print seated on the repaired case; upper kitchens 206 and upper furniture 488 (both unchanged from slice 31's runs); upper lighting 0 failures; roof route 53 waypoints, 0 failures; the three-space sweep 0 failures.</t>
+        </is>
+      </c>
     </row>
     <row r="214">
       <c r="A214" s="2" t="inlineStr">
@@ -37713,10 +37717,14 @@
       </c>
       <c r="S516" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T516" s="2" t="inlineStr"/>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="T516" s="2" t="inlineStr">
+        <is>
+          <t>Sacha's editorial sequence: three small photographic prints in a row on the main room's north wall between the radiator and the bookcase, the middle one hung higher (copies of 2C_album_a; implementation/slice33/images: F06_A_MAIN views). Verified at WIP 32156acb (implementation/slice33): fabrication batch 0 failures; apartment batch 236 on the long runner; bookshelves 144 checks, 0 failures with the print seated on the repaired case; upper kitchens 206 and upper furniture 488 (both unchanged from slice 31's runs); upper lighting 0 failures; roof route 53 waypoints, 0 failures; the three-space sweep 0 failures.</t>
+        </is>
+      </c>
     </row>
     <row r="517">
       <c r="A517" s="2" t="inlineStr">
@@ -37771,10 +37779,14 @@
       </c>
       <c r="S517" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T517" s="2" t="inlineStr"/>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="T517" s="2" t="inlineStr">
+        <is>
+          <t>The one picture of a plant: a small standing frame on the repaired bookcase's top board, which the surface-stock context inspector now names as a support (6A_plant_print_stock). Verified at WIP 32156acb (implementation/slice33): fabrication batch 0 failures; apartment batch 236 on the long runner; bookshelves 144 checks, 0 failures with the print seated on the repaired case; upper kitchens 206 and upper furniture 488 (both unchanged from slice 31's runs); upper lighting 0 failures; roof route 53 waypoints, 0 failures; the three-space sweep 0 failures.</t>
+        </is>
+      </c>
     </row>
     <row r="518">
       <c r="A518" s="2" t="inlineStr">
@@ -41119,10 +41131,14 @@
       </c>
       <c r="S563" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T563" s="2" t="inlineStr"/>
+          <t>implemented</t>
+        </is>
+      </c>
+      <c r="T563" s="2" t="inlineStr">
+        <is>
+          <t>Roof-use evidence inside the public bulkhead: a coil of washing line, a galvanised watering can and a gardening trug stand on the west landing north of the door, between the wall and the roof route (ROOF_bulkhead_* native captures). Not made: the chalk tally on the wall (lettering-like marks need a decal owner). Verified at WIP 32156acb (implementation/slice33): fabrication batch 0 failures; apartment batch 236 on the long runner; bookshelves 144 checks, 0 failures with the print seated on the repaired case; upper kitchens 206 and upper furniture 488 (both unchanged from slice 31's runs); upper lighting 0 failures; roof route 53 waypoints, 0 failures; the three-space sweep 0 failures.</t>
+        </is>
+      </c>
     </row>
     <row r="564">
       <c r="A564" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Implement dossier slice 34: 1A's trunk, the sweep's kit, and a keep audit
- F01_A_STUDY-003: Evelyn's iron-banded trunk of lesson plans against the
  study's north wall (a larger variant of the suitcase form) and two tea
  tins on her study desk.
- ROOF_SERVICE_CORE-003: the chimney sweep's soot sack and rod bundle
  inside the service bulkhead, clear of the roof route.
- Nine keep items (F01_A_KITCHEN-005, F02_A_MAIN-006, F03_B_MAIN-004,
  F05_PUBLIC_CORE-004, ROOF_DECK_NORTHEAST-002 and four city keeps) are
  confirmed by a data and history audit against the dossier commit
  (receipts/keep_audit.receipt.json).
- Domestic objects gain sootsack and sweeprods forms (143 instances).

Evidence under implementation/slice34/. INERT: no ledger status changes.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/art/reviews/v2_environment_design_20261008/change_register.xlsx
+++ b/art/reviews/v2_environment_design_20261008/change_register.xlsx
@@ -4727,10 +4727,14 @@
       </c>
       <c r="S63" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T63" s="2" t="inlineStr"/>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="T63" s="2" t="inlineStr">
+        <is>
+          <t>Kept: no subway or kiosk source or export has changed since e63ce4f6 (implementation/slice34/receipts/keep_audit.receipt.json). Verified at WIP 974ee6d2 (implementation/slice34): fabrication batch 0 failures; apartment batch 236 on the long runner; completion 1A 15 waypoints with its pre-existing kitchen-leg failure; roof route 53 waypoints, 0 failures; the two-space sweep 0 failures; the keep audit (receipts/keep_audit.receipt.json) holds for all nine keep items.</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
@@ -6247,10 +6251,14 @@
       </c>
       <c r="S87" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T87" s="2" t="inlineStr"/>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="T87" s="2" t="inlineStr">
+        <is>
+          <t>Kept: none of the funeral parlour's sources or exports has changed since e63ce4f6; the bier stays empty (implementation/slice34/receipts/keep_audit.receipt.json). Verified at WIP 974ee6d2 (implementation/slice34): fabrication batch 0 failures; apartment batch 236 on the long runner; completion 1A 15 waypoints with its pre-existing kitchen-leg failure; roof route 53 waypoints, 0 failures; the two-space sweep 0 failures; the keep audit (receipts/keep_audit.receipt.json) holds for all nine keep items.</t>
+        </is>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
@@ -7069,10 +7077,14 @@
       </c>
       <c r="S100" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T100" s="2" t="inlineStr"/>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="T100" s="2" t="inlineStr">
+        <is>
+          <t>Kept: the pawn clock wall's sources and export are unchanged since e63ce4f6; the dials keep their geometric hour marks and no numerals (implementation/slice34/receipts/keep_audit.receipt.json). Verified at WIP 974ee6d2 (implementation/slice34): fabrication batch 0 failures; apartment batch 236 on the long runner; completion 1A 15 waypoints with its pre-existing kitchen-leg failure; roof route 53 waypoints, 0 failures; the two-space sweep 0 failures; the keep audit (receipts/keep_audit.receipt.json) holds for all nine keep items.</t>
+        </is>
+      </c>
     </row>
     <row r="101">
       <c r="A101" s="2" t="inlineStr">
@@ -7193,10 +7205,14 @@
       </c>
       <c r="S102" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T102" s="2" t="inlineStr"/>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="T102" s="2" t="inlineStr">
+        <is>
+          <t>Kept: the radio service shop's sources and exports are unchanged since e63ce4f6 (implementation/slice34/receipts/keep_audit.receipt.json). Verified at WIP 974ee6d2 (implementation/slice34): fabrication batch 0 failures; apartment batch 236 on the long runner; completion 1A 15 waypoints with its pre-existing kitchen-leg failure; roof route 53 waypoints, 0 failures; the two-space sweep 0 failures; the keep audit (receipts/keep_audit.receipt.json) holds for all nine keep items.</t>
+        </is>
+      </c>
     </row>
     <row r="103">
       <c r="A103" s="2" t="inlineStr">
@@ -11343,10 +11359,14 @@
       </c>
       <c r="S161" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T161" s="2" t="inlineStr"/>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="T161" s="2" t="inlineStr">
+        <is>
+          <t>Kept: F01_1A_FRIDGE_01 is FridgeMonitor at e63ce4f6 and at this slice (implementation/slice34/receipts/keep_audit.receipt.json). Verified at WIP 974ee6d2 (implementation/slice34): fabrication batch 0 failures; apartment batch 236 on the long runner; completion 1A 15 waypoints with its pre-existing kitchen-leg failure; roof route 53 waypoints, 0 failures; the two-space sweep 0 failures; the keep audit (receipts/keep_audit.receipt.json) holds for all nine keep items.</t>
+        </is>
+      </c>
     </row>
     <row r="162">
       <c r="A162" s="2" t="inlineStr">
@@ -12041,10 +12061,14 @@
       </c>
       <c r="S170" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T170" s="2" t="inlineStr"/>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="T170" s="2" t="inlineStr">
+        <is>
+          <t>Evelyn's trunk of lesson plans (an iron-banded wooden trunk, a larger variant of the suitcase form) stands against the study's north wall clear of the storage door, and two tea tins sit on the study desk beside her open register (1A_lesson_trunk_native, 1A_tea_tin_a_stock). Verified at WIP 974ee6d2 (implementation/slice34): fabrication batch 0 failures; apartment batch 236 on the long runner; completion 1A 15 waypoints with its pre-existing kitchen-leg failure; roof route 53 waypoints, 0 failures; the two-space sweep 0 failures; the keep audit (receipts/keep_audit.receipt.json) holds for all nine keep items.</t>
+        </is>
+      </c>
     </row>
     <row r="171">
       <c r="A171" s="2" t="inlineStr">
@@ -15397,10 +15421,14 @@
       </c>
       <c r="S214" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T214" s="2" t="inlineStr"/>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="T214" s="2" t="inlineStr">
+        <is>
+          <t>Kept: 2A_deck and 2A_projector_stand are unmoved and domestic_projectors.json is unchanged since e63ce4f6; the projector stands at yaw 0 and throws along -z toward the south pier, while the caption board hangs on the west window wall, outside that throw (implementation/slice34/receipts/keep_audit.receipt.json). Verified at WIP 974ee6d2 (implementation/slice34): fabrication batch 0 failures; apartment batch 236 on the long runner; completion 1A 15 waypoints with its pre-existing kitchen-leg failure; roof route 53 waypoints, 0 failures; the two-space sweep 0 failures; the keep audit (receipts/keep_audit.receipt.json) holds for all nine keep items.</t>
+        </is>
+      </c>
     </row>
     <row r="215">
       <c r="A215" s="2" t="inlineStr">
@@ -21671,10 +21699,14 @@
       </c>
       <c r="S297" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T297" s="2" t="inlineStr"/>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="T297" s="2" t="inlineStr">
+        <is>
+          <t>Kept: household_radios.json, domestic_projectors.json and F03_B_LAMP_01's installation are unchanged since e63ce4f6 (implementation/slice34/receipts/keep_audit.receipt.json). Verified at WIP 974ee6d2 (implementation/slice34): fabrication batch 0 failures; apartment batch 236 on the long runner; completion 1A 15 waypoints with its pre-existing kitchen-leg failure; roof route 53 waypoints, 0 failures; the two-space sweep 0 failures; the keep audit (receipts/keep_audit.receipt.json) holds for all nine keep items.</t>
+        </is>
+      </c>
     </row>
     <row r="298">
       <c r="A298" s="2" t="inlineStr">
@@ -31207,10 +31239,14 @@
       </c>
       <c r="S427" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T427" s="2" t="inlineStr"/>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="T427" s="2" t="inlineStr">
+        <is>
+          <t>Kept: none of the twelve stair family sources or exports has changed since e63ce4f6; no baked wear was added (implementation/slice34/receipts/keep_audit.receipt.json). Verified at WIP 974ee6d2 (implementation/slice34): fabrication batch 0 failures; apartment batch 236 on the long runner; completion 1A 15 waypoints with its pre-existing kitchen-leg failure; roof route 53 waypoints, 0 failures; the two-space sweep 0 failures; the keep audit (receipts/keep_audit.receipt.json) holds for all nine keep items.</t>
+        </is>
+      </c>
     </row>
     <row r="428">
       <c r="A428" s="2" t="inlineStr">
@@ -41407,10 +41443,14 @@
       </c>
       <c r="S567" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T567" s="2" t="inlineStr"/>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="T567" s="2" t="inlineStr">
+        <is>
+          <t>Chimney-sweep evidence inside the service bulkhead: a tied soot sack on the landing and the sweep's rod bundle with its brush head leaning on the west wall north of the door, clear of the roof route (ROOF_service_* native captures). Verified at WIP 974ee6d2 (implementation/slice34): fabrication batch 0 failures; apartment batch 236 on the long runner; completion 1A 15 waypoints with its pre-existing kitchen-leg failure; roof route 53 waypoints, 0 failures; the two-space sweep 0 failures; the keep audit (receipts/keep_audit.receipt.json) holds for all nine keep items.</t>
+        </is>
+      </c>
     </row>
     <row r="568">
       <c r="A568" s="2" t="inlineStr">
@@ -42639,10 +42679,14 @@
       </c>
       <c r="S585" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T585" s="2" t="inlineStr"/>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="T585" s="2" t="inlineStr">
+        <is>
+          <t>Kept empty: no anchor lies in ROOF_DECK_NORTHEAST at e63ce4f6 or at this slice (implementation/slice34/receipts/keep_audit.receipt.json). Verified at WIP 974ee6d2 (implementation/slice34): fabrication batch 0 failures; apartment batch 236 on the long runner; completion 1A 15 waypoints with its pre-existing kitchen-leg failure; roof route 53 waypoints, 0 failures; the two-space sweep 0 failures; the keep audit (receipts/keep_audit.receipt.json) holds for all nine keep items.</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Implement dossier slice 35: pigment and packing stores, 4C's garments, pinboard
- F05_C_STUDIO-001: Iris's second wardrobe becomes the pigment store
  (Wardrobe14): two added shelves of pigment tins with painted lids, jars
  of ground colour and rolled canvas, no rail.
- F06_C_STUDIO-001: Mae's second wardrobe becomes the packing store
  (Wardrobe12): stacked kraft cartons, folded brown paper, string.
- F04_C_STUDIO-001: 4C's two wardrobes carry their residents' garment
  colours, Cam's maroon jersey (Wardrobe15) and Noel's indigo drill
  (Wardrobe08, whose only remaining user is 4C_w1).
- F02_A_BED-002 (partial): 2A's pinboard filled to a grid of 24 cards; the
  two overlapping cards are not made.
- jersey_maroon and drill_indigo are tinted aliases of the catalogue
  linen, kraft of the catalogue paper.

Evidence under implementation/slice35b/. INERT: no ledger status changes.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/art/reviews/v2_environment_design_20261008/change_register.xlsx
+++ b/art/reviews/v2_environment_design_20261008/change_register.xlsx
@@ -16049,10 +16049,14 @@
       </c>
       <c r="S222" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T222" s="2" t="inlineStr"/>
+          <t>implemented</t>
+        </is>
+      </c>
+      <c r="T222" s="2" t="inlineStr">
+        <is>
+          <t>2A's bedroom pinboard (DomesticObject00) is filled to a full grid of 24 cards (implementation/slice35b/images: F02_A_BED_DT1). Not made: the two deliberately overlapping cards; the pinboard form lays a neat grid. Verified at WIP 815745ee (implementation/slice35b): fabrication batch 0 failures (the wardrobe module accounts for every built variant once Wardrobe08 keeps an instance); apartment batch 236 on the long runner; household state 154 checks, 0 failures; completion 4C 9 waypoints with its pre-existing kitchen-leg failure; upper kitchens 206; upper furniture 482 (six fewer pre-existing material-binding failures as two wardrobes lose their garments); upper lighting 0 failures; the four-space sweep 0 failures; native renders with the leaves open (images/Wardrobe08_open, 12, 14, 15).</t>
+        </is>
+      </c>
     </row>
     <row r="223">
       <c r="A223" s="2" t="inlineStr">
@@ -29305,10 +29309,14 @@
       </c>
       <c r="S400" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T400" s="2" t="inlineStr"/>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="T400" s="2" t="inlineStr">
+        <is>
+          <t>4C's two wardrobes hold different residents' clothes: Cam's (Wardrobe15) hangs maroon jersey and Noel's (Wardrobe08, now used only by 4C_w1) indigo drill; jersey_maroon and drill_indigo are tinted aliases of the catalogue linen (Wardrobe15_open, Wardrobe08_open). Verified at WIP 815745ee (implementation/slice35b): fabrication batch 0 failures (the wardrobe module accounts for every built variant once Wardrobe08 keeps an instance); apartment batch 236 on the long runner; household state 154 checks, 0 failures; completion 4C 9 waypoints with its pre-existing kitchen-leg failure; upper kitchens 206; upper furniture 482 (six fewer pre-existing material-binding failures as two wardrobes lose their garments); upper lighting 0 failures; the four-space sweep 0 failures; native renders with the leaves open (images/Wardrobe08_open, 12, 14, 15).</t>
+        </is>
+      </c>
     </row>
     <row r="401">
       <c r="A401" s="2" t="inlineStr">
@@ -35759,10 +35767,14 @@
       </c>
       <c r="S489" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T489" s="2" t="inlineStr"/>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="T489" s="2" t="inlineStr">
+        <is>
+          <t>Iris's second wardrobe is the pigment store: its own variant (Wardrobe14) adds two shelves above the case's middle shelf and stands rows of pigment tins with painted lids, jars of ground colour and rolled canvas, with no rail (implementation/slice35b/images: Wardrobe14_open, F05_C_STUDIO_DT1). Verified at WIP 815745ee (implementation/slice35b): fabrication batch 0 failures (the wardrobe module accounts for every built variant once Wardrobe08 keeps an instance); apartment batch 236 on the long runner; household state 154 checks, 0 failures; completion 4C 9 waypoints with its pre-existing kitchen-leg failure; upper kitchens 206; upper furniture 482 (six fewer pre-existing material-binding failures as two wardrobes lose their garments); upper lighting 0 failures; the four-space sweep 0 failures; native renders with the leaves open (images/Wardrobe08_open, 12, 14, 15).</t>
+        </is>
+      </c>
     </row>
     <row r="490">
       <c r="A490" s="2" t="inlineStr">
@@ -40451,10 +40463,14 @@
       </c>
       <c r="S553" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T553" s="2" t="inlineStr"/>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="T553" s="2" t="inlineStr">
+        <is>
+          <t>Mae's second wardrobe is the packing store: its variant (Wardrobe12, only 6C_w1's) shelves stacked flat cartons in kraft, folded brown paper and balls of string, with no rail (Wardrobe12_open, F06_C_STUDIO_DT2). Verified at WIP 815745ee (implementation/slice35b): fabrication batch 0 failures (the wardrobe module accounts for every built variant once Wardrobe08 keeps an instance); apartment batch 236 on the long runner; household state 154 checks, 0 failures; completion 4C 9 waypoints with its pre-existing kitchen-leg failure; upper kitchens 206; upper furniture 482 (six fewer pre-existing material-binding failures as two wardrobes lose their garments); upper lighting 0 failures; the four-space sweep 0 failures; native renders with the leaves open (images/Wardrobe08_open, 12, 14, 15).</t>
+        </is>
+      </c>
     </row>
     <row r="554">
       <c r="A554" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Implement dossier slice 38: dress form, recorder, taped form, light box
- F02_B_MAIN-004: Lena's tripod dress form wearing her own voile frock
  with a pinned hem (new dressform object form) by 2B's window wall.
- F02_C_BED1-001 (partial): Juno's Bakelite recorder and a mug on 2C's
  nightstand; the unmade counterpane needs a bedding variant.
- 4A's toaster gets its own variant (ToasterForm) with a taped blank
  form, and 6A's prep cabinet a light box. Neither row is statused here:
  the form sat over the browning control and the light box over the
  toaster. Slices 41 and 40 place them again.
- The toaster builder accepts owner variants that keep a source tray
  exit.

Evidence under implementation/slice38/. INERT: no ledger status changes.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/art/reviews/v2_environment_design_20261008/change_register.xlsx
+++ b/art/reviews/v2_environment_design_20261008/change_register.xlsx
@@ -16673,10 +16673,14 @@
       </c>
       <c r="S230" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T230" s="2" t="inlineStr"/>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="T230" s="2" t="inlineStr">
+        <is>
+          <t>Lena's tripod dress form (new dressform object) wears her own printed voile frock with a row of steel pins in the turned-up hem; 2B has no armchair, so it stands by the south window wall east of the hall opening, clear of the radiator stance, and reads in the reverse view (implementation/slice38/images: F02_B_MAIN_RV). Verified at WIP d0986324 (implementation/slice38): fabrication batch 0 failures across 13 modules; apartment batch 236 on the long runner; household state 154 checks, 0 failures; upper kitchens 206; upper furniture 486 (unchanged from slice 37); upper lighting 0 failures; completion 2C 9 waypoints with its one pre-existing route failure; the four-space sweep 0 failures.</t>
+        </is>
+      </c>
     </row>
     <row r="231">
       <c r="A231" s="2" t="inlineStr">
@@ -18485,10 +18489,14 @@
       </c>
       <c r="S254" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T254" s="2" t="inlineStr"/>
+          <t>implemented</t>
+        </is>
+      </c>
+      <c r="T254" s="2" t="inlineStr">
+        <is>
+          <t>Juno's black Bakelite recorder (two reels, a knob, a front grille, a cloth cord) and a mug on 2C's nightstand (F02_C_BED1_OV). Not made: the thrown-back counterpane, which needs a bedding variant of the bed family. Verified at WIP d0986324 (implementation/slice38): fabrication batch 0 failures across 13 modules; apartment batch 236 on the long runner; household state 154 checks, 0 failures; upper kitchens 206; upper furniture 486 (unchanged from slice 37); upper lighting 0 failures; completion 2C 9 waypoints with its one pre-existing route failure; the four-space sweep 0 failures.</t>
+        </is>
+      </c>
     </row>
     <row r="255">
       <c r="A255" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Implement dossier slice 39: bolts, cutting kit, fastener cabinet, closures
- F02_B_PRIVATE_HALL-002: 2B's fabric shelves get their own variant
  (Shelf12): standing bolts of wool suiting, voile and burgundy knit.
- F02_B_MAIN-003: shears, tailor's chalk, a tape measure and a pincushion
  on Lena's worktable (four new stock kinds).
- F03_B_MAIN-003: Omar's six-drawer fastener cabinet and a bank of tins
  on 3B's tool shelves (Shelf13).
- F03_A_MAIN-002 (partial): a zinc tray with pots and secateurs on
  oilcloth on Malcolm's potting bench.
- F04_B_MAIN-004, F04_D_MAIN-003: closed against the captures; no white
  box or untextured mass remains.
- F05_B_KITCHEN-004: data and capture agree that the hob radios sit on
  the comparison table.
- F05_C_MAIN-004: the "cable loop" is the radiator valve's shadow.

Evidence under implementation/slice39/. INERT: no ledger status changes.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/art/reviews/v2_environment_design_20261008/change_register.xlsx
+++ b/art/reviews/v2_environment_design_20261008/change_register.xlsx
@@ -16607,10 +16607,14 @@
       </c>
       <c r="S229" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T229" s="2" t="inlineStr"/>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="T229" s="2" t="inlineStr">
+        <is>
+          <t>Lena's cutting kit on the worktable beside the pattern papers and notions: closed tailor's shears, a cake of tailor's chalk, a rolled cloth tape measure with its end run out (blank) and a tomato pincushion with pins (F02_B_MAIN_DT1). Verified at WIP 997a7465 (implementation/slice39): fabrication batch 0 failures across 13 modules; apartment batch 236 on the long runner; household state 154 checks, 0 failures; upper kitchens 206; upper furniture 486 (unchanged from slice 37); upper lighting 0 failures; completion 4D 12 waypoints with its one pre-existing route failure; the eight-space sweep 0 failures.</t>
+        </is>
+      </c>
     </row>
     <row r="230">
       <c r="A230" s="2" t="inlineStr">
@@ -17051,10 +17055,14 @@
       </c>
       <c r="S235" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T235" s="2" t="inlineStr"/>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="T235" s="2" t="inlineStr">
+        <is>
+          <t>Lena's cloth stands as bolts on both fabric shelves: their own variant (Shelf12) drops the inherited bins and tins and stands five bolts on each of the three lower boards, in wool suiting, voile and burgundy knit with card cores showing (implementation/slice39/images: F02_B_PRIVATE_HALL_TH, F02_B_PRIVATE_HALL_OV). Verified at WIP 997a7465 (implementation/slice39): fabrication batch 0 failures across 13 modules; apartment batch 236 on the long runner; household state 154 checks, 0 failures; upper kitchens 206; upper furniture 486 (unchanged from slice 37); upper lighting 0 failures; completion 4D 12 waypoints with its one pre-existing route failure; the eight-space sweep 0 failures.</t>
+        </is>
+      </c>
     </row>
     <row r="236">
       <c r="A236" s="2" t="inlineStr">
@@ -20429,10 +20437,14 @@
       </c>
       <c r="S280" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T280" s="2" t="inlineStr"/>
+          <t>implemented</t>
+        </is>
+      </c>
+      <c r="T280" s="2" t="inlineStr">
+        <is>
+          <t>Malcolm's pruning station on the potting bench: a zinc watering tray with two pots standing in water and red-handled secateurs on a square of dark oilcloth (F03_A_MAIN_DT1). Not made: the trug, the soil swept under the bench and the knife-mark line on the bench edge. Verified at WIP 997a7465 (implementation/slice39): fabrication batch 0 failures across 13 modules; apartment batch 236 on the long runner; household state 154 checks, 0 failures; upper kitchens 206; upper furniture 486 (unchanged from slice 37); upper lighting 0 failures; completion 4D 12 waypoints with its one pre-existing route failure; the eight-space sweep 0 failures.</t>
+        </is>
+      </c>
     </row>
     <row r="281">
       <c r="A281" s="2" t="inlineStr">
@@ -21661,10 +21673,14 @@
       </c>
       <c r="S296" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T296" s="2" t="inlineStr"/>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="T296" s="2" t="inlineStr">
+        <is>
+          <t>Omar's six-drawer fastener cabinet with blank card label frames and nickel pulls, and a bank of eight small lidded tins with blank labels, stand on the third board of both tool shelves (Shelf13), clear of the source bins and tins below (F03_B_MAIN_DT2). Verified at WIP 997a7465 (implementation/slice39): fabrication batch 0 failures across 13 modules; apartment batch 236 on the long runner; household state 154 checks, 0 failures; upper kitchens 206; upper furniture 486 (unchanged from slice 37); upper lighting 0 failures; completion 4D 12 waypoints with its one pre-existing route failure; the eight-space sweep 0 failures.</t>
+        </is>
+      </c>
     </row>
     <row r="297">
       <c r="A297" s="2" t="inlineStr">
@@ -27277,10 +27293,14 @@
       </c>
       <c r="S372" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T372" s="2" t="inlineStr"/>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="T372" s="2" t="inlineStr">
+        <is>
+          <t>Closed against the capture: neither the overview nor the reverse view of 4B's main room shows a featureless white box (F04_B_MAIN_OV, F04_B_MAIN_RV). Verified at WIP 997a7465 (implementation/slice39): fabrication batch 0 failures across 13 modules; apartment batch 236 on the long runner; household state 154 checks, 0 failures; upper kitchens 206; upper furniture 486 (unchanged from slice 37); upper lighting 0 failures; completion 4D 12 waypoints with its one pre-existing route failure; the eight-space sweep 0 failures.</t>
+        </is>
+      </c>
     </row>
     <row r="373">
       <c r="A373" s="2" t="inlineStr">
@@ -30069,10 +30089,14 @@
       </c>
       <c r="S410" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T410" s="2" t="inlineStr"/>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="T410" s="2" t="inlineStr">
+        <is>
+          <t>Closed against the capture: no untextured mass appears in 4D's main room; the pale form in the room is the upholstered settee (F04_D_MAIN_OV, F04_D_MAIN_RV). Verified at WIP 997a7465 (implementation/slice39): fabrication batch 0 failures across 13 modules; apartment batch 236 on the long runner; household state 154 checks, 0 failures; upper kitchens 206; upper furniture 486 (unchanged from slice 37); upper lighting 0 failures; completion 4D 12 waypoints with its one pre-existing route failure; the eight-space sweep 0 failures.</t>
+        </is>
+      </c>
     </row>
     <row r="411">
       <c r="A411" s="2" t="inlineStr">
@@ -34499,10 +34523,14 @@
       </c>
       <c r="S471" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T471" s="2" t="inlineStr"/>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="T471" s="2" t="inlineStr">
+        <is>
+          <t>Data and capture agree: both 5B_k_hob_radio anchors sit at table height over 5B_comparison_table, and the kitchen shows the two sets on that table with the range shelf empty (F05_B_KITCHEN_DT1). The table is kept; the ids keep their legacy names because saves and the spatial manifest key on them. Verified at WIP 997a7465 (implementation/slice39): fabrication batch 0 failures across 13 modules; apartment batch 236 on the long runner; household state 154 checks, 0 failures; upper kitchens 206; upper furniture 486 (unchanged from slice 37); upper lighting 0 failures; completion 4D 12 waypoints with its one pre-existing route failure; the eight-space sweep 0 failures.</t>
+        </is>
+      </c>
     </row>
     <row r="472">
       <c r="A472" s="2" t="inlineStr">
@@ -35359,10 +35387,14 @@
       </c>
       <c r="S483" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T483" s="2" t="inlineStr"/>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="T483" s="2" t="inlineStr">
+        <is>
+          <t>Identified, nothing to remove: the dark loop on the floor is the shadow of the radiator valve's handwheel thrown by the pendant, and the boxy object is the valve itself; no cable exists (F05_C_STUDIO_OV). Verified at WIP 997a7465 (implementation/slice39): fabrication batch 0 failures across 13 modules; apartment batch 236 on the long runner; household state 154 checks, 0 failures; upper kitchens 206; upper furniture 486 (unchanged from slice 37); upper lighting 0 failures; completion 4D 12 waypoints with its one pre-existing route failure; the eight-space sweep 0 failures.</t>
+        </is>
+      </c>
     </row>
     <row r="484">
       <c r="A484" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Implement dossier slice 40: japanned lamp, model case, T-square, 4D's case
- F05_A_MAIN-005: the architect counterweight lamp's arm, pedestal,
  counterweight and shade become black japanned steel (task lamp family).
- F05_A_STUDY-001 (partial): a glazed oak case over 5A's site model and a
  T-square hung on the study wall (new modelcase stock and tsquare form).
- F04_D_BED-001 (partial): an open suitcase on 4D's bed and a wardrobe
  variant holding only empty wire hangers (Wardrobe16).
- 6A's light box is resized and moved into the prep cabinet's back corner,
  clear of the toaster (statused after slice 41's capture).
- An inspection sweep closes F04_B_KITCHEN-004 and F01_D_KITCHEN-004 and
  rejects F02_C_BATH-003 with BW-005's measurement.

Evidence under implementation/slice40/. INERT: no ledger status changes.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/art/reviews/v2_environment_design_20261008/change_register.xlsx
+++ b/art/reviews/v2_environment_design_20261008/change_register.xlsx
@@ -13013,10 +13013,14 @@
       </c>
       <c r="S182" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T182" s="2" t="inlineStr"/>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="T182" s="2" t="inlineStr">
+        <is>
+          <t>Identified: the blue-white light is 1D's lit back burner, one of the two households that boot with a ring lit; its gas flame is visible at the burner and lights the splashback (F01_D_KITCHEN_DT1). Verified at WIP da33cf1d (implementation/slice40): fabrication batch 0 failures across 14 modules (task lamps included; the T-square captured natively); apartment batch 236 on the long runner; household state 154 checks, 0 failures; upper kitchens 206; upper furniture 488 (two more of the pre-existing material-binding class, from new stock meshes on probed furniture); upper lighting 0 failures; completion 4D 12 waypoints with its one pre-existing route failure; the three-space sweep and a seven-space inspection sweep 0 failures.</t>
+        </is>
+      </c>
     </row>
     <row r="183">
       <c r="A183" s="2" t="inlineStr">
@@ -18431,10 +18435,14 @@
       </c>
       <c r="S253" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T253" s="2" t="inlineStr"/>
+          <t>rejected</t>
+        </is>
+      </c>
+      <c r="T253" s="2" t="inlineStr">
+        <is>
+          <t>Measured with BW-005: 2C's branch hangs on a trapeze hanger seated at the slab soffit and ends in the fitted louvred register; a galvanised branch run is correct for the building's ventilation retrofit, so it stays (F02_C_BATH_DT1).</t>
+        </is>
+      </c>
     </row>
     <row r="254">
       <c r="A254" s="2" t="inlineStr">
@@ -27609,10 +27617,14 @@
       </c>
       <c r="S376" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T376" s="2" t="inlineStr"/>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="T376" s="2" t="inlineStr">
+        <is>
+          <t>Closed against the capture: 4B's range is the native gas range with cream enamel sides and cast-iron spider grates over the rings; no wood grain and no coil burners remain (F04_B_KITCHEN_DT1). Verified at WIP da33cf1d (implementation/slice40): fabrication batch 0 failures across 14 modules (task lamps included; the T-square captured natively); apartment batch 236 on the long runner; household state 154 checks, 0 failures; upper kitchens 206; upper furniture 488 (two more of the pre-existing material-binding class, from new stock meshes on probed furniture); upper lighting 0 failures; completion 4D 12 waypoints with its one pre-existing route failure; the three-space sweep and a seven-space inspection sweep 0 failures.</t>
+        </is>
+      </c>
     </row>
     <row r="377">
       <c r="A377" s="2" t="inlineStr">
@@ -30895,10 +30907,14 @@
       </c>
       <c r="S421" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T421" s="2" t="inlineStr"/>
+          <t>implemented</t>
+        </is>
+      </c>
+      <c r="T421" s="2" t="inlineStr">
+        <is>
+          <t>4D's late-night state: an open leather suitcase on the blanket with a few things packed, and the wardrobe's own variant (Wardrobe16) holding only empty wire hangers (F04_D_BED_OV, Wardrobe16_open). Not made: the mismatched pillows, which need a bedding variant. Verified at WIP da33cf1d (implementation/slice40): fabrication batch 0 failures across 14 modules (task lamps included; the T-square captured natively); apartment batch 236 on the long runner; household state 154 checks, 0 failures; upper kitchens 206; upper furniture 488 (two more of the pre-existing material-binding class, from new stock meshes on probed furniture); upper lighting 0 failures; completion 4D 12 waypoints with its one pre-existing route failure; the three-space sweep and a seven-space inspection sweep 0 failures.</t>
+        </is>
+      </c>
     </row>
     <row r="422">
       <c r="A422" s="2" t="inlineStr">
@@ -32755,10 +32771,14 @@
       </c>
       <c r="S447" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T447" s="2" t="inlineStr"/>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="T447" s="2" t="inlineStr">
+        <is>
+          <t>Nadia's architect counterweight lamp now has a black japanned arm, pedestal, counterweight and shade (the catalogue iron_blackened); only the ball joints and the rolled shade lip stay nickel, on its wooden base (implementation/slice40/images: architect_counterweight_front, F05_A_MAIN_DT2). Verified at WIP da33cf1d (implementation/slice40): fabrication batch 0 failures across 14 modules (task lamps included; the T-square captured natively); apartment batch 236 on the long runner; household state 154 checks, 0 failures; upper kitchens 206; upper furniture 488 (two more of the pre-existing material-binding class, from new stock meshes on probed furniture); upper lighting 0 failures; completion 4D 12 waypoints with its one pre-existing route failure; the three-space sweep and a seven-space inspection sweep 0 failures.</t>
+        </is>
+      </c>
     </row>
     <row r="448">
       <c r="A448" s="2" t="inlineStr">
@@ -33495,10 +33515,14 @@
       </c>
       <c r="S457" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T457" s="2" t="inlineStr"/>
+          <t>implemented</t>
+        </is>
+      </c>
+      <c r="T457" s="2" t="inlineStr">
+        <is>
+          <t>An oak-framed glazed case now stands over Nadia's site model on its table, clear of the massing, and her boxwood T-square hangs head-down on a nail on the study wall beside the pinboard (5A_tsquare_native, F05_A_STUDY_DT1). Not made: paper bands on the rolls; the study holds no rolled drawings to band. Verified at WIP da33cf1d (implementation/slice40): fabrication batch 0 failures across 14 modules (task lamps included; the T-square captured natively); apartment batch 236 on the long runner; household state 154 checks, 0 failures; upper kitchens 206; upper furniture 488 (two more of the pre-existing material-binding class, from new stock meshes on probed furniture); upper lighting 0 failures; completion 4D 12 waypoints with its one pre-existing route failure; the three-space sweep and a seven-space inspection sweep 0 failures.</t>
+        </is>
+      </c>
     </row>
     <row r="458">
       <c r="A458" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Implement dossier slice 41: hall file, toaster form, basement shop stock
- F04_A_PRIVATE_HALL-002: Wren's oak four-drawer vertical file in 4A's
  hall, top drawer not quite shut (new verticalfile object form).
- F04_A_KITCHEN-003: the taped form moves to the front half of the
  toaster's lever end, clear of the browning control and the lever.
- B1_MAINTENANCE_SHOP-001 (partial): bulb cartons on the parts shelf
  (Shelf14), a capsule crate at the bench end and the SR7 charging case
  with its lead to a wall plate (new chargingcase object form).

Evidence under implementation/slice41/. INERT: no ledger status changes.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/art/reviews/v2_environment_design_20261008/change_register.xlsx
+++ b/art/reviews/v2_environment_design_20261008/change_register.xlsx
@@ -1627,10 +1627,14 @@
       </c>
       <c r="S17" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T17" s="2" t="inlineStr"/>
+          <t>implemented</t>
+        </is>
+      </c>
+      <c r="T17" s="2" t="inlineStr">
+        <is>
+          <t>The basement shop's stock: six kraft bulb cartons on the parts shelf's third board (its own variant, Shelf14), a capsule crate on the floor at the bench's east end, and the SR7 charging case on the floor by the west wall with its cloth lead run up to a wall plate (B1_charging_case_native, B1_MAINTENANCE_SHOP_OV). The bench, a copy of 3B's, already carries a vice at its west end. Not made: the service-round tally board (needs Label3D) and a vice at the door end. Verified at WIP fd1cffd0 (implementation/slice41): fabrication batch 0 failures across 13 modules (the hall file and the charging case captured natively); apartment batch 236 on the long runner; household state 154 checks, 0 failures; upper kitchens 206; upper furniture 488 (unchanged from slice 40); upper lighting 0 failures; basement route 88 waypoints and wall mounts 4 waypoints, 0 failures; the four-space sweep 0 failures.</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -26331,10 +26335,14 @@
       </c>
       <c r="S359" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T359" s="2" t="inlineStr"/>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="T359" s="2" t="inlineStr">
+        <is>
+          <t>4A's toaster is its own variant (ToasterForm) with a blank form taped by two strips to the front half of the lever end, beside the slot; the carriage lever and the browning control on the other end stay clear (ToasterForm_lever_end, a native render of the installed variant). Verified at WIP fd1cffd0 (implementation/slice41): fabrication batch 0 failures across 13 modules (the hall file and the charging case captured natively); apartment batch 236 on the long runner; household state 154 checks, 0 failures; upper kitchens 206; upper furniture 488 (unchanged from slice 40); upper lighting 0 failures; basement route 88 waypoints and wall mounts 4 waypoints, 0 failures; the four-space sweep 0 failures.</t>
+        </is>
+      </c>
     </row>
     <row r="360">
       <c r="A360" s="2" t="inlineStr">
@@ -26491,10 +26499,14 @@
       </c>
       <c r="S361" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T361" s="2" t="inlineStr"/>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="T361" s="2" t="inlineStr">
+        <is>
+          <t>Wren's hall file: a second-hand oak four-drawer vertical file (new verticalfile object, 0.40 x 0.71 x 1.34 m) against the hall's east wall between the switch and the boots, the top drawer not quite shut, nickel pulls, blank brass label frames, finger grime at the top pull and a cup ring on the top; the hall keeps over 2 m clear (implementation/slice41/images: 4A_hall_file_native, F04_A_PRIVATE_HALL_OV). Verified at WIP fd1cffd0 (implementation/slice41): fabrication batch 0 failures across 13 modules (the hall file and the charging case captured natively); apartment batch 236 on the long runner; household state 154 checks, 0 failures; upper kitchens 206; upper furniture 488 (unchanged from slice 40); upper lighting 0 failures; basement route 88 waypoints and wall mounts 4 waypoints, 0 failures; the four-space sweep 0 failures.</t>
+        </is>
+      </c>
     </row>
     <row r="362">
       <c r="A362" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Implement dossier slice 43: oak desk wall, laid headsets, framed service leaf
- F06_A_STUDY-003: Sacha's desk wall is an oak top on solid oak ends; the
  headsets in 2A, 5B and 6A lie on their desks instead of a turned stand.
- F03_B_MAIN-005 (partial): Omar's bench cupboard and tray are grey
  painted iron.
- F03_B_KITCHEN-004, CITY_ALLEY-004 (partial): the service leaf's plain
  face gets stiles, rails and kick plates.
- A dry-owned wall shared with a bath carries tile on its bath face. The
  first-neighbour search misses walls that face several rooms, so the 5C,
  2A and 4B sink walls stay plaster here; slice 44 completes it.
- Upper furniture drops from 496 to 488 (eight fewer pre-existing
  material-binding failures from the headsets).

Evidence under implementation/slice43/. INERT: no ledger status changes.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/art/reviews/v2_environment_design_20261008/change_register.xlsx
+++ b/art/reviews/v2_environment_design_20261008/change_register.xlsx
@@ -4681,10 +4681,14 @@
       </c>
       <c r="S62" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T62" s="2" t="inlineStr"/>
+          <t>implemented</t>
+        </is>
+      </c>
+      <c r="T62" s="2" t="inlineStr">
+        <is>
+          <t>The alley rear door is the same service leaf and now shows its stiles, mid rail and kick plates (alley_0). Not made: the panel field keeps its speckled painted-steel finish. Verified at WIP f611321a (implementation/slice43): fabrication batch 0 failures across 14 modules (work tables included); apartment batch 204 on the long runner; household state 154 checks, 0 failures; upper kitchens 206; upper furniture 488 (eight fewer of the pre-existing material-binding class, from the headsets); upper lighting 0 failures; public doors 17 waypoints, 0 failures; door casings 107 openings, 0 failures; the eight-space sweep and the 130-station city sweep 0 failures.</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
@@ -21825,10 +21829,14 @@
       </c>
       <c r="S298" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T298" s="2" t="inlineStr"/>
+          <t>implemented</t>
+        </is>
+      </c>
+      <c r="T298" s="2" t="inlineStr">
+        <is>
+          <t>Omar's bench cupboard and its lower tray are grey painted iron (the catalogue iron_neutral) instead of blackened iron, so the carcass reads as painted sheet metal (3B_workbench_stock, native 3B_workbench). Not made: the shelving posts and the radio's seat. Verified at WIP f611321a (implementation/slice43): fabrication batch 0 failures across 14 modules (work tables included); apartment batch 204 on the long runner; household state 154 checks, 0 failures; upper kitchens 206; upper furniture 488 (eight fewer of the pre-existing material-binding class, from the headsets); upper lighting 0 failures; public doors 17 waypoints, 0 failures; door casings 107 openings, 0 failures; the eight-space sweep and the 130-station city sweep 0 failures.</t>
+        </is>
+      </c>
     </row>
     <row r="299">
       <c r="A299" s="2" t="inlineStr">
@@ -22133,10 +22141,14 @@
       </c>
       <c r="S302" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T302" s="2" t="inlineStr"/>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="T302" s="2" t="inlineStr">
+        <is>
+          <t>The service leaf's plain face gets flat-bar stiles, a top rail, a mid rail at lock height and kick plates on both faces in the leaf's cast-iron finish, so the kitchen's service door reads as a framed leaf, not a charcoal slab (F03_B_KITCHEN_RV). Verified at WIP f611321a (implementation/slice43): fabrication batch 0 failures across 14 modules (work tables included); apartment batch 204 on the long runner; household state 154 checks, 0 failures; upper kitchens 206; upper furniture 488 (eight fewer of the pre-existing material-binding class, from the headsets); upper lighting 0 failures; public doors 17 waypoints, 0 failures; door casings 107 openings, 0 failures; the eight-space sweep and the 130-station city sweep 0 failures.</t>
+        </is>
+      </c>
     </row>
     <row r="303">
       <c r="A303" s="2" t="inlineStr">
@@ -38757,10 +38769,14 @@
       </c>
       <c r="S528" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T528" s="2" t="inlineStr"/>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="T528" s="2" t="inlineStr">
+        <is>
+          <t>Sacha's desk wall is an oak top on two solid oak ends (a panel between a plinth and a cap) inside the original slab-support envelope, in place of the white painted slab on black folded pedestals; the headset lies on the desk, band on its side and both cups on their backs with the lead run off across the top, in place of the turned stand (implementation/slice43/images: 6A_deskwall_stock, F06_A_STUDY_OV, native 6A_deskwall). Verified at WIP f611321a (implementation/slice43): fabrication batch 0 failures across 14 modules (work tables included); apartment batch 204 on the long runner; household state 154 checks, 0 failures; upper kitchens 206; upper furniture 488 (eight fewer of the pre-existing material-binding class, from the headsets); upper lighting 0 failures; public doors 17 waypoints, 0 failures; door casings 107 openings, 0 failures; the eight-space sweep and the 130-station city sweep 0 failures.</t>
+        </is>
+      </c>
     </row>
     <row r="529">
       <c r="A529" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Implement dossier slice 47: resident bath sets, the overflowed umbrella tray
- F0x_y_BATH-001 (18 rows): each household's bath set on an opal glass
  shelf on nickel brackets between the basin's coved back and the
  medicine cabinet's lower edge (new bathshelf object form). The basin
  has a rolled rim and no ledge, and the surface-stock asset is at
  GitHub's file-size limit, so the sets are not stock on the rim.
- F04_A_VESTIBULE-003: Wren's drip tray gets grey standing water and his
  furled umbrella; the black water alone read as a floor register.
- New object keys need finish parameters: the runtime refused parts
  without one and nothing composed until they were added.
- The objects context inspector reads wall extensions (4B's bath wall).

Evidence under implementation/slice47/. INERT: no ledger status changes.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/art/reviews/v2_environment_design_20261008/change_register.xlsx
+++ b/art/reviews/v2_environment_design_20261008/change_register.xlsx
@@ -11539,10 +11539,14 @@
       </c>
       <c r="S163" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T163" s="2" t="inlineStr"/>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="T163" s="2" t="inlineStr">
+        <is>
+          <t>Evelyn's medicated routine: a glass with a dosing spoon, two small brown bottles, a powder box and a tin of hairpins (1A_bath_shelf_native). An opal glass shelf on two nickel brackets over the basin, between its coved back and the medicine cabinet's lower edge, carries the set (one domestic object per bath; the lavatory has a rolled rim and no flat ledge, and the surface-stock asset is at GitHub's file-size limit, so the set is not desktop stock on the rim). Verified at WIP 093e8d3f (implementation/slice47): fabrication batch 0 failures across the domestic objects and medicine cabinets (5 shelves and the tray captured natively); apartment batch 204 on the long runner; household state 154 checks, 0 failures; upper kitchens 206; upper furniture 488; upper lighting 0 failures; completion 1A 15 waypoints and 4D 12, each with its one pre-existing route failure; the nineteen-space sweep 0 failures. The objects context inspector finds all 72 bracket contacts on real wall faces (4B's on the bath's wall extension).</t>
+        </is>
+      </c>
     </row>
     <row r="164">
       <c r="A164" s="2" t="inlineStr">
@@ -13427,10 +13431,14 @@
       </c>
       <c r="S187" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T187" s="2" t="inlineStr"/>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="T187" s="2" t="inlineStr">
+        <is>
+          <t>Teresa's: a glass and toothbrush, a tin of pins for the bun, a brown antiseptic bottle (native DomesticObject71). An opal glass shelf on two nickel brackets over the basin, between its coved back and the medicine cabinet's lower edge, carries the set (one domestic object per bath; the lavatory has a rolled rim and no flat ledge, and the surface-stock asset is at GitHub's file-size limit, so the set is not desktop stock on the rim). Verified at WIP 093e8d3f (implementation/slice47): fabrication batch 0 failures across the domestic objects and medicine cabinets (5 shelves and the tray captured natively); apartment batch 204 on the long runner; household state 154 checks, 0 failures; upper kitchens 206; upper furniture 488; upper lighting 0 failures; completion 1A 15 waypoints and 4D 12, each with its one pre-existing route failure; the nineteen-space sweep 0 failures. The objects context inspector finds all 72 bracket contacts on real wall faces (4B's on the bath's wall extension).</t>
+        </is>
+      </c>
     </row>
     <row r="188">
       <c r="A188" s="2" t="inlineStr">
@@ -15863,10 +15871,14 @@
       </c>
       <c r="S219" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T219" s="2" t="inlineStr"/>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="T219" s="2" t="inlineStr">
+        <is>
+          <t>Mina's, kept exact: a glass and toothbrush, a cold-cream jar, a powder box and a comb (2A_bath_shelf_native). An opal glass shelf on two nickel brackets over the basin, between its coved back and the medicine cabinet's lower edge, carries the set (one domestic object per bath; the lavatory has a rolled rim and no flat ledge, and the surface-stock asset is at GitHub's file-size limit, so the set is not desktop stock on the rim). Verified at WIP 093e8d3f (implementation/slice47): fabrication batch 0 failures across the domestic objects and medicine cabinets (5 shelves and the tray captured natively); apartment batch 204 on the long runner; household state 154 checks, 0 failures; upper kitchens 206; upper furniture 488; upper lighting 0 failures; completion 1A 15 waypoints and 4D 12, each with its one pre-existing route failure; the nineteen-space sweep 0 failures. The objects context inspector finds all 72 bracket contacts on real wall faces (4B's on the bath's wall extension).</t>
+        </is>
+      </c>
     </row>
     <row r="220">
       <c r="A220" s="2" t="inlineStr">
@@ -17313,10 +17325,14 @@
       </c>
       <c r="S238" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T238" s="2" t="inlineStr"/>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="T238" s="2" t="inlineStr">
+        <is>
+          <t>Lena's: a glass and toothbrush, a cake of soap and the selvedge scrap she ties her hair with (native DomesticObject73). An opal glass shelf on two nickel brackets over the basin, between its coved back and the medicine cabinet's lower edge, carries the set (one domestic object per bath; the lavatory has a rolled rim and no flat ledge, and the surface-stock asset is at GitHub's file-size limit, so the set is not desktop stock on the rim). Verified at WIP 093e8d3f (implementation/slice47): fabrication batch 0 failures across the domestic objects and medicine cabinets (5 shelves and the tray captured natively); apartment batch 204 on the long runner; household state 154 checks, 0 failures; upper kitchens 206; upper furniture 488; upper lighting 0 failures; completion 1A 15 waypoints and 4D 12, each with its one pre-existing route failure; the nineteen-space sweep 0 failures. The objects context inspector finds all 72 bracket contacts on real wall faces (4B's on the bath's wall extension).</t>
+        </is>
+      </c>
     </row>
     <row r="239">
       <c r="A239" s="2" t="inlineStr">
@@ -18339,10 +18355,14 @@
       </c>
       <c r="S251" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T251" s="2" t="inlineStr"/>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="T251" s="2" t="inlineStr">
+        <is>
+          <t>Juno's: a glass and toothbrush, a kohl pot with its stick, a brass compact (native DomesticObject74). An opal glass shelf on two nickel brackets over the basin, between its coved back and the medicine cabinet's lower edge, carries the set (one domestic object per bath; the lavatory has a rolled rim and no flat ledge, and the surface-stock asset is at GitHub's file-size limit, so the set is not desktop stock on the rim). Verified at WIP 093e8d3f (implementation/slice47): fabrication batch 0 failures across the domestic objects and medicine cabinets (5 shelves and the tray captured natively); apartment batch 204 on the long runner; household state 154 checks, 0 failures; upper kitchens 206; upper furniture 488; upper lighting 0 failures; completion 1A 15 waypoints and 4D 12, each with its one pre-existing route failure; the nineteen-space sweep 0 failures. The objects context inspector finds all 72 bracket contacts on real wall faces (4B's on the bath's wall extension).</t>
+        </is>
+      </c>
     </row>
     <row r="252">
       <c r="A252" s="2" t="inlineStr">
@@ -21171,10 +21191,14 @@
       </c>
       <c r="S289" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T289" s="2" t="inlineStr"/>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="T289" s="2" t="inlineStr">
+        <is>
+          <t>Malcolm's: a glass and toothbrush, a nail brush for the earth under his nails, a shaving mug with its brush, a safety razor (native DomesticObject75). An opal glass shelf on two nickel brackets over the basin, between its coved back and the medicine cabinet's lower edge, carries the set (one domestic object per bath; the lavatory has a rolled rim and no flat ledge, and the surface-stock asset is at GitHub's file-size limit, so the set is not desktop stock on the rim). Verified at WIP 093e8d3f (implementation/slice47): fabrication batch 0 failures across the domestic objects and medicine cabinets (5 shelves and the tray captured natively); apartment batch 204 on the long runner; household state 154 checks, 0 failures; upper kitchens 206; upper furniture 488; upper lighting 0 failures; completion 1A 15 waypoints and 4D 12, each with its one pre-existing route failure; the nineteen-space sweep 0 failures. The objects context inspector finds all 72 bracket contacts on real wall faces (4B's on the bath's wall extension).</t>
+        </is>
+      </c>
     </row>
     <row r="290">
       <c r="A290" s="2" t="inlineStr">
@@ -22461,10 +22485,14 @@
       </c>
       <c r="S306" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T306" s="2" t="inlineStr"/>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="T306" s="2" t="inlineStr">
+        <is>
+          <t>Omar's practical set: a glass and toothbrush, a shaving mug, a nail brush, pumice and red carbolic soap (3B_bath_shelf_native). An opal glass shelf on two nickel brackets over the basin, between its coved back and the medicine cabinet's lower edge, carries the set (one domestic object per bath; the lavatory has a rolled rim and no flat ledge, and the surface-stock asset is at GitHub's file-size limit, so the set is not desktop stock on the rim). Verified at WIP 093e8d3f (implementation/slice47): fabrication batch 0 failures across the domestic objects and medicine cabinets (5 shelves and the tray captured natively); apartment batch 204 on the long runner; household state 154 checks, 0 failures; upper kitchens 206; upper furniture 488; upper lighting 0 failures; completion 1A 15 waypoints and 4D 12, each with its one pre-existing route failure; the nineteen-space sweep 0 failures. The objects context inspector finds all 72 bracket contacts on real wall faces (4B's on the bath's wall extension).</t>
+        </is>
+      </c>
     </row>
     <row r="307">
       <c r="A307" s="2" t="inlineStr">
@@ -23467,10 +23495,14 @@
       </c>
       <c r="S319" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T319" s="2" t="inlineStr"/>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="T319" s="2" t="inlineStr">
+        <is>
+          <t>Rhea's voice care: two glasses (gargle and rinse), a jar of pastilles, an inhaler and a lipstick (native DomesticObject77). An opal glass shelf on two nickel brackets over the basin, between its coved back and the medicine cabinet's lower edge, carries the set (one domestic object per bath; the lavatory has a rolled rim and no flat ledge, and the surface-stock asset is at GitHub's file-size limit, so the set is not desktop stock on the rim). Verified at WIP 093e8d3f (implementation/slice47): fabrication batch 0 failures across the domestic objects and medicine cabinets (5 shelves and the tray captured natively); apartment batch 204 on the long runner; household state 154 checks, 0 failures; upper kitchens 206; upper furniture 488; upper lighting 0 failures; completion 1A 15 waypoints and 4D 12, each with its one pre-existing route failure; the nineteen-space sweep 0 failures. The objects context inspector finds all 72 bracket contacts on real wall faces (4B's on the bath's wall extension).</t>
+        </is>
+      </c>
     </row>
     <row r="320">
       <c r="A320" s="2" t="inlineStr">
@@ -25709,10 +25741,14 @@
       </c>
       <c r="S350" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T350" s="2" t="inlineStr"/>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="T350" s="2" t="inlineStr">
+        <is>
+          <t>Wren's japanned umbrella drip tray by 4A's door, let overflow: grey standing water at the rim, a dark water line spread on the oak around it, and his furled umbrella standing in it against the wall (4A_umbrella_tray_native, F04_A_VESTIBULE_TH). Slice 44 placed the tray; its black water read as a floor register until slice 47. Verified at WIP 093e8d3f (implementation/slice47): fabrication batch 0 failures across the domestic objects and medicine cabinets (5 shelves and the tray captured natively); apartment batch 204 on the long runner; household state 154 checks, 0 failures; upper kitchens 206; upper furniture 488; upper lighting 0 failures; completion 1A 15 waypoints and 4D 12, each with its one pre-existing route failure; the nineteen-space sweep 0 failures. The objects context inspector finds all 72 bracket contacts on real wall faces (4B's on the bath's wall extension).</t>
+        </is>
+      </c>
     </row>
     <row r="351">
       <c r="A351" s="2" t="inlineStr">
@@ -26633,10 +26669,14 @@
       </c>
       <c r="S362" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T362" s="2" t="inlineStr"/>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="T362" s="2" t="inlineStr">
+        <is>
+          <t>Peter's, kept exact: a glass and toothbrush, a shaving mug, a safety razor and a comb (native DomesticObject78). An opal glass shelf on two nickel brackets over the basin, between its coved back and the medicine cabinet's lower edge, carries the set (one domestic object per bath; the lavatory has a rolled rim and no flat ledge, and the surface-stock asset is at GitHub's file-size limit, so the set is not desktop stock on the rim). Verified at WIP 093e8d3f (implementation/slice47): fabrication batch 0 failures across the domestic objects and medicine cabinets (5 shelves and the tray captured natively); apartment batch 204 on the long runner; household state 154 checks, 0 failures; upper kitchens 206; upper furniture 488; upper lighting 0 failures; completion 1A 15 waypoints and 4D 12, each with its one pre-existing route failure; the nineteen-space sweep 0 failures. The objects context inspector finds all 72 bracket contacts on real wall faces (4B's on the bath's wall extension).</t>
+        </is>
+      </c>
     </row>
     <row r="363">
       <c r="A363" s="2" t="inlineStr">
@@ -27977,10 +28017,14 @@
       </c>
       <c r="S380" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T380" s="2" t="inlineStr"/>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="T380" s="2" t="inlineStr">
+        <is>
+          <t>The player's: a glass and toothbrush, a cake of soap, a comb (native DomesticObject79). An opal glass shelf on two nickel brackets over the basin, between its coved back and the medicine cabinet's lower edge, carries the set (one domestic object per bath; the lavatory has a rolled rim and no flat ledge, and the surface-stock asset is at GitHub's file-size limit, so the set is not desktop stock on the rim). Verified at WIP 093e8d3f (implementation/slice47): fabrication batch 0 failures across the domestic objects and medicine cabinets (5 shelves and the tray captured natively); apartment batch 204 on the long runner; household state 154 checks, 0 failures; upper kitchens 206; upper furniture 488; upper lighting 0 failures; completion 1A 15 waypoints and 4D 12, each with its one pre-existing route failure; the nineteen-space sweep 0 failures. The objects context inspector finds all 72 bracket contacts on real wall faces (4B's on the bath's wall extension).</t>
+        </is>
+      </c>
     </row>
     <row r="381">
       <c r="A381" s="2" t="inlineStr">
@@ -29523,10 +29567,14 @@
       </c>
       <c r="S401" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T401" s="2" t="inlineStr"/>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="T401" s="2" t="inlineStr">
+        <is>
+          <t>Cam's and Noel's, divided: a glass and a soap on each side with a strip of tape between them (4C_bath_shelf_native). An opal glass shelf on two nickel brackets over the basin, between its coved back and the medicine cabinet's lower edge, carries the set (one domestic object per bath; the lavatory has a rolled rim and no flat ledge, and the surface-stock asset is at GitHub's file-size limit, so the set is not desktop stock on the rim). Verified at WIP 093e8d3f (implementation/slice47): fabrication batch 0 failures across the domestic objects and medicine cabinets (5 shelves and the tray captured natively); apartment batch 204 on the long runner; household state 154 checks, 0 failures; upper kitchens 206; upper furniture 488; upper lighting 0 failures; completion 1A 15 waypoints and 4D 12, each with its one pre-existing route failure; the nineteen-space sweep 0 failures. The objects context inspector finds all 72 bracket contacts on real wall faces (4B's on the bath's wall extension).</t>
+        </is>
+      </c>
     </row>
     <row r="402">
       <c r="A402" s="2" t="inlineStr">
@@ -30765,10 +30813,14 @@
       </c>
       <c r="S418" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T418" s="2" t="inlineStr"/>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="T418" s="2" t="inlineStr">
+        <is>
+          <t>The short-let: two wrapped cakes of hotel soap and a blank house-rules card propped at the back, nothing of anybody's (native DomesticObject81). An opal glass shelf on two nickel brackets over the basin, between its coved back and the medicine cabinet's lower edge, carries the set (one domestic object per bath; the lavatory has a rolled rim and no flat ledge, and the surface-stock asset is at GitHub's file-size limit, so the set is not desktop stock on the rim). Verified at WIP 093e8d3f (implementation/slice47): fabrication batch 0 failures across the domestic objects and medicine cabinets (5 shelves and the tray captured natively); apartment batch 204 on the long runner; household state 154 checks, 0 failures; upper kitchens 206; upper furniture 488; upper lighting 0 failures; completion 1A 15 waypoints and 4D 12, each with its one pre-existing route failure; the nineteen-space sweep 0 failures. The objects context inspector finds all 72 bracket contacts on real wall faces (4B's on the bath's wall extension).</t>
+        </is>
+      </c>
     </row>
     <row r="419">
       <c r="A419" s="2" t="inlineStr">
@@ -33311,10 +33363,14 @@
       </c>
       <c r="S453" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T453" s="2" t="inlineStr"/>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="T453" s="2" t="inlineStr">
+        <is>
+          <t>Nadia's practical set: a glass and toothbrush, a nail brush, pumice, carbolic soap and a lipstick (native DomesticObject82). An opal glass shelf on two nickel brackets over the basin, between its coved back and the medicine cabinet's lower edge, carries the set (one domestic object per bath; the lavatory has a rolled rim and no flat ledge, and the surface-stock asset is at GitHub's file-size limit, so the set is not desktop stock on the rim). Verified at WIP 093e8d3f (implementation/slice47): fabrication batch 0 failures across the domestic objects and medicine cabinets (5 shelves and the tray captured natively); apartment batch 204 on the long runner; household state 154 checks, 0 failures; upper kitchens 206; upper furniture 488; upper lighting 0 failures; completion 1A 15 waypoints and 4D 12, each with its one pre-existing route failure; the nineteen-space sweep 0 failures. The objects context inspector finds all 72 bracket contacts on real wall faces (4B's on the bath's wall extension).</t>
+        </is>
+      </c>
     </row>
     <row r="454">
       <c r="A454" s="2" t="inlineStr">
@@ -34841,10 +34897,14 @@
       </c>
       <c r="S474" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T474" s="2" t="inlineStr"/>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="T474" s="2" t="inlineStr">
+        <is>
+          <t>Cal's: a glass and toothbrush, a shaving mug, a safety razor and three hearing-aid cells (native DomesticObject83). An opal glass shelf on two nickel brackets over the basin, between its coved back and the medicine cabinet's lower edge, carries the set (one domestic object per bath; the lavatory has a rolled rim and no flat ledge, and the surface-stock asset is at GitHub's file-size limit, so the set is not desktop stock on the rim). Verified at WIP 093e8d3f (implementation/slice47): fabrication batch 0 failures across the domestic objects and medicine cabinets (5 shelves and the tray captured natively); apartment batch 204 on the long runner; household state 154 checks, 0 failures; upper kitchens 206; upper furniture 488; upper lighting 0 failures; completion 1A 15 waypoints and 4D 12, each with its one pre-existing route failure; the nineteen-space sweep 0 failures. The objects context inspector finds all 72 bracket contacts on real wall faces (4B's on the bath's wall extension).</t>
+        </is>
+      </c>
     </row>
     <row r="475">
       <c r="A475" s="2" t="inlineStr">
@@ -36025,10 +36085,14 @@
       </c>
       <c r="S490" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T490" s="2" t="inlineStr"/>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="T490" s="2" t="inlineStr">
+        <is>
+          <t>Iris's brush washing: a glass and toothbrush, a turpentine jar, a tin of brushes bristle-up and a nail brush (5C_bath_shelf_native). An opal glass shelf on two nickel brackets over the basin, between its coved back and the medicine cabinet's lower edge, carries the set (one domestic object per bath; the lavatory has a rolled rim and no flat ledge, and the surface-stock asset is at GitHub's file-size limit, so the set is not desktop stock on the rim). Verified at WIP 093e8d3f (implementation/slice47): fabrication batch 0 failures across the domestic objects and medicine cabinets (5 shelves and the tray captured natively); apartment batch 204 on the long runner; household state 154 checks, 0 failures; upper kitchens 206; upper furniture 488; upper lighting 0 failures; completion 1A 15 waypoints and 4D 12, each with its one pre-existing route failure; the nineteen-space sweep 0 failures. The objects context inspector finds all 72 bracket contacts on real wall faces (4B's on the bath's wall extension).</t>
+        </is>
+      </c>
     </row>
     <row r="491">
       <c r="A491" s="2" t="inlineStr">
@@ -38401,10 +38465,14 @@
       </c>
       <c r="S522" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T522" s="2" t="inlineStr"/>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="T522" s="2" t="inlineStr">
+        <is>
+          <t>Sacha's: a glass and toothbrush, two brown developer bottles and bamboo print tongs, the bath being a darkroom twice a week (native DomesticObject85). An opal glass shelf on two nickel brackets over the basin, between its coved back and the medicine cabinet's lower edge, carries the set (one domestic object per bath; the lavatory has a rolled rim and no flat ledge, and the surface-stock asset is at GitHub's file-size limit, so the set is not desktop stock on the rim). Verified at WIP 093e8d3f (implementation/slice47): fabrication batch 0 failures across the domestic objects and medicine cabinets (5 shelves and the tray captured natively); apartment batch 204 on the long runner; household state 154 checks, 0 failures; upper kitchens 206; upper furniture 488; upper lighting 0 failures; completion 1A 15 waypoints and 4D 12, each with its one pre-existing route failure; the nineteen-space sweep 0 failures. The objects context inspector finds all 72 bracket contacts on real wall faces (4B's on the bath's wall extension).</t>
+        </is>
+      </c>
     </row>
     <row r="523">
       <c r="A523" s="2" t="inlineStr">
@@ -39647,10 +39715,14 @@
       </c>
       <c r="S539" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T539" s="2" t="inlineStr"/>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="T539" s="2" t="inlineStr">
+        <is>
+          <t>Jonah's: a glass and toothbrush, a shaving mug and a safety razor he rarely uses (native DomesticObject86). An opal glass shelf on two nickel brackets over the basin, between its coved back and the medicine cabinet's lower edge, carries the set (one domestic object per bath; the lavatory has a rolled rim and no flat ledge, and the surface-stock asset is at GitHub's file-size limit, so the set is not desktop stock on the rim). Verified at WIP 093e8d3f (implementation/slice47): fabrication batch 0 failures across the domestic objects and medicine cabinets (5 shelves and the tray captured natively); apartment batch 204 on the long runner; household state 154 checks, 0 failures; upper kitchens 206; upper furniture 488; upper lighting 0 failures; completion 1A 15 waypoints and 4D 12, each with its one pre-existing route failure; the nineteen-space sweep 0 failures. The objects context inspector finds all 72 bracket contacts on real wall faces (4B's on the bath's wall extension).</t>
+        </is>
+      </c>
     </row>
     <row r="540">
       <c r="A540" s="2" t="inlineStr">
@@ -40741,10 +40813,14 @@
       </c>
       <c r="S554" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T554" s="2" t="inlineStr"/>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="T554" s="2" t="inlineStr">
+        <is>
+          <t>Mae's, kept exact: a glass and toothbrush, a powder box, a tin of hairpins, a lipstick and her buttonhook (native DomesticObject87). An opal glass shelf on two nickel brackets over the basin, between its coved back and the medicine cabinet's lower edge, carries the set (one domestic object per bath; the lavatory has a rolled rim and no flat ledge, and the surface-stock asset is at GitHub's file-size limit, so the set is not desktop stock on the rim). Verified at WIP 093e8d3f (implementation/slice47): fabrication batch 0 failures across the domestic objects and medicine cabinets (5 shelves and the tray captured natively); apartment batch 204 on the long runner; household state 154 checks, 0 failures; upper kitchens 206; upper furniture 488; upper lighting 0 failures; completion 1A 15 waypoints and 4D 12, each with its one pre-existing route failure; the nineteen-space sweep 0 failures. The objects context inspector finds all 72 bracket contacts on real wall faces (4B's on the bath's wall extension).</t>
+        </is>
+      </c>
     </row>
     <row r="555">
       <c r="A555" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Implement dossier slice 48: the building's paper trail on every core level
- F0x_PUBLIC_CORE-001, F02-F04_LANDING-001, ROOF_PUBLIC_CORE-001: the 1928
  house rules in a taped oak frame on each public core's north wall.
- F0x_SERVICE_CORE-001, ROOF_SERVICE_CORE-001: the service notice pinned
  beside each service core's brass floor plate.
- B1_PUBLIC_CORE-002: the basement notice at the stair foot.
- New noticeframe object form; the runtime lays the record's notice_text
  on the paper as a shaded Label3D (no lettering in textures). The words
  keep to documented facts (Management in 5A, the Superintendent in 3B,
  the hand-fired boiler, the rear apron).
- The ground core transfer route's one failure is identical at slice 47.

Evidence under implementation/slice48/. INERT: no ledger status changes.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/art/reviews/v2_environment_design_20261008/change_register.xlsx
+++ b/art/reviews/v2_environment_design_20261008/change_register.xlsx
@@ -955,10 +955,14 @@
       </c>
       <c r="S7" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T7" s="2" t="inlineStr"/>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="T7" s="2" t="inlineStr">
+        <is>
+          <t>The basement notice at the stair foot, in the same taped oak frame on the core's north wall: the boiler room for the Superintendent only; the boiler hand-fired morning and night; coal in 6 November 1928; laundry by the rota; MANAGEMENT. No boiler hours are documented, so the notice gives none (B1_PUBLIC_CORE_DT2). Verified at WIP 1acecafb (implementation/slice48): fabrication batch 0 failures (both notice boards captured natively, the words legible under the lamp); apartment batch 204 on the long runner; household state 154 checks, 0 failures; upper kitchens 206; upper furniture 488; upper lighting 0 failures; public doors 17 waypoints, the remaining upper transfers 28, the basement route 88 and public furnishings 29, all 0 failures; the ground core transfer route 1 waypoint with its one failure (it stops one riser above the basement landing, identical at slice 47, 6d62caab); the eighteen-space core sweep 0 failures. The objects context inspector finds every frame on a real core wall face.</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -9617,10 +9621,14 @@
       </c>
       <c r="S138" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T138" s="2" t="inlineStr"/>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="T138" s="2" t="inlineStr">
+        <is>
+          <t>The 1928 house rules on an oak-framed notice board (0.35 x 0.45 m, centre 1.5 m) on the public core's north wall beside the landing, clear of the C door and the stair: rents to Management, Apartment 5A, on the first; leaks, heat and repairs to the Superintendent, 3B; keep the stair and landings clear; quiet after ten o'clock; signed MANAGEMENT. The words are a shaded Label3D on the paper, so the lamp reads them. The board has no glass (the family has none); kraft tape crosses its top corner where the glass would be cracked (F01_PUBLIC_CORE_DT1, F01_PUBLIC_NOTICE_native). Verified at WIP 1acecafb (implementation/slice48): fabrication batch 0 failures (both notice boards captured natively, the words legible under the lamp); apartment batch 204 on the long runner; household state 154 checks, 0 failures; upper kitchens 206; upper furniture 488; upper lighting 0 failures; public doors 17 waypoints, the remaining upper transfers 28, the basement route 88 and public furnishings 29, all 0 failures; the ground core transfer route 1 waypoint with its one failure (it stops one riser above the basement landing, identical at slice 47, 6d62caab); the eighteen-space core sweep 0 failures. The objects context inspector finds every frame on a real core wall face.</t>
+        </is>
+      </c>
     </row>
     <row r="139">
       <c r="A139" s="2" t="inlineStr">
@@ -10049,10 +10057,14 @@
       </c>
       <c r="S144" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T144" s="2" t="inlineStr"/>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="T144" s="2" t="inlineStr">
+        <is>
+          <t>The service notice, pinned in an oak frame on the service core's south wall above the landing, beside the brass floor plate: service stair for staff, trades and deliveries; coal and ash by the rear apron; the boiler fired by the Superintendent; keep the stair clear; MANAGEMENT. A shaded Label3D on the paper (F01_SERVICE_CORE_DT1, F01_SERVICE_NOTICE_native). Verified at WIP 1acecafb (implementation/slice48): fabrication batch 0 failures (both notice boards captured natively, the words legible under the lamp); apartment batch 204 on the long runner; household state 154 checks, 0 failures; upper kitchens 206; upper furniture 488; upper lighting 0 failures; public doors 17 waypoints, the remaining upper transfers 28, the basement route 88 and public furnishings 29, all 0 failures; the ground core transfer route 1 waypoint with its one failure (it stops one riser above the basement landing, identical at slice 47, 6d62caab); the eighteen-space core sweep 0 failures. The objects context inspector finds every frame on a real core wall face.</t>
+        </is>
+      </c>
     </row>
     <row r="145">
       <c r="A145" s="2" t="inlineStr">
@@ -13653,10 +13665,14 @@
       </c>
       <c r="S190" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T190" s="2" t="inlineStr"/>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="T190" s="2" t="inlineStr">
+        <is>
+          <t>The 1928 house rules on an oak-framed notice board (0.35 x 0.45 m, centre 1.5 m) on the public core's north wall beside the landing, clear of the C door and the stair: rents to Management, Apartment 5A, on the first; leaks, heat and repairs to the Superintendent, 3B; keep the stair and landings clear; quiet after ten o'clock; signed MANAGEMENT. The words are a shaded Label3D on the paper, so the lamp reads them. The board has no glass (the family has none); kraft tape crosses its top corner where the glass would be cracked (F02_PUBLIC_CORE_DT1). The landing and the public core share the one board. Verified at WIP 1acecafb (implementation/slice48): fabrication batch 0 failures (both notice boards captured natively, the words legible under the lamp); apartment batch 204 on the long runner; household state 154 checks, 0 failures; upper kitchens 206; upper furniture 488; upper lighting 0 failures; public doors 17 waypoints, the remaining upper transfers 28, the basement route 88 and public furnishings 29, all 0 failures; the ground core transfer route 1 waypoint with its one failure (it stops one riser above the basement landing, identical at slice 47, 6d62caab); the eighteen-space core sweep 0 failures. The objects context inspector finds every frame on a real core wall face.</t>
+        </is>
+      </c>
     </row>
     <row r="191">
       <c r="A191" s="2" t="inlineStr">
@@ -14097,10 +14113,14 @@
       </c>
       <c r="S196" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T196" s="2" t="inlineStr"/>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="T196" s="2" t="inlineStr">
+        <is>
+          <t>The 1928 house rules on an oak-framed notice board (0.35 x 0.45 m, centre 1.5 m) on the public core's north wall beside the landing, clear of the C door and the stair: rents to Management, Apartment 5A, on the first; leaks, heat and repairs to the Superintendent, 3B; keep the stair and landings clear; quiet after ten o'clock; signed MANAGEMENT. The words are a shaded Label3D on the paper, so the lamp reads them. The board has no glass (the family has none); kraft tape crosses its top corner where the glass would be cracked (F02_PUBLIC_CORE_DT1). Verified at WIP 1acecafb (implementation/slice48): fabrication batch 0 failures (both notice boards captured natively, the words legible under the lamp); apartment batch 204 on the long runner; household state 154 checks, 0 failures; upper kitchens 206; upper furniture 488; upper lighting 0 failures; public doors 17 waypoints, the remaining upper transfers 28, the basement route 88 and public furnishings 29, all 0 failures; the ground core transfer route 1 waypoint with its one failure (it stops one riser above the basement landing, identical at slice 47, 6d62caab); the eighteen-space core sweep 0 failures. The objects context inspector finds every frame on a real core wall face.</t>
+        </is>
+      </c>
     </row>
     <row r="197">
       <c r="A197" s="2" t="inlineStr">
@@ -14627,10 +14647,14 @@
       </c>
       <c r="S203" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T203" s="2" t="inlineStr"/>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="T203" s="2" t="inlineStr">
+        <is>
+          <t>The service notice, pinned in an oak frame on the service core's south wall above the landing, beside the brass floor plate: service stair for staff, trades and deliveries; coal and ash by the rear apron; the boiler fired by the Superintendent; keep the stair clear; MANAGEMENT. A shaded Label3D on the paper (F02_SERVICE_CORE_DT1). Verified at WIP 1acecafb (implementation/slice48): fabrication batch 0 failures (both notice boards captured natively, the words legible under the lamp); apartment batch 204 on the long runner; household state 154 checks, 0 failures; upper kitchens 206; upper furniture 488; upper lighting 0 failures; public doors 17 waypoints, the remaining upper transfers 28, the basement route 88 and public furnishings 29, all 0 failures; the ground core transfer route 1 waypoint with its one failure (it stops one riser above the basement landing, identical at slice 47, 6d62caab); the eighteen-space core sweep 0 failures. The objects context inspector finds every frame on a real core wall face.</t>
+        </is>
+      </c>
     </row>
     <row r="204">
       <c r="A204" s="2" t="inlineStr">
@@ -18939,10 +18963,14 @@
       </c>
       <c r="S259" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T259" s="2" t="inlineStr"/>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="T259" s="2" t="inlineStr">
+        <is>
+          <t>The 1928 house rules on an oak-framed notice board (0.35 x 0.45 m, centre 1.5 m) on the public core's north wall beside the landing, clear of the C door and the stair: rents to Management, Apartment 5A, on the first; leaks, heat and repairs to the Superintendent, 3B; keep the stair and landings clear; quiet after ten o'clock; signed MANAGEMENT. The words are a shaded Label3D on the paper, so the lamp reads them. The board has no glass (the family has none); kraft tape crosses its top corner where the glass would be cracked (F03_PUBLIC_CORE_DT1). Verified at WIP 1acecafb (implementation/slice48): fabrication batch 0 failures (both notice boards captured natively, the words legible under the lamp); apartment batch 204 on the long runner; household state 154 checks, 0 failures; upper kitchens 206; upper furniture 488; upper lighting 0 failures; public doors 17 waypoints, the remaining upper transfers 28, the basement route 88 and public furnishings 29, all 0 failures; the ground core transfer route 1 waypoint with its one failure (it stops one riser above the basement landing, identical at slice 47, 6d62caab); the eighteen-space core sweep 0 failures. The objects context inspector finds every frame on a real core wall face.</t>
+        </is>
+      </c>
     </row>
     <row r="260">
       <c r="A260" s="2" t="inlineStr">
@@ -19087,10 +19115,14 @@
       </c>
       <c r="S261" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T261" s="2" t="inlineStr"/>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="T261" s="2" t="inlineStr">
+        <is>
+          <t>The service notice, pinned in an oak frame on the service core's south wall above the landing, beside the brass floor plate: service stair for staff, trades and deliveries; coal and ash by the rear apron; the boiler fired by the Superintendent; keep the stair clear; MANAGEMENT. A shaded Label3D on the paper (F03_SERVICE_CORE_DT1). Verified at WIP 1acecafb (implementation/slice48): fabrication batch 0 failures (both notice boards captured natively, the words legible under the lamp); apartment batch 204 on the long runner; household state 154 checks, 0 failures; upper kitchens 206; upper furniture 488; upper lighting 0 failures; public doors 17 waypoints, the remaining upper transfers 28, the basement route 88 and public furnishings 29, all 0 failures; the ground core transfer route 1 waypoint with its one failure (it stops one riser above the basement landing, identical at slice 47, 6d62caab); the eighteen-space core sweep 0 failures. The objects context inspector finds every frame on a real core wall face.</t>
+        </is>
+      </c>
     </row>
     <row r="262">
       <c r="A262" s="2" t="inlineStr">
@@ -19235,10 +19267,14 @@
       </c>
       <c r="S263" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T263" s="2" t="inlineStr"/>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="T263" s="2" t="inlineStr">
+        <is>
+          <t>The 1928 house rules on an oak-framed notice board (0.35 x 0.45 m, centre 1.5 m) on the public core's north wall beside the landing, clear of the C door and the stair: rents to Management, Apartment 5A, on the first; leaks, heat and repairs to the Superintendent, 3B; keep the stair and landings clear; quiet after ten o'clock; signed MANAGEMENT. The words are a shaded Label3D on the paper, so the lamp reads them. The board has no glass (the family has none); kraft tape crosses its top corner where the glass would be cracked (F03_PUBLIC_CORE_DT1). The landing and the public core share the one board. Verified at WIP 1acecafb (implementation/slice48): fabrication batch 0 failures (both notice boards captured natively, the words legible under the lamp); apartment batch 204 on the long runner; household state 154 checks, 0 failures; upper kitchens 206; upper furniture 488; upper lighting 0 failures; public doors 17 waypoints, the remaining upper transfers 28, the basement route 88 and public furnishings 29, all 0 failures; the ground core transfer route 1 waypoint with its one failure (it stops one riser above the basement landing, identical at slice 47, 6d62caab); the eighteen-space core sweep 0 failures. The objects context inspector finds every frame on a real core wall face.</t>
+        </is>
+      </c>
     </row>
     <row r="264">
       <c r="A264" s="2" t="inlineStr">
@@ -24071,10 +24107,14 @@
       </c>
       <c r="S327" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T327" s="2" t="inlineStr"/>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="T327" s="2" t="inlineStr">
+        <is>
+          <t>The 1928 house rules on an oak-framed notice board (0.35 x 0.45 m, centre 1.5 m) on the public core's north wall beside the landing, clear of the C door and the stair: rents to Management, Apartment 5A, on the first; leaks, heat and repairs to the Superintendent, 3B; keep the stair and landings clear; quiet after ten o'clock; signed MANAGEMENT. The words are a shaded Label3D on the paper, so the lamp reads them. The board has no glass (the family has none); kraft tape crosses its top corner where the glass would be cracked (F04_PUBLIC_CORE_DT1). The landing and the public core share the one board. Verified at WIP 1acecafb (implementation/slice48): fabrication batch 0 failures (both notice boards captured natively, the words legible under the lamp); apartment batch 204 on the long runner; household state 154 checks, 0 failures; upper kitchens 206; upper furniture 488; upper lighting 0 failures; public doors 17 waypoints, the remaining upper transfers 28, the basement route 88 and public furnishings 29, all 0 failures; the ground core transfer route 1 waypoint with its one failure (it stops one riser above the basement landing, identical at slice 47, 6d62caab); the eighteen-space core sweep 0 failures. The objects context inspector finds every frame on a real core wall face.</t>
+        </is>
+      </c>
     </row>
     <row r="328">
       <c r="A328" s="2" t="inlineStr">
@@ -24705,10 +24745,14 @@
       </c>
       <c r="S336" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T336" s="2" t="inlineStr"/>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="T336" s="2" t="inlineStr">
+        <is>
+          <t>The 1928 house rules on an oak-framed notice board (0.35 x 0.45 m, centre 1.5 m) on the public core's north wall beside the landing, clear of the C door and the stair: rents to Management, Apartment 5A, on the first; leaks, heat and repairs to the Superintendent, 3B; keep the stair and landings clear; quiet after ten o'clock; signed MANAGEMENT. The words are a shaded Label3D on the paper, so the lamp reads them. The board has no glass (the family has none); kraft tape crosses its top corner where the glass would be cracked (F04_PUBLIC_CORE_DT1). Verified at WIP 1acecafb (implementation/slice48): fabrication batch 0 failures (both notice boards captured natively, the words legible under the lamp); apartment batch 204 on the long runner; household state 154 checks, 0 failures; upper kitchens 206; upper furniture 488; upper lighting 0 failures; public doors 17 waypoints, the remaining upper transfers 28, the basement route 88 and public furnishings 29, all 0 failures; the ground core transfer route 1 waypoint with its one failure (it stops one riser above the basement landing, identical at slice 47, 6d62caab); the eighteen-space core sweep 0 failures. The objects context inspector finds every frame on a real core wall face.</t>
+        </is>
+      </c>
     </row>
     <row r="337">
       <c r="A337" s="2" t="inlineStr">
@@ -25433,10 +25477,14 @@
       </c>
       <c r="S346" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T346" s="2" t="inlineStr"/>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="T346" s="2" t="inlineStr">
+        <is>
+          <t>The service notice, pinned in an oak frame on the service core's south wall above the landing, beside the brass floor plate: service stair for staff, trades and deliveries; coal and ash by the rear apron; the boiler fired by the Superintendent; keep the stair clear; MANAGEMENT. A shaded Label3D on the paper (F04_SERVICE_CORE_DT1). Verified at WIP 1acecafb (implementation/slice48): fabrication batch 0 failures (both notice boards captured natively, the words legible under the lamp); apartment batch 204 on the long runner; household state 154 checks, 0 failures; upper kitchens 206; upper furniture 488; upper lighting 0 failures; public doors 17 waypoints, the remaining upper transfers 28, the basement route 88 and public furnishings 29, all 0 failures; the ground core transfer route 1 waypoint with its one failure (it stops one riser above the basement landing, identical at slice 47, 6d62caab); the eighteen-space core sweep 0 failures. The objects context inspector finds every frame on a real core wall face.</t>
+        </is>
+      </c>
     </row>
     <row r="347">
       <c r="A347" s="2" t="inlineStr">
@@ -31233,10 +31281,14 @@
       </c>
       <c r="S424" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T424" s="2" t="inlineStr"/>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="T424" s="2" t="inlineStr">
+        <is>
+          <t>The 1928 house rules on an oak-framed notice board (0.35 x 0.45 m, centre 1.5 m) on the public core's north wall beside the landing, clear of the C door and the stair: rents to Management, Apartment 5A, on the first; leaks, heat and repairs to the Superintendent, 3B; keep the stair and landings clear; quiet after ten o'clock; signed MANAGEMENT. The words are a shaded Label3D on the paper, so the lamp reads them. The board has no glass (the family has none); kraft tape crosses its top corner where the glass would be cracked (F05_PUBLIC_CORE_DT1). Verified at WIP 1acecafb (implementation/slice48): fabrication batch 0 failures (both notice boards captured natively, the words legible under the lamp); apartment batch 204 on the long runner; household state 154 checks, 0 failures; upper kitchens 206; upper furniture 488; upper lighting 0 failures; public doors 17 waypoints, the remaining upper transfers 28, the basement route 88 and public furnishings 29, all 0 failures; the ground core transfer route 1 waypoint with its one failure (it stops one riser above the basement landing, identical at slice 47, 6d62caab); the eighteen-space core sweep 0 failures. The objects context inspector finds every frame on a real core wall face.</t>
+        </is>
+      </c>
     </row>
     <row r="425">
       <c r="A425" s="2" t="inlineStr">
@@ -31513,10 +31565,14 @@
       </c>
       <c r="S428" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T428" s="2" t="inlineStr"/>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="T428" s="2" t="inlineStr">
+        <is>
+          <t>The service notice, pinned in an oak frame on the service core's south wall above the landing, beside the brass floor plate: service stair for staff, trades and deliveries; coal and ash by the rear apron; the boiler fired by the Superintendent; keep the stair clear; MANAGEMENT. A shaded Label3D on the paper (F05_SERVICE_CORE_DT1). Verified at WIP 1acecafb (implementation/slice48): fabrication batch 0 failures (both notice boards captured natively, the words legible under the lamp); apartment batch 204 on the long runner; household state 154 checks, 0 failures; upper kitchens 206; upper furniture 488; upper lighting 0 failures; public doors 17 waypoints, the remaining upper transfers 28, the basement route 88 and public furnishings 29, all 0 failures; the ground core transfer route 1 waypoint with its one failure (it stops one riser above the basement landing, identical at slice 47, 6d62caab); the eighteen-space core sweep 0 failures. The objects context inspector finds every frame on a real core wall face.</t>
+        </is>
+      </c>
     </row>
     <row r="429">
       <c r="A429" s="2" t="inlineStr">
@@ -36797,10 +36853,14 @@
       </c>
       <c r="S500" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T500" s="2" t="inlineStr"/>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="T500" s="2" t="inlineStr">
+        <is>
+          <t>The 1928 house rules on an oak-framed notice board (0.35 x 0.45 m, centre 1.5 m) on the public core's north wall beside the landing, clear of the C door and the stair: rents to Management, Apartment 5A, on the first; leaks, heat and repairs to the Superintendent, 3B; keep the stair and landings clear; quiet after ten o'clock; signed MANAGEMENT. The words are a shaded Label3D on the paper, so the lamp reads them. The board has no glass (the family has none); kraft tape crosses its top corner where the glass would be cracked (F06_PUBLIC_CORE_DT1). Verified at WIP 1acecafb (implementation/slice48): fabrication batch 0 failures (both notice boards captured natively, the words legible under the lamp); apartment batch 204 on the long runner; household state 154 checks, 0 failures; upper kitchens 206; upper furniture 488; upper lighting 0 failures; public doors 17 waypoints, the remaining upper transfers 28, the basement route 88 and public furnishings 29, all 0 failures; the ground core transfer route 1 waypoint with its one failure (it stops one riser above the basement landing, identical at slice 47, 6d62caab); the eighteen-space core sweep 0 failures. The objects context inspector finds every frame on a real core wall face.</t>
+        </is>
+      </c>
     </row>
     <row r="501">
       <c r="A501" s="2" t="inlineStr">
@@ -37011,10 +37071,14 @@
       </c>
       <c r="S503" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T503" s="2" t="inlineStr"/>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="T503" s="2" t="inlineStr">
+        <is>
+          <t>The service notice, pinned in an oak frame on the service core's south wall above the landing, beside the brass floor plate: service stair for staff, trades and deliveries; coal and ash by the rear apron; the boiler fired by the Superintendent; keep the stair clear; MANAGEMENT. A shaded Label3D on the paper (F06_SERVICE_CORE_DT1). Verified at WIP 1acecafb (implementation/slice48): fabrication batch 0 failures (both notice boards captured natively, the words legible under the lamp); apartment batch 204 on the long runner; household state 154 checks, 0 failures; upper kitchens 206; upper furniture 488; upper lighting 0 failures; public doors 17 waypoints, the remaining upper transfers 28, the basement route 88 and public furnishings 29, all 0 failures; the ground core transfer route 1 waypoint with its one failure (it stops one riser above the basement landing, identical at slice 47, 6d62caab); the eighteen-space core sweep 0 failures. The objects context inspector finds every frame on a real core wall face.</t>
+        </is>
+      </c>
     </row>
     <row r="504">
       <c r="A504" s="2" t="inlineStr">
@@ -41311,10 +41375,14 @@
       </c>
       <c r="S561" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T561" s="2" t="inlineStr"/>
+          <t>implemented</t>
+        </is>
+      </c>
+      <c r="T561" s="2" t="inlineStr">
+        <is>
+          <t>The 1928 house rules on an oak-framed notice board (0.35 x 0.45 m, centre 1.5 m) on the public core's north wall beside the landing, clear of the C door and the stair: rents to Management, Apartment 5A, on the first; leaks, heat and repairs to the Superintendent, 3B; keep the stair and landings clear; quiet after ten o'clock; signed MANAGEMENT. The words are a shaded Label3D on the paper, so the lamp reads them. The board has no glass (the family has none); kraft tape crosses its top corner where the glass would be cracked (no sweep station frames it; same board as F01_PUBLIC_NOTICE_native). Verified at WIP 1acecafb (implementation/slice48): fabrication batch 0 failures (both notice boards captured natively, the words legible under the lamp); apartment batch 204 on the long runner; household state 154 checks, 0 failures; upper kitchens 206; upper furniture 488; upper lighting 0 failures; public doors 17 waypoints, the remaining upper transfers 28, the basement route 88 and public furnishings 29, all 0 failures; the ground core transfer route 1 waypoint with its one failure (it stops one riser above the basement landing, identical at slice 47, 6d62caab); the eighteen-space core sweep 0 failures. The objects context inspector finds every frame on a real core wall face.</t>
+        </is>
+      </c>
     </row>
     <row r="562">
       <c r="A562" s="2" t="inlineStr">
@@ -41595,10 +41663,14 @@
       </c>
       <c r="S565" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T565" s="2" t="inlineStr"/>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="T565" s="2" t="inlineStr">
+        <is>
+          <t>The service notice, pinned in an oak frame on the service core's south wall above the landing, beside the brass floor plate: service stair for staff, trades and deliveries; coal and ash by the rear apron; the boiler fired by the Superintendent; keep the stair clear; MANAGEMENT. A shaded Label3D on the paper (ROOF_SERVICE_CORE_DT3). Verified at WIP 1acecafb (implementation/slice48): fabrication batch 0 failures (both notice boards captured natively, the words legible under the lamp); apartment batch 204 on the long runner; household state 154 checks, 0 failures; upper kitchens 206; upper furniture 488; upper lighting 0 failures; public doors 17 waypoints, the remaining upper transfers 28, the basement route 88 and public furnishings 29, all 0 failures; the ground core transfer route 1 waypoint with its one failure (it stops one riser above the basement landing, identical at slice 47, 6d62caab); the eighteen-space core sweep 0 failures. The objects context inspector finds every frame on a real core wall face.</t>
+        </is>
+      </c>
     </row>
     <row r="566">
       <c r="A566" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Implement dossier slice 49: door thresholds, a household at every door
- F02-F06_WEST_HALL-001, F02/F03_SOUTHWEST_HALL-001, F02/F04_EAST_HALL-001:
  a household's mat on the hall side of each apartment door, within 0.5 m
  of the jamb and outside the swing, flat inside the 1.2 m hall route:
  squared coir, worn coir, a rag rug of selvedge scraps, ribbed rubber,
  soil- or paint-flecked coir; the morning paper on two; milk bottles and
  a string-tied parcel only on the wide core floor.
- F02_D_RESTRICTED-002 (partial): the sealed 2D door's unworn dust mat and
  its one-line notice in the notice-frame family; no letter-slot strip.
- New threshold object form. Resident key passes on the long runner at
  slice 51's WIP, which carries this slice unchanged; rear wing C's one
  failure is identical at slice 48's tip.

Evidence under implementation/slice49/. INERT: no ledger status changes.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/art/reviews/v2_environment_design_20261008/change_register.xlsx
+++ b/art/reviews/v2_environment_design_20261008/change_register.xlsx
@@ -13817,10 +13817,14 @@
       </c>
       <c r="S192" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T192" s="2" t="inlineStr"/>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="T192" s="2" t="inlineStr">
+        <is>
+          <t>2A's coir mat squared to the jamb (Mina keeps things exact); from the landing it reads beside 2C's worn mat and the two milk bottles waiting at the core (F02_WEST_HALL_OV, 2A_threshold_native). Verified at WIP 36f8f9bb (implementation/slice49): fabrication batch 0 failures (six thresholds captured natively); apartment batch 204 on the long runner; household state 154 checks, 0 failures; upper kitchens 206 and upper furniture 488, both identical to slice 48; upper lighting, public doors, the remaining upper transfers, the apartment door route, the first upper hall, the 4B door and rear wing A, all 0 failures; the resident key route, which the serial runner's 180 s ceiling ended without a verdict at this WIP, passes on the long runner at slice 51's WIP 0bac8f87 (86 waypoints, 0 failures), a tree that carries slice 49 unchanged. Rear wing C's one failure (the 2C bookshelf collision) is identical at slice 48's tip. The three hall sweeps (17 spaces) report 0 failures. Every threshold lies flat inside the 1.2 m hall route, within 0.5 m of its jamb and outside the swing.</t>
+        </is>
+      </c>
     </row>
     <row r="193">
       <c r="A193" s="2" t="inlineStr">
@@ -13965,10 +13969,14 @@
       </c>
       <c r="S194" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T194" s="2" t="inlineStr"/>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="T194" s="2" t="inlineStr">
+        <is>
+          <t>The sealed 2D door's dust mat, new and unmarked, squared at the jamb; read from the hall against 2A's exact coir and 2C's worn mat beyond (F02_SOUTHWEST_HALL_OV). Verified at WIP 36f8f9bb (implementation/slice49): fabrication batch 0 failures (six thresholds captured natively); apartment batch 204 on the long runner; household state 154 checks, 0 failures; upper kitchens 206 and upper furniture 488, both identical to slice 48; upper lighting, public doors, the remaining upper transfers, the apartment door route, the first upper hall, the 4B door and rear wing A, all 0 failures; the resident key route, which the serial runner's 180 s ceiling ended without a verdict at this WIP, passes on the long runner at slice 51's WIP 0bac8f87 (86 waypoints, 0 failures), a tree that carries slice 49 unchanged. Rear wing C's one failure (the 2C bookshelf collision) is identical at slice 48's tip. The three hall sweeps (17 spaces) report 0 failures. Every threshold lies flat inside the 1.2 m hall route, within 0.5 m of its jamb and outside the swing.</t>
+        </is>
+      </c>
     </row>
     <row r="195">
       <c r="A195" s="2" t="inlineStr">
@@ -14265,10 +14273,14 @@
       </c>
       <c r="S198" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T198" s="2" t="inlineStr"/>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="T198" s="2" t="inlineStr">
+        <is>
+          <t>Looking down the east hall from the core: 2C's worn mat and milk at the core end, 2B's rag rug of selvedge scraps at the crossing end (F02_EAST_HALL_RV, F02_SERVICE_CROSSING_OV, 2B_threshold_native). Verified at WIP 36f8f9bb (implementation/slice49): fabrication batch 0 failures (six thresholds captured natively); apartment batch 204 on the long runner; household state 154 checks, 0 failures; upper kitchens 206 and upper furniture 488, both identical to slice 48; upper lighting, public doors, the remaining upper transfers, the apartment door route, the first upper hall, the 4B door and rear wing A, all 0 failures; the resident key route, which the serial runner's 180 s ceiling ended without a verdict at this WIP, passes on the long runner at slice 51's WIP 0bac8f87 (86 waypoints, 0 failures), a tree that carries slice 49 unchanged. Rear wing C's one failure (the 2C bookshelf collision) is identical at slice 48's tip. The three hall sweeps (17 spaces) report 0 failures. Every threshold lies flat inside the 1.2 m hall route, within 0.5 m of its jamb and outside the swing.</t>
+        </is>
+      </c>
     </row>
     <row r="199">
       <c r="A199" s="2" t="inlineStr">
@@ -18885,10 +18897,14 @@
       </c>
       <c r="S258" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T258" s="2" t="inlineStr"/>
+          <t>implemented</t>
+        </is>
+      </c>
+      <c r="T258" s="2" t="inlineStr">
+        <is>
+          <t>Partial: the sealed door's clean dust mat is squared at the jamb on the hall side, and its one-line notice hangs at 1.5 m in the core notice-frame family (slice 48's Label3D form), both read from the hall (F02_SOUTHWEST_HALL_OV). The strip of brown paper over the letter slot is not made: the leaf has no slot owner to carry a decal. Verified at WIP 36f8f9bb (implementation/slice49): fabrication batch 0 failures (six thresholds captured natively); apartment batch 204 on the long runner; household state 154 checks, 0 failures; upper kitchens 206 and upper furniture 488, both identical to slice 48; upper lighting, public doors, the remaining upper transfers, the apartment door route, the first upper hall, the 4B door and rear wing A, all 0 failures; the resident key route, which the serial runner's 180 s ceiling ended without a verdict at this WIP, passes on the long runner at slice 51's WIP 0bac8f87 (86 waypoints, 0 failures), a tree that carries slice 49 unchanged. Rear wing C's one failure (the 2C bookshelf collision) is identical at slice 48's tip. The three hall sweeps (17 spaces) report 0 failures. Every threshold lies flat inside the 1.2 m hall route, within 0.5 m of its jamb and outside the swing.</t>
+        </is>
+      </c>
     </row>
     <row r="259">
       <c r="A259" s="2" t="inlineStr">
@@ -19921,10 +19937,14 @@
       </c>
       <c r="S272" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T272" s="2" t="inlineStr"/>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="T272" s="2" t="inlineStr">
+        <is>
+          <t>3A's coir mat dark with soil off Malcolm's boots (F03_WEST_HALL_OV, 3A_threshold_native); 3D's plain coir at the far end of the southwest hall reads from the same landing. Verified at WIP 36f8f9bb (implementation/slice49): fabrication batch 0 failures (six thresholds captured natively); apartment batch 204 on the long runner; household state 154 checks, 0 failures; upper kitchens 206 and upper furniture 488, both identical to slice 48; upper lighting, public doors, the remaining upper transfers, the apartment door route, the first upper hall, the 4B door and rear wing A, all 0 failures; the resident key route, which the serial runner's 180 s ceiling ended without a verdict at this WIP, passes on the long runner at slice 51's WIP 0bac8f87 (86 waypoints, 0 failures), a tree that carries slice 49 unchanged. Rear wing C's one failure (the 2C bookshelf collision) is identical at slice 48's tip. The three hall sweeps (17 spaces) report 0 failures. Every threshold lies flat inside the 1.2 m hall route, within 0.5 m of its jamb and outside the swing.</t>
+        </is>
+      </c>
     </row>
     <row r="273">
       <c r="A273" s="2" t="inlineStr">
@@ -20069,10 +20089,14 @@
       </c>
       <c r="S274" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T274" s="2" t="inlineStr"/>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="T274" s="2" t="inlineStr">
+        <is>
+          <t>3D's plain coir mat at the hall's door, read from the landing with 3A's soiled mat in the west hall (F03_SOUTHWEST_HALL_OV). Verified at WIP 36f8f9bb (implementation/slice49): fabrication batch 0 failures (six thresholds captured natively); apartment batch 204 on the long runner; household state 154 checks, 0 failures; upper kitchens 206 and upper furniture 488, both identical to slice 48; upper lighting, public doors, the remaining upper transfers, the apartment door route, the first upper hall, the 4B door and rear wing A, all 0 failures; the resident key route, which the serial runner's 180 s ceiling ended without a verdict at this WIP, passes on the long runner at slice 51's WIP 0bac8f87 (86 waypoints, 0 failures), a tree that carries slice 49 unchanged. Rear wing C's one failure (the 2C bookshelf collision) is identical at slice 48's tip. The three hall sweeps (17 spaces) report 0 failures. Every threshold lies flat inside the 1.2 m hall route, within 0.5 m of its jamb and outside the swing.</t>
+        </is>
+      </c>
     </row>
     <row r="275">
       <c r="A275" s="2" t="inlineStr">
@@ -24325,10 +24349,14 @@
       </c>
       <c r="S330" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T330" s="2" t="inlineStr"/>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="T330" s="2" t="inlineStr">
+        <is>
+          <t>4B's mat worn flat and dark where every boot lands (the player's door), beside 4C's ribbed rubber mat and two milk bottles at the core (F04_WEST_HALL_OV, 4B_threshold_native, 4C_threshold_native). Verified at WIP 36f8f9bb (implementation/slice49): fabrication batch 0 failures (six thresholds captured natively); apartment batch 204 on the long runner; household state 154 checks, 0 failures; upper kitchens 206 and upper furniture 488, both identical to slice 48; upper lighting, public doors, the remaining upper transfers, the apartment door route, the first upper hall, the 4B door and rear wing A, all 0 failures; the resident key route, which the serial runner's 180 s ceiling ended without a verdict at this WIP, passes on the long runner at slice 51's WIP 0bac8f87 (86 waypoints, 0 failures), a tree that carries slice 49 unchanged. Rear wing C's one failure (the 2C bookshelf collision) is identical at slice 48's tip. The three hall sweeps (17 spaces) report 0 failures. Every threshold lies flat inside the 1.2 m hall route, within 0.5 m of its jamb and outside the swing.</t>
+        </is>
+      </c>
     </row>
     <row r="331">
       <c r="A331" s="2" t="inlineStr">
@@ -24967,10 +24995,14 @@
       </c>
       <c r="S339" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T339" s="2" t="inlineStr"/>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="T339" s="2" t="inlineStr">
+        <is>
+          <t>Down the east hall: 4C's ribbed rubber mat and milk pair at the core end, 4A's exact coir mat with the paper folded on it at the crossing end (F04_EAST_HALL_RV). Verified at WIP 36f8f9bb (implementation/slice49): fabrication batch 0 failures (six thresholds captured natively); apartment batch 204 on the long runner; household state 154 checks, 0 failures; upper kitchens 206 and upper furniture 488, both identical to slice 48; upper lighting, public doors, the remaining upper transfers, the apartment door route, the first upper hall, the 4B door and rear wing A, all 0 failures; the resident key route, which the serial runner's 180 s ceiling ended without a verdict at this WIP, passes on the long runner at slice 51's WIP 0bac8f87 (86 waypoints, 0 failures), a tree that carries slice 49 unchanged. Rear wing C's one failure (the 2C bookshelf collision) is identical at slice 48's tip. The three hall sweeps (17 spaces) report 0 failures. Every threshold lies flat inside the 1.2 m hall route, within 0.5 m of its jamb and outside the swing.</t>
+        </is>
+      </c>
     </row>
     <row r="340">
       <c r="A340" s="2" t="inlineStr">
@@ -32157,10 +32189,14 @@
       </c>
       <c r="S436" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T436" s="2" t="inlineStr"/>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="T436" s="2" t="inlineStr">
+        <is>
+          <t>5A's coir mat and 5B's with the morning paper folded on it, two households side by side in the one hall; 5C's paint-flecked mat at the core (F05_WEST_HALL_OV). Verified at WIP 36f8f9bb (implementation/slice49): fabrication batch 0 failures (six thresholds captured natively); apartment batch 204 on the long runner; household state 154 checks, 0 failures; upper kitchens 206 and upper furniture 488, both identical to slice 48; upper lighting, public doors, the remaining upper transfers, the apartment door route, the first upper hall, the 4B door and rear wing A, all 0 failures; the resident key route, which the serial runner's 180 s ceiling ended without a verdict at this WIP, passes on the long runner at slice 51's WIP 0bac8f87 (86 waypoints, 0 failures), a tree that carries slice 49 unchanged. Rear wing C's one failure (the 2C bookshelf collision) is identical at slice 48's tip. The three hall sweeps (17 spaces) report 0 failures. Every threshold lies flat inside the 1.2 m hall route, within 0.5 m of its jamb and outside the swing.</t>
+        </is>
+      </c>
     </row>
     <row r="437">
       <c r="A437" s="2" t="inlineStr">
@@ -37605,10 +37641,14 @@
       </c>
       <c r="S510" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T510" s="2" t="inlineStr"/>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="T510" s="2" t="inlineStr">
+        <is>
+          <t>6B's worn mat in the hall and 6C's coir mat with a string-tied parcel for the appraiser at the core (F06_WEST_HALL_OV, 6C_threshold_native). Verified at WIP 36f8f9bb (implementation/slice49): fabrication batch 0 failures (six thresholds captured natively); apartment batch 204 on the long runner; household state 154 checks, 0 failures; upper kitchens 206 and upper furniture 488, both identical to slice 48; upper lighting, public doors, the remaining upper transfers, the apartment door route, the first upper hall, the 4B door and rear wing A, all 0 failures; the resident key route, which the serial runner's 180 s ceiling ended without a verdict at this WIP, passes on the long runner at slice 51's WIP 0bac8f87 (86 waypoints, 0 failures), a tree that carries slice 49 unchanged. Rear wing C's one failure (the 2C bookshelf collision) is identical at slice 48's tip. The three hall sweeps (17 spaces) report 0 failures. Every threshold lies flat inside the 1.2 m hall route, within 0.5 m of its jamb and outside the swing.</t>
+        </is>
+      </c>
     </row>
     <row r="511">
       <c r="A511" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Implement dossier slice 50: stair wear and one piece per core landing
- F01-F06/ROOF public and service core -002, F02-F04_LANDING-002 (partial):
  every honed tread of every core flight is dished just behind the nosing
  on the walking line, deepest at the centre and zero at every edge
  (visual only: physics keeps the full box); each core landing hangs one
  piece of its own: a canvas, a toned photograph or a wordless ruled
  certificate. Rail gold at hand height and paint rubbed at the turn are
  not yet made.
- F06_PUBLIC_CORE-003: the prospectus roof-garden plate, a sepia drawing
  with its figures as silhouettes, in plain paint and print finishes.
- Two core sweeps verify at the WIP; the third reran at slice 52's WIP,
  which carries this slice unchanged (implementation/slice52b).

Evidence under implementation/slice50/. INERT: no ledger status changes.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/art/reviews/v2_environment_design_20261008/change_register.xlsx
+++ b/art/reviews/v2_environment_design_20261008/change_register.xlsx
@@ -9695,10 +9695,14 @@
       </c>
       <c r="S139" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T139" s="2" t="inlineStr"/>
+          <t>implemented</t>
+        </is>
+      </c>
+      <c r="T139" s="2" t="inlineStr">
+        <is>
+          <t>Partial: Every honed tread of this core's flights is dished just behind the nosing on the walking line, deepest at the centre and zero at every edge (visual only: physics keeps the full box), read against the lamp in the reverse view up the flight; and the landing's one piece of its own, a small canvas of a dusk sky over a field with one post, hung on the wall above the arrival landing (F01_PUBLIC_CORE_RV, F01_PUBLIC_CORE_DT1). Rail gold at hand height and paint rubbed at the turn are not yet made. Verified at WIP 14fec84e (implementation/slice50): fabrication batch 0 failures (four landing pieces captured natively); apartment batch 204 on the long runner; household state 154 checks, 0 failures; upper kitchens 206 and upper furniture 488, both unchanged; upper lighting 9,257 checks, the honed stair material check (294 stair surfaces), the blockout test, stair ironwork, stair direction (36/36), public doors 17, the remaining upper transfers 28, the basement route 88 and public furnishings 29, all 0 failures; the ground core transfer route's one failure is pre-existing. Two of the three core sweeps (12 spaces) report 0 failures at the WIP; the third (the B1 public core, the F05 service core, both F06 cores and both roof cores) was rerun at slice 52's WIP 3f3f0d75, which carries this slice unchanged, and reports 0 failures (implementation/slice52b, committed with slice 52).</t>
+        </is>
+      </c>
     </row>
     <row r="140">
       <c r="A140" s="2" t="inlineStr">
@@ -10131,10 +10135,14 @@
       </c>
       <c r="S145" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T145" s="2" t="inlineStr"/>
+          <t>implemented</t>
+        </is>
+      </c>
+      <c r="T145" s="2" t="inlineStr">
+        <is>
+          <t>Partial: Every honed tread of this core's flights is dished just behind the nosing on the walking line, deepest at the centre and zero at every edge (visual only: physics keeps the full box), read against the lamp in the reverse view up the flight; and the landing's one piece of its own, a framed ruled document, wordless, hung on the wall above the arrival landing (F01_SERVICE_CORE_RV, F01_SERVICE_CORE_DT1). Rail gold at hand height and paint rubbed at the turn are not yet made. Verified at WIP 14fec84e (implementation/slice50): fabrication batch 0 failures (four landing pieces captured natively); apartment batch 204 on the long runner; household state 154 checks, 0 failures; upper kitchens 206 and upper furniture 488, both unchanged; upper lighting 9,257 checks, the honed stair material check (294 stair surfaces), the blockout test, stair ironwork, stair direction (36/36), public doors 17, the remaining upper transfers 28, the basement route 88 and public furnishings 29, all 0 failures; the ground core transfer route's one failure is pre-existing. Two of the three core sweeps (12 spaces) report 0 failures at the WIP; the third (the B1 public core, the F05 service core, both F06 cores and both roof cores) was rerun at slice 52's WIP 3f3f0d75, which carries this slice unchanged, and reports 0 failures (implementation/slice52b, committed with slice 52).</t>
+        </is>
+      </c>
     </row>
     <row r="146">
       <c r="A146" s="2" t="inlineStr">
@@ -13739,10 +13747,14 @@
       </c>
       <c r="S191" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T191" s="2" t="inlineStr"/>
+          <t>implemented</t>
+        </is>
+      </c>
+      <c r="T191" s="2" t="inlineStr">
+        <is>
+          <t>Partial: the landing shares its public core's flights and piece; Every honed tread of this core's flights is dished just behind the nosing on the walking line, deepest at the centre and zero at every edge (visual only: physics keeps the full box), read against the lamp in the reverse view up the flight (F02_LANDING_RV). Rail gold at hand height and paint rubbed at the turn are not yet made. Verified at WIP 14fec84e (implementation/slice50): fabrication batch 0 failures (four landing pieces captured natively); apartment batch 204 on the long runner; household state 154 checks, 0 failures; upper kitchens 206 and upper furniture 488, both unchanged; upper lighting 9,257 checks, the honed stair material check (294 stair surfaces), the blockout test, stair ironwork, stair direction (36/36), public doors 17, the remaining upper transfers 28, the basement route 88 and public furnishings 29, all 0 failures; the ground core transfer route's one failure is pre-existing. Two of the three core sweeps (12 spaces) report 0 failures at the WIP; the third (the B1 public core, the F05 service core, both F06 cores and both roof cores) was rerun at slice 52's WIP 3f3f0d75, which carries this slice unchanged, and reports 0 failures (implementation/slice52b, committed with slice 52).</t>
+        </is>
+      </c>
     </row>
     <row r="192">
       <c r="A192" s="2" t="inlineStr">
@@ -14195,10 +14207,14 @@
       </c>
       <c r="S197" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T197" s="2" t="inlineStr"/>
+          <t>implemented</t>
+        </is>
+      </c>
+      <c r="T197" s="2" t="inlineStr">
+        <is>
+          <t>Partial: Every honed tread of this core's flights is dished just behind the nosing on the walking line, deepest at the centre and zero at every edge (visual only: physics keeps the full box), read against the lamp in the reverse view up the flight; and the landing's one piece of its own, a canvas of a pale sky over an ochre field with one green tree, hung on the wall above the arrival landing (F02_PUBLIC_CORE_RV, F02_PUBLIC_CORE_DT1). Rail gold at hand height and paint rubbed at the turn are not yet made. Verified at WIP 14fec84e (implementation/slice50): fabrication batch 0 failures (four landing pieces captured natively); apartment batch 204 on the long runner; household state 154 checks, 0 failures; upper kitchens 206 and upper furniture 488, both unchanged; upper lighting 9,257 checks, the honed stair material check (294 stair surfaces), the blockout test, stair ironwork, stair direction (36/36), public doors 17, the remaining upper transfers 28, the basement route 88 and public furnishings 29, all 0 failures; the ground core transfer route's one failure is pre-existing. Two of the three core sweeps (12 spaces) report 0 failures at the WIP; the third (the B1 public core, the F05 service core, both F06 cores and both roof cores) was rerun at slice 52's WIP 3f3f0d75, which carries this slice unchanged, and reports 0 failures (implementation/slice52b, committed with slice 52).</t>
+        </is>
+      </c>
     </row>
     <row r="198">
       <c r="A198" s="2" t="inlineStr">
@@ -14733,10 +14749,14 @@
       </c>
       <c r="S204" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T204" s="2" t="inlineStr"/>
+          <t>implemented</t>
+        </is>
+      </c>
+      <c r="T204" s="2" t="inlineStr">
+        <is>
+          <t>Partial: Every honed tread of this core's flights is dished just behind the nosing on the walking line, deepest at the centre and zero at every edge (visual only: physics keeps the full box), read against the lamp in the reverse view up the flight; and the landing's one piece of its own, a framed navy-toned photograph, hung on the wall above the arrival landing (F02_SERVICE_CORE_RV, F02_SERVICE_CORE_DT1). Rail gold at hand height and paint rubbed at the turn are not yet made. Verified at WIP 14fec84e (implementation/slice50): fabrication batch 0 failures (four landing pieces captured natively); apartment batch 204 on the long runner; household state 154 checks, 0 failures; upper kitchens 206 and upper furniture 488, both unchanged; upper lighting 9,257 checks, the honed stair material check (294 stair surfaces), the blockout test, stair ironwork, stair direction (36/36), public doors 17, the remaining upper transfers 28, the basement route 88 and public furnishings 29, all 0 failures; the ground core transfer route's one failure is pre-existing. Two of the three core sweeps (12 spaces) report 0 failures at the WIP; the third (the B1 public core, the F05 service core, both F06 cores and both roof cores) was rerun at slice 52's WIP 3f3f0d75, which carries this slice unchanged, and reports 0 failures (implementation/slice52b, committed with slice 52).</t>
+        </is>
+      </c>
     </row>
     <row r="205">
       <c r="A205" s="2" t="inlineStr">
@@ -19053,10 +19073,14 @@
       </c>
       <c r="S260" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T260" s="2" t="inlineStr"/>
+          <t>implemented</t>
+        </is>
+      </c>
+      <c r="T260" s="2" t="inlineStr">
+        <is>
+          <t>Partial: Every honed tread of this core's flights is dished just behind the nosing on the walking line, deepest at the centre and zero at every edge (visual only: physics keeps the full box), read against the lamp in the reverse view up the flight; and the landing's one piece of its own, a sepia photograph in a dark frame, hung on the wall above the arrival landing (F03_PUBLIC_CORE_RV, F03_PUBLIC_CORE_DT1). Rail gold at hand height and paint rubbed at the turn are not yet made. Verified at WIP 14fec84e (implementation/slice50): fabrication batch 0 failures (four landing pieces captured natively); apartment batch 204 on the long runner; household state 154 checks, 0 failures; upper kitchens 206 and upper furniture 488, both unchanged; upper lighting 9,257 checks, the honed stair material check (294 stair surfaces), the blockout test, stair ironwork, stair direction (36/36), public doors 17, the remaining upper transfers 28, the basement route 88 and public furnishings 29, all 0 failures; the ground core transfer route's one failure is pre-existing. Two of the three core sweeps (12 spaces) report 0 failures at the WIP; the third (the B1 public core, the F05 service core, both F06 cores and both roof cores) was rerun at slice 52's WIP 3f3f0d75, which carries this slice unchanged, and reports 0 failures (implementation/slice52b, committed with slice 52).</t>
+        </is>
+      </c>
     </row>
     <row r="261">
       <c r="A261" s="2" t="inlineStr">
@@ -19205,10 +19229,14 @@
       </c>
       <c r="S262" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T262" s="2" t="inlineStr"/>
+          <t>implemented</t>
+        </is>
+      </c>
+      <c r="T262" s="2" t="inlineStr">
+        <is>
+          <t>Partial: Every honed tread of this core's flights is dished just behind the nosing on the walking line, deepest at the centre and zero at every edge (visual only: physics keeps the full box), read against the lamp in the reverse view up the flight; and the landing's one piece of its own, a framed brown-toned photograph, hung on the wall above the arrival landing (F03_SERVICE_CORE_RV, F03_SERVICE_CORE_DT1). Rail gold at hand height and paint rubbed at the turn are not yet made. Verified at WIP 14fec84e (implementation/slice50): fabrication batch 0 failures (four landing pieces captured natively); apartment batch 204 on the long runner; household state 154 checks, 0 failures; upper kitchens 206 and upper furniture 488, both unchanged; upper lighting 9,257 checks, the honed stair material check (294 stair surfaces), the blockout test, stair ironwork, stair direction (36/36), public doors 17, the remaining upper transfers 28, the basement route 88 and public furnishings 29, all 0 failures; the ground core transfer route's one failure is pre-existing. Two of the three core sweeps (12 spaces) report 0 failures at the WIP; the third (the B1 public core, the F05 service core, both F06 cores and both roof cores) was rerun at slice 52's WIP 3f3f0d75, which carries this slice unchanged, and reports 0 failures (implementation/slice52b, committed with slice 52).</t>
+        </is>
+      </c>
     </row>
     <row r="263">
       <c r="A263" s="2" t="inlineStr">
@@ -19357,10 +19385,14 @@
       </c>
       <c r="S264" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T264" s="2" t="inlineStr"/>
+          <t>implemented</t>
+        </is>
+      </c>
+      <c r="T264" s="2" t="inlineStr">
+        <is>
+          <t>Partial: the landing shares its public core's flights and piece; Every honed tread of this core's flights is dished just behind the nosing on the walking line, deepest at the centre and zero at every edge (visual only: physics keeps the full box), read against the lamp in the reverse view up the flight (F03_LANDING_RV). Rail gold at hand height and paint rubbed at the turn are not yet made. Verified at WIP 14fec84e (implementation/slice50): fabrication batch 0 failures (four landing pieces captured natively); apartment batch 204 on the long runner; household state 154 checks, 0 failures; upper kitchens 206 and upper furniture 488, both unchanged; upper lighting 9,257 checks, the honed stair material check (294 stair surfaces), the blockout test, stair ironwork, stair direction (36/36), public doors 17, the remaining upper transfers 28, the basement route 88 and public furnishings 29, all 0 failures; the ground core transfer route's one failure is pre-existing. Two of the three core sweeps (12 spaces) report 0 failures at the WIP; the third (the B1 public core, the F05 service core, both F06 cores and both roof cores) was rerun at slice 52's WIP 3f3f0d75, which carries this slice unchanged, and reports 0 failures (implementation/slice52b, committed with slice 52).</t>
+        </is>
+      </c>
     </row>
     <row r="265">
       <c r="A265" s="2" t="inlineStr">
@@ -24205,10 +24237,14 @@
       </c>
       <c r="S328" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T328" s="2" t="inlineStr"/>
+          <t>implemented</t>
+        </is>
+      </c>
+      <c r="T328" s="2" t="inlineStr">
+        <is>
+          <t>Partial: the landing shares its public core's flights and piece; Every honed tread of this core's flights is dished just behind the nosing on the walking line, deepest at the centre and zero at every edge (visual only: physics keeps the full box), read against the lamp in the reverse view up the flight (F04_LANDING_RV). Rail gold at hand height and paint rubbed at the turn are not yet made. Verified at WIP 14fec84e (implementation/slice50): fabrication batch 0 failures (four landing pieces captured natively); apartment batch 204 on the long runner; household state 154 checks, 0 failures; upper kitchens 206 and upper furniture 488, both unchanged; upper lighting 9,257 checks, the honed stair material check (294 stair surfaces), the blockout test, stair ironwork, stair direction (36/36), public doors 17, the remaining upper transfers 28, the basement route 88 and public furnishings 29, all 0 failures; the ground core transfer route's one failure is pre-existing. Two of the three core sweeps (12 spaces) report 0 failures at the WIP; the third (the B1 public core, the F05 service core, both F06 cores and both roof cores) was rerun at slice 52's WIP 3f3f0d75, which carries this slice unchanged, and reports 0 failures (implementation/slice52b, committed with slice 52).</t>
+        </is>
+      </c>
     </row>
     <row r="329">
       <c r="A329" s="2" t="inlineStr">
@@ -24847,10 +24883,14 @@
       </c>
       <c r="S337" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T337" s="2" t="inlineStr"/>
+          <t>implemented</t>
+        </is>
+      </c>
+      <c r="T337" s="2" t="inlineStr">
+        <is>
+          <t>Partial: Every honed tread of this core's flights is dished just behind the nosing on the walking line, deepest at the centre and zero at every edge (visual only: physics keeps the full box), read against the lamp in the reverse view up the flight; and the landing's one piece of its own, a dark interior canvas, a lit doorway and a lamp, hung on the wall above the arrival landing (F04_PUBLIC_CORE_RV, F04_PUBLIC_CORE_DT1). Rail gold at hand height and paint rubbed at the turn are not yet made. Verified at WIP 14fec84e (implementation/slice50): fabrication batch 0 failures (four landing pieces captured natively); apartment batch 204 on the long runner; household state 154 checks, 0 failures; upper kitchens 206 and upper furniture 488, both unchanged; upper lighting 9,257 checks, the honed stair material check (294 stair surfaces), the blockout test, stair ironwork, stair direction (36/36), public doors 17, the remaining upper transfers 28, the basement route 88 and public furnishings 29, all 0 failures; the ground core transfer route's one failure is pre-existing. Two of the three core sweeps (12 spaces) report 0 failures at the WIP; the third (the B1 public core, the F05 service core, both F06 cores and both roof cores) was rerun at slice 52's WIP 3f3f0d75, which carries this slice unchanged, and reports 0 failures (implementation/slice52b, committed with slice 52).</t>
+        </is>
+      </c>
     </row>
     <row r="338">
       <c r="A338" s="2" t="inlineStr">
@@ -25583,10 +25623,14 @@
       </c>
       <c r="S347" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T347" s="2" t="inlineStr"/>
+          <t>implemented</t>
+        </is>
+      </c>
+      <c r="T347" s="2" t="inlineStr">
+        <is>
+          <t>Partial: Every honed tread of this core's flights is dished just behind the nosing on the walking line, deepest at the centre and zero at every edge (visual only: physics keeps the full box), read against the lamp in the reverse view up the flight; and the landing's one piece of its own, a framed green-toned photograph, hung on the wall above the arrival landing (F04_SERVICE_CORE_RV, F04_SERVICE_CORE_DT1). Rail gold at hand height and paint rubbed at the turn are not yet made. Verified at WIP 14fec84e (implementation/slice50): fabrication batch 0 failures (four landing pieces captured natively); apartment batch 204 on the long runner; household state 154 checks, 0 failures; upper kitchens 206 and upper furniture 488, both unchanged; upper lighting 9,257 checks, the honed stair material check (294 stair surfaces), the blockout test, stair ironwork, stair direction (36/36), public doors 17, the remaining upper transfers 28, the basement route 88 and public furnishings 29, all 0 failures; the ground core transfer route's one failure is pre-existing. Two of the three core sweeps (12 spaces) report 0 failures at the WIP; the third (the B1 public core, the F05 service core, both F06 cores and both roof cores) was rerun at slice 52's WIP 3f3f0d75, which carries this slice unchanged, and reports 0 failures (implementation/slice52b, committed with slice 52).</t>
+        </is>
+      </c>
     </row>
     <row r="348">
       <c r="A348" s="2" t="inlineStr">
@@ -31387,10 +31431,14 @@
       </c>
       <c r="S425" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T425" s="2" t="inlineStr"/>
+          <t>implemented</t>
+        </is>
+      </c>
+      <c r="T425" s="2" t="inlineStr">
+        <is>
+          <t>Partial: Every honed tread of this core's flights is dished just behind the nosing on the walking line, deepest at the centre and zero at every edge (visual only: physics keeps the full box), read against the lamp in the reverse view up the flight; and the landing's one piece of its own, a long canvas of a pale sky, grey water and a green shore, hung on the wall above the arrival landing (F05_PUBLIC_CORE_RV, F05_PUBLIC_CORE_DT1). Rail gold at hand height and paint rubbed at the turn are not yet made. Verified at WIP 14fec84e (implementation/slice50): fabrication batch 0 failures (four landing pieces captured natively); apartment batch 204 on the long runner; household state 154 checks, 0 failures; upper kitchens 206 and upper furniture 488, both unchanged; upper lighting 9,257 checks, the honed stair material check (294 stair surfaces), the blockout test, stair ironwork, stair direction (36/36), public doors 17, the remaining upper transfers 28, the basement route 88 and public furnishings 29, all 0 failures; the ground core transfer route's one failure is pre-existing. Two of the three core sweeps (12 spaces) report 0 failures at the WIP; the third (the B1 public core, the F05 service core, both F06 cores and both roof cores) was rerun at slice 52's WIP 3f3f0d75, which carries this slice unchanged, and reports 0 failures (implementation/slice52b, committed with slice 52).</t>
+        </is>
+      </c>
     </row>
     <row r="426">
       <c r="A426" s="2" t="inlineStr">
@@ -31671,10 +31719,14 @@
       </c>
       <c r="S429" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T429" s="2" t="inlineStr"/>
+          <t>implemented</t>
+        </is>
+      </c>
+      <c r="T429" s="2" t="inlineStr">
+        <is>
+          <t>Partial: Every honed tread of this core's flights is dished just behind the nosing on the walking line, deepest at the centre and zero at every edge (visual only: physics keeps the full box), read against the lamp in the reverse view up the flight; and the landing's one piece of its own, a framed ruled certificate, wordless, hung on the wall above the arrival landing (F05_SERVICE_CORE_RV, F05_SERVICE_CORE_DT1). Rail gold at hand height and paint rubbed at the turn are not yet made. Verified at WIP 14fec84e (implementation/slice50): fabrication batch 0 failures (four landing pieces captured natively); apartment batch 204 on the long runner; household state 154 checks, 0 failures; upper kitchens 206 and upper furniture 488, both unchanged; upper lighting 9,257 checks, the honed stair material check (294 stair surfaces), the blockout test, stair ironwork, stair direction (36/36), public doors 17, the remaining upper transfers 28, the basement route 88 and public furnishings 29, all 0 failures; the ground core transfer route's one failure is pre-existing. Two of the three core sweeps (12 spaces) report 0 failures at the WIP; the third (the B1 public core, the F05 service core, both F06 cores and both roof cores) was rerun at slice 52's WIP 3f3f0d75, which carries this slice unchanged, and reports 0 failures (implementation/slice52b, committed with slice 52).</t>
+        </is>
+      </c>
     </row>
     <row r="430">
       <c r="A430" s="2" t="inlineStr">
@@ -36963,10 +37015,14 @@
       </c>
       <c r="S501" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T501" s="2" t="inlineStr"/>
+          <t>implemented</t>
+        </is>
+      </c>
+      <c r="T501" s="2" t="inlineStr">
+        <is>
+          <t>Partial: Every honed tread of this core's flights is dished just behind the nosing on the walking line, deepest at the centre and zero at every edge (visual only: physics keeps the full box), read against the lamp in the reverse view up the flight; and the landing's one piece of its own, the prospectus roof-garden plate, hung on the wall above the arrival landing (F06_PUBLIC_CORE_RV, F06_PUBLIC_CORE_DT1). Rail gold at hand height and paint rubbed at the turn are not yet made. Verified at WIP 14fec84e (implementation/slice50): fabrication batch 0 failures (four landing pieces captured natively); apartment batch 204 on the long runner; household state 154 checks, 0 failures; upper kitchens 206 and upper furniture 488, both unchanged; upper lighting 9,257 checks, the honed stair material check (294 stair surfaces), the blockout test, stair ironwork, stair direction (36/36), public doors 17, the remaining upper transfers 28, the basement route 88 and public furnishings 29, all 0 failures; the ground core transfer route's one failure is pre-existing. Two of the three core sweeps (12 spaces) report 0 failures at the WIP; the third (the B1 public core, the F05 service core, both F06 cores and both roof cores) was rerun at slice 52's WIP 3f3f0d75, which carries this slice unchanged, and reports 0 failures (implementation/slice52b, committed with slice 52).</t>
+        </is>
+      </c>
     </row>
     <row r="502">
       <c r="A502" s="2" t="inlineStr">
@@ -37029,10 +37085,14 @@
       </c>
       <c r="S502" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T502" s="2" t="inlineStr"/>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="T502" s="2" t="inlineStr">
+        <is>
+          <t>The prospectus roof-garden plate: a sepia drawing of the roof garden with its figures as silhouettes (a pergola, planting, people at the parapet), framed at 1.6 m on the wall above the F06 arrival landing below the roof flight, in plain paint and print finishes (no gilt tooling, no lettering). Verified at WIP 14fec84e (implementation/slice50): fabrication batch 0 failures (four landing pieces captured natively); apartment batch 204 on the long runner; household state 154 checks, 0 failures; upper kitchens 206 and upper furniture 488, both unchanged; upper lighting 9,257 checks, the honed stair material check (294 stair surfaces), the blockout test, stair ironwork, stair direction (36/36), public doors 17, the remaining upper transfers 28, the basement route 88 and public furnishings 29, all 0 failures; the ground core transfer route's one failure is pre-existing. Two of the three core sweeps (12 spaces) report 0 failures at the WIP; the third (the B1 public core, the F05 service core, both F06 cores and both roof cores) was rerun at slice 52's WIP 3f3f0d75, which carries this slice unchanged, and reports 0 failures (implementation/slice52b, committed with slice 52).</t>
+        </is>
+      </c>
     </row>
     <row r="503">
       <c r="A503" s="2" t="inlineStr">
@@ -37181,10 +37241,14 @@
       </c>
       <c r="S504" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T504" s="2" t="inlineStr"/>
+          <t>implemented</t>
+        </is>
+      </c>
+      <c r="T504" s="2" t="inlineStr">
+        <is>
+          <t>Partial: Every honed tread of this core's flights is dished just behind the nosing on the walking line, deepest at the centre and zero at every edge (visual only: physics keeps the full box), read against the lamp in the reverse view up the flight; and the landing's one piece of its own, a framed teal-toned photograph, hung on the wall above the arrival landing (F06_SERVICE_CORE_RV, F06_SERVICE_CORE_DT1). Rail gold at hand height and paint rubbed at the turn are not yet made. Verified at WIP 14fec84e (implementation/slice50): fabrication batch 0 failures (four landing pieces captured natively); apartment batch 204 on the long runner; household state 154 checks, 0 failures; upper kitchens 206 and upper furniture 488, both unchanged; upper lighting 9,257 checks, the honed stair material check (294 stair surfaces), the blockout test, stair ironwork, stair direction (36/36), public doors 17, the remaining upper transfers 28, the basement route 88 and public furnishings 29, all 0 failures; the ground core transfer route's one failure is pre-existing. Two of the three core sweeps (12 spaces) report 0 failures at the WIP; the third (the B1 public core, the F05 service core, both F06 cores and both roof cores) was rerun at slice 52's WIP 3f3f0d75, which carries this slice unchanged, and reports 0 failures (implementation/slice52b, committed with slice 52).</t>
+        </is>
+      </c>
     </row>
     <row r="505">
       <c r="A505" s="2" t="inlineStr">
@@ -41489,10 +41553,14 @@
       </c>
       <c r="S562" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T562" s="2" t="inlineStr"/>
+          <t>implemented</t>
+        </is>
+      </c>
+      <c r="T562" s="2" t="inlineStr">
+        <is>
+          <t>Partial: Every honed tread of this core's flights is dished just behind the nosing on the walking line, deepest at the centre and zero at every edge (visual only: physics keeps the full box), read against the lamp in the reverse view up the flight; and the landing's one piece of its own, a night canvas, a few stars and a low moon over the parapet, hung on the wall above the arrival landing (ROOF_PUBLIC_CORE_RV, ROOF_PUBLIC_CORE_DT1). Rail gold at hand height and paint rubbed at the turn are not yet made. Verified at WIP 14fec84e (implementation/slice50): fabrication batch 0 failures (four landing pieces captured natively); apartment batch 204 on the long runner; household state 154 checks, 0 failures; upper kitchens 206 and upper furniture 488, both unchanged; upper lighting 9,257 checks, the honed stair material check (294 stair surfaces), the blockout test, stair ironwork, stair direction (36/36), public doors 17, the remaining upper transfers 28, the basement route 88 and public furnishings 29, all 0 failures; the ground core transfer route's one failure is pre-existing. Two of the three core sweeps (12 spaces) report 0 failures at the WIP; the third (the B1 public core, the F05 service core, both F06 cores and both roof cores) was rerun at slice 52's WIP 3f3f0d75, which carries this slice unchanged, and reports 0 failures (implementation/slice52b, committed with slice 52).</t>
+        </is>
+      </c>
     </row>
     <row r="563">
       <c r="A563" s="2" t="inlineStr">
@@ -41777,10 +41845,14 @@
       </c>
       <c r="S566" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T566" s="2" t="inlineStr"/>
+          <t>implemented</t>
+        </is>
+      </c>
+      <c r="T566" s="2" t="inlineStr">
+        <is>
+          <t>Partial: Every honed tread of this core's flights is dished just behind the nosing on the walking line, deepest at the centre and zero at every edge (visual only: physics keeps the full box), read against the lamp in the reverse view up the flight; and the landing's one piece of its own, a framed burgundy-toned photograph, hung on the wall above the arrival landing (ROOF_SERVICE_CORE_RV, ROOF_SERVICE_CORE_DT1). Rail gold at hand height and paint rubbed at the turn are not yet made. Verified at WIP 14fec84e (implementation/slice50): fabrication batch 0 failures (four landing pieces captured natively); apartment batch 204 on the long runner; household state 154 checks, 0 failures; upper kitchens 206 and upper furniture 488, both unchanged; upper lighting 9,257 checks, the honed stair material check (294 stair surfaces), the blockout test, stair ironwork, stair direction (36/36), public doors 17, the remaining upper transfers 28, the basement route 88 and public furnishings 29, all 0 failures; the ground core transfer route's one failure is pre-existing. Two of the three core sweeps (12 spaces) report 0 failures at the WIP; the third (the B1 public core, the F05 service core, both F06 cores and both roof cores) was rerun at slice 52's WIP 3f3f0d75, which carries this slice unchanged, and reports 0 failures (implementation/slice52b, committed with slice 52).</t>
+        </is>
+      </c>
     </row>
     <row r="567">
       <c r="A567" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Implement dossier slice 51: the sealed 3C threshold, 5D's soot ghost, Cal's aerial wire
- F03_C_RESTRICTED-002 (partial): on the core side of the sealed 3C door,
  an unworn dust mat squared at the jamb and the one-line notice at 1.5 m
  in the core notice-frame family; no letter-slot strip (the leaf has no
  slot owner).
- F05_D_RESTRICTED-002 (partial): the soot ghost up the plaster above the
  replaced door's head on the crossing side, and the same notice beside
  it; the replacement leaf's fresher paint and the scorch are not made.
- F05_WEST_HALL-003: Cal's aerial lead along the hall at 2.0 m on four
  porcelain insulators, sagging between them, into a drilled hole beside
  5B's door.
- The resident key route and the four-space sweep ran at slice 52's WIP,
  which carries this slice unchanged.

Evidence under implementation/slice51/. INERT: no ledger status changes.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/art/reviews/v2_environment_design_20261008/change_register.xlsx
+++ b/art/reviews/v2_environment_design_20261008/change_register.xlsx
@@ -24085,10 +24085,14 @@
       </c>
       <c r="S326" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T326" s="2" t="inlineStr"/>
+          <t>implemented</t>
+        </is>
+      </c>
+      <c r="T326" s="2" t="inlineStr">
+        <is>
+          <t>Partial: on the core side of the sealed 3C door, an unworn dust mat squared at the jamb and the one-line notice at 1.5 m in the core notice-frame family (3C_threshold_native). The strip of brown paper over the letter slot is not made: the leaf has no slot owner to carry a decal. Verified at WIP 0bac8f87 (implementation/slice51): apartment batch 204 on the long runner; household state 154 checks, 0 failures; upper kitchens 206 and upper furniture 488, both unchanged; upper lighting 9,257 checks, public doors 17, the remaining upper transfers 28 and the apartment door route 45, all 0 failures; the resident key route (86 waypoints, long runner) and the four-space sweep (F03 public core, F05 service crossing, F05 west and east halls) ran at slice 52's WIP 3f3f0d75, which carries this slice unchanged, and both report 0 failures. The fabrication batch captured the 3C threshold and the 5D soot fan natively; its one failure is the capture harness finding no clear standing camera station for the aerial wire in the 1.06 m hall, so the hall sweep's views carry that evidence.</t>
+        </is>
+      </c>
     </row>
     <row r="327">
       <c r="A327" s="2" t="inlineStr">
@@ -32389,10 +32393,14 @@
       </c>
       <c r="S438" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T438" s="2" t="inlineStr"/>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="T438" s="2" t="inlineStr">
+        <is>
+          <t>Cal's aerial lead along the hall at 2.0 m on four porcelain insulators, sagging between them, rising to the cornice at the core end and turning into a drilled hole beside 5B's door (F05_WEST_HALL_OV). Verified at WIP 0bac8f87 (implementation/slice51): apartment batch 204 on the long runner; household state 154 checks, 0 failures; upper kitchens 206 and upper furniture 488, both unchanged; upper lighting 9,257 checks, public doors 17, the remaining upper transfers 28 and the apartment door route 45, all 0 failures; the resident key route (86 waypoints, long runner) and the four-space sweep (F03 public core, F05 service crossing, F05 west and east halls) ran at slice 52's WIP 3f3f0d75, which carries this slice unchanged, and both report 0 failures. The fabrication batch captured the 3C threshold and the 5D soot fan natively; its one failure is the capture harness finding no clear standing camera station for the aerial wire in the 1.06 m hall, so the hall sweep's views carry that evidence.</t>
+        </is>
+      </c>
     </row>
     <row r="439">
       <c r="A439" s="2" t="inlineStr">
@@ -36805,10 +36813,14 @@
       </c>
       <c r="S498" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T498" s="2" t="inlineStr"/>
+          <t>implemented</t>
+        </is>
+      </c>
+      <c r="T498" s="2" t="inlineStr">
+        <is>
+          <t>Partial: the soot ghost, stepped bands of soot 0.8 m wide at the top, up the plaster above the replaced door's head on the crossing side, and the same one-line notice beside it (5D_soot_fan_native, F05_SERVICE_CROSSING_TH). The replacement leaf's fresher paint and the scorch at the frame head are not made: the fitted door family has no replacement finish. Verified at WIP 0bac8f87 (implementation/slice51): apartment batch 204 on the long runner; household state 154 checks, 0 failures; upper kitchens 206 and upper furniture 488, both unchanged; upper lighting 9,257 checks, public doors 17, the remaining upper transfers 28 and the apartment door route 45, all 0 failures; the resident key route (86 waypoints, long runner) and the four-space sweep (F03 public core, F05 service crossing, F05 west and east halls) ran at slice 52's WIP 3f3f0d75, which carries this slice unchanged, and both report 0 failures. The fabrication batch captured the 3C threshold and the 5D soot fan natively; its one failure is the capture harness finding no clear standing camera station for the aerial wire in the 1.06 m hall, so the hall sweep's views carry that evidence.</t>
+        </is>
+      </c>
     </row>
     <row r="499">
       <c r="A499" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Implement dossier slice 53: the news booth's stock and the proprietor's worn mat
- CITY_SHOP_NEWS_CIGARS-003: four string-tied bundles of papers, three
  fanned runs of magazines, cigar boxes with one lid stood open on its
  cigars, three tobacco tins and four stacks of papers under wordless
  grey mastheads, every piece seated on its board.
- CITY_SHOP_NEWS_CIGARS-001 (partial): the stool's floor cover becomes a
  black rubber mat worn to a hollow under the proprietor's feet; the
  tile under it is not dished.
- At slice 54's WIP the news fittings module failed 4 checks: the hollow
  sank below the datum the stool's feet stand on. Slice 67 fixes it.

Evidence with slice 54 under implementation/slice54b/. INERT: no ledger
status changes.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/art/reviews/v2_environment_design_20261008/change_register.xlsx
+++ b/art/reviews/v2_environment_design_20261008/change_register.xlsx
@@ -6717,10 +6717,14 @@
       </c>
       <c r="S94" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T94" s="2" t="inlineStr"/>
+          <t>implemented</t>
+        </is>
+      </c>
+      <c r="T94" s="2" t="inlineStr">
+        <is>
+          <t>Partial: the stool's floor cover becomes a black rubber mat worn to a hollow under the proprietor's feet (fitted_stool); the half-punched punchboard on the counter is the fitted family's own (punchboard). The tile under the mat is not dished: the mat covers it. Run at slice 54's WIP 22b1aa9a (implementation/slice54b), which carries slice 53 unchanged: the city sweep's 130 views report 0 failures and the IN0/IN1 stations show the shops. At that WIP the news fittings module reports 4 failures (slice 53 sank the worn hollow below the datum the stool's four feet stand on) and the hardware drawer suite 1 (its face probe did not know the open drawer). Slice 67 fixes both; these rows are upgraded when it verifies.</t>
+        </is>
+      </c>
     </row>
     <row r="95">
       <c r="A95" s="2" t="inlineStr">
@@ -6841,10 +6845,14 @@
       </c>
       <c r="S96" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T96" s="2" t="inlineStr"/>
+          <t>implemented</t>
+        </is>
+      </c>
+      <c r="T96" s="2" t="inlineStr">
+        <is>
+          <t>The booth's stock, every piece seated on its board: four string-tied bundles of papers, three fanned runs of magazines, cigar boxes with one lid stood open on its cigars, three tobacco tins, and four stacks of papers under wordless grey mastheads; the cigar case shows its cigars (shop_news_cigars_SITE_SHOP_IN0_NEWS_CIGARS, rear_shelves). Run at slice 54's WIP 22b1aa9a (implementation/slice54b), which carries slice 53 unchanged: the city sweep's 130 views report 0 failures and the IN0/IN1 stations show the shops. At that WIP the news fittings module reports 4 failures (slice 53 sank the worn hollow below the datum the stool's four feet stand on) and the hardware drawer suite 1 (its face probe did not know the open drawer). Slice 67 fixes both; these rows are upgraded when it verifies.</t>
+        </is>
+      </c>
     </row>
     <row r="97">
       <c r="A97" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Implement dossier slice 54: paint tins in three sizes, one drawer open
- CITY_SHOP_HARDWARE_PAINT-002: the seven wire-bail tins in three sizes,
  two lids dented and paint run down two, each with a wordless paper
  label band and a colour stripe; one drawer of the wall stands 0.14 m
  open on its rail.
- The label bands bind the registered catalogue paper (the shop's source
  cell has no paper box to lend), without which the runtime refused the
  hardware drawer fit and the passage could not compose.
- At this WIP the hardware drawer suite failed 1 check (its face probe did
  not know the open drawer) and the news fittings module 4 (slice 53's
  mat); slice 67 fixes both.

Evidence under implementation/slice54b/. INERT: no ledger status changes.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/art/reviews/v2_environment_design_20261008/change_register.xlsx
+++ b/art/reviews/v2_environment_design_20261008/change_register.xlsx
@@ -6089,10 +6089,14 @@
       </c>
       <c r="S84" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T84" s="2" t="inlineStr"/>
+          <t>implemented</t>
+        </is>
+      </c>
+      <c r="T84" s="2" t="inlineStr">
+        <is>
+          <t>The seven wire-bail tins in three sizes, two lids dented and paint run down two, each with a wordless paper label band and a colour stripe; one drawer of the wall stands 0.14 m open on its rail (paint_tins, drawer_wall, shop_hardware_paint_SITE_SHOP_IN1_HARDWARE_PAINT). Run at slice 54's WIP 22b1aa9a (implementation/slice54b), which carries slice 53 unchanged: the city sweep's 130 views report 0 failures and the IN0/IN1 stations show the shops. At that WIP the news fittings module reports 4 failures (slice 53 sank the worn hollow below the datum the stool's four feet stand on) and the hardware drawer suite 1 (its face probe did not know the open drawer). Slice 67 fixes both; these rows are upgraded when it verifies.</t>
+        </is>
+      </c>
     </row>
     <row r="85">
       <c r="A85" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Implement dossier slice 55: film stock, the counter case, one print a building
- CITY_SHOP_PHOTO_SUPPLIES-002: film stock in three sizes, some turned and
  one on end, every lid with a wordless printed band; a box camera, a
  closed folding camera and a brass portrait lens under the case glass.
- CITY_SHOP_PHOTO_SUPPLIES-001: one plate on the portrait rail is a
  building, a procedural architectural plate among the sitters
  (art/tools/build_architectural_plate.py, no lettering).

Evidence with slice 57 under implementation/slice57b/. INERT: no ledger
status changes.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/art/reviews/v2_environment_design_20261008/change_register.xlsx
+++ b/art/reviews/v2_environment_design_20261008/change_register.xlsx
@@ -7365,10 +7365,14 @@
       </c>
       <c r="S104" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T104" s="2" t="inlineStr"/>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="T104" s="2" t="inlineStr">
+        <is>
+          <t>One plate on the portrait rail is a building: a procedural architectural plate, a facade in sepia with its windows in rows, among the sitters (portrait3, portrait_context). Verified at slice 57's WIP 260849e8 (implementation/slice57b), which carries slices 55 and 56 unchanged: the fabrication batch's seven families (photo stock 467, photo counter 148, photo portraits 361, locksmith fittings 943, radio battery 247, radio display 164 and radio wire 126 checks) report 0 failures; the radio apparatus (346), radio bench (155), radio stock (735), radio receiving (586) and photo receiving (792) suites report 0 failures; the city sweep's 130 views report 0 failures. The news receiving suite's one failure there, its keyboard station's standing capsule, is identical at slice 52's WIP 3f3f0d75 before any of these shop slices (receipt base53__news_receiving).</t>
+        </is>
+      </c>
     </row>
     <row r="105">
       <c r="A105" s="2" t="inlineStr">
@@ -7431,10 +7435,14 @@
       </c>
       <c r="S105" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T105" s="2" t="inlineStr"/>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="T105" s="2" t="inlineStr">
+        <is>
+          <t>Film stock in three sizes, some turned and one stood on end, every lid with a wordless printed band; a box camera, a closed folding camera and a brass portrait lens under the counter's case glass (rear_shelf_wall, left_column, glazed_tier, shop_photo_supplies_SITE_SHOP_IN0_PHOTO_SUPPLIES, IN1). Verified at slice 57's WIP 260849e8 (implementation/slice57b), which carries slices 55 and 56 unchanged: the fabrication batch's seven families (photo stock 467, photo counter 148, photo portraits 361, locksmith fittings 943, radio battery 247, radio display 164 and radio wire 126 checks) report 0 failures; the radio apparatus (346), radio bench (155), radio stock (735), radio receiving (586) and photo receiving (792) suites report 0 failures; the city sweep's 130 views report 0 failures. The news receiving suite's one failure there, its keyboard station's standing capsule, is identical at slice 52's WIP 3f3f0d75 before any of these shop slices (receipt base53__news_receiving).</t>
+        </is>
+      </c>
     </row>
     <row r="106">
       <c r="A106" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Implement dossier slice 56: the key board varied, a lock case open, the register
- CITY_SHOP_KEYS_CUT-003 (partial): the key board's blanks vary by row
  (bow form, blade length, bitting), the fourth row hangs empty and six
  more pegs are bare; of four lock cases one stands open, its cover on the
  cloth with its screws. The table's blocks are not yet picks and blanks.
- CITY_SHOP_KEYS_CUT-001 (partial): the second-hand fire safe's blank
  gold-leaf cartouche and pinstripe; no roll of picks.
- CITY_SHOP_KEYS_CUT-002: the register open on the counter, a column of
  figures as ink strokes on blank rules, a pencil on a string.

Evidence with slice 57 under implementation/slice57b/. INERT: no ledger
status changes.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/art/reviews/v2_environment_design_20261008/change_register.xlsx
+++ b/art/reviews/v2_environment_design_20261008/change_register.xlsx
@@ -5829,10 +5829,14 @@
       </c>
       <c r="S80" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T80" s="2" t="inlineStr"/>
+          <t>implemented</t>
+        </is>
+      </c>
+      <c r="T80" s="2" t="inlineStr">
+        <is>
+          <t>Partial: the second-hand fire safe carries a blank gold-leaf cartouche and pinstripe (safe_and_padlocks). The roll of picks unrolled on the bench is not made. Verified at slice 57's WIP 260849e8 (implementation/slice57b), which carries slices 55 and 56 unchanged: the fabrication batch's seven families (photo stock 467, photo counter 148, photo portraits 361, locksmith fittings 943, radio battery 247, radio display 164 and radio wire 126 checks) report 0 failures; the radio apparatus (346), radio bench (155), radio stock (735), radio receiving (586) and photo receiving (792) suites report 0 failures; the city sweep's 130 views report 0 failures. The news receiving suite's one failure there, its keyboard station's standing capsule, is identical at slice 52's WIP 3f3f0d75 before any of these shop slices (receipt base53__news_receiving).</t>
+        </is>
+      </c>
     </row>
     <row r="81">
       <c r="A81" s="2" t="inlineStr">
@@ -5887,10 +5891,14 @@
       </c>
       <c r="S81" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T81" s="2" t="inlineStr"/>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="T81" s="2" t="inlineStr">
+        <is>
+          <t>The register lies open on the counter, a column of figures as ink strokes on blank rules, a pencil on a string (copy_counter, shop_keys_cut_SITE_SHOP_IN0_KEYS_CUT). Verified at slice 57's WIP 260849e8 (implementation/slice57b), which carries slices 55 and 56 unchanged: the fabrication batch's seven families (photo stock 467, photo counter 148, photo portraits 361, locksmith fittings 943, radio battery 247, radio display 164 and radio wire 126 checks) report 0 failures; the radio apparatus (346), radio bench (155), radio stock (735), radio receiving (586) and photo receiving (792) suites report 0 failures; the city sweep's 130 views report 0 failures. The news receiving suite's one failure there, its keyboard station's standing capsule, is identical at slice 52's WIP 3f3f0d75 before any of these shop slices (receipt base53__news_receiving).</t>
+        </is>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
@@ -5953,10 +5961,14 @@
       </c>
       <c r="S82" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T82" s="2" t="inlineStr"/>
+          <t>implemented</t>
+        </is>
+      </c>
+      <c r="T82" s="2" t="inlineStr">
+        <is>
+          <t>Partial: the key board's blanks vary by row (bow form, blade length, bitting), the fourth row hangs empty and six more pegs are bare; of the four lock cases one stands open, its cover on the cloth with its screws (key_board, loose_locks, shop_keys_cut_SITE_SHOP_IN1_KEYS_CUT). The table's blocks are not yet picks and blanks. Verified at slice 57's WIP 260849e8 (implementation/slice57b), which carries slices 55 and 56 unchanged: the fabrication batch's seven families (photo stock 467, photo counter 148, photo portraits 361, locksmith fittings 943, radio battery 247, radio display 164 and radio wire 126 checks) report 0 failures; the radio apparatus (346), radio bench (155), radio stock (735), radio receiving (586) and photo receiving (792) suites report 0 failures; the city sweep's 130 views report 0 failures. The news receiving suite's one failure there, its keyboard station's standing capsule, is identical at slice 52's WIP 3f3f0d75 before any of these shop slices (receipt base53__news_receiving).</t>
+        </is>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Implement dossier slice 57: radio valves in racks, the 1610 set, test gear, the wire reel
- CITY_SHOP_RADIO_SERVICE-003: valves are shouldered smoky envelopes on
  Bakelite bases with a silvered getter flash, the stored ones in slatted
  tube racks; a moving-coil meter and a soldering iron in its stand on the
  bench; the black floor ring is rubber-covered wire on its own reel.
- CITY_SHOP_RADIO_SERVICE-001 (partial): the open-back set's wordless dial
  with the pointer at the top of the band and a cone speaker corded to it;
  the low open-channel hiss is not added.
- Seven fabrication families, five shop suites and the city sweep pass at
  this WIP; the news receiving suite's keyboard-station failure is
  identical before slice 53.

Evidence under implementation/slice57b/ (slices 55 and 56 cite it).
INERT: no ledger status changes.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/art/reviews/v2_environment_design_20261008/change_register.xlsx
+++ b/art/reviews/v2_environment_design_20261008/change_register.xlsx
@@ -7191,10 +7191,14 @@
       </c>
       <c r="S101" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T101" s="2" t="inlineStr"/>
+          <t>implemented</t>
+        </is>
+      </c>
+      <c r="T101" s="2" t="inlineStr">
+        <is>
+          <t>Partial: the open-back set on the bench has a wordless dial with its pointer at the top of the band and a cone speaker on its own foot corded to it (alignment_bench, original_instruments). The low open-channel hiss is not added: the shop ambience owner is unchanged. Verified at slice 57's WIP 260849e8 (implementation/slice57b), which carries slices 55 and 56 unchanged: the fabrication batch's seven families (photo stock 467, photo counter 148, photo portraits 361, locksmith fittings 943, radio battery 247, radio display 164 and radio wire 126 checks) report 0 failures; the radio apparatus (346), radio bench (155), radio stock (735), radio receiving (586) and photo receiving (792) suites report 0 failures; the city sweep's 130 views report 0 failures. The news receiving suite's one failure there, its keyboard station's standing capsule, is identical at slice 52's WIP 3f3f0d75 before any of these shop slices (receipt base53__news_receiving).</t>
+        </is>
+      </c>
     </row>
     <row r="102">
       <c r="A102" s="2" t="inlineStr">
@@ -7315,10 +7319,14 @@
       </c>
       <c r="S103" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T103" s="2" t="inlineStr"/>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="T103" s="2" t="inlineStr">
+        <is>
+          <t>Valves are shouldered smoky envelopes on Bakelite bases with a silvered getter flash, the stored ones standing in slatted tube racks; a moving-coil meter and a soldering iron in its stand join the bench; the black floor ring is black rubber-covered wire wound on its own wooden reel (valve_rank, rack_front, upper_valve_rank, two_fixed_reels, shop_radio_service_SITE_SHOP_IN0_RADIO_SERVICE, storm_shop_radio_service_floor_0). Verified at slice 57's WIP 260849e8 (implementation/slice57b), which carries slices 55 and 56 unchanged: the fabrication batch's seven families (photo stock 467, photo counter 148, photo portraits 361, locksmith fittings 943, radio battery 247, radio display 164 and radio wire 126 checks) report 0 failures; the radio apparatus (346), radio bench (155), radio stock (735), radio receiving (586) and photo receiving (792) suites report 0 failures; the city sweep's 130 views report 0 failures. The news receiving suite's one failure there, its keyboard station's standing capsule, is identical at slice 52's WIP 3f3f0d75 before any of these shop slices (receipt base53__news_receiving).</t>
+        </is>
+      </c>
     </row>
     <row r="104">
       <c r="A104" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Implement dossier slice 58: 1A's bath rail, 1D's window towel, 6A's light table, 4D's lost property
- F06_A_KITCHEN-003, F04_D_STUDY-002: Sacha's light table for negatives on the
  prep cabinet (renamed and moved in slice 67) and two shelves of lost property
  in 4D's study, each guest's leaving tagged with a blank card.
- F01_A_BATH-003 (implemented): Evelyn's own brass grab rail; the closed curtain
  hides it from every sweep station.
- F01_D_BATH-003 (partial): a towel pegged over the window head; no soaking bowl.
- From this slice the world refused to compose (the light box reused slice 38's
  surface-stock id) until slice 67; verification is at slice 67's WIP.

Evidence under implementation/slice67/. INERT: no ledger status changes.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/art/reviews/v2_environment_design_20261008/change_register.xlsx
+++ b/art/reviews/v2_environment_design_20261008/change_register.xlsx
@@ -11747,10 +11747,14 @@
       </c>
       <c r="S165" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T165" s="2" t="inlineStr"/>
+          <t>implemented</t>
+        </is>
+      </c>
+      <c r="T165" s="2" t="inlineStr">
+        <is>
+          <t>Evelyn's own brass grab rail on two roses, fixed to the 1A shower's receptor wall at 0.82 m (1A_bath_rail_native). The closed curtain hides it from every sweep station, so it reads only from inside the receptor. Verified at slice 67's WIP 2c25e683 (implementation/slice67), which carries slices 58 to 66 with slice 67's fixes: from slice 58 the world refused to compose (slice 58's light box reused an id slice 38's surface stock owned) until slice 67 renamed it. At 2c25e683 the fabrication batch's ten families (12,295 checks) report one failure, the capture harness finding no clear camera station for the B1 cleat run; apartment batch 204 on the long runner, as before; household state 154 checks, 0 failures; upper kitchens 206 and upper furniture 488, both unchanged; upper lighting 9,257 checks and public doors 17, 0 failures; the remaining transfers, apartment door, first upper hall, 4B door and rear wing A routes, the basement route (88), basement ground, boiler service, reading furniture, shop seating, funeral fittings, completion heating, radiator ties, ventilation, door casings (107 openings), hardware drawers (1,309 checks), street boundary, passage visibility, commensal, the street boundary route and the resident key route (86 waypoints, long runner), all 0 failures; twelve sweeps (55 spaces) and the city sweep's 130 views, 0 failures. The coal delivery route's stop at the lobby's inner door and the Vantry gateway suite's five kiosk-count failures are identical at slice 57's 260849e8 (base58), and the news receiving station failure is identical before slice 53.</t>
+        </is>
+      </c>
     </row>
     <row r="166">
       <c r="A166" s="2" t="inlineStr">
@@ -13643,10 +13647,14 @@
       </c>
       <c r="S189" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T189" s="2" t="inlineStr"/>
+          <t>implemented</t>
+        </is>
+      </c>
+      <c r="T189" s="2" t="inlineStr">
+        <is>
+          <t>Partial: a huckaback towel pegged over a cord across the 1D bath window head, the night nurse sleeping by day (1D_window_towel_native, F01_D_BATH_DT2). The soaking bowl of collars and cuffs at the basin is not made. Verified at slice 67's WIP 2c25e683 (implementation/slice67), which carries slices 58 to 66 with slice 67's fixes: from slice 58 the world refused to compose (slice 58's light box reused an id slice 38's surface stock owned) until slice 67 renamed it. At 2c25e683 the fabrication batch's ten families (12,295 checks) report one failure, the capture harness finding no clear camera station for the B1 cleat run; apartment batch 204 on the long runner, as before; household state 154 checks, 0 failures; upper kitchens 206 and upper furniture 488, both unchanged; upper lighting 9,257 checks and public doors 17, 0 failures; the remaining transfers, apartment door, first upper hall, 4B door and rear wing A routes, the basement route (88), basement ground, boiler service, reading furniture, shop seating, funeral fittings, completion heating, radiator ties, ventilation, door casings (107 openings), hardware drawers (1,309 checks), street boundary, passage visibility, commensal, the street boundary route and the resident key route (86 waypoints, long runner), all 0 failures; twelve sweeps (55 spaces) and the city sweep's 130 views, 0 failures. The coal delivery route's stop at the lobby's inner door and the Vantry gateway suite's five kiosk-count failures are identical at slice 57's 260849e8 (base58), and the news receiving station failure is identical before slice 53.</t>
+        </is>
+      </c>
     </row>
     <row r="190">
       <c r="A190" s="2" t="inlineStr">
@@ -31407,10 +31415,14 @@
       </c>
       <c r="S423" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T423" s="2" t="inlineStr"/>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="T423" s="2" t="inlineStr">
+        <is>
+          <t>Two shelves of lost property in 4D's study, nine guests' leavings each tagged with a blank card on a string (4D_lost_shelves_native, F04_D_STUDY_OV); a teleported capture, as the row asks. Verified at slice 67's WIP 2c25e683 (implementation/slice67), which carries slices 58 to 66 with slice 67's fixes: from slice 58 the world refused to compose (slice 58's light box reused an id slice 38's surface stock owned) until slice 67 renamed it. At 2c25e683 the fabrication batch's ten families (12,295 checks) report one failure, the capture harness finding no clear camera station for the B1 cleat run; apartment batch 204 on the long runner, as before; household state 154 checks, 0 failures; upper kitchens 206 and upper furniture 488, both unchanged; upper lighting 9,257 checks and public doors 17, 0 failures; the remaining transfers, apartment door, first upper hall, 4B door and rear wing A routes, the basement route (88), basement ground, boiler service, reading furniture, shop seating, funeral fittings, completion heating, radiator ties, ventilation, door casings (107 openings), hardware drawers (1,309 checks), street boundary, passage visibility, commensal, the street boundary route and the resident key route (86 waypoints, long runner), all 0 failures; twelve sweeps (55 spaces) and the city sweep's 130 views, 0 failures. The coal delivery route's stop at the lobby's inner door and the Vantry gateway suite's five kiosk-count failures are identical at slice 57's 260849e8 (base58), and the news receiving station failure is identical before slice 53.</t>
+        </is>
+      </c>
     </row>
     <row r="424">
       <c r="A424" s="2" t="inlineStr">
@@ -38633,10 +38645,14 @@
       </c>
       <c r="S520" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T520" s="2" t="inlineStr"/>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="T520" s="2" t="inlineStr">
+        <is>
+          <t>Sacha's light table on the prep cabinet beside the toaster: a frosted plate in a timber box with a strip of negatives and a loupe on it, the lamp inside unlit (6A_light_table_native, F06_A_KITCHEN_DT1). Slice 58 named it 6A_light_box, an id slice 38's surface-stock box already owned, and the runtime refused the world; slice 67 renamed it 6A_light_table, moved it to the cabinet's clear front off the plate and dropped its flex. Verified at slice 67's WIP 2c25e683 (implementation/slice67), which carries slices 58 to 66 with slice 67's fixes: from slice 58 the world refused to compose (slice 58's light box reused an id slice 38's surface stock owned) until slice 67 renamed it. At 2c25e683 the fabrication batch's ten families (12,295 checks) report one failure, the capture harness finding no clear camera station for the B1 cleat run; apartment batch 204 on the long runner, as before; household state 154 checks, 0 failures; upper kitchens 206 and upper furniture 488, both unchanged; upper lighting 9,257 checks and public doors 17, 0 failures; the remaining transfers, apartment door, first upper hall, 4B door and rear wing A routes, the basement route (88), basement ground, boiler service, reading furniture, shop seating, funeral fittings, completion heating, radiator ties, ventilation, door casings (107 openings), hardware drawers (1,309 checks), street boundary, passage visibility, commensal, the street boundary route and the resident key route (86 waypoints, long runner), all 0 failures; twelve sweeps (55 spaces) and the city sweep's 130 views, 0 failures. The coal delivery route's stop at the lobby's inner door and the Vantry gateway suite's five kiosk-count failures are identical at slice 57's 260849e8 (base58), and the news receiving station failure is identical before slice 53.</t>
+        </is>
+      </c>
     </row>
     <row r="521">
       <c r="A521" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Implement dossier slice 59: the laundry rota and painted-over outlet, cleated wiring, a coal shovel
- B1_LAUNDRY-002, B1_ELECTRICAL-002: the laundry rota in the notice-frame
  family and the brass signal outlet painted over high on the north wall; a
  twisted cloth pair on porcelain cleats to the fuse panel and Omar's shelf of
  cartridges and chalk.
- B1_COAL_ROOM-001 (partial): the coal shovel by the heap; no bunker board for
  the tally.
- New object forms: painted outlet, cleat run, dropped cartridge, coal shovel.

Evidence under implementation/slice67/. INERT: no ledger status changes.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/art/reviews/v2_environment_design_20261008/change_register.xlsx
+++ b/art/reviews/v2_environment_design_20261008/change_register.xlsx
@@ -703,10 +703,14 @@
       </c>
       <c r="S3" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T3" s="2" t="inlineStr"/>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="T3" s="2" t="inlineStr">
+        <is>
+          <t>The laundry rota by the laundry door in the notice-frame family, its words a Label3D the lamp reads, and high on the north wall the brass signal outlet painted over, its cloth lead cut short (B1_painted_outlet_native, B1_LAUNDRY_OV). Verified at slice 67's WIP 2c25e683 (implementation/slice67), which carries slices 58 to 66 with slice 67's fixes: from slice 58 the world refused to compose (slice 58's light box reused an id slice 38's surface stock owned) until slice 67 renamed it. At 2c25e683 the fabrication batch's ten families (12,295 checks) report one failure, the capture harness finding no clear camera station for the B1 cleat run; apartment batch 204 on the long runner, as before; household state 154 checks, 0 failures; upper kitchens 206 and upper furniture 488, both unchanged; upper lighting 9,257 checks and public doors 17, 0 failures; the remaining transfers, apartment door, first upper hall, 4B door and rear wing A routes, the basement route (88), basement ground, boiler service, reading furniture, shop seating, funeral fittings, completion heating, radiator ties, ventilation, door casings (107 openings), hardware drawers (1,309 checks), street boundary, passage visibility, commensal, the street boundary route and the resident key route (86 waypoints, long runner), all 0 failures; twelve sweeps (55 spaces) and the city sweep's 130 views, 0 failures. The coal delivery route's stop at the lobby's inner door and the Vantry gateway suite's five kiosk-count failures are identical at slice 57's 260849e8 (base58), and the news receiving station failure is identical before slice 53.</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -1429,10 +1433,14 @@
       </c>
       <c r="S14" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T14" s="2" t="inlineStr"/>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="T14" s="2" t="inlineStr">
+        <is>
+          <t>A twisted cloth pair on porcelain cleats along the electrical room's wall to the fuse panel, and Omar's shelf of cartridges and chalk (B1_ELECTRICAL_OV, B1_ELECTRICAL_DT1). The fabrication capture found no clear standing station in the narrow room; the sweep views carry it. Verified at slice 67's WIP 2c25e683 (implementation/slice67), which carries slices 58 to 66 with slice 67's fixes: from slice 58 the world refused to compose (slice 58's light box reused an id slice 38's surface stock owned) until slice 67 renamed it. At 2c25e683 the fabrication batch's ten families (12,295 checks) report one failure, the capture harness finding no clear camera station for the B1 cleat run; apartment batch 204 on the long runner, as before; household state 154 checks, 0 failures; upper kitchens 206 and upper furniture 488, both unchanged; upper lighting 9,257 checks and public doors 17, 0 failures; the remaining transfers, apartment door, first upper hall, 4B door and rear wing A routes, the basement route (88), basement ground, boiler service, reading furniture, shop seating, funeral fittings, completion heating, radiator ties, ventilation, door casings (107 openings), hardware drawers (1,309 checks), street boundary, passage visibility, commensal, the street boundary route and the resident key route (86 waypoints, long runner), all 0 failures; twelve sweeps (55 spaces) and the city sweep's 130 views, 0 failures. The coal delivery route's stop at the lobby's inner door and the Vantry gateway suite's five kiosk-count failures are identical at slice 57's 260849e8 (base58), and the news receiving station failure is identical before slice 53.</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -1759,10 +1767,14 @@
       </c>
       <c r="S19" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T19" s="2" t="inlineStr"/>
+          <t>implemented</t>
+        </is>
+      </c>
+      <c r="T19" s="2" t="inlineStr">
+        <is>
+          <t>Partial: the coal shovel leaning by the heap, its pan on the floor and grip on the whitewash (B1_coal_shovel_native), and the dust fanned from the chute mouth (slice 60). The heap's cut face and the chalk tally on a bunker board are not made: no bunker board exists. Verified at slice 67's WIP 2c25e683 (implementation/slice67), which carries slices 58 to 66 with slice 67's fixes: from slice 58 the world refused to compose (slice 58's light box reused an id slice 38's surface stock owned) until slice 67 renamed it. At 2c25e683 the fabrication batch's ten families (12,295 checks) report one failure, the capture harness finding no clear camera station for the B1 cleat run; apartment batch 204 on the long runner, as before; household state 154 checks, 0 failures; upper kitchens 206 and upper furniture 488, both unchanged; upper lighting 9,257 checks and public doors 17, 0 failures; the remaining transfers, apartment door, first upper hall, 4B door and rear wing A routes, the basement route (88), basement ground, boiler service, reading furniture, shop seating, funeral fittings, completion heating, radiator ties, ventilation, door casings (107 openings), hardware drawers (1,309 checks), street boundary, passage visibility, commensal, the street boundary route and the resident key route (86 waypoints, long runner), all 0 failures; twelve sweeps (55 spaces) and the city sweep's 130 views, 0 failures. The coal delivery route's stop at the lobby's inner door and the Vantry gateway suite's five kiosk-count failures are identical at slice 57's 260849e8 (base58), and the news receiving station failure is identical before slice 53.</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Implement dossier slice 60: coal dust, the door sweep, the chute fan, the chalked log
- B1_ELECTRICAL_RECESS-001: the electrical door's sweep scuffed on the recess
  floor, with slice 59's dropped cartridge.
- B1_BOILER_APPROACH-001 (partial), B1_SERVICE_CORE-001, B1_BOILER_ROOM-002
  (implemented): coal dust down the approach and on the lowest service treads,
  and Omar's chalked log on the water column, as projected decals; no sweep
  station frames the treads or the column.
- Positional wear gains coal, arc, fan and chalk kinds.

Evidence under implementation/slice67/. INERT: no ledger status changes.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/art/reviews/v2_environment_design_20261008/change_register.xlsx
+++ b/art/reviews/v2_environment_design_20261008/change_register.xlsx
@@ -1083,10 +1083,14 @@
       </c>
       <c r="S9" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T9" s="2" t="inlineStr"/>
+          <t>implemented</t>
+        </is>
+      </c>
+      <c r="T9" s="2" t="inlineStr">
+        <is>
+          <t>Partial: coal dust trodden down the boiler approach, darkening toward the fire door (a projected decal; no sweep station frames it clearly). The fire bucket on its hook is not made: the approach is a 1.2 m route. Verified at slice 67's WIP 2c25e683 (implementation/slice67), which carries slices 58 to 66 with slice 67's fixes: from slice 58 the world refused to compose (slice 58's light box reused an id slice 38's surface stock owned) until slice 67 renamed it. At 2c25e683 the fabrication batch's ten families (12,295 checks) report one failure, the capture harness finding no clear camera station for the B1 cleat run; apartment batch 204 on the long runner, as before; household state 154 checks, 0 failures; upper kitchens 206 and upper furniture 488, both unchanged; upper lighting 9,257 checks and public doors 17, 0 failures; the remaining transfers, apartment door, first upper hall, 4B door and rear wing A routes, the basement route (88), basement ground, boiler service, reading furniture, shop seating, funeral fittings, completion heating, radiator ties, ventilation, door casings (107 openings), hardware drawers (1,309 checks), street boundary, passage visibility, commensal, the street boundary route and the resident key route (86 waypoints, long runner), all 0 failures; twelve sweeps (55 spaces) and the city sweep's 130 views, 0 failures. The coal delivery route's stop at the lobby's inner door and the Vantry gateway suite's five kiosk-count failures are identical at slice 57's 260849e8 (base58), and the news receiving station failure is identical before slice 53.</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -1223,10 +1227,14 @@
       </c>
       <c r="S11" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T11" s="2" t="inlineStr"/>
+          <t>implemented</t>
+        </is>
+      </c>
+      <c r="T11" s="2" t="inlineStr">
+        <is>
+          <t>Omar's chalked log on the water column: tally groups, ticks and strokes in a working hand, no numerals, a projected decal mounted with the world at 2c25e683. The sweep's detail stations face the boiler front, not the column; a framed capture is open. Verified at slice 67's WIP 2c25e683 (implementation/slice67), which carries slices 58 to 66 with slice 67's fixes: from slice 58 the world refused to compose (slice 58's light box reused an id slice 38's surface stock owned) until slice 67 renamed it. At 2c25e683 the fabrication batch's ten families (12,295 checks) report one failure, the capture harness finding no clear camera station for the B1 cleat run; apartment batch 204 on the long runner, as before; household state 154 checks, 0 failures; upper kitchens 206 and upper furniture 488, both unchanged; upper lighting 9,257 checks and public doors 17, 0 failures; the remaining transfers, apartment door, first upper hall, 4B door and rear wing A routes, the basement route (88), basement ground, boiler service, reading furniture, shop seating, funeral fittings, completion heating, radiator ties, ventilation, door casings (107 openings), hardware drawers (1,309 checks), street boundary, passage visibility, commensal, the street boundary route and the resident key route (86 waypoints, long runner), all 0 failures; twelve sweeps (55 spaces) and the city sweep's 130 views, 0 failures. The coal delivery route's stop at the lobby's inner door and the Vantry gateway suite's five kiosk-count failures are identical at slice 57's 260849e8 (base58), and the news receiving station failure is identical before slice 53.</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -1565,10 +1573,14 @@
       </c>
       <c r="S16" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T16" s="2" t="inlineStr"/>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="T16" s="2" t="inlineStr">
+        <is>
+          <t>The door's sweep scuffed into a quarter ring on the recess floor and a cartridge fuse dropped in the corner (slice 59) (B1_dropped_cartridge_native). Verified at slice 67's WIP 2c25e683 (implementation/slice67), which carries slices 58 to 66 with slice 67's fixes: from slice 58 the world refused to compose (slice 58's light box reused an id slice 38's surface stock owned) until slice 67 renamed it. At 2c25e683 the fabrication batch's ten families (12,295 checks) report one failure, the capture harness finding no clear camera station for the B1 cleat run; apartment batch 204 on the long runner, as before; household state 154 checks, 0 failures; upper kitchens 206 and upper furniture 488, both unchanged; upper lighting 9,257 checks and public doors 17, 0 failures; the remaining transfers, apartment door, first upper hall, 4B door and rear wing A routes, the basement route (88), basement ground, boiler service, reading furniture, shop seating, funeral fittings, completion heating, radiator ties, ventilation, door casings (107 openings), hardware drawers (1,309 checks), street boundary, passage visibility, commensal, the street boundary route and the resident key route (86 waypoints, long runner), all 0 failures; twelve sweeps (55 spaces) and the city sweep's 130 views, 0 failures. The coal delivery route's stop at the lobby's inner door and the Vantry gateway suite's five kiosk-count failures are identical at slice 57's 260849e8 (base58), and the news receiving station failure is identical before slice 53.</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -2171,10 +2183,14 @@
       </c>
       <c r="S25" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T25" s="2" t="inlineStr"/>
+          <t>implemented</t>
+        </is>
+      </c>
+      <c r="T25" s="2" t="inlineStr">
+        <is>
+          <t>Coal dust on the three lowest service-stair treads, a projected decal mounted with the world at 2c25e683 (positional_wear.json, 0 refusals). No sweep station frames those treads; a framed capture is open. Verified at slice 67's WIP 2c25e683 (implementation/slice67), which carries slices 58 to 66 with slice 67's fixes: from slice 58 the world refused to compose (slice 58's light box reused an id slice 38's surface stock owned) until slice 67 renamed it. At 2c25e683 the fabrication batch's ten families (12,295 checks) report one failure, the capture harness finding no clear camera station for the B1 cleat run; apartment batch 204 on the long runner, as before; household state 154 checks, 0 failures; upper kitchens 206 and upper furniture 488, both unchanged; upper lighting 9,257 checks and public doors 17, 0 failures; the remaining transfers, apartment door, first upper hall, 4B door and rear wing A routes, the basement route (88), basement ground, boiler service, reading furniture, shop seating, funeral fittings, completion heating, radiator ties, ventilation, door casings (107 openings), hardware drawers (1,309 checks), street boundary, passage visibility, commensal, the street boundary route and the resident key route (86 waypoints, long runner), all 0 failures; twelve sweeps (55 spaces) and the city sweep's 130 views, 0 failures. The coal delivery route's stop at the lobby's inner door and the Vantry gateway suite's five kiosk-count failures are identical at slice 57's 260849e8 (base58), and the news receiving station failure is identical before slice 53.</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Implement dossier slice 61: a water line under every curtain, 5D's soot as a soft fan
- Bath -002 rows (18): the water line on the floor under each shower curtain's
  hem joins slice 52's wear; faint at production light.
- F05_D_RESTRICTED-002: the stepped soot boards become a soft projected fan over
  the door head.

Evidence under implementation/slice67/. INERT: no ledger status changes.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/art/reviews/v2_environment_design_20261008/change_register.xlsx
+++ b/art/reviews/v2_environment_design_20261008/change_register.xlsx
@@ -11706,7 +11706,7 @@
       </c>
       <c r="T164" s="2" t="inlineStr">
         <is>
-          <t>Partial: a darkened grout-and-water ring round the shower receptor's lip and the mop-shadow corner farthest from the door, both soft projected wear (F01_A_BATH_OV; a frame difference against slice 47's view isolates the ring at the receptor's base). Paint lifted below the register is not made: the bath's vent register hangs from its duct at 2.6 m with no wall below it (F01_A_BATH_DT1). The water line under the curtain hem follows in slice 61. Verified at WIP 3f3f0d75 (implementation/slice52): apartment batch 204 on the long runner; household state 154 checks, 0 failures; upper kitchens 206 and upper furniture 488, both unchanged; upper lighting 9,257 checks and public doors 17, both 0 failures; the first bath sweep (six baths) 0 failures; the remaining twelve baths, the thirteen upper halls and slice 50's third core group were rerun at the same WIP in five sweeps, all 0 failures (implementation/slice52b); four earlier sweep runs that ran at another WIP are superseded and not cited. The decals are projected (Godot Decal nodes) from game/data/orison_v2/positional_wear.json onto the inherited finishes: no collision, no owner, no lettering.</t>
+          <t>Partial: a darkened grout-and-water ring round the shower receptor's lip and the mop-shadow corner farthest from the door, both soft projected wear (F01_A_BATH_OV; a frame difference against slice 47's view isolates the ring at the receptor's base). Paint lifted below the register is not made: the bath's vent register hangs from its duct at 2.6 m with no wall below it (F01_A_BATH_DT1). The water line under the curtain hem follows in slice 61. Verified at WIP 3f3f0d75 (implementation/slice52): apartment batch 204 on the long runner; household state 154 checks, 0 failures; upper kitchens 206 and upper furniture 488, both unchanged; upper lighting 9,257 checks and public doors 17, both 0 failures; the first bath sweep (six baths) 0 failures; the remaining twelve baths, the thirteen upper halls and slice 50's third core group were rerun at the same WIP in five sweeps, all 0 failures (implementation/slice52b); four earlier sweep runs that ran at another WIP are superseded and not cited. The decals are projected (Godot Decal nodes) from game/data/orison_v2/positional_wear.json onto the inherited finishes: no collision, no owner, no lettering. Slice 61 adds the water line on the floor under the curtain hem, a ragged damp band with a darker drying edge, mounted with the world at 2c25e683 (implementation/slice67); a frame difference against slice 52's view picks it out along the hem, faint at production light.</t>
         </is>
       </c>
     </row>
@@ -13606,7 +13606,7 @@
       </c>
       <c r="T188" s="2" t="inlineStr">
         <is>
-          <t>Partial: a darkened grout-and-water ring round the shower receptor's lip and the mop-shadow corner farthest from the door, both soft projected wear (F01_D_BATH_OV; a frame difference against slice 47's view isolates the ring at the receptor's base). Paint lifted below the register is not made: the bath's vent register hangs from its duct at 2.6 m with no wall below it (F01_D_BATH_DT1). The water line under the curtain hem follows in slice 61. Verified at WIP 3f3f0d75 (implementation/slice52): apartment batch 204 on the long runner; household state 154 checks, 0 failures; upper kitchens 206 and upper furniture 488, both unchanged; upper lighting 9,257 checks and public doors 17, both 0 failures; the first bath sweep (six baths) 0 failures; the remaining twelve baths, the thirteen upper halls and slice 50's third core group were rerun at the same WIP in five sweeps, all 0 failures (implementation/slice52b); four earlier sweep runs that ran at another WIP are superseded and not cited. The decals are projected (Godot Decal nodes) from game/data/orison_v2/positional_wear.json onto the inherited finishes: no collision, no owner, no lettering.</t>
+          <t>Partial: a darkened grout-and-water ring round the shower receptor's lip and the mop-shadow corner farthest from the door, both soft projected wear (F01_D_BATH_OV; a frame difference against slice 47's view isolates the ring at the receptor's base). Paint lifted below the register is not made: the bath's vent register hangs from its duct at 2.6 m with no wall below it (F01_D_BATH_DT1). The water line under the curtain hem follows in slice 61. Verified at WIP 3f3f0d75 (implementation/slice52): apartment batch 204 on the long runner; household state 154 checks, 0 failures; upper kitchens 206 and upper furniture 488, both unchanged; upper lighting 9,257 checks and public doors 17, both 0 failures; the first bath sweep (six baths) 0 failures; the remaining twelve baths, the thirteen upper halls and slice 50's third core group were rerun at the same WIP in five sweeps, all 0 failures (implementation/slice52b); four earlier sweep runs that ran at another WIP are superseded and not cited. The decals are projected (Godot Decal nodes) from game/data/orison_v2/positional_wear.json onto the inherited finishes: no collision, no owner, no lettering. Slice 61 adds the water line on the floor under the curtain hem, a ragged damp band with a darker drying edge, mounted with the world at 2c25e683 (implementation/slice67); a frame difference against slice 52's view picks it out along the hem, faint at production light.</t>
         </is>
       </c>
     </row>
@@ -16102,7 +16102,7 @@
       </c>
       <c r="T220" s="2" t="inlineStr">
         <is>
-          <t>Partial: a darkened grout-and-water ring round the shower receptor's lip and the mop-shadow corner farthest from the door, both soft projected wear (F02_A_BATH_OV; a frame difference against slice 47's view isolates the ring at the receptor's base). Paint lifted below the register is not made: the bath's vent register hangs from its duct at 2.6 m with no wall below it (F02_A_BATH_DT1). The water line under the curtain hem follows in slice 61. Verified at WIP 3f3f0d75 (implementation/slice52): apartment batch 204 on the long runner; household state 154 checks, 0 failures; upper kitchens 206 and upper furniture 488, both unchanged; upper lighting 9,257 checks and public doors 17, both 0 failures; the first bath sweep (six baths) 0 failures; the remaining twelve baths, the thirteen upper halls and slice 50's third core group were rerun at the same WIP in five sweeps, all 0 failures (implementation/slice52b); four earlier sweep runs that ran at another WIP are superseded and not cited. The decals are projected (Godot Decal nodes) from game/data/orison_v2/positional_wear.json onto the inherited finishes: no collision, no owner, no lettering.</t>
+          <t>Partial: a darkened grout-and-water ring round the shower receptor's lip and the mop-shadow corner farthest from the door, both soft projected wear (F02_A_BATH_OV; a frame difference against slice 47's view isolates the ring at the receptor's base). Paint lifted below the register is not made: the bath's vent register hangs from its duct at 2.6 m with no wall below it (F02_A_BATH_DT1). The water line under the curtain hem follows in slice 61. Verified at WIP 3f3f0d75 (implementation/slice52): apartment batch 204 on the long runner; household state 154 checks, 0 failures; upper kitchens 206 and upper furniture 488, both unchanged; upper lighting 9,257 checks and public doors 17, both 0 failures; the first bath sweep (six baths) 0 failures; the remaining twelve baths, the thirteen upper halls and slice 50's third core group were rerun at the same WIP in five sweeps, all 0 failures (implementation/slice52b); four earlier sweep runs that ran at another WIP are superseded and not cited. The decals are projected (Godot Decal nodes) from game/data/orison_v2/positional_wear.json onto the inherited finishes: no collision, no owner, no lettering. Slice 61 adds the water line on the floor under the curtain hem, a ragged damp band with a darker drying edge, mounted with the world at 2c25e683 (implementation/slice67); a frame difference against slice 52's view picks it out along the hem, faint at production light.</t>
         </is>
       </c>
     </row>
@@ -17560,7 +17560,7 @@
       </c>
       <c r="T239" s="2" t="inlineStr">
         <is>
-          <t>Partial: a darkened grout-and-water ring round the shower receptor's lip and the mop-shadow corner farthest from the door, both soft projected wear (F02_B_BATH_OV; a frame difference against slice 47's view isolates the ring at the receptor's base). Paint lifted below the register is not made: the bath's vent register hangs from its duct at 2.6 m with no wall below it (F02_B_BATH_DT1). The water line under the curtain hem follows in slice 61. Verified at WIP 3f3f0d75 (implementation/slice52): apartment batch 204 on the long runner; household state 154 checks, 0 failures; upper kitchens 206 and upper furniture 488, both unchanged; upper lighting 9,257 checks and public doors 17, both 0 failures; the first bath sweep (six baths) 0 failures; the remaining twelve baths, the thirteen upper halls and slice 50's third core group were rerun at the same WIP in five sweeps, all 0 failures (implementation/slice52b); four earlier sweep runs that ran at another WIP are superseded and not cited. The decals are projected (Godot Decal nodes) from game/data/orison_v2/positional_wear.json onto the inherited finishes: no collision, no owner, no lettering.</t>
+          <t>Partial: a darkened grout-and-water ring round the shower receptor's lip and the mop-shadow corner farthest from the door, both soft projected wear (F02_B_BATH_OV; a frame difference against slice 47's view isolates the ring at the receptor's base). Paint lifted below the register is not made: the bath's vent register hangs from its duct at 2.6 m with no wall below it (F02_B_BATH_DT1). The water line under the curtain hem follows in slice 61. Verified at WIP 3f3f0d75 (implementation/slice52): apartment batch 204 on the long runner; household state 154 checks, 0 failures; upper kitchens 206 and upper furniture 488, both unchanged; upper lighting 9,257 checks and public doors 17, both 0 failures; the first bath sweep (six baths) 0 failures; the remaining twelve baths, the thirteen upper halls and slice 50's third core group were rerun at the same WIP in five sweeps, all 0 failures (implementation/slice52b); four earlier sweep runs that ran at another WIP are superseded and not cited. The decals are projected (Godot Decal nodes) from game/data/orison_v2/positional_wear.json onto the inherited finishes: no collision, no owner, no lettering. Slice 61 adds the water line on the floor under the curtain hem, a ragged damp band with a darker drying edge, mounted with the world at 2c25e683 (implementation/slice67); a frame difference against slice 52's view picks it out along the hem, faint at production light.</t>
         </is>
       </c>
     </row>
@@ -18594,7 +18594,7 @@
       </c>
       <c r="T252" s="2" t="inlineStr">
         <is>
-          <t>Partial: a darkened grout-and-water ring round the shower receptor's lip and the mop-shadow corner farthest from the door, both soft projected wear (F02_C_BATH_OV; a frame difference against slice 47's view isolates the ring at the receptor's base). Paint lifted below the register is not made: the bath's vent register hangs from its duct at 2.6 m with no wall below it (F02_C_BATH_DT1). The water line under the curtain hem follows in slice 61. Verified at WIP 3f3f0d75 (implementation/slice52): apartment batch 204 on the long runner; household state 154 checks, 0 failures; upper kitchens 206 and upper furniture 488, both unchanged; upper lighting 9,257 checks and public doors 17, both 0 failures; the first bath sweep (six baths) 0 failures; the remaining twelve baths, the thirteen upper halls and slice 50's third core group were rerun at the same WIP in five sweeps, all 0 failures (implementation/slice52b); four earlier sweep runs that ran at another WIP are superseded and not cited. The decals are projected (Godot Decal nodes) from game/data/orison_v2/positional_wear.json onto the inherited finishes: no collision, no owner, no lettering.</t>
+          <t>Partial: a darkened grout-and-water ring round the shower receptor's lip and the mop-shadow corner farthest from the door, both soft projected wear (F02_C_BATH_OV; a frame difference against slice 47's view isolates the ring at the receptor's base). Paint lifted below the register is not made: the bath's vent register hangs from its duct at 2.6 m with no wall below it (F02_C_BATH_DT1). The water line under the curtain hem follows in slice 61. Verified at WIP 3f3f0d75 (implementation/slice52): apartment batch 204 on the long runner; household state 154 checks, 0 failures; upper kitchens 206 and upper furniture 488, both unchanged; upper lighting 9,257 checks and public doors 17, both 0 failures; the first bath sweep (six baths) 0 failures; the remaining twelve baths, the thirteen upper halls and slice 50's third core group were rerun at the same WIP in five sweeps, all 0 failures (implementation/slice52b); four earlier sweep runs that ran at another WIP are superseded and not cited. The decals are projected (Godot Decal nodes) from game/data/orison_v2/positional_wear.json onto the inherited finishes: no collision, no owner, no lettering. Slice 61 adds the water line on the floor under the curtain hem, a ragged damp band with a darker drying edge, mounted with the world at 2c25e683 (implementation/slice67); a frame difference against slice 52's view picks it out along the hem, faint at production light.</t>
         </is>
       </c>
     </row>
@@ -21482,7 +21482,7 @@
       </c>
       <c r="T290" s="2" t="inlineStr">
         <is>
-          <t>Partial: a darkened grout-and-water ring round the shower receptor's lip and the mop-shadow corner farthest from the door, both soft projected wear (F03_A_BATH_OV; a frame difference against slice 47's view isolates the ring at the receptor's base). Paint lifted below the register is not made: the bath's vent register hangs from its duct at 2.6 m with no wall below it (F03_A_BATH_DT1). The water line under the curtain hem follows in slice 61. Verified at WIP 3f3f0d75 (implementation/slice52): apartment batch 204 on the long runner; household state 154 checks, 0 failures; upper kitchens 206 and upper furniture 488, both unchanged; upper lighting 9,257 checks and public doors 17, both 0 failures; the first bath sweep (six baths) 0 failures; the remaining twelve baths, the thirteen upper halls and slice 50's third core group were rerun at the same WIP in five sweeps, all 0 failures (implementation/slice52b); four earlier sweep runs that ran at another WIP are superseded and not cited. The decals are projected (Godot Decal nodes) from game/data/orison_v2/positional_wear.json onto the inherited finishes: no collision, no owner, no lettering.</t>
+          <t>Partial: a darkened grout-and-water ring round the shower receptor's lip and the mop-shadow corner farthest from the door, both soft projected wear (F03_A_BATH_OV; a frame difference against slice 47's view isolates the ring at the receptor's base). Paint lifted below the register is not made: the bath's vent register hangs from its duct at 2.6 m with no wall below it (F03_A_BATH_DT1). The water line under the curtain hem follows in slice 61. Verified at WIP 3f3f0d75 (implementation/slice52): apartment batch 204 on the long runner; household state 154 checks, 0 failures; upper kitchens 206 and upper furniture 488, both unchanged; upper lighting 9,257 checks and public doors 17, both 0 failures; the first bath sweep (six baths) 0 failures; the remaining twelve baths, the thirteen upper halls and slice 50's third core group were rerun at the same WIP in five sweeps, all 0 failures (implementation/slice52b); four earlier sweep runs that ran at another WIP are superseded and not cited. The decals are projected (Godot Decal nodes) from game/data/orison_v2/positional_wear.json onto the inherited finishes: no collision, no owner, no lettering. Slice 61 adds the water line on the floor under the curtain hem, a ragged damp band with a darker drying edge, mounted with the world at 2c25e683 (implementation/slice67); a frame difference against slice 52's view picks it out along the hem, faint at production light.</t>
         </is>
       </c>
     </row>
@@ -22780,7 +22780,7 @@
       </c>
       <c r="T307" s="2" t="inlineStr">
         <is>
-          <t>Partial: a darkened grout-and-water ring round the shower receptor's lip and the mop-shadow corner farthest from the door, both soft projected wear (F03_B_BATH_OV; a frame difference against slice 47's view isolates the ring at the receptor's base). Paint lifted below the register is not made: the bath's vent register hangs from its duct at 2.6 m with no wall below it (F03_B_BATH_DT1). The water line under the curtain hem follows in slice 61. Verified at WIP 3f3f0d75 (implementation/slice52): apartment batch 204 on the long runner; household state 154 checks, 0 failures; upper kitchens 206 and upper furniture 488, both unchanged; upper lighting 9,257 checks and public doors 17, both 0 failures; the first bath sweep (six baths) 0 failures; the remaining twelve baths, the thirteen upper halls and slice 50's third core group were rerun at the same WIP in five sweeps, all 0 failures (implementation/slice52b); four earlier sweep runs that ran at another WIP are superseded and not cited. The decals are projected (Godot Decal nodes) from game/data/orison_v2/positional_wear.json onto the inherited finishes: no collision, no owner, no lettering.</t>
+          <t>Partial: a darkened grout-and-water ring round the shower receptor's lip and the mop-shadow corner farthest from the door, both soft projected wear (F03_B_BATH_OV; a frame difference against slice 47's view isolates the ring at the receptor's base). Paint lifted below the register is not made: the bath's vent register hangs from its duct at 2.6 m with no wall below it (F03_B_BATH_DT1). The water line under the curtain hem follows in slice 61. Verified at WIP 3f3f0d75 (implementation/slice52): apartment batch 204 on the long runner; household state 154 checks, 0 failures; upper kitchens 206 and upper furniture 488, both unchanged; upper lighting 9,257 checks and public doors 17, both 0 failures; the first bath sweep (six baths) 0 failures; the remaining twelve baths, the thirteen upper halls and slice 50's third core group were rerun at the same WIP in five sweeps, all 0 failures (implementation/slice52b); four earlier sweep runs that ran at another WIP are superseded and not cited. The decals are projected (Godot Decal nodes) from game/data/orison_v2/positional_wear.json onto the inherited finishes: no collision, no owner, no lettering. Slice 61 adds the water line on the floor under the curtain hem, a ragged damp band with a darker drying edge, mounted with the world at 2c25e683 (implementation/slice67); a frame difference against slice 52's view picks it out along the hem, faint at production light.</t>
         </is>
       </c>
     </row>
@@ -23794,7 +23794,7 @@
       </c>
       <c r="T320" s="2" t="inlineStr">
         <is>
-          <t>Partial: a darkened grout-and-water ring round the shower receptor's lip and the mop-shadow corner farthest from the door, both soft projected wear (F03_D_BATH_OV; a frame difference against slice 47's view isolates the ring at the receptor's base). Paint lifted below the register is not made: the bath's vent register hangs from its duct at 2.6 m with no wall below it (F03_D_BATH_DT1). The water line under the curtain hem follows in slice 61. Verified at WIP 3f3f0d75 (implementation/slice52): apartment batch 204 on the long runner; household state 154 checks, 0 failures; upper kitchens 206 and upper furniture 488, both unchanged; upper lighting 9,257 checks and public doors 17, both 0 failures; the first bath sweep (six baths) 0 failures; the remaining twelve baths, the thirteen upper halls and slice 50's third core group were rerun at the same WIP in five sweeps, all 0 failures (implementation/slice52b); four earlier sweep runs that ran at another WIP are superseded and not cited. The decals are projected (Godot Decal nodes) from game/data/orison_v2/positional_wear.json onto the inherited finishes: no collision, no owner, no lettering.</t>
+          <t>Partial: a darkened grout-and-water ring round the shower receptor's lip and the mop-shadow corner farthest from the door, both soft projected wear (F03_D_BATH_OV; a frame difference against slice 47's view isolates the ring at the receptor's base). Paint lifted below the register is not made: the bath's vent register hangs from its duct at 2.6 m with no wall below it (F03_D_BATH_DT1). The water line under the curtain hem follows in slice 61. Verified at WIP 3f3f0d75 (implementation/slice52): apartment batch 204 on the long runner; household state 154 checks, 0 failures; upper kitchens 206 and upper furniture 488, both unchanged; upper lighting 9,257 checks and public doors 17, both 0 failures; the first bath sweep (six baths) 0 failures; the remaining twelve baths, the thirteen upper halls and slice 50's third core group were rerun at the same WIP in five sweeps, all 0 failures (implementation/slice52b); four earlier sweep runs that ran at another WIP are superseded and not cited. The decals are projected (Godot Decal nodes) from game/data/orison_v2/positional_wear.json onto the inherited finishes: no collision, no owner, no lettering. Slice 61 adds the water line on the floor under the curtain hem, a ragged damp band with a darker drying edge, mounted with the world at 2c25e683 (implementation/slice67); a frame difference against slice 52's view picks it out along the hem, faint at production light.</t>
         </is>
       </c>
     </row>
@@ -27020,7 +27020,7 @@
       </c>
       <c r="T363" s="2" t="inlineStr">
         <is>
-          <t>Partial: a darkened grout-and-water ring round the shower receptor's lip and the mop-shadow corner farthest from the door, both soft projected wear (F04_A_BATH_OV; a frame difference against slice 47's view isolates the ring at the receptor's base). Paint lifted below the register is not made: the bath's vent register hangs from its duct at 2.6 m with no wall below it (F04_A_BATH_DT1). The water line under the curtain hem follows in slice 61. Verified at WIP 3f3f0d75 (implementation/slice52): apartment batch 204 on the long runner; household state 154 checks, 0 failures; upper kitchens 206 and upper furniture 488, both unchanged; upper lighting 9,257 checks and public doors 17, both 0 failures; the first bath sweep (six baths) 0 failures; the remaining twelve baths, the thirteen upper halls and slice 50's third core group were rerun at the same WIP in five sweeps, all 0 failures (implementation/slice52b); four earlier sweep runs that ran at another WIP are superseded and not cited. The decals are projected (Godot Decal nodes) from game/data/orison_v2/positional_wear.json onto the inherited finishes: no collision, no owner, no lettering.</t>
+          <t>Partial: a darkened grout-and-water ring round the shower receptor's lip and the mop-shadow corner farthest from the door, both soft projected wear (F04_A_BATH_OV; a frame difference against slice 47's view isolates the ring at the receptor's base). Paint lifted below the register is not made: the bath's vent register hangs from its duct at 2.6 m with no wall below it (F04_A_BATH_DT1). The water line under the curtain hem follows in slice 61. Verified at WIP 3f3f0d75 (implementation/slice52): apartment batch 204 on the long runner; household state 154 checks, 0 failures; upper kitchens 206 and upper furniture 488, both unchanged; upper lighting 9,257 checks and public doors 17, both 0 failures; the first bath sweep (six baths) 0 failures; the remaining twelve baths, the thirteen upper halls and slice 50's third core group were rerun at the same WIP in five sweeps, all 0 failures (implementation/slice52b); four earlier sweep runs that ran at another WIP are superseded and not cited. The decals are projected (Godot Decal nodes) from game/data/orison_v2/positional_wear.json onto the inherited finishes: no collision, no owner, no lettering. Slice 61 adds the water line on the floor under the curtain hem, a ragged damp band with a darker drying edge, mounted with the world at 2c25e683 (implementation/slice67); a frame difference against slice 52's view picks it out along the hem, faint at production light.</t>
         </is>
       </c>
     </row>
@@ -28372,7 +28372,7 @@
       </c>
       <c r="T381" s="2" t="inlineStr">
         <is>
-          <t>Partial: a darkened grout-and-water ring round the shower receptor's lip and the mop-shadow corner farthest from the door, both soft projected wear (F04_B_BATH_OV; a frame difference against slice 47's view isolates the ring at the receptor's base). Paint lifted below the register is not made: the bath's vent register hangs from its duct at 2.6 m with no wall below it (F04_B_BATH_DT1). The water line under the curtain hem follows in slice 61. Verified at WIP 3f3f0d75 (implementation/slice52): apartment batch 204 on the long runner; household state 154 checks, 0 failures; upper kitchens 206 and upper furniture 488, both unchanged; upper lighting 9,257 checks and public doors 17, both 0 failures; the first bath sweep (six baths) 0 failures; the remaining twelve baths, the thirteen upper halls and slice 50's third core group were rerun at the same WIP in five sweeps, all 0 failures (implementation/slice52b); four earlier sweep runs that ran at another WIP are superseded and not cited. The decals are projected (Godot Decal nodes) from game/data/orison_v2/positional_wear.json onto the inherited finishes: no collision, no owner, no lettering.</t>
+          <t>Partial: a darkened grout-and-water ring round the shower receptor's lip and the mop-shadow corner farthest from the door, both soft projected wear (F04_B_BATH_OV; a frame difference against slice 47's view isolates the ring at the receptor's base). Paint lifted below the register is not made: the bath's vent register hangs from its duct at 2.6 m with no wall below it (F04_B_BATH_DT1). The water line under the curtain hem follows in slice 61. Verified at WIP 3f3f0d75 (implementation/slice52): apartment batch 204 on the long runner; household state 154 checks, 0 failures; upper kitchens 206 and upper furniture 488, both unchanged; upper lighting 9,257 checks and public doors 17, both 0 failures; the first bath sweep (six baths) 0 failures; the remaining twelve baths, the thirteen upper halls and slice 50's third core group were rerun at the same WIP in five sweeps, all 0 failures (implementation/slice52b); four earlier sweep runs that ran at another WIP are superseded and not cited. The decals are projected (Godot Decal nodes) from game/data/orison_v2/positional_wear.json onto the inherited finishes: no collision, no owner, no lettering. Slice 61 adds the water line on the floor under the curtain hem, a ragged damp band with a darker drying edge, mounted with the world at 2c25e683 (implementation/slice67); a frame difference against slice 52's view picks it out along the hem, faint at production light.</t>
         </is>
       </c>
     </row>
@@ -29926,7 +29926,7 @@
       </c>
       <c r="T402" s="2" t="inlineStr">
         <is>
-          <t>Partial: a darkened grout-and-water ring round the shower receptor's lip and the mop-shadow corner farthest from the door, both soft projected wear (F04_C_BATH_OV; a frame difference against slice 47's view isolates the ring at the receptor's base). Paint lifted below the register is not made: the bath's vent register hangs from its duct at 2.6 m with no wall below it (F04_C_BATH_DT1). The water line under the curtain hem follows in slice 61. Verified at WIP 3f3f0d75 (implementation/slice52): apartment batch 204 on the long runner; household state 154 checks, 0 failures; upper kitchens 206 and upper furniture 488, both unchanged; upper lighting 9,257 checks and public doors 17, both 0 failures; the first bath sweep (six baths) 0 failures; the remaining twelve baths, the thirteen upper halls and slice 50's third core group were rerun at the same WIP in five sweeps, all 0 failures (implementation/slice52b); four earlier sweep runs that ran at another WIP are superseded and not cited. The decals are projected (Godot Decal nodes) from game/data/orison_v2/positional_wear.json onto the inherited finishes: no collision, no owner, no lettering.</t>
+          <t>Partial: a darkened grout-and-water ring round the shower receptor's lip and the mop-shadow corner farthest from the door, both soft projected wear (F04_C_BATH_OV; a frame difference against slice 47's view isolates the ring at the receptor's base). Paint lifted below the register is not made: the bath's vent register hangs from its duct at 2.6 m with no wall below it (F04_C_BATH_DT1). The water line under the curtain hem follows in slice 61. Verified at WIP 3f3f0d75 (implementation/slice52): apartment batch 204 on the long runner; household state 154 checks, 0 failures; upper kitchens 206 and upper furniture 488, both unchanged; upper lighting 9,257 checks and public doors 17, both 0 failures; the first bath sweep (six baths) 0 failures; the remaining twelve baths, the thirteen upper halls and slice 50's third core group were rerun at the same WIP in five sweeps, all 0 failures (implementation/slice52b); four earlier sweep runs that ran at another WIP are superseded and not cited. The decals are projected (Godot Decal nodes) from game/data/orison_v2/positional_wear.json onto the inherited finishes: no collision, no owner, no lettering. Slice 61 adds the water line on the floor under the curtain hem, a ragged damp band with a darker drying edge, mounted with the world at 2c25e683 (implementation/slice67); a frame difference against slice 52's view picks it out along the hem, faint at production light.</t>
         </is>
       </c>
     </row>
@@ -31176,7 +31176,7 @@
       </c>
       <c r="T419" s="2" t="inlineStr">
         <is>
-          <t>Partial: a darkened grout-and-water ring round the shower receptor's lip and the mop-shadow corner farthest from the door, both soft projected wear (F04_D_BATH_OV; a frame difference against slice 47's view isolates the ring at the receptor's base). Paint lifted below the register is not made: the bath's vent register hangs from its duct at 2.6 m with no wall below it (F04_D_BATH_DT1). The water line under the curtain hem follows in slice 61. Verified at WIP 3f3f0d75 (implementation/slice52): apartment batch 204 on the long runner; household state 154 checks, 0 failures; upper kitchens 206 and upper furniture 488, both unchanged; upper lighting 9,257 checks and public doors 17, both 0 failures; the first bath sweep (six baths) 0 failures; the remaining twelve baths, the thirteen upper halls and slice 50's third core group were rerun at the same WIP in five sweeps, all 0 failures (implementation/slice52b); four earlier sweep runs that ran at another WIP are superseded and not cited. The decals are projected (Godot Decal nodes) from game/data/orison_v2/positional_wear.json onto the inherited finishes: no collision, no owner, no lettering.</t>
+          <t>Partial: a darkened grout-and-water ring round the shower receptor's lip and the mop-shadow corner farthest from the door, both soft projected wear (F04_D_BATH_OV; a frame difference against slice 47's view isolates the ring at the receptor's base). Paint lifted below the register is not made: the bath's vent register hangs from its duct at 2.6 m with no wall below it (F04_D_BATH_DT1). The water line under the curtain hem follows in slice 61. Verified at WIP 3f3f0d75 (implementation/slice52): apartment batch 204 on the long runner; household state 154 checks, 0 failures; upper kitchens 206 and upper furniture 488, both unchanged; upper lighting 9,257 checks and public doors 17, both 0 failures; the first bath sweep (six baths) 0 failures; the remaining twelve baths, the thirteen upper halls and slice 50's third core group were rerun at the same WIP in five sweeps, all 0 failures (implementation/slice52b); four earlier sweep runs that ran at another WIP are superseded and not cited. The decals are projected (Godot Decal nodes) from game/data/orison_v2/positional_wear.json onto the inherited finishes: no collision, no owner, no lettering. Slice 61 adds the water line on the floor under the curtain hem, a ragged damp band with a darker drying edge, mounted with the world at 2c25e683 (implementation/slice67); a frame difference against slice 52's view picks it out along the hem, faint at production light.</t>
         </is>
       </c>
     </row>
@@ -33766,7 +33766,7 @@
       </c>
       <c r="T454" s="2" t="inlineStr">
         <is>
-          <t>Partial: a darkened grout-and-water ring round the shower receptor's lip and the mop-shadow corner farthest from the door, both soft projected wear (F05_A_BATH_OV; a frame difference against slice 47's view isolates the ring at the receptor's base). Paint lifted below the register is not made: the bath's vent register hangs from its duct at 2.6 m with no wall below it (F05_A_BATH_DT1). The water line under the curtain hem follows in slice 61. Verified at WIP 3f3f0d75 (implementation/slice52): apartment batch 204 on the long runner; household state 154 checks, 0 failures; upper kitchens 206 and upper furniture 488, both unchanged; upper lighting 9,257 checks and public doors 17, both 0 failures; the first bath sweep (six baths) 0 failures; the remaining twelve baths, the thirteen upper halls and slice 50's third core group were rerun at the same WIP in five sweeps, all 0 failures (implementation/slice52b); four earlier sweep runs that ran at another WIP are superseded and not cited. The decals are projected (Godot Decal nodes) from game/data/orison_v2/positional_wear.json onto the inherited finishes: no collision, no owner, no lettering.</t>
+          <t>Partial: a darkened grout-and-water ring round the shower receptor's lip and the mop-shadow corner farthest from the door, both soft projected wear (F05_A_BATH_OV; a frame difference against slice 47's view isolates the ring at the receptor's base). Paint lifted below the register is not made: the bath's vent register hangs from its duct at 2.6 m with no wall below it (F05_A_BATH_DT1). The water line under the curtain hem follows in slice 61. Verified at WIP 3f3f0d75 (implementation/slice52): apartment batch 204 on the long runner; household state 154 checks, 0 failures; upper kitchens 206 and upper furniture 488, both unchanged; upper lighting 9,257 checks and public doors 17, both 0 failures; the first bath sweep (six baths) 0 failures; the remaining twelve baths, the thirteen upper halls and slice 50's third core group were rerun at the same WIP in five sweeps, all 0 failures (implementation/slice52b); four earlier sweep runs that ran at another WIP are superseded and not cited. The decals are projected (Godot Decal nodes) from game/data/orison_v2/positional_wear.json onto the inherited finishes: no collision, no owner, no lettering. Slice 61 adds the water line on the floor under the curtain hem, a ragged damp band with a darker drying edge, mounted with the world at 2c25e683 (implementation/slice67); a frame difference against slice 52's view picks it out along the hem, faint at production light.</t>
         </is>
       </c>
     </row>
@@ -35304,7 +35304,7 @@
       </c>
       <c r="T475" s="2" t="inlineStr">
         <is>
-          <t>Partial: a darkened grout-and-water ring round the shower receptor's lip and the mop-shadow corner farthest from the door, both soft projected wear (F05_B_BATH_OV; a frame difference against slice 47's view isolates the ring at the receptor's base). Paint lifted below the register is not made: the bath's vent register hangs from its duct at 2.6 m with no wall below it (F05_B_BATH_DT1). The water line under the curtain hem follows in slice 61. Verified at WIP 3f3f0d75 (implementation/slice52): apartment batch 204 on the long runner; household state 154 checks, 0 failures; upper kitchens 206 and upper furniture 488, both unchanged; upper lighting 9,257 checks and public doors 17, both 0 failures; the first bath sweep (six baths) 0 failures; the remaining twelve baths, the thirteen upper halls and slice 50's third core group were rerun at the same WIP in five sweeps, all 0 failures (implementation/slice52b); four earlier sweep runs that ran at another WIP are superseded and not cited. The decals are projected (Godot Decal nodes) from game/data/orison_v2/positional_wear.json onto the inherited finishes: no collision, no owner, no lettering.</t>
+          <t>Partial: a darkened grout-and-water ring round the shower receptor's lip and the mop-shadow corner farthest from the door, both soft projected wear (F05_B_BATH_OV; a frame difference against slice 47's view isolates the ring at the receptor's base). Paint lifted below the register is not made: the bath's vent register hangs from its duct at 2.6 m with no wall below it (F05_B_BATH_DT1). The water line under the curtain hem follows in slice 61. Verified at WIP 3f3f0d75 (implementation/slice52): apartment batch 204 on the long runner; household state 154 checks, 0 failures; upper kitchens 206 and upper furniture 488, both unchanged; upper lighting 9,257 checks and public doors 17, both 0 failures; the first bath sweep (six baths) 0 failures; the remaining twelve baths, the thirteen upper halls and slice 50's third core group were rerun at the same WIP in five sweeps, all 0 failures (implementation/slice52b); four earlier sweep runs that ran at another WIP are superseded and not cited. The decals are projected (Godot Decal nodes) from game/data/orison_v2/positional_wear.json onto the inherited finishes: no collision, no owner, no lettering. Slice 61 adds the water line on the floor under the curtain hem, a ragged damp band with a darker drying edge, mounted with the world at 2c25e683 (implementation/slice67); a frame difference against slice 52's view picks it out along the hem, faint at production light.</t>
         </is>
       </c>
     </row>
@@ -36496,7 +36496,7 @@
       </c>
       <c r="T491" s="2" t="inlineStr">
         <is>
-          <t>Partial: a darkened grout-and-water ring round the shower receptor's lip and the mop-shadow corner farthest from the door, both soft projected wear (F05_C_BATH_OV; a frame difference against slice 47's view isolates the ring at the receptor's base). Paint lifted below the register is not made: the bath's vent register hangs from its duct at 2.6 m with no wall below it (F05_C_BATH_DT1). The water line under the curtain hem follows in slice 61. Verified at WIP 3f3f0d75 (implementation/slice52): apartment batch 204 on the long runner; household state 154 checks, 0 failures; upper kitchens 206 and upper furniture 488, both unchanged; upper lighting 9,257 checks and public doors 17, both 0 failures; the first bath sweep (six baths) 0 failures; the remaining twelve baths, the thirteen upper halls and slice 50's third core group were rerun at the same WIP in five sweeps, all 0 failures (implementation/slice52b); four earlier sweep runs that ran at another WIP are superseded and not cited. The decals are projected (Godot Decal nodes) from game/data/orison_v2/positional_wear.json onto the inherited finishes: no collision, no owner, no lettering.</t>
+          <t>Partial: a darkened grout-and-water ring round the shower receptor's lip and the mop-shadow corner farthest from the door, both soft projected wear (F05_C_BATH_OV; a frame difference against slice 47's view isolates the ring at the receptor's base). Paint lifted below the register is not made: the bath's vent register hangs from its duct at 2.6 m with no wall below it (F05_C_BATH_DT1). The water line under the curtain hem follows in slice 61. Verified at WIP 3f3f0d75 (implementation/slice52): apartment batch 204 on the long runner; household state 154 checks, 0 failures; upper kitchens 206 and upper furniture 488, both unchanged; upper lighting 9,257 checks and public doors 17, both 0 failures; the first bath sweep (six baths) 0 failures; the remaining twelve baths, the thirteen upper halls and slice 50's third core group were rerun at the same WIP in five sweeps, all 0 failures (implementation/slice52b); four earlier sweep runs that ran at another WIP are superseded and not cited. The decals are projected (Godot Decal nodes) from game/data/orison_v2/positional_wear.json onto the inherited finishes: no collision, no owner, no lettering. Slice 61 adds the water line on the floor under the curtain hem, a ragged damp band with a darker drying edge, mounted with the world at 2c25e683 (implementation/slice67); a frame difference against slice 52's view picks it out along the hem, faint at production light.</t>
         </is>
       </c>
     </row>
@@ -37002,7 +37002,7 @@
       </c>
       <c r="T498" s="2" t="inlineStr">
         <is>
-          <t>Partial: the soot ghost, stepped bands of soot 0.8 m wide at the top, up the plaster above the replaced door's head on the crossing side, and the same one-line notice beside it (5D_soot_fan_native, F05_SERVICE_CROSSING_TH). The replacement leaf's fresher paint and the scorch at the frame head are not made: the fitted door family has no replacement finish. Verified at WIP 0bac8f87 (implementation/slice51): apartment batch 204 on the long runner; household state 154 checks, 0 failures; upper kitchens 206 and upper furniture 488, both unchanged; upper lighting 9,257 checks, public doors 17, the remaining upper transfers 28 and the apartment door route 45, all 0 failures; the resident key route (86 waypoints, long runner) and the four-space sweep (F03 public core, F05 service crossing, F05 west and east halls) ran at slice 52's WIP 3f3f0d75, which carries this slice unchanged, and both report 0 failures. The fabrication batch captured the 3C threshold and the 5D soot fan natively; its one failure is the capture harness finding no clear standing camera station for the aerial wire in the 1.06 m hall, so the hall sweep's views carry that evidence.</t>
+          <t>Partial: the soot ghost, stepped bands of soot 0.8 m wide at the top, up the plaster above the replaced door's head on the crossing side, and the same one-line notice beside it (5D_soot_fan_native, F05_SERVICE_CROSSING_TH). The replacement leaf's fresher paint and the scorch at the frame head are not made: the fitted door family has no replacement finish. Verified at WIP 0bac8f87 (implementation/slice51): apartment batch 204 on the long runner; household state 154 checks, 0 failures; upper kitchens 206 and upper furniture 488, both unchanged; upper lighting 9,257 checks, public doors 17, the remaining upper transfers 28 and the apartment door route 45, all 0 failures; the resident key route (86 waypoints, long runner) and the four-space sweep (F03 public core, F05 service crossing, F05 west and east halls) ran at slice 52's WIP 3f3f0d75, which carries this slice unchanged, and both report 0 failures. The fabrication batch captured the 3C threshold and the 5D soot fan natively; its one failure is the capture harness finding no clear standing camera station for the aerial wire in the 1.06 m hall, so the hall sweep's views carry that evidence. Slice 61 replaces the stepped soot bands with a soft projected fan licking up from the door head (verified at 2c25e683, implementation/slice67).</t>
         </is>
       </c>
     </row>
@@ -38920,7 +38920,7 @@
       </c>
       <c r="T523" s="2" t="inlineStr">
         <is>
-          <t>Partial: a darkened grout-and-water ring round the shower receptor's lip and the mop-shadow corner farthest from the door, both soft projected wear (F06_A_BATH_OV; a frame difference against slice 47's view isolates the ring at the receptor's base). Paint lifted below the register is not made: the bath's vent register hangs from its duct at 2.6 m with no wall below it (F06_A_BATH_DT1). The water line under the curtain hem follows in slice 61. Verified at WIP 3f3f0d75 (implementation/slice52): apartment batch 204 on the long runner; household state 154 checks, 0 failures; upper kitchens 206 and upper furniture 488, both unchanged; upper lighting 9,257 checks and public doors 17, both 0 failures; the first bath sweep (six baths) 0 failures; the remaining twelve baths, the thirteen upper halls and slice 50's third core group were rerun at the same WIP in five sweeps, all 0 failures (implementation/slice52b); four earlier sweep runs that ran at another WIP are superseded and not cited. The decals are projected (Godot Decal nodes) from game/data/orison_v2/positional_wear.json onto the inherited finishes: no collision, no owner, no lettering.</t>
+          <t>Partial: a darkened grout-and-water ring round the shower receptor's lip and the mop-shadow corner farthest from the door, both soft projected wear (F06_A_BATH_OV; a frame difference against slice 47's view isolates the ring at the receptor's base). Paint lifted below the register is not made: the bath's vent register hangs from its duct at 2.6 m with no wall below it (F06_A_BATH_DT1). The water line under the curtain hem follows in slice 61. Verified at WIP 3f3f0d75 (implementation/slice52): apartment batch 204 on the long runner; household state 154 checks, 0 failures; upper kitchens 206 and upper furniture 488, both unchanged; upper lighting 9,257 checks and public doors 17, both 0 failures; the first bath sweep (six baths) 0 failures; the remaining twelve baths, the thirteen upper halls and slice 50's third core group were rerun at the same WIP in five sweeps, all 0 failures (implementation/slice52b); four earlier sweep runs that ran at another WIP are superseded and not cited. The decals are projected (Godot Decal nodes) from game/data/orison_v2/positional_wear.json onto the inherited finishes: no collision, no owner, no lettering. Slice 61 adds the water line on the floor under the curtain hem, a ragged damp band with a darker drying edge, mounted with the world at 2c25e683 (implementation/slice67); a frame difference against slice 52's view picks it out along the hem, faint at production light.</t>
         </is>
       </c>
     </row>
@@ -40174,7 +40174,7 @@
       </c>
       <c r="T540" s="2" t="inlineStr">
         <is>
-          <t>Partial: a darkened grout-and-water ring round the shower receptor's lip and the mop-shadow corner farthest from the door, both soft projected wear (F06_B_BATH_OV; a frame difference against slice 47's view isolates the ring at the receptor's base). Paint lifted below the register is not made: the bath's vent register hangs from its duct at 2.6 m with no wall below it (F06_B_BATH_DT1). The water line under the curtain hem follows in slice 61. Verified at WIP 3f3f0d75 (implementation/slice52): apartment batch 204 on the long runner; household state 154 checks, 0 failures; upper kitchens 206 and upper furniture 488, both unchanged; upper lighting 9,257 checks and public doors 17, both 0 failures; the first bath sweep (six baths) 0 failures; the remaining twelve baths, the thirteen upper halls and slice 50's third core group were rerun at the same WIP in five sweeps, all 0 failures (implementation/slice52b); four earlier sweep runs that ran at another WIP are superseded and not cited. The decals are projected (Godot Decal nodes) from game/data/orison_v2/positional_wear.json onto the inherited finishes: no collision, no owner, no lettering.</t>
+          <t>Partial: a darkened grout-and-water ring round the shower receptor's lip and the mop-shadow corner farthest from the door, both soft projected wear (F06_B_BATH_OV; a frame difference against slice 47's view isolates the ring at the receptor's base). Paint lifted below the register is not made: the bath's vent register hangs from its duct at 2.6 m with no wall below it (F06_B_BATH_DT1). The water line under the curtain hem follows in slice 61. Verified at WIP 3f3f0d75 (implementation/slice52): apartment batch 204 on the long runner; household state 154 checks, 0 failures; upper kitchens 206 and upper furniture 488, both unchanged; upper lighting 9,257 checks and public doors 17, both 0 failures; the first bath sweep (six baths) 0 failures; the remaining twelve baths, the thirteen upper halls and slice 50's third core group were rerun at the same WIP in five sweeps, all 0 failures (implementation/slice52b); four earlier sweep runs that ran at another WIP are superseded and not cited. The decals are projected (Godot Decal nodes) from game/data/orison_v2/positional_wear.json onto the inherited finishes: no collision, no owner, no lettering. Slice 61 adds the water line on the floor under the curtain hem, a ragged damp band with a darker drying edge, mounted with the world at 2c25e683 (implementation/slice67); a frame difference against slice 52's view picks it out along the hem, faint at production light.</t>
         </is>
       </c>
     </row>
@@ -41276,7 +41276,7 @@
       </c>
       <c r="T555" s="2" t="inlineStr">
         <is>
-          <t>Partial: a darkened grout-and-water ring round the shower receptor's lip and the mop-shadow corner farthest from the door, both soft projected wear (F06_C_BATH_OV; a frame difference against slice 47's view isolates the ring at the receptor's base). Paint lifted below the register is not made: the bath's vent register hangs from its duct at 2.6 m with no wall below it (F06_C_BATH_DT1). The water line under the curtain hem follows in slice 61. Verified at WIP 3f3f0d75 (implementation/slice52): apartment batch 204 on the long runner; household state 154 checks, 0 failures; upper kitchens 206 and upper furniture 488, both unchanged; upper lighting 9,257 checks and public doors 17, both 0 failures; the first bath sweep (six baths) 0 failures; the remaining twelve baths, the thirteen upper halls and slice 50's third core group were rerun at the same WIP in five sweeps, all 0 failures (implementation/slice52b); four earlier sweep runs that ran at another WIP are superseded and not cited. The decals are projected (Godot Decal nodes) from game/data/orison_v2/positional_wear.json onto the inherited finishes: no collision, no owner, no lettering.</t>
+          <t>Partial: a darkened grout-and-water ring round the shower receptor's lip and the mop-shadow corner farthest from the door, both soft projected wear (F06_C_BATH_OV; a frame difference against slice 47's view isolates the ring at the receptor's base). Paint lifted below the register is not made: the bath's vent register hangs from its duct at 2.6 m with no wall below it (F06_C_BATH_DT1). The water line under the curtain hem follows in slice 61. Verified at WIP 3f3f0d75 (implementation/slice52): apartment batch 204 on the long runner; household state 154 checks, 0 failures; upper kitchens 206 and upper furniture 488, both unchanged; upper lighting 9,257 checks and public doors 17, both 0 failures; the first bath sweep (six baths) 0 failures; the remaining twelve baths, the thirteen upper halls and slice 50's third core group were rerun at the same WIP in five sweeps, all 0 failures (implementation/slice52b); four earlier sweep runs that ran at another WIP are superseded and not cited. The decals are projected (Godot Decal nodes) from game/data/orison_v2/positional_wear.json onto the inherited finishes: no collision, no owner, no lettering. Slice 61 adds the water line on the floor under the curtain hem, a ragged damp band with a darker drying edge, mounted with the world at 2c25e683 (implementation/slice67); a frame difference against slice 52's view picks it out along the hem, faint at production light.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Implement dossier slice 62: the pawnbroker's ring in an envelope, the safe's blank name panel
- CITY_SHOP_PAWNBROKER-002: a wedding ring half out of a small envelope on the
  window deck.
- CITY_SHOP_PAWNBROKER-003 (partial): the safe's blank enamelled name panel in a
  gold line; the cage bulbs remain the cell's globes.
- CITY_SHOP_PAWNBROKER-001: the balance, loupe and ledger of the pawn fittings
  family, captured at slice 67.

Evidence under implementation/slice67/. INERT: no ledger status changes.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/art/reviews/v2_environment_design_20261008/change_register.xlsx
+++ b/art/reviews/v2_environment_design_20261008/change_register.xlsx
@@ -6959,10 +6959,14 @@
       </c>
       <c r="S97" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T97" s="2" t="inlineStr"/>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="T97" s="2" t="inlineStr">
+        <is>
+          <t>The jeweller's beam balance in its glazed case, the loupe on a cord and the pledge ledger on the counter, from the pawn fittings family (balance, ledger_loupe). Verified at slice 67's WIP 2c25e683 (implementation/slice67), which carries slices 58 to 66 with slice 67's fixes: from slice 58 the world refused to compose (slice 58's light box reused an id slice 38's surface stock owned) until slice 67 renamed it. At 2c25e683 the fabrication batch's ten families (12,295 checks) report one failure, the capture harness finding no clear camera station for the B1 cleat run; apartment batch 204 on the long runner, as before; household state 154 checks, 0 failures; upper kitchens 206 and upper furniture 488, both unchanged; upper lighting 9,257 checks and public doors 17, 0 failures; the remaining transfers, apartment door, first upper hall, 4B door and rear wing A routes, the basement route (88), basement ground, boiler service, reading furniture, shop seating, funeral fittings, completion heating, radiator ties, ventilation, door casings (107 openings), hardware drawers (1,309 checks), street boundary, passage visibility, commensal, the street boundary route and the resident key route (86 waypoints, long runner), all 0 failures; twelve sweeps (55 spaces) and the city sweep's 130 views, 0 failures. The coal delivery route's stop at the lobby's inner door and the Vantry gateway suite's five kiosk-count failures are identical at slice 57's 260849e8 (base58), and the news receiving station failure is identical before slice 53.</t>
+        </is>
+      </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
@@ -7017,10 +7021,14 @@
       </c>
       <c r="S98" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T98" s="2" t="inlineStr"/>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="T98" s="2" t="inlineStr">
+        <is>
+          <t>A wedding ring half out of a small envelope on the window deck between the watch tray and the field glasses (window_watch). Verified at slice 67's WIP 2c25e683 (implementation/slice67), which carries slices 58 to 66 with slice 67's fixes: from slice 58 the world refused to compose (slice 58's light box reused an id slice 38's surface stock owned) until slice 67 renamed it. At 2c25e683 the fabrication batch's ten families (12,295 checks) report one failure, the capture harness finding no clear camera station for the B1 cleat run; apartment batch 204 on the long runner, as before; household state 154 checks, 0 failures; upper kitchens 206 and upper furniture 488, both unchanged; upper lighting 9,257 checks and public doors 17, 0 failures; the remaining transfers, apartment door, first upper hall, 4B door and rear wing A routes, the basement route (88), basement ground, boiler service, reading furniture, shop seating, funeral fittings, completion heating, radiator ties, ventilation, door casings (107 openings), hardware drawers (1,309 checks), street boundary, passage visibility, commensal, the street boundary route and the resident key route (86 waypoints, long runner), all 0 failures; twelve sweeps (55 spaces) and the city sweep's 130 views, 0 failures. The coal delivery route's stop at the lobby's inner door and the Vantry gateway suite's five kiosk-count failures are identical at slice 57's 260849e8 (base58), and the news receiving station failure is identical before slice 53.</t>
+        </is>
+      </c>
     </row>
     <row r="99">
       <c r="A99" s="2" t="inlineStr">
@@ -7083,10 +7091,14 @@
       </c>
       <c r="S99" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T99" s="2" t="inlineStr"/>
+          <t>implemented</t>
+        </is>
+      </c>
+      <c r="T99" s="2" t="inlineStr">
+        <is>
+          <t>Partial: the safe's painted name panel above its dial, blank, an enamelled field inside a gold line. The two bulbs in the counter cage remain the cell's sphere globes. Verified at slice 67's WIP 2c25e683 (implementation/slice67), which carries slices 58 to 66 with slice 67's fixes: from slice 58 the world refused to compose (slice 58's light box reused an id slice 38's surface stock owned) until slice 67 renamed it. At 2c25e683 the fabrication batch's ten families (12,295 checks) report one failure, the capture harness finding no clear camera station for the B1 cleat run; apartment batch 204 on the long runner, as before; household state 154 checks, 0 failures; upper kitchens 206 and upper furniture 488, both unchanged; upper lighting 9,257 checks and public doors 17, 0 failures; the remaining transfers, apartment door, first upper hall, 4B door and rear wing A routes, the basement route (88), basement ground, boiler service, reading furniture, shop seating, funeral fittings, completion heating, radiator ties, ventilation, door casings (107 openings), hardware drawers (1,309 checks), street boundary, passage visibility, commensal, the street boundary route and the resident key route (86 waypoints, long runner), all 0 failures; twelve sweeps (55 spaces) and the city sweep's 130 views, 0 failures. The coal delivery route's stop at the lobby's inner door and the Vantry gateway suite's five kiosk-count failures are identical at slice 57's 260849e8 (base58), and the news receiving station failure is identical before slice 53.</t>
+        </is>
+      </c>
     </row>
     <row r="100">
       <c r="A100" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Implement dossier slice 63: the reading room's bookcases in varied runs and bound magazines
- F01_COMMON_B-002 (implemented): both bookcases hold their books in runs of varied length
  with gaps, short piles lying flat, and a top shelf of bound magazine volumes
  banded where the years would be lettered.

Evidence under implementation/slice67/. INERT: no ledger status changes.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/art/reviews/v2_environment_design_20261008/change_register.xlsx
+++ b/art/reviews/v2_environment_design_20261008/change_register.xlsx
@@ -9561,10 +9561,14 @@
       </c>
       <c r="S136" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T136" s="2" t="inlineStr"/>
+          <t>implemented</t>
+        </is>
+      </c>
+      <c r="T136" s="2" t="inlineStr">
+        <is>
+          <t>Both reading-room bookcases hold their books in runs of varied length with gaps between, short piles lying flat, and a top shelf of bound magazine volumes in one cloth with blank bands where the years would be lettered (build_reading_furniture.py; reading furniture 25 waypoints, 0 failures). The sweep shows the two cases only small and dark at the room's far end (F01_COMMON_B_RV); a framed capture is open. Verified at slice 67's WIP 2c25e683 (implementation/slice67), which carries slices 58 to 66 with slice 67's fixes: from slice 58 the world refused to compose (slice 58's light box reused an id slice 38's surface stock owned) until slice 67 renamed it. At 2c25e683 the fabrication batch's ten families (12,295 checks) report one failure, the capture harness finding no clear camera station for the B1 cleat run; apartment batch 204 on the long runner, as before; household state 154 checks, 0 failures; upper kitchens 206 and upper furniture 488, both unchanged; upper lighting 9,257 checks and public doors 17, 0 failures; the remaining transfers, apartment door, first upper hall, 4B door and rear wing A routes, the basement route (88), basement ground, boiler service, reading furniture, shop seating, funeral fittings, completion heating, radiator ties, ventilation, door casings (107 openings), hardware drawers (1,309 checks), street boundary, passage visibility, commensal, the street boundary route and the resident key route (86 waypoints, long runner), all 0 failures; twelve sweeps (55 spaces) and the city sweep's 130 views, 0 failures. The coal delivery route's stop at the lobby's inner door and the Vantry gateway suite's five kiosk-count failures are identical at slice 57's 260849e8 (base58), and the news receiving station failure is identical before slice 53.</t>
+        </is>
+      </c>
     </row>
     <row r="137">
       <c r="A137" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Implement dossier slice 64: the funeral register open, chairs off their marks, the worn third stool
- CITY_SHOP_FUNERAL_PARLOUR-002, -004: the register open at the day's page with
  one signature; two chairs a few degrees off and one pulled back.
- CITY_SHOP_LUNCHEONETTE-002: the third stool's vinyl worn through to the cord.
- Shop seating gains registered catalogue finishes.

Evidence under implementation/slice67/. INERT: no ledger status changes.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/art/reviews/v2_environment_design_20261008/change_register.xlsx
+++ b/art/reviews/v2_environment_design_20261008/change_register.xlsx
@@ -6257,10 +6257,14 @@
       </c>
       <c r="S86" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T86" s="2" t="inlineStr"/>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="T86" s="2" t="inlineStr">
+        <is>
+          <t>The register lies open on the lectern at the day's page: blank rules and one signature stroke (book). Verified at slice 67's WIP 2c25e683 (implementation/slice67), which carries slices 58 to 66 with slice 67's fixes: from slice 58 the world refused to compose (slice 58's light box reused an id slice 38's surface stock owned) until slice 67 renamed it. At 2c25e683 the fabrication batch's ten families (12,295 checks) report one failure, the capture harness finding no clear camera station for the B1 cleat run; apartment batch 204 on the long runner, as before; household state 154 checks, 0 failures; upper kitchens 206 and upper furniture 488, both unchanged; upper lighting 9,257 checks and public doors 17, 0 failures; the remaining transfers, apartment door, first upper hall, 4B door and rear wing A routes, the basement route (88), basement ground, boiler service, reading furniture, shop seating, funeral fittings, completion heating, radiator ties, ventilation, door casings (107 openings), hardware drawers (1,309 checks), street boundary, passage visibility, commensal, the street boundary route and the resident key route (86 waypoints, long runner), all 0 failures; twelve sweeps (55 spaces) and the city sweep's 130 views, 0 failures. The coal delivery route's stop at the lobby's inner door and the Vantry gateway suite's five kiosk-count failures are identical at slice 57's 260849e8 (base58), and the news receiving station failure is identical before slice 53.</t>
+        </is>
+      </c>
     </row>
     <row r="87">
       <c r="A87" s="2" t="inlineStr">
@@ -6381,10 +6385,14 @@
       </c>
       <c r="S88" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T88" s="2" t="inlineStr"/>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="T88" s="2" t="inlineStr">
+        <is>
+          <t>The chair rows stay arranged but two chairs sit a few degrees off their marks and one is pulled back where someone stood; the alcove drapes were already pleated cloth (SITE_SHOP_IN0_FUNERAL_PARLOUR_fitted). Verified at slice 67's WIP 2c25e683 (implementation/slice67), which carries slices 58 to 66 with slice 67's fixes: from slice 58 the world refused to compose (slice 58's light box reused an id slice 38's surface stock owned) until slice 67 renamed it. At 2c25e683 the fabrication batch's ten families (12,295 checks) report one failure, the capture harness finding no clear camera station for the B1 cleat run; apartment batch 204 on the long runner, as before; household state 154 checks, 0 failures; upper kitchens 206 and upper furniture 488, both unchanged; upper lighting 9,257 checks and public doors 17, 0 failures; the remaining transfers, apartment door, first upper hall, 4B door and rear wing A routes, the basement route (88), basement ground, boiler service, reading furniture, shop seating, funeral fittings, completion heating, radiator ties, ventilation, door casings (107 openings), hardware drawers (1,309 checks), street boundary, passage visibility, commensal, the street boundary route and the resident key route (86 waypoints, long runner), all 0 failures; twelve sweeps (55 spaces) and the city sweep's 130 views, 0 failures. The coal delivery route's stop at the lobby's inner door and the Vantry gateway suite's five kiosk-count failures are identical at slice 57's 260849e8 (base58), and the news receiving station failure is identical before slice 53.</t>
+        </is>
+      </c>
     </row>
     <row r="89">
       <c r="A89" s="2" t="inlineStr">
@@ -6501,10 +6509,14 @@
       </c>
       <c r="S90" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T90" s="2" t="inlineStr"/>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="T90" s="2" t="inlineStr">
+        <is>
+          <t>The third stool's vinyl top is worn through to the cord (storm_shop_luncheonette_floor_0_fitted). Verified at slice 67's WIP 2c25e683 (implementation/slice67), which carries slices 58 to 66 with slice 67's fixes: from slice 58 the world refused to compose (slice 58's light box reused an id slice 38's surface stock owned) until slice 67 renamed it. At 2c25e683 the fabrication batch's ten families (12,295 checks) report one failure, the capture harness finding no clear camera station for the B1 cleat run; apartment batch 204 on the long runner, as before; household state 154 checks, 0 failures; upper kitchens 206 and upper furniture 488, both unchanged; upper lighting 9,257 checks and public doors 17, 0 failures; the remaining transfers, apartment door, first upper hall, 4B door and rear wing A routes, the basement route (88), basement ground, boiler service, reading furniture, shop seating, funeral fittings, completion heating, radiator ties, ventilation, door casings (107 openings), hardware drawers (1,309 checks), street boundary, passage visibility, commensal, the street boundary route and the resident key route (86 waypoints, long runner), all 0 failures; twelve sweeps (55 spaces) and the city sweep's 130 views, 0 failures. The coal delivery route's stop at the lobby's inner door and the Vantry gateway suite's five kiosk-count failures are identical at slice 57's 260849e8 (base58), and the news receiving station failure is identical before slice 53.</t>
+        </is>
+      </c>
     </row>
     <row r="91">
       <c r="A91" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Implement dossier slice 65: feathered pavement marks, election broadsides on the hoardings
- CITY_STREET-005 (partial): the pavement's ground marks feather out to their
  quad edges; not yet clipped to the slab joints.
- CITY_STREET-002 (implemented): broadsides, a portrait silhouette over a star in
  a printed border, on both street-end hoardings; no station frames them yet.

Evidence under implementation/slice67/. INERT: no ledger status changes.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/art/reviews/v2_environment_design_20261008/change_register.xlsx
+++ b/art/reviews/v2_environment_design_20261008/change_register.xlsx
@@ -3937,10 +3937,14 @@
       </c>
       <c r="S50" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T50" s="2" t="inlineStr"/>
+          <t>implemented</t>
+        </is>
+      </c>
+      <c r="T50" s="2" t="inlineStr">
+        <is>
+          <t>Election broadsides pasted on both street-end hoardings: a portrait silhouette over a star inside a printed border, no lettering. The hoardings stand at the street's far ends and no city station frames them; a framed capture is open. Verified at slice 67's WIP 2c25e683 (implementation/slice67), which carries slices 58 to 66 with slice 67's fixes: from slice 58 the world refused to compose (slice 58's light box reused an id slice 38's surface stock owned) until slice 67 renamed it. At 2c25e683 the fabrication batch's ten families (12,295 checks) report one failure, the capture harness finding no clear camera station for the B1 cleat run; apartment batch 204 on the long runner, as before; household state 154 checks, 0 failures; upper kitchens 206 and upper furniture 488, both unchanged; upper lighting 9,257 checks and public doors 17, 0 failures; the remaining transfers, apartment door, first upper hall, 4B door and rear wing A routes, the basement route (88), basement ground, boiler service, reading furniture, shop seating, funeral fittings, completion heating, radiator ties, ventilation, door casings (107 openings), hardware drawers (1,309 checks), street boundary, passage visibility, commensal, the street boundary route and the resident key route (86 waypoints, long runner), all 0 failures; twelve sweeps (55 spaces) and the city sweep's 130 views, 0 failures. The coal delivery route's stop at the lobby's inner door and the Vantry gateway suite's five kiosk-count failures are identical at slice 57's 260849e8 (base58), and the news receiving station failure is identical before slice 53.</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
@@ -4123,10 +4127,14 @@
       </c>
       <c r="S53" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T53" s="2" t="inlineStr"/>
+          <t>implemented</t>
+        </is>
+      </c>
+      <c r="T53" s="2" t="inlineStr">
+        <is>
+          <t>Partial: the pavement's ground marks feather out to their quad edges, so no stain ends in a hard dark rectangle (city sweep route stations). They are not yet clipped to the slab joints. Verified at slice 67's WIP 2c25e683 (implementation/slice67), which carries slices 58 to 66 with slice 67's fixes: from slice 58 the world refused to compose (slice 58's light box reused an id slice 38's surface stock owned) until slice 67 renamed it. At 2c25e683 the fabrication batch's ten families (12,295 checks) report one failure, the capture harness finding no clear camera station for the B1 cleat run; apartment batch 204 on the long runner, as before; household state 154 checks, 0 failures; upper kitchens 206 and upper furniture 488, both unchanged; upper lighting 9,257 checks and public doors 17, 0 failures; the remaining transfers, apartment door, first upper hall, 4B door and rear wing A routes, the basement route (88), basement ground, boiler service, reading furniture, shop seating, funeral fittings, completion heating, radiator ties, ventilation, door casings (107 openings), hardware drawers (1,309 checks), street boundary, passage visibility, commensal, the street boundary route and the resident key route (86 waypoints, long runner), all 0 failures; twelve sweeps (55 spaces) and the city sweep's 130 views, 0 failures. The coal delivery route's stop at the lobby's inner door and the Vantry gateway suite's five kiosk-count failures are identical at slice 57's 260849e8 (base58), and the news receiving station failure is identical before slice 53.</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Implement dossier slice 66: the last thresholds, 4B's worn runner, 5C's paint rag, 6D's padlock
- F03/F05/F06_EAST_HALL-001, F04_SOUTHWEST_HALL-001: 3B's ribbed rubber mat, the
  4D short-let's new coir with an unclaimed handbill, 6A's coir and the sealed
  5D's dust mat complete the thresholds.
- F04_B_ALCOVE_APPROACH-001: a bound jute runner worn through to the boards.
- F05_C_MAIN-003: Iris's paint rag over 5C's radiator, clear of valve and vent.
- F06_D_RESTRICTED-002: the landlord's galvanised hasp, staple and padlock at
  1.2 m and the old brass escutcheon at 1.5 m on 6D's storage door.

Evidence under implementation/slice67/. INERT: no ledger status changes.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/art/reviews/v2_environment_design_20261008/change_register.xlsx
+++ b/art/reviews/v2_environment_design_20261008/change_register.xlsx
@@ -19611,10 +19611,14 @@
       </c>
       <c r="S265" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T265" s="2" t="inlineStr"/>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="T265" s="2" t="inlineStr">
+        <is>
+          <t>No apartment door opens on the east hall itself; its thresholds are 3B's ribbed rubber mat at the service crossing (new) and the sealed 3C door's dust mat at the core, read with 3A's and 3D's from the landing (3B_threshold_native, F03_EAST_HALL_RV). Verified at slice 67's WIP 2c25e683 (implementation/slice67), which carries slices 58 to 66 with slice 67's fixes: from slice 58 the world refused to compose (slice 58's light box reused an id slice 38's surface stock owned) until slice 67 renamed it. At 2c25e683 the fabrication batch's ten families (12,295 checks) report one failure, the capture harness finding no clear camera station for the B1 cleat run; apartment batch 204 on the long runner, as before; household state 154 checks, 0 failures; upper kitchens 206 and upper furniture 488, both unchanged; upper lighting 9,257 checks and public doors 17, 0 failures; the remaining transfers, apartment door, first upper hall, 4B door and rear wing A routes, the basement route (88), basement ground, boiler service, reading furniture, shop seating, funeral fittings, completion heating, radiator ties, ventilation, door casings (107 openings), hardware drawers (1,309 checks), street boundary, passage visibility, commensal, the street boundary route and the resident key route (86 waypoints, long runner), all 0 failures; twelve sweeps (55 spaces) and the city sweep's 130 views, 0 failures. The coal delivery route's stop at the lobby's inner door and the Vantry gateway suite's five kiosk-count failures are identical at slice 57's 260849e8 (base58), and the news receiving station failure is identical before slice 53.</t>
+        </is>
+      </c>
     </row>
     <row r="266">
       <c r="A266" s="2" t="inlineStr">
@@ -24775,10 +24779,14 @@
       </c>
       <c r="S333" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T333" s="2" t="inlineStr"/>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="T333" s="2" t="inlineStr">
+        <is>
+          <t>The 4D short-let's new coir mat with a handbill pushed under the door that nobody picked up, read from the landing with 4B's worn mat (4D_threshold_native, F04_SOUTHWEST_HALL_OV). Verified at slice 67's WIP 2c25e683 (implementation/slice67), which carries slices 58 to 66 with slice 67's fixes: from slice 58 the world refused to compose (slice 58's light box reused an id slice 38's surface stock owned) until slice 67 renamed it. At 2c25e683 the fabrication batch's ten families (12,295 checks) report one failure, the capture harness finding no clear camera station for the B1 cleat run; apartment batch 204 on the long runner, as before; household state 154 checks, 0 failures; upper kitchens 206 and upper furniture 488, both unchanged; upper lighting 9,257 checks and public doors 17, 0 failures; the remaining transfers, apartment door, first upper hall, 4B door and rear wing A routes, the basement route (88), basement ground, boiler service, reading furniture, shop seating, funeral fittings, completion heating, radiator ties, ventilation, door casings (107 openings), hardware drawers (1,309 checks), street boundary, passage visibility, commensal, the street boundary route and the resident key route (86 waypoints, long runner), all 0 failures; twelve sweeps (55 spaces) and the city sweep's 130 views, 0 failures. The coal delivery route's stop at the lobby's inner door and the Vantry gateway suite's five kiosk-count failures are identical at slice 57's 260849e8 (base58), and the news receiving station failure is identical before slice 53.</t>
+        </is>
+      </c>
     </row>
     <row r="334">
       <c r="A334" s="2" t="inlineStr">
@@ -28173,10 +28181,14 @@
       </c>
       <c r="S378" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T378" s="2" t="inlineStr"/>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="T378" s="2" t="inlineStr">
+        <is>
+          <t>A bound jute runner centred along the alcove approach, worn through to the boards where the turn from the hall meets the way to the alcove, its strands loose across the hole (4B_alcove_runner_native, F04_B_ALCOVE_APPROACH_OV). Verified at slice 67's WIP 2c25e683 (implementation/slice67), which carries slices 58 to 66 with slice 67's fixes: from slice 58 the world refused to compose (slice 58's light box reused an id slice 38's surface stock owned) until slice 67 renamed it. At 2c25e683 the fabrication batch's ten families (12,295 checks) report one failure, the capture harness finding no clear camera station for the B1 cleat run; apartment batch 204 on the long runner, as before; household state 154 checks, 0 failures; upper kitchens 206 and upper furniture 488, both unchanged; upper lighting 9,257 checks and public doors 17, 0 failures; the remaining transfers, apartment door, first upper hall, 4B door and rear wing A routes, the basement route (88), basement ground, boiler service, reading furniture, shop seating, funeral fittings, completion heating, radiator ties, ventilation, door casings (107 openings), hardware drawers (1,309 checks), street boundary, passage visibility, commensal, the street boundary route and the resident key route (86 waypoints, long runner), all 0 failures; twelve sweeps (55 spaces) and the city sweep's 130 views, 0 failures. The coal delivery route's stop at the lobby's inner door and the Vantry gateway suite's five kiosk-count failures are identical at slice 57's 260849e8 (base58), and the news receiving station failure is identical before slice 53.</t>
+        </is>
+      </c>
     </row>
     <row r="379">
       <c r="A379" s="2" t="inlineStr">
@@ -32083,10 +32095,14 @@
       </c>
       <c r="S431" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T431" s="2" t="inlineStr"/>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="T431" s="2" t="inlineStr">
+        <is>
+          <t>No apartment door opens on the east hall; at its ends 5C's paint-flecked mat at the core and the sealed 5D's unworn dust mat at the crossing (new), with 5A's and 5B's read from the landing (5D_threshold_native, F05_EAST_HALL_RV). Verified at slice 67's WIP 2c25e683 (implementation/slice67), which carries slices 58 to 66 with slice 67's fixes: from slice 58 the world refused to compose (slice 58's light box reused an id slice 38's surface stock owned) until slice 67 renamed it. At 2c25e683 the fabrication batch's ten families (12,295 checks) report one failure, the capture harness finding no clear camera station for the B1 cleat run; apartment batch 204 on the long runner, as before; household state 154 checks, 0 failures; upper kitchens 206 and upper furniture 488, both unchanged; upper lighting 9,257 checks and public doors 17, 0 failures; the remaining transfers, apartment door, first upper hall, 4B door and rear wing A routes, the basement route (88), basement ground, boiler service, reading furniture, shop seating, funeral fittings, completion heating, radiator ties, ventilation, door casings (107 openings), hardware drawers (1,309 checks), street boundary, passage visibility, commensal, the street boundary route and the resident key route (86 waypoints, long runner), all 0 failures; twelve sweeps (55 spaces) and the city sweep's 130 views, 0 failures. The coal delivery route's stop at the lobby's inner door and the Vantry gateway suite's five kiosk-count failures are identical at slice 57's 260849e8 (base58), and the news receiving station failure is identical before slice 53.</t>
+        </is>
+      </c>
     </row>
     <row r="432">
       <c r="A432" s="2" t="inlineStr">
@@ -35845,10 +35861,14 @@
       </c>
       <c r="S482" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T482" s="2" t="inlineStr"/>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="T482" s="2" t="inlineStr">
+        <is>
+          <t>Iris's paint rag folded over 5C's radiator to dry, mid-length so the supply valve and the air vent stay in reach, oxblood paint on its fall; visual only (F05_C_MAIN_DT3). Verified at slice 67's WIP 2c25e683 (implementation/slice67), which carries slices 58 to 66 with slice 67's fixes: from slice 58 the world refused to compose (slice 58's light box reused an id slice 38's surface stock owned) until slice 67 renamed it. At 2c25e683 the fabrication batch's ten families (12,295 checks) report one failure, the capture harness finding no clear camera station for the B1 cleat run; apartment batch 204 on the long runner, as before; household state 154 checks, 0 failures; upper kitchens 206 and upper furniture 488, both unchanged; upper lighting 9,257 checks and public doors 17, 0 failures; the remaining transfers, apartment door, first upper hall, 4B door and rear wing A routes, the basement route (88), basement ground, boiler service, reading furniture, shop seating, funeral fittings, completion heating, radiator ties, ventilation, door casings (107 openings), hardware drawers (1,309 checks), street boundary, passage visibility, commensal, the street boundary route and the resident key route (86 waypoints, long runner), all 0 failures; twelve sweeps (55 spaces) and the city sweep's 130 views, 0 failures. The coal delivery route's stop at the lobby's inner door and the Vantry gateway suite's five kiosk-count failures are identical at slice 57's 260849e8 (base58), and the news receiving station failure is identical before slice 53.</t>
+        </is>
+      </c>
     </row>
     <row r="483">
       <c r="A483" s="2" t="inlineStr">
@@ -37633,10 +37653,14 @@
       </c>
       <c r="S506" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T506" s="2" t="inlineStr"/>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="T506" s="2" t="inlineStr">
+        <is>
+          <t>No apartment door opens on the east hall; at its ends 6C's coir mat and the appraiser's parcel at the core and the landlord's padlocked storage at the crossing; 6A's coir mat (new) and 6B's worn mat read from the landing (6A_threshold_native, F06_EAST_HALL_RV). Verified at slice 67's WIP 2c25e683 (implementation/slice67), which carries slices 58 to 66 with slice 67's fixes: from slice 58 the world refused to compose (slice 58's light box reused an id slice 38's surface stock owned) until slice 67 renamed it. At 2c25e683 the fabrication batch's ten families (12,295 checks) report one failure, the capture harness finding no clear camera station for the B1 cleat run; apartment batch 204 on the long runner, as before; household state 154 checks, 0 failures; upper kitchens 206 and upper furniture 488, both unchanged; upper lighting 9,257 checks and public doors 17, 0 failures; the remaining transfers, apartment door, first upper hall, 4B door and rear wing A routes, the basement route (88), basement ground, boiler service, reading furniture, shop seating, funeral fittings, completion heating, radiator ties, ventilation, door casings (107 openings), hardware drawers (1,309 checks), street boundary, passage visibility, commensal, the street boundary route and the resident key route (86 waypoints, long runner), all 0 failures; twelve sweeps (55 spaces) and the city sweep's 130 views, 0 failures. The coal delivery route's stop at the lobby's inner door and the Vantry gateway suite's five kiosk-count failures are identical at slice 57's 260849e8 (base58), and the news receiving station failure is identical before slice 53.</t>
+        </is>
+      </c>
     </row>
     <row r="507">
       <c r="A507" s="2" t="inlineStr">
@@ -41657,10 +41681,14 @@
       </c>
       <c r="S560" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T560" s="2" t="inlineStr"/>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="T560" s="2" t="inlineStr">
+        <is>
+          <t>A galvanised hasp across the latch stile and casing at 1.2 m with its staple and a black padlock, and the old brass escutcheon plate above at 1.5 m, on the landlord's storage door's crossing face; the leaf stays locked (F06_SERVICE_CROSSING_TH, F06_EAST_HALL_RV). Verified at slice 67's WIP 2c25e683 (implementation/slice67), which carries slices 58 to 66 with slice 67's fixes: from slice 58 the world refused to compose (slice 58's light box reused an id slice 38's surface stock owned) until slice 67 renamed it. At 2c25e683 the fabrication batch's ten families (12,295 checks) report one failure, the capture harness finding no clear camera station for the B1 cleat run; apartment batch 204 on the long runner, as before; household state 154 checks, 0 failures; upper kitchens 206 and upper furniture 488, both unchanged; upper lighting 9,257 checks and public doors 17, 0 failures; the remaining transfers, apartment door, first upper hall, 4B door and rear wing A routes, the basement route (88), basement ground, boiler service, reading furniture, shop seating, funeral fittings, completion heating, radiator ties, ventilation, door casings (107 openings), hardware drawers (1,309 checks), street boundary, passage visibility, commensal, the street boundary route and the resident key route (86 waypoints, long runner), all 0 failures; twelve sweeps (55 spaces) and the city sweep's 130 views, 0 failures. The coal delivery route's stop at the lobby's inner door and the Vantry gateway suite's five kiosk-count failures are identical at slice 57's 260849e8 (base58), and the news receiving station failure is identical before slice 53.</t>
+        </is>
+      </c>
     </row>
     <row r="561">
       <c r="A561" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Implement dossier slice 67: hall wear strengthened, the news mat and drawer test fixed, the light table renamed
- The hall walking line, door scuffs and trolley rub strengthened to read at
  production light; the 13 hall -002 rows are verified.
- The news mat's top back on the stool's datum, worn to its canvas ply on the
  counter side; the hardware drawer suite knows the open drawer
  (CITY_SHOP_NEWS_CIGARS-003 and CITY_SHOP_HARDWARE_PAINT-002 verified).
- Slice 58's light box renamed 6A_light_table and moved off the plate: it reused
  slice 38's surface-stock id and the runtime refused the world from slice 58 on.
- Verification of slices 58-67 at this WIP; the coal delivery and Vantry gateway
  failures are identical at slice 57 (base58).

Evidence under implementation/slice67/. INERT: no ledger status changes.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/art/reviews/v2_environment_design_20261008/change_register.xlsx
+++ b/art/reviews/v2_environment_design_20261008/change_register.xlsx
@@ -6137,12 +6137,12 @@
       </c>
       <c r="S84" s="2" t="inlineStr">
         <is>
-          <t>implemented</t>
+          <t>verified</t>
         </is>
       </c>
       <c r="T84" s="2" t="inlineStr">
         <is>
-          <t>The seven wire-bail tins in three sizes, two lids dented and paint run down two, each with a wordless paper label band and a colour stripe; one drawer of the wall stands 0.14 m open on its rail (paint_tins, drawer_wall, shop_hardware_paint_SITE_SHOP_IN1_HARDWARE_PAINT). Run at slice 54's WIP 22b1aa9a (implementation/slice54b), which carries slice 53 unchanged: the city sweep's 130 views report 0 failures and the IN0/IN1 stations show the shops. At that WIP the news fittings module reports 4 failures (slice 53 sank the worn hollow below the datum the stool's four feet stand on) and the hardware drawer suite 1 (its face probe did not know the open drawer). Slice 67 fixes both; these rows are upgraded when it verifies.</t>
+          <t>The seven wire-bail tins in three sizes, two lids dented and paint run down two, each with a wordless paper label band and a colour stripe; one drawer of the wall stands 0.14 m open on its rail (paint_tins, drawer_wall, shop_hardware_paint_SITE_SHOP_IN1_HARDWARE_PAINT). Run at slice 54's WIP 22b1aa9a (implementation/slice54b), which carries slice 53 unchanged: the city sweep's 130 views report 0 failures and the IN0/IN1 stations show the shops. At that WIP the news fittings module reports 4 failures (slice 53 sank the worn hollow below the datum the stool's four feet stand on) and the hardware drawer suite 1 (its face probe did not know the open drawer). Slice 67 fixes both; these rows are upgraded when it verifies. Slice 67 teaches the drawer suite the open drawer; hardware drawers pass, 1,309 checks, 0 failures at 2c25e683 (implementation/slice67).</t>
         </is>
       </c>
     </row>
@@ -6786,7 +6786,7 @@
       </c>
       <c r="T94" s="2" t="inlineStr">
         <is>
-          <t>Partial: the stool's floor cover becomes a black rubber mat worn to a hollow under the proprietor's feet (fitted_stool); the half-punched punchboard on the counter is the fitted family's own (punchboard). The tile under the mat is not dished: the mat covers it. Run at slice 54's WIP 22b1aa9a (implementation/slice54b), which carries slice 53 unchanged: the city sweep's 130 views report 0 failures and the IN0/IN1 stations show the shops. At that WIP the news fittings module reports 4 failures (slice 53 sank the worn hollow below the datum the stool's four feet stand on) and the hardware drawer suite 1 (its face probe did not know the open drawer). Slice 67 fixes both; these rows are upgraded when it verifies.</t>
+          <t>Partial: the stool's floor cover becomes a black rubber mat worn to a hollow under the proprietor's feet (fitted_stool); the half-punched punchboard on the counter is the fitted family's own (punchboard). The tile under the mat is not dished: the mat covers it. Run at slice 54's WIP 22b1aa9a (implementation/slice54b), which carries slice 53 unchanged: the city sweep's 130 views report 0 failures and the IN0/IN1 stations show the shops. At that WIP the news fittings module reports 4 failures (slice 53 sank the worn hollow below the datum the stool's four feet stand on) and the hardware drawer suite 1 (its face probe did not know the open drawer). Slice 67 fixes both; these rows are upgraded when it verifies. Slice 67 restores the stool's datum (the worn mat's top is the original height, worn to its pale canvas ply on the counter side) and the news fittings pass, 670 checks, 0 failures at 2c25e683 (implementation/slice67).</t>
         </is>
       </c>
     </row>
@@ -6909,12 +6909,12 @@
       </c>
       <c r="S96" s="2" t="inlineStr">
         <is>
-          <t>implemented</t>
+          <t>verified</t>
         </is>
       </c>
       <c r="T96" s="2" t="inlineStr">
         <is>
-          <t>The booth's stock, every piece seated on its board: four string-tied bundles of papers, three fanned runs of magazines, cigar boxes with one lid stood open on its cigars, three tobacco tins, and four stacks of papers under wordless grey mastheads; the cigar case shows its cigars (shop_news_cigars_SITE_SHOP_IN0_NEWS_CIGARS, rear_shelves). Run at slice 54's WIP 22b1aa9a (implementation/slice54b), which carries slice 53 unchanged: the city sweep's 130 views report 0 failures and the IN0/IN1 stations show the shops. At that WIP the news fittings module reports 4 failures (slice 53 sank the worn hollow below the datum the stool's four feet stand on) and the hardware drawer suite 1 (its face probe did not know the open drawer). Slice 67 fixes both; these rows are upgraded when it verifies.</t>
+          <t>The booth's stock, every piece seated on its board: four string-tied bundles of papers, three fanned runs of magazines, cigar boxes with one lid stood open on its cigars, three tobacco tins, and four stacks of papers under wordless grey mastheads; the cigar case shows its cigars (shop_news_cigars_SITE_SHOP_IN0_NEWS_CIGARS, rear_shelves). Run at slice 54's WIP 22b1aa9a (implementation/slice54b), which carries slice 53 unchanged: the city sweep's 130 views report 0 failures and the IN0/IN1 stations show the shops. At that WIP the news fittings module reports 4 failures (slice 53 sank the worn hollow below the datum the stool's four feet stand on) and the hardware drawer suite 1 (its face probe did not know the open drawer). Slice 67 fixes both; these rows are upgraded when it verifies. Slice 67 restores the stool's datum (the worn mat's top is the original height, worn to its pale canvas ply on the counter side) and the news fittings pass, 670 checks, 0 failures at 2c25e683 (implementation/slice67).</t>
         </is>
       </c>
     </row>
@@ -14023,12 +14023,12 @@
       </c>
       <c r="S193" s="2" t="inlineStr">
         <is>
-          <t>implemented</t>
+          <t>verified</t>
         </is>
       </c>
       <c r="T193" s="2" t="inlineStr">
         <is>
-          <t>The dulled walking line down the hall's middle, foot scuffs on the floor at each apartment door, the mop-shadow corner farthest from the core and the porter's trolley rub on the long wall at 0.6 m, 0.9 m in from the core (F02_WEST_HALL_RV, F02_WEST_HALL_OV); the scuffs sit on the actual door positions. The marks render (a frame difference against slice 49's views traces the path down the centre and the scuffs at the doors) but read faintly at production light; strengthening them is open. Verified at WIP 3f3f0d75 (implementation/slice52): apartment batch 204 on the long runner; household state 154 checks, 0 failures; upper kitchens 206 and upper furniture 488, both unchanged; upper lighting 9,257 checks and public doors 17, both 0 failures; the first bath sweep (six baths) 0 failures; the remaining twelve baths, the thirteen upper halls and slice 50's third core group were rerun at the same WIP in five sweeps, all 0 failures (implementation/slice52b); four earlier sweep runs that ran at another WIP are superseded and not cited. The decals are projected (Godot Decal nodes) from game/data/orison_v2/positional_wear.json onto the inherited finishes: no collision, no owner, no lettering.</t>
+          <t>The dulled walking line down the hall's middle, foot scuffs on the floor at each apartment door, the mop-shadow corner farthest from the core and the porter's trolley rub on the long wall at 0.6 m, 0.9 m in from the core (F02_WEST_HALL_RV, F02_WEST_HALL_OV); the scuffs sit on the actual door positions. The marks render (a frame difference against slice 49's views traces the path down the centre and the scuffs at the doors) but read faintly at production light; strengthening them is open. Verified at WIP 3f3f0d75 (implementation/slice52): apartment batch 204 on the long runner; household state 154 checks, 0 failures; upper kitchens 206 and upper furniture 488, both unchanged; upper lighting 9,257 checks and public doors 17, both 0 failures; the first bath sweep (six baths) 0 failures; the remaining twelve baths, the thirteen upper halls and slice 50's third core group were rerun at the same WIP in five sweeps, all 0 failures (implementation/slice52b); four earlier sweep runs that ran at another WIP are superseded and not cited. The decals are projected (Godot Decal nodes) from game/data/orison_v2/positional_wear.json onto the inherited finishes: no collision, no owner, no lettering. Slice 67 strengthens the walking line, door scuffs and trolley rub to read at production light (verified at 2c25e683, implementation/slice67).</t>
         </is>
       </c>
     </row>
@@ -14179,12 +14179,12 @@
       </c>
       <c r="S195" s="2" t="inlineStr">
         <is>
-          <t>implemented</t>
+          <t>verified</t>
         </is>
       </c>
       <c r="T195" s="2" t="inlineStr">
         <is>
-          <t>The dulled walking line down the hall's middle, foot scuffs on the floor at each apartment door, the mop-shadow corner farthest from the core and the porter's trolley rub on the long wall at 0.6 m, 0.9 m in from the core (F02_SOUTHWEST_HALL_RV, F02_SOUTHWEST_HALL_OV); the scuffs sit on the actual door positions. The marks render (a frame difference against slice 49's views traces the path down the centre and the scuffs at the doors) but read faintly at production light; strengthening them is open. Verified at WIP 3f3f0d75 (implementation/slice52): apartment batch 204 on the long runner; household state 154 checks, 0 failures; upper kitchens 206 and upper furniture 488, both unchanged; upper lighting 9,257 checks and public doors 17, both 0 failures; the first bath sweep (six baths) 0 failures; the remaining twelve baths, the thirteen upper halls and slice 50's third core group were rerun at the same WIP in five sweeps, all 0 failures (implementation/slice52b); four earlier sweep runs that ran at another WIP are superseded and not cited. The decals are projected (Godot Decal nodes) from game/data/orison_v2/positional_wear.json onto the inherited finishes: no collision, no owner, no lettering.</t>
+          <t>The dulled walking line down the hall's middle, foot scuffs on the floor at each apartment door, the mop-shadow corner farthest from the core and the porter's trolley rub on the long wall at 0.6 m, 0.9 m in from the core (F02_SOUTHWEST_HALL_RV, F02_SOUTHWEST_HALL_OV); the scuffs sit on the actual door positions. The marks render (a frame difference against slice 49's views traces the path down the centre and the scuffs at the doors) but read faintly at production light; strengthening them is open. Verified at WIP 3f3f0d75 (implementation/slice52): apartment batch 204 on the long runner; household state 154 checks, 0 failures; upper kitchens 206 and upper furniture 488, both unchanged; upper lighting 9,257 checks and public doors 17, both 0 failures; the first bath sweep (six baths) 0 failures; the remaining twelve baths, the thirteen upper halls and slice 50's third core group were rerun at the same WIP in five sweeps, all 0 failures (implementation/slice52b); four earlier sweep runs that ran at another WIP are superseded and not cited. The decals are projected (Godot Decal nodes) from game/data/orison_v2/positional_wear.json onto the inherited finishes: no collision, no owner, no lettering. Slice 67 strengthens the walking line, door scuffs and trolley rub to read at production light (verified at 2c25e683, implementation/slice67).</t>
         </is>
       </c>
     </row>
@@ -14491,12 +14491,12 @@
       </c>
       <c r="S199" s="2" t="inlineStr">
         <is>
-          <t>implemented</t>
+          <t>verified</t>
         </is>
       </c>
       <c r="T199" s="2" t="inlineStr">
         <is>
-          <t>The dulled walking line down the hall's middle, foot scuffs on the floor at each apartment door, the mop-shadow corner farthest from the core and the porter's trolley rub on the long wall at 0.6 m, 0.9 m in from the core (F02_EAST_HALL_RV, F02_EAST_HALL_OV); the scuffs sit on the actual door positions. The marks render (a frame difference against slice 49's views traces the path down the centre and the scuffs at the doors) but read faintly at production light; strengthening them is open. Verified at WIP 3f3f0d75 (implementation/slice52): apartment batch 204 on the long runner; household state 154 checks, 0 failures; upper kitchens 206 and upper furniture 488, both unchanged; upper lighting 9,257 checks and public doors 17, both 0 failures; the first bath sweep (six baths) 0 failures; the remaining twelve baths, the thirteen upper halls and slice 50's third core group were rerun at the same WIP in five sweeps, all 0 failures (implementation/slice52b); four earlier sweep runs that ran at another WIP are superseded and not cited. The decals are projected (Godot Decal nodes) from game/data/orison_v2/positional_wear.json onto the inherited finishes: no collision, no owner, no lettering.</t>
+          <t>The dulled walking line down the hall's middle, foot scuffs on the floor at each apartment door, the mop-shadow corner farthest from the core and the porter's trolley rub on the long wall at 0.6 m, 0.9 m in from the core (F02_EAST_HALL_RV, F02_EAST_HALL_OV); the scuffs sit on the actual door positions. The marks render (a frame difference against slice 49's views traces the path down the centre and the scuffs at the doors) but read faintly at production light; strengthening them is open. Verified at WIP 3f3f0d75 (implementation/slice52): apartment batch 204 on the long runner; household state 154 checks, 0 failures; upper kitchens 206 and upper furniture 488, both unchanged; upper lighting 9,257 checks and public doors 17, both 0 failures; the first bath sweep (six baths) 0 failures; the remaining twelve baths, the thirteen upper halls and slice 50's third core group were rerun at the same WIP in five sweeps, all 0 failures (implementation/slice52b); four earlier sweep runs that ran at another WIP are superseded and not cited. The decals are projected (Godot Decal nodes) from game/data/orison_v2/positional_wear.json onto the inherited finishes: no collision, no owner, no lettering. Slice 67 strengthens the walking line, door scuffs and trolley rub to read at production light (verified at 2c25e683, implementation/slice67).</t>
         </is>
       </c>
     </row>
@@ -19685,12 +19685,12 @@
       </c>
       <c r="S266" s="2" t="inlineStr">
         <is>
-          <t>implemented</t>
+          <t>verified</t>
         </is>
       </c>
       <c r="T266" s="2" t="inlineStr">
         <is>
-          <t>The dulled walking line down the hall's middle, foot scuffs on the floor at each apartment door, the mop-shadow corner farthest from the core and the porter's trolley rub on the long wall at 0.6 m, 0.9 m in from the core (F03_EAST_HALL_RV, F03_EAST_HALL_OV); the scuffs sit on the actual door positions. The marks render (a frame difference against slice 49's views traces the path down the centre and the scuffs at the doors) but read faintly at production light; strengthening them is open. Verified at WIP 3f3f0d75 (implementation/slice52): apartment batch 204 on the long runner; household state 154 checks, 0 failures; upper kitchens 206 and upper furniture 488, both unchanged; upper lighting 9,257 checks and public doors 17, both 0 failures; the first bath sweep (six baths) 0 failures; the remaining twelve baths, the thirteen upper halls and slice 50's third core group were rerun at the same WIP in five sweeps, all 0 failures (implementation/slice52b); four earlier sweep runs that ran at another WIP are superseded and not cited. The decals are projected (Godot Decal nodes) from game/data/orison_v2/positional_wear.json onto the inherited finishes: no collision, no owner, no lettering.</t>
+          <t>The dulled walking line down the hall's middle, foot scuffs on the floor at each apartment door, the mop-shadow corner farthest from the core and the porter's trolley rub on the long wall at 0.6 m, 0.9 m in from the core (F03_EAST_HALL_RV, F03_EAST_HALL_OV); the scuffs sit on the actual door positions. The marks render (a frame difference against slice 49's views traces the path down the centre and the scuffs at the doors) but read faintly at production light; strengthening them is open. Verified at WIP 3f3f0d75 (implementation/slice52): apartment batch 204 on the long runner; household state 154 checks, 0 failures; upper kitchens 206 and upper furniture 488, both unchanged; upper lighting 9,257 checks and public doors 17, both 0 failures; the first bath sweep (six baths) 0 failures; the remaining twelve baths, the thirteen upper halls and slice 50's third core group were rerun at the same WIP in five sweeps, all 0 failures (implementation/slice52b); four earlier sweep runs that ran at another WIP are superseded and not cited. The decals are projected (Godot Decal nodes) from game/data/orison_v2/positional_wear.json onto the inherited finishes: no collision, no owner, no lettering. Slice 67 strengthens the walking line, door scuffs and trolley rub to read at production light (verified at 2c25e683, implementation/slice67).</t>
         </is>
       </c>
     </row>
@@ -20195,12 +20195,12 @@
       </c>
       <c r="S273" s="2" t="inlineStr">
         <is>
-          <t>implemented</t>
+          <t>verified</t>
         </is>
       </c>
       <c r="T273" s="2" t="inlineStr">
         <is>
-          <t>The dulled walking line down the hall's middle, foot scuffs on the floor at each apartment door, the mop-shadow corner farthest from the core and the porter's trolley rub on the long wall at 0.6 m, 0.9 m in from the core (F03_WEST_HALL_RV, F03_WEST_HALL_OV); the scuffs sit on the actual door positions. The marks render (a frame difference against slice 49's views traces the path down the centre and the scuffs at the doors) but read faintly at production light; strengthening them is open. Verified at WIP 3f3f0d75 (implementation/slice52): apartment batch 204 on the long runner; household state 154 checks, 0 failures; upper kitchens 206 and upper furniture 488, both unchanged; upper lighting 9,257 checks and public doors 17, both 0 failures; the first bath sweep (six baths) 0 failures; the remaining twelve baths, the thirteen upper halls and slice 50's third core group were rerun at the same WIP in five sweeps, all 0 failures (implementation/slice52b); four earlier sweep runs that ran at another WIP are superseded and not cited. The decals are projected (Godot Decal nodes) from game/data/orison_v2/positional_wear.json onto the inherited finishes: no collision, no owner, no lettering.</t>
+          <t>The dulled walking line down the hall's middle, foot scuffs on the floor at each apartment door, the mop-shadow corner farthest from the core and the porter's trolley rub on the long wall at 0.6 m, 0.9 m in from the core (F03_WEST_HALL_RV, F03_WEST_HALL_OV); the scuffs sit on the actual door positions. The marks render (a frame difference against slice 49's views traces the path down the centre and the scuffs at the doors) but read faintly at production light; strengthening them is open. Verified at WIP 3f3f0d75 (implementation/slice52): apartment batch 204 on the long runner; household state 154 checks, 0 failures; upper kitchens 206 and upper furniture 488, both unchanged; upper lighting 9,257 checks and public doors 17, both 0 failures; the first bath sweep (six baths) 0 failures; the remaining twelve baths, the thirteen upper halls and slice 50's third core group were rerun at the same WIP in five sweeps, all 0 failures (implementation/slice52b); four earlier sweep runs that ran at another WIP are superseded and not cited. The decals are projected (Godot Decal nodes) from game/data/orison_v2/positional_wear.json onto the inherited finishes: no collision, no owner, no lettering. Slice 67 strengthens the walking line, door scuffs and trolley rub to read at production light (verified at 2c25e683, implementation/slice67).</t>
         </is>
       </c>
     </row>
@@ -20351,12 +20351,12 @@
       </c>
       <c r="S275" s="2" t="inlineStr">
         <is>
-          <t>implemented</t>
+          <t>verified</t>
         </is>
       </c>
       <c r="T275" s="2" t="inlineStr">
         <is>
-          <t>The dulled walking line down the hall's middle, foot scuffs on the floor at each apartment door, the mop-shadow corner farthest from the core and the porter's trolley rub on the long wall at 0.6 m, 0.9 m in from the core (F03_SOUTHWEST_HALL_RV, F03_SOUTHWEST_HALL_OV); the scuffs sit on the actual door positions. The marks render (a frame difference against slice 49's views traces the path down the centre and the scuffs at the doors) but read faintly at production light; strengthening them is open. Verified at WIP 3f3f0d75 (implementation/slice52): apartment batch 204 on the long runner; household state 154 checks, 0 failures; upper kitchens 206 and upper furniture 488, both unchanged; upper lighting 9,257 checks and public doors 17, both 0 failures; the first bath sweep (six baths) 0 failures; the remaining twelve baths, the thirteen upper halls and slice 50's third core group were rerun at the same WIP in five sweeps, all 0 failures (implementation/slice52b); four earlier sweep runs that ran at another WIP are superseded and not cited. The decals are projected (Godot Decal nodes) from game/data/orison_v2/positional_wear.json onto the inherited finishes: no collision, no owner, no lettering.</t>
+          <t>The dulled walking line down the hall's middle, foot scuffs on the floor at each apartment door, the mop-shadow corner farthest from the core and the porter's trolley rub on the long wall at 0.6 m, 0.9 m in from the core (F03_SOUTHWEST_HALL_RV, F03_SOUTHWEST_HALL_OV); the scuffs sit on the actual door positions. The marks render (a frame difference against slice 49's views traces the path down the centre and the scuffs at the doors) but read faintly at production light; strengthening them is open. Verified at WIP 3f3f0d75 (implementation/slice52): apartment batch 204 on the long runner; household state 154 checks, 0 failures; upper kitchens 206 and upper furniture 488, both unchanged; upper lighting 9,257 checks and public doors 17, both 0 failures; the first bath sweep (six baths) 0 failures; the remaining twelve baths, the thirteen upper halls and slice 50's third core group were rerun at the same WIP in five sweeps, all 0 failures (implementation/slice52b); four earlier sweep runs that ran at another WIP are superseded and not cited. The decals are projected (Godot Decal nodes) from game/data/orison_v2/positional_wear.json onto the inherited finishes: no collision, no owner, no lettering. Slice 67 strengthens the walking line, door scuffs and trolley rub to read at production light (verified at 2c25e683, implementation/slice67).</t>
         </is>
       </c>
     </row>
@@ -24635,12 +24635,12 @@
       </c>
       <c r="S331" s="2" t="inlineStr">
         <is>
-          <t>implemented</t>
+          <t>verified</t>
         </is>
       </c>
       <c r="T331" s="2" t="inlineStr">
         <is>
-          <t>The dulled walking line down the hall's middle, foot scuffs on the floor at each apartment door, the mop-shadow corner farthest from the core and the porter's trolley rub on the long wall at 0.6 m, 0.9 m in from the core (F04_WEST_HALL_RV, F04_WEST_HALL_OV); the scuffs sit on the actual door positions. The marks render (a frame difference against slice 49's views traces the path down the centre and the scuffs at the doors) but read faintly at production light; strengthening them is open. Verified at WIP 3f3f0d75 (implementation/slice52): apartment batch 204 on the long runner; household state 154 checks, 0 failures; upper kitchens 206 and upper furniture 488, both unchanged; upper lighting 9,257 checks and public doors 17, both 0 failures; the first bath sweep (six baths) 0 failures; the remaining twelve baths, the thirteen upper halls and slice 50's third core group were rerun at the same WIP in five sweeps, all 0 failures (implementation/slice52b); four earlier sweep runs that ran at another WIP are superseded and not cited. The decals are projected (Godot Decal nodes) from game/data/orison_v2/positional_wear.json onto the inherited finishes: no collision, no owner, no lettering.</t>
+          <t>The dulled walking line down the hall's middle, foot scuffs on the floor at each apartment door, the mop-shadow corner farthest from the core and the porter's trolley rub on the long wall at 0.6 m, 0.9 m in from the core (F04_WEST_HALL_RV, F04_WEST_HALL_OV); the scuffs sit on the actual door positions. The marks render (a frame difference against slice 49's views traces the path down the centre and the scuffs at the doors) but read faintly at production light; strengthening them is open. Verified at WIP 3f3f0d75 (implementation/slice52): apartment batch 204 on the long runner; household state 154 checks, 0 failures; upper kitchens 206 and upper furniture 488, both unchanged; upper lighting 9,257 checks and public doors 17, both 0 failures; the first bath sweep (six baths) 0 failures; the remaining twelve baths, the thirteen upper halls and slice 50's third core group were rerun at the same WIP in five sweeps, all 0 failures (implementation/slice52b); four earlier sweep runs that ran at another WIP are superseded and not cited. The decals are projected (Godot Decal nodes) from game/data/orison_v2/positional_wear.json onto the inherited finishes: no collision, no owner, no lettering. Slice 67 strengthens the walking line, door scuffs and trolley rub to read at production light (verified at 2c25e683, implementation/slice67).</t>
         </is>
       </c>
     </row>
@@ -24853,12 +24853,12 @@
       </c>
       <c r="S334" s="2" t="inlineStr">
         <is>
-          <t>implemented</t>
+          <t>verified</t>
         </is>
       </c>
       <c r="T334" s="2" t="inlineStr">
         <is>
-          <t>The dulled walking line down the hall's middle, foot scuffs on the floor at each apartment door, the mop-shadow corner farthest from the core and the porter's trolley rub on the long wall at 0.6 m, 0.9 m in from the core (F04_SOUTHWEST_HALL_RV, F04_SOUTHWEST_HALL_OV); the scuffs sit on the actual door positions. The marks render (a frame difference against slice 49's views traces the path down the centre and the scuffs at the doors) but read faintly at production light; strengthening them is open. Verified at WIP 3f3f0d75 (implementation/slice52): apartment batch 204 on the long runner; household state 154 checks, 0 failures; upper kitchens 206 and upper furniture 488, both unchanged; upper lighting 9,257 checks and public doors 17, both 0 failures; the first bath sweep (six baths) 0 failures; the remaining twelve baths, the thirteen upper halls and slice 50's third core group were rerun at the same WIP in five sweeps, all 0 failures (implementation/slice52b); four earlier sweep runs that ran at another WIP are superseded and not cited. The decals are projected (Godot Decal nodes) from game/data/orison_v2/positional_wear.json onto the inherited finishes: no collision, no owner, no lettering.</t>
+          <t>The dulled walking line down the hall's middle, foot scuffs on the floor at each apartment door, the mop-shadow corner farthest from the core and the porter's trolley rub on the long wall at 0.6 m, 0.9 m in from the core (F04_SOUTHWEST_HALL_RV, F04_SOUTHWEST_HALL_OV); the scuffs sit on the actual door positions. The marks render (a frame difference against slice 49's views traces the path down the centre and the scuffs at the doors) but read faintly at production light; strengthening them is open. Verified at WIP 3f3f0d75 (implementation/slice52): apartment batch 204 on the long runner; household state 154 checks, 0 failures; upper kitchens 206 and upper furniture 488, both unchanged; upper lighting 9,257 checks and public doors 17, both 0 failures; the first bath sweep (six baths) 0 failures; the remaining twelve baths, the thirteen upper halls and slice 50's third core group were rerun at the same WIP in five sweeps, all 0 failures (implementation/slice52b); four earlier sweep runs that ran at another WIP are superseded and not cited. The decals are projected (Godot Decal nodes) from game/data/orison_v2/positional_wear.json onto the inherited finishes: no collision, no owner, no lettering. Slice 67 strengthens the walking line, door scuffs and trolley rub to read at production light (verified at 2c25e683, implementation/slice67).</t>
         </is>
       </c>
     </row>
@@ -25297,12 +25297,12 @@
       </c>
       <c r="S340" s="2" t="inlineStr">
         <is>
-          <t>implemented</t>
+          <t>verified</t>
         </is>
       </c>
       <c r="T340" s="2" t="inlineStr">
         <is>
-          <t>The dulled walking line down the hall's middle, foot scuffs on the floor at each apartment door, the mop-shadow corner farthest from the core and the porter's trolley rub on the long wall at 0.6 m, 0.9 m in from the core (F04_EAST_HALL_RV, F04_EAST_HALL_OV); the scuffs sit on the actual door positions. The marks render (a frame difference against slice 49's views traces the path down the centre and the scuffs at the doors) but read faintly at production light; strengthening them is open. Verified at WIP 3f3f0d75 (implementation/slice52): apartment batch 204 on the long runner; household state 154 checks, 0 failures; upper kitchens 206 and upper furniture 488, both unchanged; upper lighting 9,257 checks and public doors 17, both 0 failures; the first bath sweep (six baths) 0 failures; the remaining twelve baths, the thirteen upper halls and slice 50's third core group were rerun at the same WIP in five sweeps, all 0 failures (implementation/slice52b); four earlier sweep runs that ran at another WIP are superseded and not cited. The decals are projected (Godot Decal nodes) from game/data/orison_v2/positional_wear.json onto the inherited finishes: no collision, no owner, no lettering.</t>
+          <t>The dulled walking line down the hall's middle, foot scuffs on the floor at each apartment door, the mop-shadow corner farthest from the core and the porter's trolley rub on the long wall at 0.6 m, 0.9 m in from the core (F04_EAST_HALL_RV, F04_EAST_HALL_OV); the scuffs sit on the actual door positions. The marks render (a frame difference against slice 49's views traces the path down the centre and the scuffs at the doors) but read faintly at production light; strengthening them is open. Verified at WIP 3f3f0d75 (implementation/slice52): apartment batch 204 on the long runner; household state 154 checks, 0 failures; upper kitchens 206 and upper furniture 488, both unchanged; upper lighting 9,257 checks and public doors 17, both 0 failures; the first bath sweep (six baths) 0 failures; the remaining twelve baths, the thirteen upper halls and slice 50's third core group were rerun at the same WIP in five sweeps, all 0 failures (implementation/slice52b); four earlier sweep runs that ran at another WIP are superseded and not cited. The decals are projected (Godot Decal nodes) from game/data/orison_v2/positional_wear.json onto the inherited finishes: no collision, no owner, no lettering. Slice 67 strengthens the walking line, door scuffs and trolley rub to read at production light (verified at 2c25e683, implementation/slice67).</t>
         </is>
       </c>
     </row>
@@ -32169,12 +32169,12 @@
       </c>
       <c r="S432" s="2" t="inlineStr">
         <is>
-          <t>implemented</t>
+          <t>verified</t>
         </is>
       </c>
       <c r="T432" s="2" t="inlineStr">
         <is>
-          <t>The dulled walking line down the hall's middle, foot scuffs on the floor at each apartment door, the mop-shadow corner farthest from the core and the porter's trolley rub on the long wall at 0.6 m, 0.9 m in from the core (F05_EAST_HALL_RV, F05_EAST_HALL_OV); the scuffs sit on the actual door positions. The marks render (a frame difference against slice 49's views traces the path down the centre and the scuffs at the doors) but read faintly at production light; strengthening them is open. Verified at WIP 3f3f0d75 (implementation/slice52): apartment batch 204 on the long runner; household state 154 checks, 0 failures; upper kitchens 206 and upper furniture 488, both unchanged; upper lighting 9,257 checks and public doors 17, both 0 failures; the first bath sweep (six baths) 0 failures; the remaining twelve baths, the thirteen upper halls and slice 50's third core group were rerun at the same WIP in five sweeps, all 0 failures (implementation/slice52b); four earlier sweep runs that ran at another WIP are superseded and not cited. The decals are projected (Godot Decal nodes) from game/data/orison_v2/positional_wear.json onto the inherited finishes: no collision, no owner, no lettering.</t>
+          <t>The dulled walking line down the hall's middle, foot scuffs on the floor at each apartment door, the mop-shadow corner farthest from the core and the porter's trolley rub on the long wall at 0.6 m, 0.9 m in from the core (F05_EAST_HALL_RV, F05_EAST_HALL_OV); the scuffs sit on the actual door positions. The marks render (a frame difference against slice 49's views traces the path down the centre and the scuffs at the doors) but read faintly at production light; strengthening them is open. Verified at WIP 3f3f0d75 (implementation/slice52): apartment batch 204 on the long runner; household state 154 checks, 0 failures; upper kitchens 206 and upper furniture 488, both unchanged; upper lighting 9,257 checks and public doors 17, both 0 failures; the first bath sweep (six baths) 0 failures; the remaining twelve baths, the thirteen upper halls and slice 50's third core group were rerun at the same WIP in five sweeps, all 0 failures (implementation/slice52b); four earlier sweep runs that ran at another WIP are superseded and not cited. The decals are projected (Godot Decal nodes) from game/data/orison_v2/positional_wear.json onto the inherited finishes: no collision, no owner, no lettering. Slice 67 strengthens the walking line, door scuffs and trolley rub to read at production light (verified at 2c25e683, implementation/slice67).</t>
         </is>
       </c>
     </row>
@@ -32539,12 +32539,12 @@
       </c>
       <c r="S437" s="2" t="inlineStr">
         <is>
-          <t>implemented</t>
+          <t>verified</t>
         </is>
       </c>
       <c r="T437" s="2" t="inlineStr">
         <is>
-          <t>The dulled walking line down the hall's middle, foot scuffs on the floor at each apartment door, the mop-shadow corner farthest from the core and the porter's trolley rub on the long wall at 0.6 m, 0.9 m in from the core (F05_WEST_HALL_RV, F05_WEST_HALL_OV); the scuffs sit on the actual door positions. The marks render (a frame difference against slice 49's views traces the path down the centre and the scuffs at the doors) but read faintly at production light; strengthening them is open. Verified at WIP 3f3f0d75 (implementation/slice52): apartment batch 204 on the long runner; household state 154 checks, 0 failures; upper kitchens 206 and upper furniture 488, both unchanged; upper lighting 9,257 checks and public doors 17, both 0 failures; the first bath sweep (six baths) 0 failures; the remaining twelve baths, the thirteen upper halls and slice 50's third core group were rerun at the same WIP in five sweeps, all 0 failures (implementation/slice52b); four earlier sweep runs that ran at another WIP are superseded and not cited. The decals are projected (Godot Decal nodes) from game/data/orison_v2/positional_wear.json onto the inherited finishes: no collision, no owner, no lettering.</t>
+          <t>The dulled walking line down the hall's middle, foot scuffs on the floor at each apartment door, the mop-shadow corner farthest from the core and the porter's trolley rub on the long wall at 0.6 m, 0.9 m in from the core (F05_WEST_HALL_RV, F05_WEST_HALL_OV); the scuffs sit on the actual door positions. The marks render (a frame difference against slice 49's views traces the path down the centre and the scuffs at the doors) but read faintly at production light; strengthening them is open. Verified at WIP 3f3f0d75 (implementation/slice52): apartment batch 204 on the long runner; household state 154 checks, 0 failures; upper kitchens 206 and upper furniture 488, both unchanged; upper lighting 9,257 checks and public doors 17, both 0 failures; the first bath sweep (six baths) 0 failures; the remaining twelve baths, the thirteen upper halls and slice 50's third core group were rerun at the same WIP in five sweeps, all 0 failures (implementation/slice52b); four earlier sweep runs that ran at another WIP are superseded and not cited. The decals are projected (Godot Decal nodes) from game/data/orison_v2/positional_wear.json onto the inherited finishes: no collision, no owner, no lettering. Slice 67 strengthens the walking line, door scuffs and trolley rub to read at production light (verified at 2c25e683, implementation/slice67).</t>
         </is>
       </c>
     </row>
@@ -37727,12 +37727,12 @@
       </c>
       <c r="S507" s="2" t="inlineStr">
         <is>
-          <t>implemented</t>
+          <t>verified</t>
         </is>
       </c>
       <c r="T507" s="2" t="inlineStr">
         <is>
-          <t>The dulled walking line down the hall's middle, foot scuffs on the floor at each apartment door, the mop-shadow corner farthest from the core and the porter's trolley rub on the long wall at 0.6 m, 0.9 m in from the core (F06_EAST_HALL_RV, F06_EAST_HALL_OV); the scuffs sit on the actual door positions. The marks render (a frame difference against slice 49's views traces the path down the centre and the scuffs at the doors) but read faintly at production light; strengthening them is open. Verified at WIP 3f3f0d75 (implementation/slice52): apartment batch 204 on the long runner; household state 154 checks, 0 failures; upper kitchens 206 and upper furniture 488, both unchanged; upper lighting 9,257 checks and public doors 17, both 0 failures; the first bath sweep (six baths) 0 failures; the remaining twelve baths, the thirteen upper halls and slice 50's third core group were rerun at the same WIP in five sweeps, all 0 failures (implementation/slice52b); four earlier sweep runs that ran at another WIP are superseded and not cited. The decals are projected (Godot Decal nodes) from game/data/orison_v2/positional_wear.json onto the inherited finishes: no collision, no owner, no lettering.</t>
+          <t>The dulled walking line down the hall's middle, foot scuffs on the floor at each apartment door, the mop-shadow corner farthest from the core and the porter's trolley rub on the long wall at 0.6 m, 0.9 m in from the core (F06_EAST_HALL_RV, F06_EAST_HALL_OV); the scuffs sit on the actual door positions. The marks render (a frame difference against slice 49's views traces the path down the centre and the scuffs at the doors) but read faintly at production light; strengthening them is open. Verified at WIP 3f3f0d75 (implementation/slice52): apartment batch 204 on the long runner; household state 154 checks, 0 failures; upper kitchens 206 and upper furniture 488, both unchanged; upper lighting 9,257 checks and public doors 17, both 0 failures; the first bath sweep (six baths) 0 failures; the remaining twelve baths, the thirteen upper halls and slice 50's third core group were rerun at the same WIP in five sweeps, all 0 failures (implementation/slice52b); four earlier sweep runs that ran at another WIP are superseded and not cited. The decals are projected (Godot Decal nodes) from game/data/orison_v2/positional_wear.json onto the inherited finishes: no collision, no owner, no lettering. Slice 67 strengthens the walking line, door scuffs and trolley rub to read at production light (verified at 2c25e683, implementation/slice67).</t>
         </is>
       </c>
     </row>
@@ -38039,12 +38039,12 @@
       </c>
       <c r="S511" s="2" t="inlineStr">
         <is>
-          <t>implemented</t>
+          <t>verified</t>
         </is>
       </c>
       <c r="T511" s="2" t="inlineStr">
         <is>
-          <t>The dulled walking line down the hall's middle, foot scuffs on the floor at each apartment door, the mop-shadow corner farthest from the core and the porter's trolley rub on the long wall at 0.6 m, 0.9 m in from the core (F06_WEST_HALL_RV, F06_WEST_HALL_OV); the scuffs sit on the actual door positions. The marks render (a frame difference against slice 49's views traces the path down the centre and the scuffs at the doors) but read faintly at production light; strengthening them is open. Verified at WIP 3f3f0d75 (implementation/slice52): apartment batch 204 on the long runner; household state 154 checks, 0 failures; upper kitchens 206 and upper furniture 488, both unchanged; upper lighting 9,257 checks and public doors 17, both 0 failures; the first bath sweep (six baths) 0 failures; the remaining twelve baths, the thirteen upper halls and slice 50's third core group were rerun at the same WIP in five sweeps, all 0 failures (implementation/slice52b); four earlier sweep runs that ran at another WIP are superseded and not cited. The decals are projected (Godot Decal nodes) from game/data/orison_v2/positional_wear.json onto the inherited finishes: no collision, no owner, no lettering.</t>
+          <t>The dulled walking line down the hall's middle, foot scuffs on the floor at each apartment door, the mop-shadow corner farthest from the core and the porter's trolley rub on the long wall at 0.6 m, 0.9 m in from the core (F06_WEST_HALL_RV, F06_WEST_HALL_OV); the scuffs sit on the actual door positions. The marks render (a frame difference against slice 49's views traces the path down the centre and the scuffs at the doors) but read faintly at production light; strengthening them is open. Verified at WIP 3f3f0d75 (implementation/slice52): apartment batch 204 on the long runner; household state 154 checks, 0 failures; upper kitchens 206 and upper furniture 488, both unchanged; upper lighting 9,257 checks and public doors 17, both 0 failures; the first bath sweep (six baths) 0 failures; the remaining twelve baths, the thirteen upper halls and slice 50's third core group were rerun at the same WIP in five sweeps, all 0 failures (implementation/slice52b); four earlier sweep runs that ran at another WIP are superseded and not cited. The decals are projected (Godot Decal nodes) from game/data/orison_v2/positional_wear.json onto the inherited finishes: no collision, no owner, no lettering. Slice 67 strengthens the walking line, door scuffs and trolley rub to read at production light (verified at 2c25e683, implementation/slice67).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Implement dossier slice 68: the house tank in staves, the mail bank overfull and ajar, 1A's corrected notice
- ROOF_DECK_WEST-004: the house tank's body in timber staves, not brick.
- F01_A_VESTIBULE-003: Evelyn's notice struck through in red pencil with a
  correction slip, pinned inside 1A's entry leaf (the opener reads leaf_notice).
- F01_MAIL_TELEPHONE-001 (partial): two boxes overfull and two doors ajar on a
  letter; no station frames the bank closely yet.
- The completion source back in step with 4D's case (a projection staleness).

Evidence under implementation/slice68/. INERT: no ledger status changes.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/art/reviews/v2_environment_design_20261008/change_register.xlsx
+++ b/art/reviews/v2_environment_design_20261008/change_register.xlsx
@@ -9255,10 +9255,14 @@
       </c>
       <c r="S131" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T131" s="2" t="inlineStr"/>
+          <t>implemented</t>
+        </is>
+      </c>
+      <c r="T131" s="2" t="inlineStr">
+        <is>
+          <t>Partial: two boxes overfull (2C, 4D), their letters drawn into the window cards, and two doors ajar on a letter (1D, 5B); the mail bank suite passes. No sweep station frames the bank closely enough to read its eighteen windows; a close capture is open. Verified at slice 75's WIP 088f987a (implementation/slice68), which carries slices 68 to 75. At 088f987a the fabrication batch's domestic objects and reading nook (11,108 checks) report 0 failures; the mail bank suite passes; wall mounts, roof drainage, public doors (17 waypoints), door casings (107 openings), the apartment door route (45), the golden repair route (94), hardware stock (1,418 checks), hardware drawers (1,309), diner overhead (99), diner counter (160), diner till (130), cobbler fittings (753), laundry fittings (1,139), laundry trade (347) and the laundry route (17), all 0 failures; the roof route 53 waypoints, 0 failures on the long runner after its 180 s run hit the ceiling; three sweeps (nine spaces) and the city sweep's 130 views, 0 failures. The completion interiors suite's one route failure, at 1A's fridge, is identical at the merge-base baseline.</t>
+        </is>
+      </c>
     </row>
     <row r="132">
       <c r="A132" s="2" t="inlineStr">
@@ -10609,10 +10613,14 @@
       </c>
       <c r="S150" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T150" s="2" t="inlineStr"/>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="T150" s="2" t="inlineStr">
+        <is>
+          <t>Evelyn's corrected notice pinned inside 1A's entry leaf at 1.5 m, clear of the knob: a sheet struck through in red pencil with a correction slip pasted over it, no lettering; the leaf's opener reads the record's leaf_notice (F01_A_VESTIBULE_RV, crops/1A_corrected_notice). Verified at slice 75's WIP 088f987a (implementation/slice68), which carries slices 68 to 75. At 088f987a the fabrication batch's domestic objects and reading nook (11,108 checks) report 0 failures; the mail bank suite passes; wall mounts, roof drainage, public doors (17 waypoints), door casings (107 openings), the apartment door route (45), the golden repair route (94), hardware stock (1,418 checks), hardware drawers (1,309), diner overhead (99), diner counter (160), diner till (130), cobbler fittings (753), laundry fittings (1,139), laundry trade (347) and the laundry route (17), all 0 failures; the roof route 53 waypoints, 0 failures on the long runner after its 180 s run hit the ceiling; three sweeps (nine spaces) and the city sweep's 130 views, 0 failures. The completion interiors suite's one route failure, at 1A's fridge, is identical at the merge-base baseline.</t>
+        </is>
+      </c>
     </row>
     <row r="151">
       <c r="A151" s="2" t="inlineStr">
@@ -42483,10 +42491,14 @@
       </c>
       <c r="S571" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T571" s="2" t="inlineStr"/>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="T571" s="2" t="inlineStr">
+        <is>
+          <t>The house tank's body takes the tank-staves finish: upright timber staves where the review saw brick, on its timber legs and cradle (ROOF_DECK_WEST_DT2, crops/tank_staves). Verified at slice 75's WIP 088f987a (implementation/slice68), which carries slices 68 to 75. At 088f987a the fabrication batch's domestic objects and reading nook (11,108 checks) report 0 failures; the mail bank suite passes; wall mounts, roof drainage, public doors (17 waypoints), door casings (107 openings), the apartment door route (45), the golden repair route (94), hardware stock (1,418 checks), hardware drawers (1,309), diner overhead (99), diner counter (160), diner till (130), cobbler fittings (753), laundry fittings (1,139), laundry trade (347) and the laundry route (17), all 0 failures; the roof route 53 waypoints, 0 failures on the long runner after its 180 s run hit the ceiling; three sweeps (nine spaces) and the city sweep's 130 views, 0 failures. The completion interiors suite's one route failure, at 1A's fridge, is identical at the merge-base baseline.</t>
+        </is>
+      </c>
     </row>
     <row r="572">
       <c r="A572" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Implement dossier slice 69: the hardware counter's bell and night card, the capsule box; shop labels
- CITY_SHOP_HARDWARE_PAINT-001 (partial): the brass bell and the night-service
  card at the counter's north end; the box of transmitter capsules on the rack
  is not framed by any capture.
- Shop families gain an optional labels list (Label3D words on the paper).

Evidence under implementation/slice68/. INERT: no ledger status changes.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/art/reviews/v2_environment_design_20261008/change_register.xlsx
+++ b/art/reviews/v2_environment_design_20261008/change_register.xlsx
@@ -6071,10 +6071,14 @@
       </c>
       <c r="S83" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T83" s="2" t="inlineStr"/>
+          <t>implemented</t>
+        </is>
+      </c>
+      <c r="T83" s="2" t="inlineStr">
+        <is>
+          <t>Partial: the brass counter bell and the night-service card (Label3D: NIGHT SERVICE RING BELL STOP) at the counter's north end read in the service-counter capture (crops/hardware_bell_card). The open box of carbon transmitter capsules sits on the north rack's third shelf at the counter end and passes the stock checks, but no capture frames it. Verified at slice 75's WIP 088f987a (implementation/slice68), which carries slices 68 to 75. At 088f987a the fabrication batch's domestic objects and reading nook (11,108 checks) report 0 failures; the mail bank suite passes; wall mounts, roof drainage, public doors (17 waypoints), door casings (107 openings), the apartment door route (45), the golden repair route (94), hardware stock (1,418 checks), hardware drawers (1,309), diner overhead (99), diner counter (160), diner till (130), cobbler fittings (753), laundry fittings (1,139), laundry trade (347) and the laundry route (17), all 0 failures; the roof route 53 waypoints, 0 failures on the long runner after its 180 s run hit the ceiling; three sweeps (nine spaces) and the city sweep's 130 views, 0 failures. The completion interiors suite's one route failure, at 1A's fridge, is identical at the merge-base baseline.</t>
+        </is>
+      </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Implement dossier slice 71: the luncheonette's sugar shakers and a jar of pickled eggs
- CITY_SHOP_LUNCHEONETTE-001: two sugar shakers and a jar of pickled eggs on the
  counter in the cell's own glass, with slice 70's menu board and the existing
  ceiling fan.

Evidence under implementation/slice68/. INERT: no ledger status changes.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/art/reviews/v2_environment_design_20261008/change_register.xlsx
+++ b/art/reviews/v2_environment_design_20261008/change_register.xlsx
@@ -6463,10 +6463,14 @@
       </c>
       <c r="S89" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T89" s="2" t="inlineStr"/>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="T89" s="2" t="inlineStr">
+        <is>
+          <t>The menu board in three columns of white push-in letters (slice 70, Label3D), two sugar shakers and a jar of pickled eggs in the cell's own glass on the counter (slice 71), under the diner overhead family's ceiling fan (menu_face, fan_canopy, crops/diner_shakers_eggs). Verified at slice 75's WIP 088f987a (implementation/slice68), which carries slices 68 to 75. At 088f987a the fabrication batch's domestic objects and reading nook (11,108 checks) report 0 failures; the mail bank suite passes; wall mounts, roof drainage, public doors (17 waypoints), door casings (107 openings), the apartment door route (45), the golden repair route (94), hardware stock (1,418 checks), hardware drawers (1,309), diner overhead (99), diner counter (160), diner till (130), cobbler fittings (753), laundry fittings (1,139), laundry trade (347) and the laundry route (17), all 0 failures; the roof route 53 waypoints, 0 failures on the long runner after its 180 s run hit the ceiling; three sweeps (nine spaces) and the city sweep's 130 views, 0 failures. The completion interiors suite's one route failure, at 1A's fridge, is identical at the merge-base baseline.</t>
+        </is>
+      </c>
     </row>
     <row r="90">
       <c r="A90" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Implement dossier slice 72: the basement toolboard a shadow board, one tool out
- B1_MAINTENANCE_SHOP-002: a painted outline behind every tool on the
  basement toolboard and one outline empty on its peg.

Evidence under implementation/slice68/. INERT: no ledger status changes.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/art/reviews/v2_environment_design_20261008/change_register.xlsx
+++ b/art/reviews/v2_environment_design_20261008/change_register.xlsx
@@ -1717,10 +1717,14 @@
       </c>
       <c r="S18" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T18" s="2" t="inlineStr"/>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="T18" s="2" t="inlineStr">
+        <is>
+          <t>The toolboard is a shadow board: a painted outline behind every tool and one outline empty on its peg, the screwdriver out on a job (b1_toolboard_native, crops/toolboard_silhouettes). Verified at slice 75's WIP 088f987a (implementation/slice68), which carries slices 68 to 75. At 088f987a the fabrication batch's domestic objects and reading nook (11,108 checks) report 0 failures; the mail bank suite passes; wall mounts, roof drainage, public doors (17 waypoints), door casings (107 openings), the apartment door route (45), the golden repair route (94), hardware stock (1,418 checks), hardware drawers (1,309), diner overhead (99), diner counter (160), diner till (130), cobbler fittings (753), laundry fittings (1,139), laundry trade (347) and the laundry route (17), all 0 failures; the roof route 53 waypoints, 0 failures on the long runner after its 180 s run hit the ceiling; three sweeps (nine spaces) and the city sweep's 130 views, 0 failures. The completion interiors suite's one route failure, at 1A's fridge, is identical at the merge-base baseline.</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Implement dossier slice 73: the basement nook's reader, a book tented on the cushion
- B1_PUBLIC_CORE-001: a book left open face down on the north seat's cushion,
  built in the cushion's own assembly so the table's sixty volumes stay.

Evidence under implementation/slice68/. INERT: no ledger status changes.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/art/reviews/v2_environment_design_20261008/change_register.xlsx
+++ b/art/reviews/v2_environment_design_20261008/change_register.xlsx
@@ -901,10 +901,14 @@
       </c>
       <c r="S6" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T6" s="2" t="inlineStr"/>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="T6" s="2" t="inlineStr">
+        <is>
+          <t>The nook's reader: a book left open face down on the north seat's cushion, its covers tented over the spine, beside the mug and the pile on the table; built in the cushion's own assembly so the table's sixty retained volumes stay as they were (B1_NOOK_LAMP_context, crops/nook_tented_book). Verified at slice 75's WIP 088f987a (implementation/slice68), which carries slices 68 to 75. At 088f987a the fabrication batch's domestic objects and reading nook (11,108 checks) report 0 failures; the mail bank suite passes; wall mounts, roof drainage, public doors (17 waypoints), door casings (107 openings), the apartment door route (45), the golden repair route (94), hardware stock (1,418 checks), hardware drawers (1,309), diner overhead (99), diner counter (160), diner till (130), cobbler fittings (753), laundry fittings (1,139), laundry trade (347) and the laundry route (17), all 0 failures; the roof route 53 waypoints, 0 failures on the long runner after its 180 s run hit the ceiling; three sweeps (nine spaces) and the city sweep's 130 views, 0 failures. The completion interiors suite's one route failure, at 1A's fridge, is identical at the merge-base baseline.</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Implement dossier slice 74: the cobbler's floor in leather dust, the dark pairs brown leather
- CITY_SHOP_SHOE_REBUILDING-003 (partial): the floor's dust warm leather, not
  near-black, and the dark pairs brown leather; the red cube, a second bulb and
  the ladder remain.
- CITY_SHOP_SHOE_REBUILDING-001: the last rack and waiting seat already in the
  cobbler family, captured.

Evidence under implementation/slice68/. INERT: no ledger status changes.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/art/reviews/v2_environment_design_20261008/change_register.xlsx
+++ b/art/reviews/v2_environment_design_20261008/change_register.xlsx
@@ -5683,10 +5683,14 @@
       </c>
       <c r="S77" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T77" s="2" t="inlineStr"/>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="T77" s="2" t="inlineStr">
+        <is>
+          <t>Already present in the cobbler fittings family and captured at 088f987a: the slanted rack of iron lasts and shoes on the party wall and the low waiting seat by the door (last_rack, waiting_seat). Verified at slice 75's WIP 088f987a (implementation/slice68), which carries slices 68 to 75. At 088f987a the fabrication batch's domestic objects and reading nook (11,108 checks) report 0 failures; the mail bank suite passes; wall mounts, roof drainage, public doors (17 waypoints), door casings (107 openings), the apartment door route (45), the golden repair route (94), hardware stock (1,418 checks), hardware drawers (1,309), diner overhead (99), diner counter (160), diner till (130), cobbler fittings (753), laundry fittings (1,139), laundry trade (347) and the laundry route (17), all 0 failures; the roof route 53 waypoints, 0 failures on the long runner after its 180 s run hit the ceiling; three sweeps (nine spaces) and the city sweep's 130 views, 0 failures. The completion interiors suite's one route failure, at 1A's fridge, is identical at the merge-base baseline.</t>
+        </is>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
@@ -5807,10 +5811,14 @@
       </c>
       <c r="S79" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T79" s="2" t="inlineStr"/>
+          <t>implemented</t>
+        </is>
+      </c>
+      <c r="T79" s="2" t="inlineStr">
+        <is>
+          <t>Partial: the floor's dust is a warm leather dust instead of near-black and the dark pairs are brown leather with form (floor_dust, last_rack, shoe_rack). The red cube, the second cage bulb over the bench and the ladder are not done. Verified at slice 75's WIP 088f987a (implementation/slice68), which carries slices 68 to 75. At 088f987a the fabrication batch's domestic objects and reading nook (11,108 checks) report 0 failures; the mail bank suite passes; wall mounts, roof drainage, public doors (17 waypoints), door casings (107 openings), the apartment door route (45), the golden repair route (94), hardware stock (1,418 checks), hardware drawers (1,309), diner overhead (99), diner counter (160), diner till (130), cobbler fittings (753), laundry fittings (1,139), laundry trade (347) and the laundry route (17), all 0 failures; the roof route 53 waypoints, 0 failures on the long runner after its 180 s run hit the ceiling; three sweeps (nine spaces) and the city sweep's 130 views, 0 failures. The completion interiors suite's one route failure, at 1A's fridge, is identical at the merge-base baseline.</t>
+        </is>
+      </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Implement dossier slice 75: the laundry's ticket halves in four ages, the oldest parcel row
- CITY_SHOP_MODEL_LAUNDRY-001: the ticket halves on the wire in four ages of
  paper and the top parcel row's wrapping darker.
- Verification of slices 68-75 at this WIP (`slice68`); completion interiors'
  fridge stop is identical at the merge-base baseline.

Evidence under implementation/slice68/. INERT: no ledger status changes.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/art/reviews/v2_environment_design_20261008/change_register.xlsx
+++ b/art/reviews/v2_environment_design_20261008/change_register.xlsx
@@ -5493,10 +5493,14 @@
       </c>
       <c r="S74" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T74" s="2" t="inlineStr"/>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="T74" s="2" t="inlineStr">
+        <is>
+          <t>The ticket halves on the wire in four ages of paper, fresh to a year old, and the top parcel row the oldest, its wrapping darker (tickets, parcel_wall); tinted catalogue paper keys. Verified at slice 75's WIP 088f987a (implementation/slice68), which carries slices 68 to 75. At 088f987a the fabrication batch's domestic objects and reading nook (11,108 checks) report 0 failures; the mail bank suite passes; wall mounts, roof drainage, public doors (17 waypoints), door casings (107 openings), the apartment door route (45), the golden repair route (94), hardware stock (1,418 checks), hardware drawers (1,309), diner overhead (99), diner counter (160), diner till (130), cobbler fittings (753), laundry fittings (1,139), laundry trade (347) and the laundry route (17), all 0 failures; the roof route 53 waypoints, 0 failures on the long runner after its 180 s run hit the ceiling; three sweeps (nine spaces) and the city sweep's 130 views, 0 failures. The completion interiors suite's one route failure, at 1A's fridge, is identical at the merge-base baseline.</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Implement dossier slice 76: the coal chute seated on a boarded bunker; the coal route through the vestibule
- B1_COAL_ROOM-002: a boarded bunker round the fabricated heap, its front board
  gate worked down to two boards with the lifted pair against the wall, and the
  chute's lower lip resting on a bearer across the side walls.
- B1_COAL_ROOM-003 (partial): the heap is already the fabricated mound; grime on
  the whitewash remains.
- The coal delivery route predated the vestibule leaves and stopped at the inner
  door; it now opens both, so the coal heap suite runs end to end.

Evidence under implementation/slice80/. INERT: no ledger status changes.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/art/reviews/v2_environment_design_20261008/change_register.xlsx
+++ b/art/reviews/v2_environment_design_20261008/change_register.xlsx
@@ -1857,10 +1857,14 @@
       </c>
       <c r="S20" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T20" s="2" t="inlineStr"/>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="T20" s="2" t="inlineStr">
+        <is>
+          <t>The chute's lower lip rests on a timber bearer laid across a boarded bunker round the heap: side walls of four horizontal boards from the south wall, a front board gate in slotted posts worked down to two boards with the lifted pair standing against the wall, in coal-dusted dark wood (B1_COAL_ROOM_OV, B1_COAL_ROOM_DT2, coal_bunker, delivery_chute_and_bunker). The coal delivery route predated the vestibule leaves and stopped at the inner door; it now opens both, and the coal heap suite runs end to end. Verified at slice 80's WIP 1d65072d and its runtime-identical predecessor 129e02d3 (implementation/slice80), which carry slices 76 to 80. The patrol stations suite reports seven boxes, seven marks and seven delivered, 0 failures, and V1's watch register (87/87), watch pair (118/118) and tour key (65/65) suites pass; the fabrication batch's domestic objects and service instruments (12,350 checks) report two capture-harness refusals and no fabrication failure (the tour card is not its notice variant's first instance; the tubs leave no clear camera station in front of the rinse taps); the coal heap route 36 waypoints with 9 heap contacts, the laundry route 17 waypoints, the blockout and M08F suites, all 0 failures; four sweeps (twelve spaces), 0 failures. The M08E spatial suite's one failure and the mail access route's one failure are identical at slice 75's 088f987a (base80). The static gate board at 1d65072d matches slice 35's on all 49 gates.</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -1919,10 +1923,14 @@
       </c>
       <c r="S21" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T21" s="2" t="inlineStr"/>
+          <t>implemented</t>
+        </is>
+      </c>
+      <c r="T21" s="2" t="inlineStr">
+        <is>
+          <t>Partial: the heap is the fabricated mound (coal_heap.glb with collision on its own slope; all fourteen old heap boxes retired), now held in slice 76's boarded bunker. Grime on the whitewash beyond slice 60's chute fan is not done. Verified at slice 80's WIP 1d65072d and its runtime-identical predecessor 129e02d3 (implementation/slice80), which carry slices 76 to 80. The patrol stations suite reports seven boxes, seven marks and seven delivered, 0 failures, and V1's watch register (87/87), watch pair (118/118) and tour key (65/65) suites pass; the fabrication batch's domestic objects and service instruments (12,350 checks) report two capture-harness refusals and no fabrication failure (the tour card is not its notice variant's first instance; the tubs leave no clear camera station in front of the rinse taps); the coal heap route 36 waypoints with 9 heap contacts, the laundry route 17 waypoints, the blockout and M08F suites, all 0 failures; four sweeps (twelve spaces), 0 failures. The M08E spatial suite's one failure and the mail access route's one failure are identical at slice 75's 088f987a (base80). The static gate board at 1d65072d matches slice 35's on all 49 gates.</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Implement dossier slice 78: the rinse tubs' taps out of the wet stack, their waste back into it
- B1_LAUNDRY-004: hot and cold out of the west wet stack's face to a pair of
  long-reach bibs over each rinse tub, and a cast-iron waste taking both drain
  tails back into the stack; with slice 77 the laundry's water is complete.
- The domestic-object context inspector treats a solid blockout riser's faces as
  retained walls.

Evidence under implementation/slice80/. INERT: no ledger status changes.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/art/reviews/v2_environment_design_20261008/change_register.xlsx
+++ b/art/reviews/v2_environment_design_20261008/change_register.xlsx
@@ -835,10 +835,14 @@
       </c>
       <c r="S5" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T5" s="2" t="inlineStr"/>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="T5" s="2" t="inlineStr">
+        <is>
+          <t>The laundry's water, slices 77 and 78. The washers: cold and hot mains out of the west wall through flanges, on clips above the hanging belt, a drop and brass bib cock at each machine with a rubber hose to its own fill cock, and a cast-iron floor gully taking each drain hose (washer_supply). The rinse tubs: cold and hot out of the west wet stack's face to a pair of long-reach bibs over each tub's back rim, and a cast-iron waste taking both brass drain tails back into the stack (rinse_taps, B1_LAUNDRY views). The context inspector now treats a solid riser's faces as walls. Verified at slice 80's WIP 1d65072d and its runtime-identical predecessor 129e02d3 (implementation/slice80), which carry slices 76 to 80. The patrol stations suite reports seven boxes, seven marks and seven delivered, 0 failures, and V1's watch register (87/87), watch pair (118/118) and tour key (65/65) suites pass; the fabrication batch's domestic objects and service instruments (12,350 checks) report two capture-harness refusals and no fabrication failure (the tour card is not its notice variant's first instance; the tubs leave no clear camera station in front of the rinse taps); the coal heap route 36 waypoints with 9 heap contacts, the laundry route 17 waypoints, the blockout and M08F suites, all 0 failures; four sweeps (twelve spaces), 0 failures. The M08E spatial suite's one failure and the mail access route's one failure are identical at slice 75's 088f987a (base80). The static gate board at 1d65072d matches slice 35's on all 49 gates.</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Implement dossier slice 79: the night watch's kettle on a gas ring and the tour card
- F01_WATCH-002: a gas ring and enamel kettle on a bracketed shelf on the wall
  the watch room shares with the lobby, fed by a rubber tube from a brass cock,
  and the tour card (Label3D) naming slice 80's patrol boxes.

Evidence under implementation/slice80/. INERT: no ledger status changes.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/art/reviews/v2_environment_design_20261008/change_register.xlsx
+++ b/art/reviews/v2_environment_design_20261008/change_register.xlsx
@@ -9225,10 +9225,14 @@
       </c>
       <c r="S130" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T130" s="2" t="inlineStr"/>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="T130" s="2" t="inlineStr">
+        <is>
+          <t>The night watch's kettle: a cast-iron gas ring with a cream enamel kettle on a deal shelf on iron brackets, on the wall the watch room shares with the lobby, fed by a rubber tube from a brass cock on a gas pipe out of the wall (F01_watch_kettle_native, watch_kettle); and the tour card on the north wall near the key guard, its words a Label3D naming the patrol boxes (F01_WATCH views). Verified at slice 80's WIP 1d65072d and its runtime-identical predecessor 129e02d3 (implementation/slice80), which carry slices 76 to 80. The patrol stations suite reports seven boxes, seven marks and seven delivered, 0 failures, and V1's watch register (87/87), watch pair (118/118) and tour key (65/65) suites pass; the fabrication batch's domestic objects and service instruments (12,350 checks) report two capture-harness refusals and no fabrication failure (the tour card is not its notice variant's first instance; the tubs leave no clear camera station in front of the rinse taps); the coal heap route 36 waypoints with 9 heap contacts, the laundry route 17 waypoints, the blockout and M08F suites, all 0 failures; four sweeps (twelve spaces), 0 failures. The M08E spatial suite's one failure and the mail access route's one failure are identical at slice 75's 088f987a (base80). The static gate board at 1d65072d matches slice 35's on all 49 gates.</t>
+        </is>
+      </c>
     </row>
     <row r="131">
       <c r="A131" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Implement dossier slice 80: a patrol station on every floor; the signal register with seven drops
- At the owner's direction (2026-10-10), V2 mounts a watchman's signal box on
  every floor: station 1 at the boiler, 2 to 6 on the core's north wall of
  floors 2 to 6, 7 in the lobby beside the watch room. They are
  the existing WatchStationProp, on the existing network and worked with the
  existing tour key; OrisonV2PatrolStationsTest proves a full round.
- The signal register grows from four drops to seven; its native fabrication is
  rebuilt from a fresh source census (unchanged parts identical to the old one).
- Verification of slices 76-80 at this WIP (`slice80`).

Evidence under implementation/slice80/. INERT: no ledger status changes.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/art/reviews/v2_environment_design_20261008/change_register.xlsx
+++ b/art/reviews/v2_environment_design_20261008/change_register.xlsx
@@ -9299,12 +9299,12 @@
       </c>
       <c r="S131" s="2" t="inlineStr">
         <is>
-          <t>implemented</t>
+          <t>verified</t>
         </is>
       </c>
       <c r="T131" s="2" t="inlineStr">
         <is>
-          <t>Partial: two boxes overfull (2C, 4D), their letters drawn into the window cards, and two doors ajar on a letter (1D, 5B); the mail bank suite passes. No sweep station frames the bank closely enough to read its eighteen windows; a close capture is open. Verified at slice 75's WIP 088f987a (implementation/slice68), which carries slices 68 to 75. At 088f987a the fabrication batch's domestic objects and reading nook (11,108 checks) report 0 failures; the mail bank suite passes; wall mounts, roof drainage, public doors (17 waypoints), door casings (107 openings), the apartment door route (45), the golden repair route (94), hardware stock (1,418 checks), hardware drawers (1,309), diner overhead (99), diner counter (160), diner till (130), cobbler fittings (753), laundry fittings (1,139), laundry trade (347) and the laundry route (17), all 0 failures; the roof route 53 waypoints, 0 failures on the long runner after its 180 s run hit the ceiling; three sweeps (nine spaces) and the city sweep's 130 views, 0 failures. The completion interiors suite's one route failure, at 1A's fridge, is identical at the merge-base baseline.</t>
+          <t>Partial: two boxes overfull (2C, 4D), their letters drawn into the window cards, and two doors ajar on a letter (1D, 5B); the mail bank suite passes. No sweep station frames the bank closely enough to read its eighteen windows; a close capture is open. Verified at slice 75's WIP 088f987a (implementation/slice68), which carries slices 68 to 75. At 088f987a the fabrication batch's domestic objects and reading nook (11,108 checks) report 0 failures; the mail bank suite passes; wall mounts, roof drainage, public doors (17 waypoints), door casings (107 openings), the apartment door route (45), the golden repair route (94), hardware stock (1,418 checks), hardware drawers (1,309), diner overhead (99), diner counter (160), diner till (130), cobbler fittings (753), laundry fittings (1,139), laundry trade (347) and the laundry route (17), all 0 failures; the roof route 53 waypoints, 0 failures on the long runner after its 180 s run hit the ceiling; three sweeps (nine spaces) and the city sweep's 130 views, 0 failures. The completion interiors suite's one route failure, at 1A's fridge, is identical at the merge-base baseline. A close capture from the mail room at 1d65072d (implementation/slice80, mail_bank_room) reads the bank: card windows on the box doors, the two overfull boxes with letters showing, the two doors ajar on a letter and the empty recesses.</t>
         </is>
       </c>
     </row>
@@ -9431,10 +9431,14 @@
       </c>
       <c r="S133" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T133" s="2" t="inlineStr"/>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="T133" s="2" t="inlineStr">
+        <is>
+          <t>Checked from the mail room's side: the bank's face, its eighteen windows and the slot, faces into the mail room toward its door (mail_bank_room), and the porter board faces into the watch room (F01_WATCH_OV); V1's backs-to-the-corridor facing does not reproduce in V2. Verified at slice 80's WIP 1d65072d and its runtime-identical predecessor 129e02d3 (implementation/slice80), which carry slices 76 to 80. The patrol stations suite reports seven boxes, seven marks and seven delivered, 0 failures, and V1's watch register (87/87), watch pair (118/118) and tour key (65/65) suites pass; the fabrication batch's domestic objects and service instruments (12,350 checks) report two capture-harness refusals and no fabrication failure (the tour card is not its notice variant's first instance; the tubs leave no clear camera station in front of the rinse taps); the coal heap route 36 waypoints with 9 heap contacts, the laundry route 17 waypoints, the blockout and M08F suites, all 0 failures; four sweeps (twelve spaces), 0 failures. The M08E spatial suite's one failure and the mail access route's one failure are identical at slice 75's 088f987a (base80). The static gate board at 1d65072d matches slice 35's on all 49 gates.</t>
+        </is>
+      </c>
     </row>
     <row r="134">
       <c r="A134" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Dossier slice 81: every remaining row statused, each with its reason
- The rows this pass leaves unbuilt are marked deferred (or rejected) with the
  reason each waits: the service spine (BW-006 and its 17 rows), the roof decks'
  sloped support path, the bar's census-bound fabrications, the bodega's missing
  family, the monitor-top kitchen rows' contradictory text, pinned sources
  (5B's larder, the ventilation registers), protected shop layout, catalogue
  gaps (linoleum, chain-link, emissive), light budget and owner rulings.
- Closed from captures: the lobby's V1 rows, the passage hours at 20:00, the
  street's storm state, F04_B_ALCOVE_APPROACH-002 and F05_SERVICE_CROSSING-002
  (not defects); F03_SOUTHWEST_HALL-003's diagonal identified as a picture rail.

Evidence under implementation/slice81/. INERT: no ledger status changes.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/art/reviews/v2_environment_design_20261008/change_register.xlsx
+++ b/art/reviews/v2_environment_design_20261008/change_register.xlsx
@@ -1029,10 +1029,14 @@
       </c>
       <c r="S8" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T8" s="2" t="inlineStr"/>
+          <t>deferred</t>
+        </is>
+      </c>
+      <c r="T8" s="2" t="inlineStr">
+        <is>
+          <t>Still present at 088f987a (B1_PUBLIC_CORE_DT1): a hard bright line at the pier and wall seam beside the stair foot, light through a gap in the shell. Deferred to a shell-joint pass.</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -1305,10 +1309,14 @@
       </c>
       <c r="S12" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T12" s="2" t="inlineStr"/>
+          <t>deferred</t>
+        </is>
+      </c>
+      <c r="T12" s="2" t="inlineStr">
+        <is>
+          <t>Deferred to a lighting-budget decision. Lit, two cage bulbs exceed the 16/16 budget the row names; the unlit warm-emissive alternative needs an emissive finish, and neither the material catalogue nor the fixed-lighting or domestic families carries one.</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -2079,10 +2087,14 @@
       </c>
       <c r="S23" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T23" s="2" t="inlineStr"/>
+          <t>deferred</t>
+        </is>
+      </c>
+      <c r="T23" s="2" t="inlineStr">
+        <is>
+          <t>Deferred. Chain-link reads only through an alpha-scissor finish, which the material catalogue does not have; a new catalogue material comes first (RUL-008).</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -2639,10 +2651,14 @@
       </c>
       <c r="S31" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T31" s="2" t="inlineStr"/>
+          <t>deferred</t>
+        </is>
+      </c>
+      <c r="T31" s="2" t="inlineStr">
+        <is>
+          <t>Deferred: shell work in the blockout and stair generators. The service halls are 1.2 m routes edge to edge, so risers need a chase rather than the hall; the service lift landing and a service stair finish distinct from the public marble are generator changes, as is the dado. The 17 maintenance-evidence rows on the spine wait on it.</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -2705,10 +2721,14 @@
       </c>
       <c r="S32" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T32" s="2" t="inlineStr"/>
+          <t>deferred</t>
+        </is>
+      </c>
+      <c r="T32" s="2" t="inlineStr">
+        <is>
+          <t>Deferred. Window treatments for every apartment window need blind and curtain variants in the window joinery family and a per-unit state driven by the sleep schedules; CITY_FACADE-001 waits on the same family.</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
@@ -2771,10 +2791,14 @@
       </c>
       <c r="S33" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T33" s="2" t="inlineStr"/>
+          <t>deferred</t>
+        </is>
+      </c>
+      <c r="T33" s="2" t="inlineStr">
+        <is>
+          <t>Deferred. Elsewhere in this pass slice 44 gave three households their bedding states and slice 61 put a water line under every curtain hem; the slack variant across the completion beds, the curtains' drawn and gathered variation with hems, flush cabinet mirrors and the receptor hems remain.</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -3179,10 +3203,14 @@
       </c>
       <c r="S39" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T39" s="2" t="inlineStr"/>
+          <t>deferred</t>
+        </is>
+      </c>
+      <c r="T39" s="2" t="inlineStr">
+        <is>
+          <t>Deferred to a shell pass. The white brick is the face of retained masonry and the wet stack where no plaster finish quad is emitted (the B1 laundry's stack shows it too); the fix is the shell builder's side-aware plaster emission.</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
@@ -3479,10 +3507,14 @@
       </c>
       <c r="S43" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T43" s="2" t="inlineStr"/>
+          <t>deferred</t>
+        </is>
+      </c>
+      <c r="T43" s="2" t="inlineStr">
+        <is>
+          <t>Deferred. Mouldings and hardware for the completion wardrobes, nightstands, wall cupboards and the sixteen base cabinets are a casework family pass across F04 and F05.</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
@@ -3545,10 +3577,14 @@
       </c>
       <c r="S44" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T44" s="2" t="inlineStr"/>
+          <t>deferred</t>
+        </is>
+      </c>
+      <c r="T44" s="2" t="inlineStr">
+        <is>
+          <t>Deferred. The terrazzo aggregate scale is in the catalogue's terrazzo maps; re-authoring them at 5 to 15 mm chips with brass strips is a material-catalogue change.</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
@@ -3615,10 +3651,14 @@
       </c>
       <c r="S45" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T45" s="2" t="inlineStr"/>
+          <t>deferred</t>
+        </is>
+      </c>
+      <c r="T45" s="2" t="inlineStr">
+        <is>
+          <t>Deferred: the material catalogue has no linoleum; a battleship-linoleum entry comes before the kitchen floor variant.</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
@@ -3755,10 +3795,14 @@
       </c>
       <c r="S47" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T47" s="2" t="inlineStr"/>
+          <t>deferred</t>
+        </is>
+      </c>
+      <c r="T47" s="2" t="inlineStr">
+        <is>
+          <t>Open. At 088f987a the city sweep's rear stations still show ten of eleven rear rooms bare, with the shared brown cubes and an empty shelf; only the funeral parlour reads (site_rear_*_floor_0). The trade receiving families exist (the laundry receiver is captured by its own suite) but none is framed in its rear cell. Re-anchoring them and a cage bulb per rear room are deferred to a rear-room pass.</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
@@ -3899,10 +3943,14 @@
       </c>
       <c r="S49" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T49" s="2" t="inlineStr"/>
+          <t>deferred</t>
+        </is>
+      </c>
+      <c r="T49" s="2" t="inlineStr">
+        <is>
+          <t>Deferred. Ash cans need a street-furniture owner inside the street's route and containment tests, and the droppings' fly shimmer is gated on the commensals ruling (C2).</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
@@ -4019,10 +4067,14 @@
       </c>
       <c r="S51" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T51" s="2" t="inlineStr"/>
+          <t>deferred</t>
+        </is>
+      </c>
+      <c r="T51" s="2" t="inlineStr">
+        <is>
+          <t>Deferred: a steam plume is a WeatherFX billboard, outside this pass's static families.</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
@@ -4081,10 +4133,14 @@
       </c>
       <c r="S52" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T52" s="2" t="inlineStr"/>
+          <t>deferred</t>
+        </is>
+      </c>
+      <c r="T52" s="2" t="inlineStr">
+        <is>
+          <t>Deferred: sound only (the acoustic and weather bed); no visual dossier change.</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
@@ -4217,10 +4273,14 @@
       </c>
       <c r="S54" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T54" s="2" t="inlineStr"/>
+          <t>deferred</t>
+        </is>
+      </c>
+      <c r="T54" s="2" t="inlineStr">
+        <is>
+          <t>Deferred to a city-shell pass: the closure masses, alley walls and their finishes are the city generator's geometry. Brick maps, window grids and cornices on every closure mass are open.</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
@@ -4283,10 +4343,14 @@
       </c>
       <c r="S55" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T55" s="2" t="inlineStr"/>
+          <t>deferred</t>
+        </is>
+      </c>
+      <c r="T55" s="2" t="inlineStr">
+        <is>
+          <t>Measured, deferred. The city sweep with the simulated storm (WEATHER_SIMULATE=storm, WEATHER_SEED 7) at 129e02d3 renders the same as the clear sweep, a mean pixel difference of 0.12 in 255 on facade_front_wide (implementation/slice81, both sweeps 130 views, 0 failures): the V2 runtime composes no weather owner, so the brief's quiet storm (live rain, near rain suppressed, the puddle pass) is V1's weather, not yet ported. The dry road and clear sky are therefore what V2 ships, not a capture accident; the storm's port is the open work.</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
@@ -4349,10 +4413,14 @@
       </c>
       <c r="S56" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T56" s="2" t="inlineStr"/>
+          <t>deferred</t>
+        </is>
+      </c>
+      <c r="T56" s="2" t="inlineStr">
+        <is>
+          <t>Deferred with BW-007: ice cards and curtain states need the window joinery family's states.</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
@@ -4415,10 +4483,14 @@
       </c>
       <c r="S57" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T57" s="2" t="inlineStr"/>
+          <t>deferred</t>
+        </is>
+      </c>
+      <c r="T57" s="2" t="inlineStr">
+        <is>
+          <t>Deferred: positional wear on the front door's handle, lock, bell push, mat and stone is a facade wear pass.</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
@@ -4547,10 +4619,14 @@
       </c>
       <c r="S59" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T59" s="2" t="inlineStr"/>
+          <t>deferred</t>
+        </is>
+      </c>
+      <c r="T59" s="2" t="inlineStr">
+        <is>
+          <t>Deferred: rut and leaf-litter decals on the alley ground are an alley wear pass.</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
@@ -4605,10 +4681,14 @@
       </c>
       <c r="S60" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T60" s="2" t="inlineStr"/>
+          <t>deferred</t>
+        </is>
+      </c>
+      <c r="T60" s="2" t="inlineStr">
+        <is>
+          <t>Deferred to a city-shell pass: the closure masses, alley walls and their finishes are the city generator's geometry. One lit pane on the north neighbour's back is a shell emissive.</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
@@ -4675,10 +4755,14 @@
       </c>
       <c r="S61" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T61" s="2" t="inlineStr"/>
+          <t>deferred</t>
+        </is>
+      </c>
+      <c r="T61" s="2" t="inlineStr">
+        <is>
+          <t>Deferred to a city-shell pass: the closure masses, alley walls and their finishes are the city generator's geometry. Painted cast-iron leaders with stain fans, coping on the wall tops and a finished closing plane are open.</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
@@ -4861,10 +4945,14 @@
       </c>
       <c r="S64" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T64" s="2" t="inlineStr"/>
+          <t>deferred</t>
+        </is>
+      </c>
+      <c r="T64" s="2" t="inlineStr">
+        <is>
+          <t>Deferred: the reflected train light and the stirring scrap are lighting and weather effects.</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
@@ -4919,10 +5007,14 @@
       </c>
       <c r="S65" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T65" s="2" t="inlineStr"/>
+          <t>deferred</t>
+        </is>
+      </c>
+      <c r="T65" s="2" t="inlineStr">
+        <is>
+          <t>Deferred: a second station at the kerb opposite the kiosk is a sweep addition; not a defect until seen closer, as the row says.</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
@@ -4993,10 +5085,14 @@
       </c>
       <c r="S66" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T66" s="2" t="inlineStr"/>
+          <t>deferred</t>
+        </is>
+      </c>
+      <c r="T66" s="2" t="inlineStr">
+        <is>
+          <t>Deferred. The bodega has no V2 fittings family to carry new stock or replace its stand-ins: its interior is the passage's generic shelf stock, so the cards, notions counter, ledger and register need a bodega family first.</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
@@ -5063,10 +5159,14 @@
       </c>
       <c r="S67" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T67" s="2" t="inlineStr"/>
+          <t>deferred</t>
+        </is>
+      </c>
+      <c r="T67" s="2" t="inlineStr">
+        <is>
+          <t>Deferred. The bodega has no V2 fittings family to carry new stock or replace its stand-ins: its interior is the passage's generic shelf stock, so the cards, notions counter, ledger and register need a bodega family first.</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
@@ -5121,10 +5221,14 @@
       </c>
       <c r="S68" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T68" s="2" t="inlineStr"/>
+          <t>deferred</t>
+        </is>
+      </c>
+      <c r="T68" s="2" t="inlineStr">
+        <is>
+          <t>Deferred. The bodega has no V2 fittings family to carry new stock or replace its stand-ins: its interior is the passage's generic shelf stock, so the cards, notions counter, ledger and register need a bodega family first.</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
@@ -5183,10 +5287,14 @@
       </c>
       <c r="S69" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T69" s="2" t="inlineStr"/>
+          <t>deferred</t>
+        </is>
+      </c>
+      <c r="T69" s="2" t="inlineStr">
+        <is>
+          <t>Deferred. The bodega has no V2 fittings family to carry new stock or replace its stand-ins: its interior is the passage's generic shelf stock, so the cards, notions counter, ledger and register need a bodega family first.</t>
+        </is>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
@@ -5257,10 +5365,14 @@
       </c>
       <c r="S70" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T70" s="2" t="inlineStr"/>
+          <t>deferred</t>
+        </is>
+      </c>
+      <c r="T70" s="2" t="inlineStr">
+        <is>
+          <t>Deferred. The bodega has no V2 fittings family to carry new stock or replace its stand-ins: its interior is the passage's generic shelf stock, so the cards, notions counter, ledger and register need a bodega family first.</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
@@ -5319,10 +5431,14 @@
       </c>
       <c r="S71" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T71" s="2" t="inlineStr"/>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="T71" s="2" t="inlineStr">
+        <is>
+          <t>Checked: at the sweep's hour the passage hours director reports OPEN with ten grilles folded (sweep_city log: [PASSAGE HOURS] OPEN; 10 grilles folded; 10 close after 02:00, the hardware store keeps night service), and the shop interior stations show lit, trading shops. The director's clock binding is correct.</t>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
@@ -5385,10 +5501,14 @@
       </c>
       <c r="S72" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T72" s="2" t="inlineStr"/>
+          <t>deferred</t>
+        </is>
+      </c>
+      <c r="T72" s="2" t="inlineStr">
+        <is>
+          <t>Deferred: the parcel shelf, the ghost sign on the throat's brick and the anachronistic tube are passage additions for a later pass.</t>
+        </is>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
@@ -5443,10 +5563,14 @@
       </c>
       <c r="S73" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T73" s="2" t="inlineStr"/>
+          <t>deferred</t>
+        </is>
+      </c>
+      <c r="T73" s="2" t="inlineStr">
+        <is>
+          <t>Deferred: the directory's extra line is a passage directory change for a later pass.</t>
+        </is>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
@@ -5567,10 +5691,14 @@
       </c>
       <c r="S75" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T75" s="2" t="inlineStr"/>
+          <t>deferred</t>
+        </is>
+      </c>
+      <c r="T75" s="2" t="inlineStr">
+        <is>
+          <t>Deferred: the gas ring's glow, a steam billboard and a wet floor mask are effects.</t>
+        </is>
+      </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
@@ -5633,10 +5761,14 @@
       </c>
       <c r="S76" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T76" s="2" t="inlineStr"/>
+          <t>deferred</t>
+        </is>
+      </c>
+      <c r="T76" s="2" t="inlineStr">
+        <is>
+          <t>Deferred. The garments on the rail are the fitted family's flat shirt boards; cloth-batch garments with folds need the cloth pipeline. The parcel wall is the laundry trade family's wrapped parcels (slice 75 aged its top row).</t>
+        </is>
+      </c>
     </row>
     <row r="77">
       <c r="A77" s="2" t="inlineStr">
@@ -5761,10 +5893,14 @@
       </c>
       <c r="S78" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T78" s="2" t="inlineStr"/>
+          <t>deferred</t>
+        </is>
+      </c>
+      <c r="T78" s="2" t="inlineStr">
+        <is>
+          <t>Deferred: a dust film with a clean rectangle under the ledger is a cobbler counter wear pass.</t>
+        </is>
+      </c>
     </row>
     <row r="79">
       <c r="A79" s="2" t="inlineStr">
@@ -6243,10 +6379,14 @@
       </c>
       <c r="S85" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T85" s="2" t="inlineStr"/>
+          <t>deferred</t>
+        </is>
+      </c>
+      <c r="T85" s="2" t="inlineStr">
+        <is>
+          <t>Deferred. Free-standing caskets need new source records, and the shops' source layout is in the protected building_layout.json (RUL-004).</t>
+        </is>
+      </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
@@ -6627,10 +6767,14 @@
       </c>
       <c r="S91" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T91" s="2" t="inlineStr"/>
+          <t>deferred</t>
+        </is>
+      </c>
+      <c r="T91" s="2" t="inlineStr">
+        <is>
+          <t>Deferred. The register now reads with its keys in the diner till family (counter_service at 088f987a); the cream pole and the black cabinet remain to be identified and modelled (diner_backbar.md's cooler).</t>
+        </is>
+      </c>
     </row>
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
@@ -6693,10 +6837,14 @@
       </c>
       <c r="S92" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T92" s="2" t="inlineStr"/>
+          <t>deferred</t>
+        </is>
+      </c>
+      <c r="T92" s="2" t="inlineStr">
+        <is>
+          <t>Deferred to a lighting-budget decision: the carboy backlight is a practical light.</t>
+        </is>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
@@ -6759,10 +6907,14 @@
       </c>
       <c r="S93" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T93" s="2" t="inlineStr"/>
+          <t>deferred</t>
+        </is>
+      </c>
+      <c r="T93" s="2" t="inlineStr">
+        <is>
+          <t>Deferred: the show-globe glazing (with -001), nickel fountain taps and drawer slips are a druggist fittings pass.</t>
+        </is>
+      </c>
     </row>
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
@@ -6883,10 +7035,14 @@
       </c>
       <c r="S95" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T95" s="2" t="inlineStr"/>
+          <t>deferred</t>
+        </is>
+      </c>
+      <c r="T95" s="2" t="inlineStr">
+        <is>
+          <t>Deferred for canon: the headline is the election result in telegram grammar, and the Bible does not yet fix the line; slice 65's broadsides are wordless.</t>
+        </is>
+      </c>
     </row>
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
@@ -7645,10 +7801,14 @@
       </c>
       <c r="S106" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T106" s="2" t="inlineStr"/>
+          <t>deferred</t>
+        </is>
+      </c>
+      <c r="T106" s="2" t="inlineStr">
+        <is>
+          <t>Deferred to a bar pass. The bar's fittings are native fabrications bound to source censuses by SHA-256 (bar_furniture, bar_pool, bar_stage, bar_instruments); each addition is a census re-capture and refabrication, the path slice 80 took for the signal register.</t>
+        </is>
+      </c>
     </row>
     <row r="107">
       <c r="A107" s="2" t="inlineStr">
@@ -7707,10 +7867,14 @@
       </c>
       <c r="S107" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T107" s="2" t="inlineStr"/>
+          <t>deferred</t>
+        </is>
+      </c>
+      <c r="T107" s="2" t="inlineStr">
+        <is>
+          <t>Deferred to a bar pass. The bar's fittings are native fabrications bound to source censuses by SHA-256 (bar_furniture, bar_pool, bar_stage, bar_instruments); each addition is a census re-capture and refabrication, the path slice 80 took for the signal register.</t>
+        </is>
+      </c>
     </row>
     <row r="108">
       <c r="A108" s="2" t="inlineStr">
@@ -7765,10 +7929,14 @@
       </c>
       <c r="S108" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T108" s="2" t="inlineStr"/>
+          <t>deferred</t>
+        </is>
+      </c>
+      <c r="T108" s="2" t="inlineStr">
+        <is>
+          <t>Deferred: gated on an owner ruling on Prohibition (the row's own condition).</t>
+        </is>
+      </c>
     </row>
     <row r="109">
       <c r="A109" s="2" t="inlineStr">
@@ -7827,10 +7995,14 @@
       </c>
       <c r="S109" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T109" s="2" t="inlineStr"/>
+          <t>deferred</t>
+        </is>
+      </c>
+      <c r="T109" s="2" t="inlineStr">
+        <is>
+          <t>Deferred to a bar pass. The bar's fittings are native fabrications bound to source censuses by SHA-256 (bar_furniture, bar_pool, bar_stage, bar_instruments); each addition is a census re-capture and refabrication, the path slice 80 took for the signal register.</t>
+        </is>
+      </c>
     </row>
     <row r="110">
       <c r="A110" s="2" t="inlineStr">
@@ -7897,10 +8069,14 @@
       </c>
       <c r="S110" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T110" s="2" t="inlineStr"/>
+          <t>deferred</t>
+        </is>
+      </c>
+      <c r="T110" s="2" t="inlineStr">
+        <is>
+          <t>Deferred to a bar pass. The bar's fittings are native fabrications bound to source censuses by SHA-256 (bar_furniture, bar_pool, bar_stage, bar_instruments); each addition is a census re-capture and refabrication, the path slice 80 took for the signal register.</t>
+        </is>
+      </c>
     </row>
     <row r="111">
       <c r="A111" s="2" t="inlineStr">
@@ -7955,10 +8131,14 @@
       </c>
       <c r="S111" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T111" s="2" t="inlineStr"/>
+          <t>deferred</t>
+        </is>
+      </c>
+      <c r="T111" s="2" t="inlineStr">
+        <is>
+          <t>Deferred to a bar pass. The bar's fittings are native fabrications bound to source censuses by SHA-256 (bar_furniture, bar_pool, bar_stage, bar_instruments); each addition is a census re-capture and refabrication, the path slice 80 took for the signal register.</t>
+        </is>
+      </c>
     </row>
     <row r="112">
       <c r="A112" s="2" t="inlineStr">
@@ -8013,10 +8193,14 @@
       </c>
       <c r="S112" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T112" s="2" t="inlineStr"/>
+          <t>deferred</t>
+        </is>
+      </c>
+      <c r="T112" s="2" t="inlineStr">
+        <is>
+          <t>Deferred to a bar pass. The bar's fittings are native fabrications bound to source censuses by SHA-256 (bar_furniture, bar_pool, bar_stage, bar_instruments); each addition is a census re-capture and refabrication, the path slice 80 took for the signal register.</t>
+        </is>
+      </c>
     </row>
     <row r="113">
       <c r="A113" s="2" t="inlineStr">
@@ -8071,10 +8255,14 @@
       </c>
       <c r="S113" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T113" s="2" t="inlineStr"/>
+          <t>deferred</t>
+        </is>
+      </c>
+      <c r="T113" s="2" t="inlineStr">
+        <is>
+          <t>Deferred: gated on an owner ruling on Prohibition (the row's own condition).</t>
+        </is>
+      </c>
     </row>
     <row r="114">
       <c r="A114" s="2" t="inlineStr">
@@ -8137,10 +8325,14 @@
       </c>
       <c r="S114" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T114" s="2" t="inlineStr"/>
+          <t>deferred</t>
+        </is>
+      </c>
+      <c r="T114" s="2" t="inlineStr">
+        <is>
+          <t>Deferred to a bar pass. The bar's fittings are native fabrications bound to source censuses by SHA-256 (bar_furniture, bar_pool, bar_stage, bar_instruments); each addition is a census re-capture and refabrication, the path slice 80 took for the signal register.</t>
+        </is>
+      </c>
     </row>
     <row r="115">
       <c r="A115" s="2" t="inlineStr">
@@ -8203,10 +8395,14 @@
       </c>
       <c r="S115" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T115" s="2" t="inlineStr"/>
+          <t>deferred</t>
+        </is>
+      </c>
+      <c r="T115" s="2" t="inlineStr">
+        <is>
+          <t>Deferred to a bar pass. The bar's fittings are native fabrications bound to source censuses by SHA-256 (bar_furniture, bar_pool, bar_stage, bar_instruments); each addition is a census re-capture and refabrication, the path slice 80 took for the signal register.</t>
+        </is>
+      </c>
     </row>
     <row r="116">
       <c r="A116" s="2" t="inlineStr">
@@ -8269,10 +8465,14 @@
       </c>
       <c r="S116" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T116" s="2" t="inlineStr"/>
+          <t>deferred</t>
+        </is>
+      </c>
+      <c r="T116" s="2" t="inlineStr">
+        <is>
+          <t>Deferred to a bar pass. The bar's fittings are native fabrications bound to source censuses by SHA-256 (bar_furniture, bar_pool, bar_stage, bar_instruments); each addition is a census re-capture and refabrication, the path slice 80 took for the signal register.</t>
+        </is>
+      </c>
     </row>
     <row r="117">
       <c r="A117" s="2" t="inlineStr">
@@ -8335,10 +8535,14 @@
       </c>
       <c r="S117" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T117" s="2" t="inlineStr"/>
+          <t>deferred</t>
+        </is>
+      </c>
+      <c r="T117" s="2" t="inlineStr">
+        <is>
+          <t>Deferred to a bar pass. The bar's fittings are native fabrications bound to source censuses by SHA-256 (bar_furniture, bar_pool, bar_stage, bar_instruments); each addition is a census re-capture and refabrication, the path slice 80 took for the signal register.</t>
+        </is>
+      </c>
     </row>
     <row r="118">
       <c r="A118" s="2" t="inlineStr">
@@ -8401,10 +8605,14 @@
       </c>
       <c r="S118" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T118" s="2" t="inlineStr"/>
+          <t>deferred</t>
+        </is>
+      </c>
+      <c r="T118" s="2" t="inlineStr">
+        <is>
+          <t>Deferred to a bar pass. The bar's fittings are native fabrications bound to source censuses by SHA-256 (bar_furniture, bar_pool, bar_stage, bar_instruments); each addition is a census re-capture and refabrication, the path slice 80 took for the signal register.</t>
+        </is>
+      </c>
     </row>
     <row r="119">
       <c r="A119" s="2" t="inlineStr">
@@ -8479,10 +8687,14 @@
       </c>
       <c r="S119" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T119" s="2" t="inlineStr"/>
+          <t>deferred</t>
+        </is>
+      </c>
+      <c r="T119" s="2" t="inlineStr">
+        <is>
+          <t>Deferred. The aprons are city-owned exterior ground inside the front entry route and containment tests; no static-object family mounts there yet.</t>
+        </is>
+      </c>
     </row>
     <row r="120">
       <c r="A120" s="2" t="inlineStr">
@@ -8537,10 +8749,14 @@
       </c>
       <c r="S120" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T120" s="2" t="inlineStr"/>
+          <t>deferred</t>
+        </is>
+      </c>
+      <c r="T120" s="2" t="inlineStr">
+        <is>
+          <t>Deferred with CITY_SHOP_NEWS_CIGARS-002 for the election canon, and the apron owner.</t>
+        </is>
+      </c>
     </row>
     <row r="121">
       <c r="A121" s="2" t="inlineStr">
@@ -8603,10 +8819,14 @@
       </c>
       <c r="S121" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T121" s="2" t="inlineStr"/>
+          <t>deferred</t>
+        </is>
+      </c>
+      <c r="T121" s="2" t="inlineStr">
+        <is>
+          <t>Deferred. The rear apron is city-owned ground inside the service alley's route test; no static-object family mounts there yet.</t>
+        </is>
+      </c>
     </row>
     <row r="122">
       <c r="A122" s="2" t="inlineStr">
@@ -9015,10 +9235,14 @@
       </c>
       <c r="S127" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T127" s="2" t="inlineStr"/>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="T127" s="2" t="inlineStr">
+        <is>
+          <t>Closed: no teal order-board slabs and no floating nameplates in any lobby tile at 088f987a (F01_LOBBY OV, RV, TH, DT1 to DT3); the V1 rows do not reproduce in V2.</t>
+        </is>
+      </c>
     </row>
     <row r="128">
       <c r="A128" s="2" t="inlineStr">
@@ -9077,10 +9301,14 @@
       </c>
       <c r="S128" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T128" s="2" t="inlineStr"/>
+          <t>verified</t>
+        </is>
+      </c>
+      <c r="T128" s="2" t="inlineStr">
+        <is>
+          <t>Closed: no yellow numbered placard and no white brick patch in the lobby at 088f987a (F01_LOBBY_OV, F01_LOBBY_RV).</t>
+        </is>
+      </c>
     </row>
     <row r="129">
       <c r="A129" s="2" t="inlineStr">
@@ -9699,10 +9927,14 @@
       </c>
       <c r="S137" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T137" s="2" t="inlineStr"/>
+          <t>deferred</t>
+        </is>
+      </c>
+      <c r="T137" s="2" t="inlineStr">
+        <is>
+          <t>Deferred to a city-shell pass: the closure masses, alley walls and their finishes are the city generator's geometry. The reading room's windows look onto the light court's unfinished face.</t>
+        </is>
+      </c>
     </row>
     <row r="138">
       <c r="A138" s="2" t="inlineStr">
@@ -9995,10 +10227,14 @@
       </c>
       <c r="S141" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T141" s="2" t="inlineStr"/>
+          <t>deferred</t>
+        </is>
+      </c>
+      <c r="T141" s="2" t="inlineStr">
+        <is>
+          <t>Deferred with BW-006. The service spine's halls are 1.2 m wide and the whole width is the route, so the riser cluster, crate and hose this row asks for have no place outside it until BW-006 gives the spine its risers in a chase, its dado and its lighting.</t>
+        </is>
+      </c>
     </row>
     <row r="142">
       <c r="A142" s="2" t="inlineStr">
@@ -10073,10 +10309,14 @@
       </c>
       <c r="S142" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T142" s="2" t="inlineStr"/>
+          <t>deferred</t>
+        </is>
+      </c>
+      <c r="T142" s="2" t="inlineStr">
+        <is>
+          <t>Deferred with BW-006. The service spine's halls are 1.2 m wide and the whole width is the route, so the riser cluster, crate and hose this row asks for have no place outside it until BW-006 gives the spine its risers in a chase, its dado and its lighting.</t>
+        </is>
+      </c>
     </row>
     <row r="143">
       <c r="A143" s="2" t="inlineStr">
@@ -10139,10 +10379,14 @@
       </c>
       <c r="S143" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T143" s="2" t="inlineStr"/>
+          <t>deferred</t>
+        </is>
+      </c>
+      <c r="T143" s="2" t="inlineStr">
+        <is>
+          <t>Deferred with BW-006: the dumbwaiter stands on the 1.2 m route and there is no floor outside it for a sack truck and crates.</t>
+        </is>
+      </c>
     </row>
     <row r="144">
       <c r="A144" s="2" t="inlineStr">
@@ -10353,10 +10597,14 @@
       </c>
       <c r="S146" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T146" s="2" t="inlineStr"/>
+          <t>deferred</t>
+        </is>
+      </c>
+      <c r="T146" s="2" t="inlineStr">
+        <is>
+          <t>Deferred with BW-006: the service core's door leaf and landing panel are the spine's finish.</t>
+        </is>
+      </c>
     </row>
     <row r="147">
       <c r="A147" s="2" t="inlineStr">
@@ -11333,10 +11581,14 @@
       </c>
       <c r="S158" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T158" s="2" t="inlineStr"/>
+          <t>deferred</t>
+        </is>
+      </c>
+      <c r="T158" s="2" t="inlineStr">
+        <is>
+          <t>Deferred for an owner restatement. The row's title asks for monitor-top electric evidence, but its construction (an ice card in the kitchen window, a zinc drip tray with a tide line) is icebox evidence, and this household's fridge is a FridgeMonitor in household_fridges.json; a monitor-top unit takes no ice. The icebox households already have their drip pans (slice 18).</t>
+        </is>
+      </c>
     </row>
     <row r="159">
       <c r="A159" s="2" t="inlineStr">
@@ -14629,10 +14881,14 @@
       </c>
       <c r="S200" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T200" s="2" t="inlineStr"/>
+          <t>deferred</t>
+        </is>
+      </c>
+      <c r="T200" s="2" t="inlineStr">
+        <is>
+          <t>Deferred with BW-006. The service spine's halls are 1.2 m wide and the whole width is the route, so the riser cluster, crate and hose this row asks for have no place outside it until BW-006 gives the spine its risers in a chase, its dado and its lighting.</t>
+        </is>
+      </c>
     </row>
     <row r="201">
       <c r="A201" s="2" t="inlineStr">
@@ -14707,10 +14963,14 @@
       </c>
       <c r="S201" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T201" s="2" t="inlineStr"/>
+          <t>deferred</t>
+        </is>
+      </c>
+      <c r="T201" s="2" t="inlineStr">
+        <is>
+          <t>Deferred with BW-006. The service spine's halls are 1.2 m wide and the whole width is the route, so the riser cluster, crate and hose this row asks for have no place outside it until BW-006 gives the spine its risers in a chase, its dado and its lighting.</t>
+        </is>
+      </c>
     </row>
     <row r="202">
       <c r="A202" s="2" t="inlineStr">
@@ -14785,10 +15045,14 @@
       </c>
       <c r="S202" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T202" s="2" t="inlineStr"/>
+          <t>deferred</t>
+        </is>
+      </c>
+      <c r="T202" s="2" t="inlineStr">
+        <is>
+          <t>Deferred with BW-006. The service spine's halls are 1.2 m wide and the whole width is the route, so the riser cluster, crate and hose this row asks for have no place outside it until BW-006 gives the spine its risers in a chase, its dado and its lighting.</t>
+        </is>
+      </c>
     </row>
     <row r="203">
       <c r="A203" s="2" t="inlineStr">
@@ -14999,10 +15263,14 @@
       </c>
       <c r="S205" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T205" s="2" t="inlineStr"/>
+          <t>deferred</t>
+        </is>
+      </c>
+      <c r="T205" s="2" t="inlineStr">
+        <is>
+          <t>Deferred with BW-006: the plain service stair and the service lift landing are generator changes.</t>
+        </is>
+      </c>
     </row>
     <row r="206">
       <c r="A206" s="2" t="inlineStr">
@@ -15565,10 +15833,14 @@
       </c>
       <c r="S212" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T212" s="2" t="inlineStr"/>
+          <t>deferred</t>
+        </is>
+      </c>
+      <c r="T212" s="2" t="inlineStr">
+        <is>
+          <t>Deferred. The radio's table, the projector stand and the deck on the coffee table are placed, and a cable form with clips along the skirting from each device to the plate beside the switch is a follow-up.</t>
+        </is>
+      </c>
     </row>
     <row r="213">
       <c r="A213" s="2" t="inlineStr">
@@ -19885,10 +20157,14 @@
       </c>
       <c r="S268" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T268" s="2" t="inlineStr"/>
+          <t>deferred</t>
+        </is>
+      </c>
+      <c r="T268" s="2" t="inlineStr">
+        <is>
+          <t>Deferred with BW-006. The service spine's halls are 1.2 m wide and the whole width is the route, so the riser cluster, crate and hose this row asks for have no place outside it until BW-006 gives the spine its risers in a chase, its dado and its lighting.</t>
+        </is>
+      </c>
     </row>
     <row r="269">
       <c r="A269" s="2" t="inlineStr">
@@ -19943,10 +20219,14 @@
       </c>
       <c r="S269" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T269" s="2" t="inlineStr"/>
+          <t>deferred</t>
+        </is>
+      </c>
+      <c r="T269" s="2" t="inlineStr">
+        <is>
+          <t>Deferred with BW-006: the crossing's ceiling planes are the spine's shell geometry.</t>
+        </is>
+      </c>
     </row>
     <row r="270">
       <c r="A270" s="2" t="inlineStr">
@@ -20021,10 +20301,14 @@
       </c>
       <c r="S270" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T270" s="2" t="inlineStr"/>
+          <t>deferred</t>
+        </is>
+      </c>
+      <c r="T270" s="2" t="inlineStr">
+        <is>
+          <t>Deferred with BW-006. The service spine's halls are 1.2 m wide and the whole width is the route, so the riser cluster, crate and hose this row asks for have no place outside it until BW-006 gives the spine its risers in a chase, its dado and its lighting.</t>
+        </is>
+      </c>
     </row>
     <row r="271">
       <c r="A271" s="2" t="inlineStr">
@@ -20099,10 +20383,14 @@
       </c>
       <c r="S271" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T271" s="2" t="inlineStr"/>
+          <t>deferred</t>
+        </is>
+      </c>
+      <c r="T271" s="2" t="inlineStr">
+        <is>
+          <t>Deferred with BW-006. The service spine's halls are 1.2 m wide and the whole width is the route, so the riser cluster, crate and hose this row asks for have no place outside it until BW-006 gives the spine its risers in a chase, its dado and its lighting.</t>
+        </is>
+      </c>
     </row>
     <row r="272">
       <c r="A272" s="2" t="inlineStr">
@@ -20469,10 +20757,14 @@
       </c>
       <c r="S276" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T276" s="2" t="inlineStr"/>
+          <t>deferred</t>
+        </is>
+      </c>
+      <c r="T276" s="2" t="inlineStr">
+        <is>
+          <t>Identified, deferred. A node probe of the hall's upper volume at b2cf2b70 finds no pipe, only walls, ceilings and 3D's vestibule; the diagonal is the picture rail on the west wall, which stops mid-wall short of 3D's door casing and reads as a loose rod in perspective (f03sw_rail). Ending it at the casing is a millwork-pass item.</t>
+        </is>
+      </c>
     </row>
     <row r="277">
       <c r="A277" s="2" t="inlineStr">
@@ -21179,10 +21471,14 @@
       </c>
       <c r="S285" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T285" s="2" t="inlineStr"/>
+          <t>deferred</t>
+        </is>
+      </c>
+      <c r="T285" s="2" t="inlineStr">
+        <is>
+          <t>Deferred for an owner restatement. The row's title asks for monitor-top electric evidence, but its construction (an ice card in the kitchen window, a zinc drip tray with a tide line) is icebox evidence, and this household's fridge is a FridgeMonitor in household_fridges.json; a monitor-top unit takes no ice. The icebox households already have their drip pans (slice 18).</t>
+        </is>
+      </c>
     </row>
     <row r="286">
       <c r="A286" s="2" t="inlineStr">
@@ -25201,10 +25497,14 @@
       </c>
       <c r="S338" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T338" s="2" t="inlineStr"/>
+          <t>deferred</t>
+        </is>
+      </c>
+      <c r="T338" s="2" t="inlineStr">
+        <is>
+          <t>Deferred: the landing doors' painted-steel finish, sight glass and sill belong to the lift (elevator.gd), and the brick around them is BW-015's plaster emission.</t>
+        </is>
+      </c>
     </row>
     <row r="339">
       <c r="A339" s="2" t="inlineStr">
@@ -25497,10 +25797,14 @@
       </c>
       <c r="S342" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T342" s="2" t="inlineStr"/>
+          <t>deferred</t>
+        </is>
+      </c>
+      <c r="T342" s="2" t="inlineStr">
+        <is>
+          <t>Deferred with BW-006. The service spine's halls are 1.2 m wide and the whole width is the route, so the riser cluster, crate and hose this row asks for have no place outside it until BW-006 gives the spine its risers in a chase, its dado and its lighting.</t>
+        </is>
+      </c>
     </row>
     <row r="343">
       <c r="A343" s="2" t="inlineStr">
@@ -25563,10 +25867,14 @@
       </c>
       <c r="S343" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T343" s="2" t="inlineStr"/>
+          <t>deferred</t>
+        </is>
+      </c>
+      <c r="T343" s="2" t="inlineStr">
+        <is>
+          <t>Deferred with BW-006: the crossing's wainscot relief and floor strip are spine finish.</t>
+        </is>
+      </c>
     </row>
     <row r="344">
       <c r="A344" s="2" t="inlineStr">
@@ -25641,10 +25949,14 @@
       </c>
       <c r="S344" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T344" s="2" t="inlineStr"/>
+          <t>deferred</t>
+        </is>
+      </c>
+      <c r="T344" s="2" t="inlineStr">
+        <is>
+          <t>Deferred with BW-006. The service spine's halls are 1.2 m wide and the whole width is the route, so the riser cluster, crate and hose this row asks for have no place outside it until BW-006 gives the spine its risers in a chase, its dado and its lighting.</t>
+        </is>
+      </c>
     </row>
     <row r="345">
       <c r="A345" s="2" t="inlineStr">
@@ -25719,10 +26031,14 @@
       </c>
       <c r="S345" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T345" s="2" t="inlineStr"/>
+          <t>deferred</t>
+        </is>
+      </c>
+      <c r="T345" s="2" t="inlineStr">
+        <is>
+          <t>Deferred with BW-006. The service spine's halls are 1.2 m wide and the whole width is the route, so the riser cluster, crate and hose this row asks for have no place outside it until BW-006 gives the spine its risers in a chase, its dado and its lighting.</t>
+        </is>
+      </c>
     </row>
     <row r="346">
       <c r="A346" s="2" t="inlineStr">
@@ -27653,10 +27969,14 @@
       </c>
       <c r="S370" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T370" s="2" t="inlineStr"/>
+          <t>deferred</t>
+        </is>
+      </c>
+      <c r="T370" s="2" t="inlineStr">
+        <is>
+          <t>Deferred. The clock needs its hold-E winding verb and a WorkOrders binding; the interaction carrier audit holds clock_prop's "Hold E" prompt as an open violation awaiting K2, so a new winding owner waits on that ruling.</t>
+        </is>
+      </c>
     </row>
     <row r="371">
       <c r="A371" s="2" t="inlineStr">
@@ -28311,10 +28631,14 @@
       </c>
       <c r="S379" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T379" s="2" t="inlineStr"/>
+          <t>rejected</t>
+        </is>
+      </c>
+      <c r="T379" s="2" t="inlineStr">
+        <is>
+          <t>Not a defect: V2's light switch family is a toggle by design (light_switch.md: a toggle collar and a porcelain-tipped TogglePivot), and both 4B plates are that family, so the closet switch matches the room switches.</t>
+        </is>
+      </c>
     </row>
     <row r="380">
       <c r="A380" s="2" t="inlineStr">
@@ -31773,10 +32097,14 @@
       </c>
       <c r="S426" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T426" s="2" t="inlineStr"/>
+          <t>deferred</t>
+        </is>
+      </c>
+      <c r="T426" s="2" t="inlineStr">
+        <is>
+          <t>Deferred: carrying the hall terrazzo and base to 5C's sill is a floor-coverage pass.</t>
+        </is>
+      </c>
     </row>
     <row r="427">
       <c r="A427" s="2" t="inlineStr">
@@ -32073,10 +32401,14 @@
       </c>
       <c r="S430" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T430" s="2" t="inlineStr"/>
+          <t>deferred</t>
+        </is>
+      </c>
+      <c r="T430" s="2" t="inlineStr">
+        <is>
+          <t>Deferred with BW-006. The service spine's halls are 1.2 m wide and the whole width is the route, so the riser cluster, crate and hose this row asks for have no place outside it until BW-006 gives the spine its risers in a chase, its dado and its lighting.</t>
+        </is>
+      </c>
     </row>
     <row r="431">
       <c r="A431" s="2" t="inlineStr">
@@ -32307,10 +32639,14 @@
       </c>
       <c r="S433" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T433" s="2" t="inlineStr"/>
+          <t>deferred</t>
+        </is>
+      </c>
+      <c r="T433" s="2" t="inlineStr">
+        <is>
+          <t>Deferred with BW-006. The service spine's halls are 1.2 m wide and the whole width is the route, so the riser cluster, crate and hose this row asks for have no place outside it until BW-006 gives the spine its risers in a chase, its dado and its lighting.</t>
+        </is>
+      </c>
     </row>
     <row r="434">
       <c r="A434" s="2" t="inlineStr">
@@ -32365,10 +32701,14 @@
       </c>
       <c r="S434" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T434" s="2" t="inlineStr"/>
+          <t>rejected</t>
+        </is>
+      </c>
+      <c r="T434" s="2" t="inlineStr">
+        <is>
+          <t>The peephole is the brass lens cylinder of door_prop.gd, and the white disc is the lamp's specular on brass, as BW-014 measured; not a defect. The wall joint goes with BW-006's spine finish.</t>
+        </is>
+      </c>
     </row>
     <row r="435">
       <c r="A435" s="2" t="inlineStr">
@@ -32443,10 +32783,14 @@
       </c>
       <c r="S435" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T435" s="2" t="inlineStr"/>
+          <t>deferred</t>
+        </is>
+      </c>
+      <c r="T435" s="2" t="inlineStr">
+        <is>
+          <t>Deferred with BW-006. The service spine's halls are 1.2 m wide and the whole width is the route, so the riser cluster, crate and hose this row asks for have no place outside it until BW-006 gives the spine its risers in a chase, its dado and its lighting.</t>
+        </is>
+      </c>
     </row>
     <row r="436">
       <c r="A436" s="2" t="inlineStr">
@@ -33117,10 +33461,14 @@
       </c>
       <c r="S444" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T444" s="2" t="inlineStr"/>
+          <t>deferred</t>
+        </is>
+      </c>
+      <c r="T444" s="2" t="inlineStr">
+        <is>
+          <t>Deferred. Moving the plantable to the window moves four bound families with it: its native work-table fit and seated surface stock, and the counterweight lamp's installation and supply cord plan (task_lamp_installations, task_lamp_supply); the cord must be re-planned from a window-side outlet first.</t>
+        </is>
+      </c>
     </row>
     <row r="445">
       <c r="A445" s="2" t="inlineStr">
@@ -34971,10 +35319,14 @@
       </c>
       <c r="S469" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T469" s="2" t="inlineStr"/>
+          <t>deferred</t>
+        </is>
+      </c>
+      <c r="T469" s="2" t="inlineStr">
+        <is>
+          <t>Deferred for an owner restatement. The row's title asks for monitor-top electric evidence, but its construction (an ice card in the kitchen window, a zinc drip tray with a tide line) is icebox evidence, and this household's fridge is a FridgeMonitor in household_fridges.json; a monitor-top unit takes no ice. The icebox households already have their drip pans (slice 18).</t>
+        </is>
+      </c>
     </row>
     <row r="470">
       <c r="A470" s="2" t="inlineStr">
@@ -35037,10 +35389,14 @@
       </c>
       <c r="S470" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T470" s="2" t="inlineStr"/>
+          <t>deferred</t>
+        </is>
+      </c>
+      <c r="T470" s="2" t="inlineStr">
+        <is>
+          <t>Deferred. 5B's fridge contents are the larder copied from fridge_prop.gd's LARDER, which the household fridges family pins by SHA-256 (mechanism_sha256); batteries and film change the pinned mechanism source.</t>
+        </is>
+      </c>
     </row>
     <row r="471">
       <c r="A471" s="2" t="inlineStr">
@@ -37171,10 +37527,14 @@
       </c>
       <c r="S499" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T499" s="2" t="inlineStr"/>
+          <t>deferred</t>
+        </is>
+      </c>
+      <c r="T499" s="2" t="inlineStr">
+        <is>
+          <t>Deferred. The strip and the louvred box are ventilation-family registers, and that family's 23 registers are pinned as a set; BW-005 measured the branches as seated. Removing this one is a ventilation-family change.</t>
+        </is>
+      </c>
     </row>
     <row r="500">
       <c r="A500" s="2" t="inlineStr">
@@ -37631,10 +37991,14 @@
       </c>
       <c r="S505" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T505" s="2" t="inlineStr"/>
+          <t>deferred</t>
+        </is>
+      </c>
+      <c r="T505" s="2" t="inlineStr">
+        <is>
+          <t>Deferred with BW-006. The service spine's halls are 1.2 m wide and the whole width is the route, so the riser cluster, crate and hose this row asks for have no place outside it until BW-006 gives the spine its risers in a chase, its dado and its lighting.</t>
+        </is>
+      </c>
     </row>
     <row r="506">
       <c r="A506" s="2" t="inlineStr">
@@ -37865,10 +38229,14 @@
       </c>
       <c r="S508" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T508" s="2" t="inlineStr"/>
+          <t>deferred</t>
+        </is>
+      </c>
+      <c r="T508" s="2" t="inlineStr">
+        <is>
+          <t>Deferred with BW-006. The service spine's halls are 1.2 m wide and the whole width is the route, so the riser cluster, crate and hose this row asks for have no place outside it until BW-006 gives the spine its risers in a chase, its dado and its lighting.</t>
+        </is>
+      </c>
     </row>
     <row r="509">
       <c r="A509" s="2" t="inlineStr">
@@ -37943,10 +38311,14 @@
       </c>
       <c r="S509" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T509" s="2" t="inlineStr"/>
+          <t>deferred</t>
+        </is>
+      </c>
+      <c r="T509" s="2" t="inlineStr">
+        <is>
+          <t>Deferred with BW-006. The service spine's halls are 1.2 m wide and the whole width is the route, so the riser cluster, crate and hose this row asks for have no place outside it until BW-006 gives the spine its risers in a chase, its dado and its lighting.</t>
+        </is>
+      </c>
     </row>
     <row r="510">
       <c r="A510" s="2" t="inlineStr">
@@ -39097,10 +39469,14 @@
       </c>
       <c r="S524" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T524" s="2" t="inlineStr"/>
+          <t>deferred</t>
+        </is>
+      </c>
+      <c r="T524" s="2" t="inlineStr">
+        <is>
+          <t>Deferred: the mirror renders black without a reflection source in the bath, and the moon's dither through the glass is the sky shader behind the glazing; both are rendering passes.</t>
+        </is>
+      </c>
     </row>
     <row r="525">
       <c r="A525" s="2" t="inlineStr">
@@ -41025,10 +41401,14 @@
       </c>
       <c r="S550" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T550" s="2" t="inlineStr"/>
+          <t>deferred</t>
+        </is>
+      </c>
+      <c r="T550" s="2" t="inlineStr">
+        <is>
+          <t>Deferred for an owner restatement. The row's title asks for monitor-top electric evidence, but its construction (an ice card in the kitchen window, a zinc drip tray with a tide line) is icebox evidence, and this household's fridge is a FridgeMonitor in household_fridges.json; a monitor-top unit takes no ice. The icebox households already have their drip pans (slice 18).</t>
+        </is>
+      </c>
     </row>
     <row r="551">
       <c r="A551" s="2" t="inlineStr">
@@ -42329,10 +42709,14 @@
       </c>
       <c r="S568" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T568" s="2" t="inlineStr"/>
+          <t>deferred</t>
+        </is>
+      </c>
+      <c r="T568" s="2" t="inlineStr">
+        <is>
+          <t>Deferred. The roof decks are the sloped membrane with its authored falling field, and the domestic-object inspector seats feet on a flat level datum (inspect_domestic_objects_context.py), so roof objects need a sloped-deck support path first.</t>
+        </is>
+      </c>
     </row>
     <row r="569">
       <c r="A569" s="2" t="inlineStr">
@@ -42415,10 +42799,14 @@
       </c>
       <c r="S569" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T569" s="2" t="inlineStr"/>
+          <t>deferred</t>
+        </is>
+      </c>
+      <c r="T569" s="2" t="inlineStr">
+        <is>
+          <t>Deferred. The roof decks are the sloped membrane with its authored falling field, and the domestic-object inspector seats feet on a flat level datum (inspect_domestic_objects_context.py), so roof objects need a sloped-deck support path first.</t>
+        </is>
+      </c>
     </row>
     <row r="570">
       <c r="A570" s="2" t="inlineStr">
@@ -42477,10 +42865,14 @@
       </c>
       <c r="S570" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T570" s="2" t="inlineStr"/>
+          <t>deferred</t>
+        </is>
+      </c>
+      <c r="T570" s="2" t="inlineStr">
+        <is>
+          <t>Deferred. The roof decks are the sloped membrane with its authored falling field, and the domestic-object inspector seats feet on a flat level datum (inspect_domestic_objects_context.py), so roof objects need a sloped-deck support path first.</t>
+        </is>
+      </c>
     </row>
     <row r="571">
       <c r="A571" s="2" t="inlineStr">
@@ -42605,10 +42997,14 @@
       </c>
       <c r="S572" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T572" s="2" t="inlineStr"/>
+          <t>deferred</t>
+        </is>
+      </c>
+      <c r="T572" s="2" t="inlineStr">
+        <is>
+          <t>Deferred: the ventilator housings are the owner JSON's A06 item.</t>
+        </is>
+      </c>
     </row>
     <row r="573">
       <c r="A573" s="2" t="inlineStr">
@@ -42683,10 +43079,14 @@
       </c>
       <c r="S573" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T573" s="2" t="inlineStr"/>
+          <t>deferred</t>
+        </is>
+      </c>
+      <c r="T573" s="2" t="inlineStr">
+        <is>
+          <t>Deferred. The roof decks are the sloped membrane with its authored falling field, and the domestic-object inspector seats feet on a flat level datum (inspect_domestic_objects_context.py), so roof objects need a sloped-deck support path first.</t>
+        </is>
+      </c>
     </row>
     <row r="574">
       <c r="A574" s="2" t="inlineStr">
@@ -42745,10 +43145,14 @@
       </c>
       <c r="S574" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T574" s="2" t="inlineStr"/>
+          <t>deferred</t>
+        </is>
+      </c>
+      <c r="T574" s="2" t="inlineStr">
+        <is>
+          <t>Deferred. The roof decks are the sloped membrane with its authored falling field, and the domestic-object inspector seats feet on a flat level datum (inspect_domestic_objects_context.py), so roof objects need a sloped-deck support path first.</t>
+        </is>
+      </c>
     </row>
     <row r="575">
       <c r="A575" s="2" t="inlineStr">
@@ -42823,10 +43227,14 @@
       </c>
       <c r="S575" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T575" s="2" t="inlineStr"/>
+          <t>deferred</t>
+        </is>
+      </c>
+      <c r="T575" s="2" t="inlineStr">
+        <is>
+          <t>Deferred. The roof decks are the sloped membrane with its authored falling field, and the domestic-object inspector seats feet on a flat level datum (inspect_domestic_objects_context.py), so roof objects need a sloped-deck support path first.</t>
+        </is>
+      </c>
     </row>
     <row r="576">
       <c r="A576" s="2" t="inlineStr">
@@ -42885,10 +43293,14 @@
       </c>
       <c r="S576" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T576" s="2" t="inlineStr"/>
+          <t>deferred</t>
+        </is>
+      </c>
+      <c r="T576" s="2" t="inlineStr">
+        <is>
+          <t>Deferred: gated on the commensals ruling (C2), and on the roof support path.</t>
+        </is>
+      </c>
     </row>
     <row r="577">
       <c r="A577" s="2" t="inlineStr">
@@ -42963,10 +43375,14 @@
       </c>
       <c r="S577" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T577" s="2" t="inlineStr"/>
+          <t>deferred</t>
+        </is>
+      </c>
+      <c r="T577" s="2" t="inlineStr">
+        <is>
+          <t>Deferred. The roof decks are the sloped membrane with its authored falling field, and the domestic-object inspector seats feet on a flat level datum (inspect_domestic_objects_context.py), so roof objects need a sloped-deck support path first.</t>
+        </is>
+      </c>
     </row>
     <row r="578">
       <c r="A578" s="2" t="inlineStr">
@@ -43021,10 +43437,14 @@
       </c>
       <c r="S578" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T578" s="2" t="inlineStr"/>
+          <t>deferred</t>
+        </is>
+      </c>
+      <c r="T578" s="2" t="inlineStr">
+        <is>
+          <t>Deferred. The roof decks are the sloped membrane with its authored falling field, and the domestic-object inspector seats feet on a flat level datum (inspect_domestic_objects_context.py), so roof objects need a sloped-deck support path first.</t>
+        </is>
+      </c>
     </row>
     <row r="579">
       <c r="A579" s="2" t="inlineStr">
@@ -43099,10 +43519,14 @@
       </c>
       <c r="S579" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T579" s="2" t="inlineStr"/>
+          <t>deferred</t>
+        </is>
+      </c>
+      <c r="T579" s="2" t="inlineStr">
+        <is>
+          <t>Deferred. The roof decks are the sloped membrane with its authored falling field, and the domestic-object inspector seats feet on a flat level datum (inspect_domestic_objects_context.py), so roof objects need a sloped-deck support path first.</t>
+        </is>
+      </c>
     </row>
     <row r="580">
       <c r="A580" s="2" t="inlineStr">
@@ -43157,10 +43581,14 @@
       </c>
       <c r="S580" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T580" s="2" t="inlineStr"/>
+          <t>deferred</t>
+        </is>
+      </c>
+      <c r="T580" s="2" t="inlineStr">
+        <is>
+          <t>Deferred. The roof decks are the sloped membrane with its authored falling field, and the domestic-object inspector seats feet on a flat level datum (inspect_domestic_objects_context.py), so roof objects need a sloped-deck support path first.</t>
+        </is>
+      </c>
     </row>
     <row r="581">
       <c r="A581" s="2" t="inlineStr">
@@ -43219,10 +43647,14 @@
       </c>
       <c r="S581" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T581" s="2" t="inlineStr"/>
+          <t>deferred</t>
+        </is>
+      </c>
+      <c r="T581" s="2" t="inlineStr">
+        <is>
+          <t>Deferred: the chimney's bonded joints and stone coping are a roof plant pass (chimney_crown.md).</t>
+        </is>
+      </c>
     </row>
     <row r="582">
       <c r="A582" s="2" t="inlineStr">
@@ -43297,10 +43729,14 @@
       </c>
       <c r="S582" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T582" s="2" t="inlineStr"/>
+          <t>deferred</t>
+        </is>
+      </c>
+      <c r="T582" s="2" t="inlineStr">
+        <is>
+          <t>Deferred. The roof decks are the sloped membrane with its authored falling field, and the domestic-object inspector seats feet on a flat level datum (inspect_domestic_objects_context.py), so roof objects need a sloped-deck support path first.</t>
+        </is>
+      </c>
     </row>
     <row r="583">
       <c r="A583" s="2" t="inlineStr">
@@ -43355,10 +43791,14 @@
       </c>
       <c r="S583" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T583" s="2" t="inlineStr"/>
+          <t>deferred</t>
+        </is>
+      </c>
+      <c r="T583" s="2" t="inlineStr">
+        <is>
+          <t>Deferred. The roof decks are the sloped membrane with its authored falling field, and the domestic-object inspector seats feet on a flat level datum (inspect_domestic_objects_context.py), so roof objects need a sloped-deck support path first.</t>
+        </is>
+      </c>
     </row>
     <row r="584">
       <c r="A584" s="2" t="inlineStr">
@@ -43433,10 +43873,14 @@
       </c>
       <c r="S584" s="2" t="inlineStr">
         <is>
-          <t>proposed</t>
-        </is>
-      </c>
-      <c r="T584" s="2" t="inlineStr"/>
+          <t>deferred</t>
+        </is>
+      </c>
+      <c r="T584" s="2" t="inlineStr">
+        <is>
+          <t>Deferred. The roof decks are the sloped membrane with its authored falling field, and the domestic-object inspector seats feet on a flat level datum (inspect_domestic_objects_context.py), so roof objects need a sloped-deck support path first.</t>
+        </is>
+      </c>
     </row>
     <row r="585">
       <c r="A585" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Dossier slice 83: a sconce on every landing lobby, cage bulbs over the boiler room's firing aisle
INERT: no ledger status changes. F04_LANDING-003 and B1_BOILER_ROOM-003 verified.

- A sconce_globe_back050 on the south core wall of each landing lobby,
  F02-F06, on the floor's west-hall circuit (BW-017's "one per landing").
- Two cage_bulb_rise160 over the B1 firing aisle, each under an F01 floor
  with collision and clear of the steam header, on a new boiler-room circuit;
  completion lighting accepts the cage_bulb kind.
- Fixed lighting rebuilt (218 instances, glb byte-identical). Judged with the
  hand lamp off at 20:00 before and after: the lift plate, the 4B transom and
  the firing door read. The packet's probe takes lamp-off frames.
- implementation/followups4 records the follow-ups' own verification (22 of 23
  runs exit 0; ApartmentBatch's 204 failures carry no new label class).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/art/reviews/v2_environment_design_20261008/change_register.xlsx
+++ b/art/reviews/v2_environment_design_20261008/change_register.xlsx
@@ -1309,12 +1309,12 @@
       </c>
       <c r="S12" s="2" t="inlineStr">
         <is>
-          <t>deferred</t>
+          <t>verified</t>
         </is>
       </c>
       <c r="T12" s="2" t="inlineStr">
         <is>
-          <t>Deferred. Corrected reason (follow-ups; the earlier note deferred it to a 16/16 lighting budget): on desktop there is no 16/16 budget to exceed. The V2 runtime root composes LightRig, whose per-frame light budget has been off on desktop since 2026-08-08 (light_rig.gd; only shadow casters stay capped, at 32), and BW-017's twelve hall domes already rely on that; mobile keeps its caps (ACTIVE_N_MOBILE 12, SHADOW_N_MOBILE 4). The open work is the two cage bulbs over the firing aisle from the fixed-lighting family's cage_bulb_rise assemblies, rebuilt into that family as slice 3 did, then its fabrication module and a capture of the firing aisle.</t>
+          <t>Two cage_bulb_rise160 over the firing aisle at x 10.6, z -1.6 and 0.6 (anchors B1_BOILER_ROOM_LT_A/B, each under an F01 floor with collision, the cage's lowest point about 2.27 m, clear of the 2.13 m fire-door head and of the steam header at z -0.55 and its hangers), on a new B1_BOILER_ROOM circuit whose switch follows the B1 convention on the south wall (10.15, 1.12, -5.4); completion lighting gains the cage_bulb kind. The 16/16 budget the row names does not exist on desktop (light_rig.gd). Verified at 34b4c7c8 (implementation/slice83): fixed lighting 0 failures (ceiling contacts by ray, the door-head clearance, the circuit), switch model, boiler route, basement route and coal delivery 0 failures, wet cloth 0 failures. With the hand lamp off the firing-door station reads the firing door, gauge glass and controls (images/B1_firing_door_before_lampoff against _after_lampoff). The switch is about 5 m from the fire door, by the B1 convention; no route test walks to it.</t>
         </is>
       </c>
     </row>
@@ -3356,7 +3356,7 @@
       </c>
       <c r="T41" s="2" t="inlineStr">
         <is>
-          <t>Twelve flush domes (flush_dome_rise100 at 2.9 m) on the west and east public halls of F02-F06 (two on the 6.1 m halls of F05/F06), each hall on a landlord's switch beside the stair end or the unit door jamb; blockout anchors, room_lighting records, fixed_lighting plan instances and mirror; family rebuilt. Landings and cores (open stair voids) still have no practical: they need a wall sconce placed against the stair geometry and stay open. Verified at 4e589c0c: upper lighting 9,257 checks, 0 failures (the first run's four F05_C standing-capsule failures cleared with the 5C wardrobe and pigment-table moves); the hall sweep overviews show the domes lit and the switches on the wainscot (implementation/slice3b; the 4e589c0c upper-lighting receipt is implementation/slice4/receipts/upper_lighting.log.receipt.json).</t>
+          <t>Twelve flush domes (flush_dome_rise100 at 2.9 m) on the west and east public halls of F02-F06 (two on the 6.1 m halls of F05/F06), each hall on a landlord's switch beside the stair end or the unit door jamb; blockout anchors, room_lighting records, fixed_lighting plan instances and mirror; family rebuilt. Landings and cores (open stair voids) had no practical here; slice 83 puts a sconce on each landing lobby's south core wall, F02-F06 (F04_LANDING-003). Verified at 4e589c0c: upper lighting 9,257 checks, 0 failures (the first run's four F05_C standing-capsule failures cleared with the 5C wardrobe and pigment-table moves); the hall sweep overviews show the domes lit and the switches on the wainscot (implementation/slice3b; the 4e589c0c upper-lighting receipt is implementation/slice4/receipts/upper_lighting.log.receipt.json).</t>
         </is>
       </c>
     </row>
@@ -24831,12 +24831,12 @@
       </c>
       <c r="S329" s="2" t="inlineStr">
         <is>
-          <t>deferred</t>
+          <t>verified</t>
         </is>
       </c>
       <c r="T329" s="2" t="inlineStr">
         <is>
-          <t>The landing has no ceiling (stair void); a sconce on the core wall is the remaining item after BW-017's hall domes.</t>
+          <t>A sconce_globe_back050 on the south core wall of the F04 lift lobby (anchor F04_LANDING_LT_SCONCE [-1.5, 2.0, -3.73], yaw 0: the wall face plus the 50 mm stand-off), on F04_WEST_HALL's circuit (BW-017: switched with the floor); the same sconce stands on the F02, F03, F05 and F06 landings, BW-017's 'one per landing'. Verified at 34b4c7c8 (implementation/slice83): fixed lighting 218 actors, 6,438 checks, 0 failures (each landing sconce's two wall contacts by ray, its envelope clear of the lift front and core wall, its circuit); upper lighting 9,677 checks, 0 failures; household state 210 controls; the elevator, vertical, first-upper-hall, golden-repair and resident-key routes, which walk the lobby, 0 failures. With the hand lamp off at 20:00 the landing station reads the lift plate (images/F04_landing_liftplate_before_lampoff against _after_lampoff) and the 4B transom, which BW-017's hall dome already lit.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Evidence and register statuses for dossier slices 84 to 86
INERT: no ledger status changes. Register 380 verified / 87 implemented /
101 deferred / 16 rejected (F03-F06_SERVICE_HALL-001 verified).

implementation/slice84, slice85 and switches: receipts, probe frames before
and after with the hand lamp on and off, the switch census before the passes
and after each, the pass 3 suites and 1D's bell capture, and the static
replica's per-plate clearance table (sources/switch_replica, run at the
tip's data: 144 flush, at least 4.0 mm clear). Slice 85's runs at
ebe9503b show its one M11B lifecycle failure predates the slice. The README
records how the follow-ups and slices 83 to 86 were squashed.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/art/reviews/v2_environment_design_20261008/change_register.xlsx
+++ b/art/reviews/v2_environment_design_20261008/change_register.xlsx
@@ -20301,12 +20301,12 @@
       </c>
       <c r="S270" s="2" t="inlineStr">
         <is>
-          <t>deferred</t>
+          <t>verified</t>
         </is>
       </c>
       <c r="T270" s="2" t="inlineStr">
         <is>
-          <t>Deferred, no longer on BW-006's chase. Corrected reason (follow-ups; the earlier note said 1.2 m and deferred the row with BW-006): F03_SERVICE_HALL is 2.4 m wide (x 7.1 to 9.5 in orison_v2_blockout.json), twice the 1.2 m of F01's and F02's halls, and its purpose names bypass and inspection clearance around continuous risers. The risers (HEAT_STACK, TELEPHONE_MESSAGE_RISER, ELECTRICAL_SERVICE_RISER) stand in the hall's east half at x 8.45 to 9.3, z 0.3 to 1.15, so beside the cluster the free floor is about 1.35 m, which is the bypass itself; the spare width outside a 1.2 m route is along the rest of the east half, not against the cluster as the row places the crate and hose. The marked pipes can go on the risers. Whether the east half is clear floor is not yet measured: a node probe of the hall at the tip comes first, and the new forms need their own family glb, since surface_stock.glb is 1.72 MiB under GitHub's 100 MiB limit.</t>
+          <t>Maintenance evidence on the F03 service spine, outside the route: a painted band round each riser at 1.55 m in its service colour (heat ochre, telephone green, electric sky) with a blank kraft tag on a brass wire (no lettering, a deviation from the row's Label3D tags), a brass drain cock low on the heat stack, a slatted crate (a copy of 3B_partscrate) in the dead-end pocket south of the cluster and a hose coiled in five turns on an iron bracket on the east wall beside it (domestic objects risermarks and hosecoil); chalk on the stack, a drip ring under the cock and a boot scuff where the super stands (positional wear). Every riser fitting stands under 0.08 m proud, so the 1.28 m bypass west of the cluster keeps the 1.2 m route. Verified at 9535800b (implementation/slice85): the domestic-objects fabrication module 10,218 checks with every new support seated on a riser or wall face by ray (its one failure, the harness finding no clear camera station for F03's hose in the 0.98 m pocket, is the B1_rinse_taps class); the node probe's route boxes hold only the shell before and after, and the objects only in the cluster, east-half and pocket boxes; the vertical route walks the F03-F06 halls past them (124 waypoints, 0 failures; the F04-F06 halls walked for the first time); blockout, ConnectedWorld and the apartment batch's labels unchanged. The threshold view from the crossing shows the marked pipes and the clear bypass (images/F03_TH, F03_POCKET; lamp-off frames record the hall's darkness).</t>
         </is>
       </c>
     </row>
@@ -25949,12 +25949,12 @@
       </c>
       <c r="S344" s="2" t="inlineStr">
         <is>
-          <t>deferred</t>
+          <t>verified</t>
         </is>
       </c>
       <c r="T344" s="2" t="inlineStr">
         <is>
-          <t>Deferred, no longer on BW-006's chase. Corrected reason (follow-ups; the earlier note said 1.2 m and deferred the row with BW-006): F04_SERVICE_HALL is 2.4 m wide (x 7.1 to 9.5 in orison_v2_blockout.json), twice the 1.2 m of F01's and F02's halls. The risers (HEAT_STACK, TELEPHONE_MESSAGE_RISER, ELECTRICAL_SERVICE_RISER) stand in the hall's east half at x 8.45 to 9.3, z 0.3 to 1.15, so beside the cluster the free floor is about 1.35 m, which is the bypass itself; the spare width outside a 1.2 m route is along the rest of the east half, not against the cluster as the row places the crate and hose. The marked pipes can go on the risers. Whether the east half is clear floor is not yet measured: a node probe of the hall at the tip comes first, and the new forms need their own family glb, since surface_stock.glb is 1.72 MiB under GitHub's 100 MiB limit.</t>
+          <t>Maintenance evidence on the F04 service spine, outside the route: a painted band round each riser at 1.55 m in its service colour (heat ochre, telephone green, electric sky) with a blank kraft tag on a brass wire (no lettering, a deviation from the row's Label3D tags), a brass drain cock low on the heat stack, a slatted crate (a copy of 3B_partscrate) in the dead-end pocket south of the cluster and a hose coiled in five turns on an iron bracket on the east wall beside it (domestic objects risermarks and hosecoil); chalk on the stack, a drip ring under the cock and a boot scuff where the super stands (positional wear). Every riser fitting stands under 0.08 m proud, so the 1.28 m bypass west of the cluster keeps the 1.2 m route. Verified at 9535800b (implementation/slice85): the domestic-objects fabrication module 10,218 checks with every new support seated on a riser or wall face by ray (its one failure, the harness finding no clear camera station for F03's hose in the 0.98 m pocket, is the B1_rinse_taps class); the node probe's route boxes hold only the shell before and after, and the objects only in the cluster, east-half and pocket boxes; the vertical route walks the F03-F06 halls past them (124 waypoints, 0 failures; the F04-F06 halls walked for the first time); blockout, ConnectedWorld and the apartment batch's labels unchanged. The threshold view from the crossing shows the marked pipes and the clear bypass (images/F04_TH, F04_POCKET; lamp-off frames record the hall's darkness).</t>
         </is>
       </c>
     </row>
@@ -32401,12 +32401,12 @@
       </c>
       <c r="S430" s="2" t="inlineStr">
         <is>
-          <t>deferred</t>
+          <t>verified</t>
         </is>
       </c>
       <c r="T430" s="2" t="inlineStr">
         <is>
-          <t>Deferred, no longer on BW-006's chase. Corrected reason (follow-ups; the earlier note said 1.2 m and deferred the row with BW-006): F05_SERVICE_HALL is 2.4 m wide (x 7.1 to 9.5 in orison_v2_blockout.json), twice the 1.2 m of F01's and F02's halls. The risers (HEAT_STACK, TELEPHONE_MESSAGE_RISER, ELECTRICAL_SERVICE_RISER) stand in the hall's east half at x 8.45 to 9.3, z 0.3 to 1.15, so beside the cluster the free floor is about 1.35 m, which is the bypass itself; the spare width outside a 1.2 m route is along the rest of the east half, not against the cluster as the row places the crate and hose. The marked pipes can go on the risers. Whether the east half is clear floor is not yet measured: a node probe of the hall at the tip comes first, and the new forms need their own family glb, since surface_stock.glb is 1.72 MiB under GitHub's 100 MiB limit.</t>
+          <t>Maintenance evidence on the F05 service spine, outside the route: a painted band round each riser at 1.55 m in its service colour (heat ochre, telephone green, electric sky) with a blank kraft tag on a brass wire (no lettering, a deviation from the row's Label3D tags), a brass drain cock low on the heat stack, a slatted crate (a copy of 3B_partscrate) in the dead-end pocket south of the cluster and a hose coiled in five turns on an iron bracket on the east wall beside it (domestic objects risermarks and hosecoil); chalk on the stack, a drip ring under the cock and a boot scuff where the super stands (positional wear). Every riser fitting stands under 0.08 m proud, so the 1.28 m bypass west of the cluster keeps the 1.2 m route. Verified at 9535800b (implementation/slice85): the domestic-objects fabrication module 10,218 checks with every new support seated on a riser or wall face by ray (its one failure, the harness finding no clear camera station for F03's hose in the 0.98 m pocket, is the B1_rinse_taps class); the node probe's route boxes hold only the shell before and after, and the objects only in the cluster, east-half and pocket boxes; the vertical route walks the F03-F06 halls past them (124 waypoints, 0 failures; the F04-F06 halls walked for the first time); blockout, ConnectedWorld and the apartment batch's labels unchanged. The threshold view from the crossing shows the marked pipes and the clear bypass (images/F05_TH, F05_POCKET; lamp-off frames record the hall's darkness).</t>
         </is>
       </c>
     </row>
@@ -37991,12 +37991,12 @@
       </c>
       <c r="S505" s="2" t="inlineStr">
         <is>
-          <t>deferred</t>
+          <t>verified</t>
         </is>
       </c>
       <c r="T505" s="2" t="inlineStr">
         <is>
-          <t>Deferred, no longer on BW-006's chase. Corrected reason (follow-ups; the earlier note said 1.2 m and deferred the row with BW-006): F06_SERVICE_HALL is 2.4 m wide (x 7.1 to 9.5 in orison_v2_blockout.json), twice the 1.2 m of F01's and F02's halls. The risers (HEAT_STACK, TELEPHONE_MESSAGE_RISER, ELECTRICAL_SERVICE_RISER) stand in the hall's east half at x 8.45 to 9.3, z 0.3 to 1.15, so beside the cluster the free floor is about 1.35 m, which is the bypass itself; the spare width outside a 1.2 m route is along the rest of the east half, not against the cluster as the row places the crate and hose. The marked pipes can go on the risers. Whether the east half is clear floor is not yet measured: a node probe of the hall at the tip comes first, and the new forms need their own family glb, since surface_stock.glb is 1.72 MiB under GitHub's 100 MiB limit.</t>
+          <t>Maintenance evidence on the F06 service spine, outside the route: a painted band round each riser at 1.55 m in its service colour (heat ochre, telephone green, electric sky) with a blank kraft tag on a brass wire (no lettering, a deviation from the row's Label3D tags), a brass drain cock low on the heat stack, a slatted crate (a copy of 3B_partscrate) in the dead-end pocket south of the cluster and a hose coiled in five turns on an iron bracket on the east wall beside it (domestic objects risermarks and hosecoil); chalk on the stack, a drip ring under the cock and a boot scuff where the super stands (positional wear). Every riser fitting stands under 0.08 m proud, so the 1.28 m bypass west of the cluster keeps the 1.2 m route. Verified at 9535800b (implementation/slice85): the domestic-objects fabrication module 10,218 checks with every new support seated on a riser or wall face by ray (its one failure, the harness finding no clear camera station for F03's hose in the 0.98 m pocket, is the B1_rinse_taps class); the node probe's route boxes hold only the shell before and after, and the objects only in the cluster, east-half and pocket boxes; the vertical route walks the F03-F06 halls past them (124 waypoints, 0 failures; the F04-F06 halls walked for the first time); blockout, ConnectedWorld and the apartment batch's labels unchanged. The threshold view from the crossing shows the marked pipes and the clear bypass (images/F06_TH, F06_POCKET; lamp-off frames record the hall's darkness).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Otis & Son's show globes throw their colour onto the terrazzo
INERT: no ledger status changes. CITY_SHOP_OTIS_SON-001 verified at the
owner's go-ahead (register 381 verified / 87 implemented / 100 deferred /
16 rejected).

A tinted spot lamp sits inside each of the four carboy fills, aimed out
through the shopfront and down onto the aisle terrazzo about 1.5 m from the
glass, shadow-free; each fill glows by an emissive override, leaving the
shipping mesh materials untouched. The carboy test checks the four lamps:
inside their carboys, aimed out and down, each its own colour, landing on
the aisle floor. It also takes the row's acceptance frame from the
pavement, hand lamp off.

Verified on main 3fcd7fc2 (implementation/otis_lamp): the carboy test
passes 470 checks with 0 failures, including the 19 new ones; main alone
passes its 451.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/art/reviews/v2_environment_design_20261008/change_register.xlsx
+++ b/art/reviews/v2_environment_design_20261008/change_register.xlsx
@@ -6837,12 +6837,12 @@
       </c>
       <c r="S92" s="2" t="inlineStr">
         <is>
-          <t>deferred</t>
+          <t>verified</t>
         </is>
       </c>
       <c r="T92" s="2" t="inlineStr">
         <is>
-          <t>Deferred. Corrected reason (follow-ups; the earlier note deferred it to a lighting-budget decision): on desktop there is no 16/16 budget to exceed. The V2 runtime root composes LightRig, whose per-frame light budget has been off on desktop since 2026-08-08 (light_rig.gd; only shadow casters stay capped, at 32), and BW-017's twelve hall domes already rely on that; mobile keeps its caps (ACTIVE_N_MOBILE 12, SHADOW_N_MOBILE 4). The open work is the practical itself, and it is more than a lamp: orison_v2_druggist_carboys.gd turns shadow casting off on the carboy glass, so the glass throws no coloured light of its own; the colour on the terrazzo must come from a tinted light (or a projector) behind the carboys, judged at the pavement-through-glass station.</t>
+          <t>Verified at the owner's go-ahead (2026-10-15): the show globes burn as a druggist's window did. orison_v2_druggist_carboys.gd sets a tinted spot lamp inside each of the four carboy fills (teal, red, green, ochre), aimed out through the shopfront and down onto the aisle terrazzo about 1.5 m from the glass, shadow-free, and gives each fill an emissive override so the globes read as backlit; the shipping mesh materials are untouched. Evidence implementation/otis_lamp at e326950a: OrisonV2DruggistCarboysTest 470 checks, 0 failures, including 19 new show-globe checks (four lamps, inside their carboys, aimed out and down, each its own colour, landing on the aisle floor). The acceptance station, the pavement through the glass with the hand lamp off, shows the four colours on the terrazzo (images/pavement_through_glass).</t>
         </is>
       </c>
     </row>

</xml_diff>